<commit_message>
chore(assets): reserve player skill effect assets in art list
</commit_message>
<xml_diff>
--- a/outputs/01a0bf14-7f85-7282-bb8d-672064556a58/美术资产清单.xlsx
+++ b/outputs/01a0bf14-7f85-7282-bb8d-672064556a58/美术资产清单.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="美术资产清单" sheetId="1" r:id="R35c90178587741f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="源文件盘点" sheetId="2" r:id="Rd8d76a28c5cb4bff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="美术资产清单" sheetId="1" r:id="Ra513a2f0424f4cd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="源文件盘点" sheetId="2" r:id="R5db7b97349564186"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VisualAssets" displayName="VisualAssets" ref="A5:I48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VisualAssets" displayName="VisualAssets" ref="A5:I72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="分类"/>
@@ -348,7 +348,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>范围：当前网页原型及工作区源素材；中国象棋七类按敌我分列，未出现的棋种标为未实现。</x:v>
+        <x:v>范围：当前网页原型及工作区源素材；传统棋子按敌我分列，技能效果只预留己方，敌方按被动单位处理。</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -361,7 +361,7 @@
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>共 43 项视觉元素；传统棋子 14 款（标准双方各 16 枚），另有项目转职 2 款；旧目录源图片 1 个。</x:v>
+        <x:v>共 67 项视觉元素；传统棋子 14 款，项目转职 2 款；己方技能效果预留 24 项；旧目录源图片 1 个。</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -1055,28 +1055,28 @@
         <x:v>A-023</x:v>
       </x:c>
       <x:c r="B28" s="8" t="str">
-        <x:v>操作标记</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C28" s="8" t="str">
-        <x:v>当前选中棋位</x:v>
+        <x:v>全体｜击杀成长反馈</x:v>
       </x:c>
       <x:c r="D28" s="8" t="str">
-        <x:v>1种</x:v>
+        <x:v>9棋种通用</x:v>
       </x:c>
       <x:c r="E28" s="8" t="str">
-        <x:v>选棋后标记起点</x:v>
+        <x:v>己方棋子击杀后 Lv、SP 与击杀数增加</x:v>
       </x:c>
       <x:c r="F28" s="8" t="str">
-        <x:v>黄色半透明圆点</x:v>
+        <x:v>仅数值文字刷新；无独立特效资产</x:v>
       </x:c>
       <x:c r="G28" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H28" s="8" t="str">
-        <x:v>web/js/app.js:33-34</x:v>
+        <x:v>web/js/rules.js:38; web/js/app.js:37-40</x:v>
       </x:c>
       <x:c r="I28" s="8" t="str">
-        <x:v>需与其他标记可区分</x:v>
+        <x:v>建议包含棋子归属、等级提升和 SP 获得反馈</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="32" customHeight="1">
@@ -1084,28 +1084,28 @@
         <x:v>A-024</x:v>
       </x:c>
       <x:c r="B29" s="8" t="str">
-        <x:v>操作标记</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C29" s="8" t="str">
-        <x:v>合法移动落点</x:v>
+        <x:v>全体｜强健升级</x:v>
       </x:c>
       <x:c r="D29" s="8" t="str">
-        <x:v>1种</x:v>
+        <x:v>9棋种通用</x:v>
       </x:c>
       <x:c r="E29" s="8" t="str">
-        <x:v>移动选择</x:v>
+        <x:v>己方存活棋子当前／最大 HP +1</x:v>
       </x:c>
       <x:c r="F29" s="8" t="str">
-        <x:v>蓝色半透明圆点</x:v>
+        <x:v>仅按钮和 HP 数值刷新</x:v>
       </x:c>
       <x:c r="G29" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H29" s="8" t="str">
-        <x:v>web/js/app.js:33-34</x:v>
+        <x:v>web/js/app.js:42; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I29" s="8" t="str">
-        <x:v>需兼顾窄屏识别</x:v>
+        <x:v>帅、仕、相、马、车、炮、兵、弓兵、枪兵共用；仕／相规则仍 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="32" customHeight="1">
@@ -1113,28 +1113,28 @@
         <x:v>A-025</x:v>
       </x:c>
       <x:c r="B30" s="8" t="str">
-        <x:v>操作标记</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C30" s="8" t="str">
-        <x:v>攻击与冲击目标</x:v>
+        <x:v>帅｜专属技能效果预留</x:v>
       </x:c>
       <x:c r="D30" s="8" t="str">
-        <x:v>1种</x:v>
+        <x:v>1槽</x:v>
       </x:c>
       <x:c r="E30" s="8" t="str">
-        <x:v>攻击或车冲击</x:v>
+        <x:v>己方帅未来专属技能</x:v>
       </x:c>
       <x:c r="F30" s="8" t="str">
-        <x:v>红色半透明圆点</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="G30" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>预留（规则TBD）</x:v>
       </x:c>
       <x:c r="H30" s="8" t="str">
-        <x:v>web/js/app.js:33-34</x:v>
+        <x:v>用户要求预留所有己方棋子技能效果</x:v>
       </x:c>
       <x:c r="I30" s="8" t="str">
-        <x:v>需与移动落点可区分</x:v>
+        <x:v>当前只有通用强健；技能名称、触发和表现 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="32" customHeight="1">
@@ -1142,28 +1142,28 @@
         <x:v>A-026</x:v>
       </x:c>
       <x:c r="B31" s="8" t="str">
-        <x:v>操作标记</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C31" s="8" t="str">
-        <x:v>方向攻击范围</x:v>
+        <x:v>仕｜专属技能效果预留</x:v>
       </x:c>
       <x:c r="D31" s="8" t="str">
-        <x:v>1种</x:v>
+        <x:v>1槽</x:v>
       </x:c>
       <x:c r="E31" s="8" t="str">
-        <x:v>弓／枪四向预览</x:v>
+        <x:v>己方仕未来专属技能</x:v>
       </x:c>
       <x:c r="F31" s="8" t="str">
-        <x:v>黄色路径圆点</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="G31" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>预留（规则TBD）</x:v>
       </x:c>
       <x:c r="H31" s="8" t="str">
-        <x:v>web/js/app.js:59</x:v>
+        <x:v>用户要求预留所有己方棋子技能效果</x:v>
       </x:c>
       <x:c r="I31" s="8" t="str">
-        <x:v>正式范围表现 TBD</x:v>
+        <x:v>己方仕尚未进入规则；技能名称、触发和表现 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="32" customHeight="1">
@@ -1171,28 +1171,28 @@
         <x:v>A-027</x:v>
       </x:c>
       <x:c r="B32" s="8" t="str">
-        <x:v>操作标记</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C32" s="8" t="str">
-        <x:v>炮击路径与炮架</x:v>
+        <x:v>相｜专属技能效果预留</x:v>
       </x:c>
       <x:c r="D32" s="8" t="str">
-        <x:v>2种</x:v>
+        <x:v>1槽</x:v>
       </x:c>
       <x:c r="E32" s="8" t="str">
-        <x:v>炮击预览</x:v>
+        <x:v>己方相未来专属技能</x:v>
       </x:c>
       <x:c r="F32" s="8" t="str">
-        <x:v>黄色路径点＋紫色炮架点</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="G32" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>预留（规则TBD）</x:v>
       </x:c>
       <x:c r="H32" s="8" t="str">
-        <x:v>web/js/app.js:34</x:v>
+        <x:v>用户要求预留所有己方棋子技能效果</x:v>
       </x:c>
       <x:c r="I32" s="8" t="str">
-        <x:v>必须辨识炮架与主目标</x:v>
+        <x:v>己方相尚未进入规则；技能名称、触发和表现 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="32" customHeight="1">
@@ -1200,28 +1200,28 @@
         <x:v>A-028</x:v>
       </x:c>
       <x:c r="B33" s="8" t="str">
-        <x:v>操作标记</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C33" s="8" t="str">
-        <x:v>炮主目标</x:v>
+        <x:v>马｜专属技能效果预留</x:v>
       </x:c>
       <x:c r="D33" s="8" t="str">
-        <x:v>1种</x:v>
+        <x:v>1槽</x:v>
       </x:c>
       <x:c r="E33" s="8" t="str">
-        <x:v>炮击预览</x:v>
+        <x:v>己方马未来专属技能</x:v>
       </x:c>
       <x:c r="F33" s="8" t="str">
-        <x:v>红色目标点</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="G33" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>预留（规则TBD）</x:v>
       </x:c>
       <x:c r="H33" s="8" t="str">
-        <x:v>web/js/app.js:34</x:v>
+        <x:v>docs/us/US-001-m0-player-skills.md:2.2</x:v>
       </x:c>
       <x:c r="I33" s="8" t="str">
-        <x:v>扩散格视觉表现 TBD</x:v>
+        <x:v>当前马只有基础走法和通用强健；专属技能 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="32" customHeight="1">
@@ -1229,28 +1229,28 @@
         <x:v>A-029</x:v>
       </x:c>
       <x:c r="B34" s="8" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C34" s="8" t="str">
-        <x:v>战斗背景与主布局</x:v>
+        <x:v>车｜疾行移动</x:v>
       </x:c>
       <x:c r="D34" s="8" t="str">
-        <x:v>桌面／窄屏</x:v>
+        <x:v>直线4方向</x:v>
       </x:c>
       <x:c r="E34" s="8" t="str">
-        <x:v>棋盘外背景与分区</x:v>
+        <x:v>执行独立普通移动</x:v>
       </x:c>
       <x:c r="F34" s="8" t="str">
-        <x:v>CSS 纯色与响应式布局</x:v>
+        <x:v>棋位圆点与瞬时位移；无移动特效资产</x:v>
       </x:c>
       <x:c r="G34" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H34" s="8" t="str">
-        <x:v>web/index.html:8-14</x:v>
+        <x:v>web/js/app.js:59,64; web/js/rules.js:31,43</x:v>
       </x:c>
       <x:c r="I34" s="8" t="str">
-        <x:v>正式背景、装饰 TBD</x:v>
+        <x:v>表现起点、路径、终点和剩余移动额度</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="32" customHeight="1">
@@ -1258,28 +1258,28 @@
         <x:v>A-030</x:v>
       </x:c>
       <x:c r="B35" s="8" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C35" s="8" t="str">
-        <x:v>顶部状态栏</x:v>
+        <x:v>车｜疾行升级</x:v>
       </x:c>
       <x:c r="D35" s="8" t="str">
-        <x:v>1套</x:v>
+        <x:v>1套／等级变化</x:v>
       </x:c>
       <x:c r="E35" s="8" t="str">
-        <x:v>波次、回合、HP、金币、击杀</x:v>
+        <x:v>普通移动距离 +1</x:v>
       </x:c>
       <x:c r="F35" s="8" t="str">
-        <x:v>CSS 卡片＋文字</x:v>
+        <x:v>仅技能按钮和距离数值刷新</x:v>
       </x:c>
       <x:c r="G35" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H35" s="8" t="str">
-        <x:v>web/index.html:11,23</x:v>
+        <x:v>web/js/app.js:50; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>图标需求 TBD</x:v>
+        <x:v>最高 7 格；升级反馈需区别于实际移动</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="32" customHeight="1">
@@ -1287,28 +1287,28 @@
         <x:v>A-031</x:v>
       </x:c>
       <x:c r="B36" s="8" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C36" s="8" t="str">
-        <x:v>我方单位列表与棋子徽记</x:v>
+        <x:v>车｜冲击</x:v>
       </x:c>
       <x:c r="D36" s="8" t="str">
-        <x:v>1套</x:v>
+        <x:v>直线4方向</x:v>
       </x:c>
       <x:c r="E36" s="8" t="str">
-        <x:v>选棋及单位状态</x:v>
+        <x:v>冲向空格或敌人</x:v>
       </x:c>
       <x:c r="F36" s="8" t="str">
-        <x:v>CSS 卡片＋汉字徽记</x:v>
+        <x:v>目标圆点和文字预览；无冲击特效资产</x:v>
       </x:c>
       <x:c r="G36" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H36" s="8" t="str">
-        <x:v>web/index.html:12,26; web/js/app.js:37</x:v>
+        <x:v>web/js/app.js:59,64; web/js/rules.js:42-46</x:v>
       </x:c>
       <x:c r="I36" s="8" t="str">
-        <x:v>沿用棋子识别系统</x:v>
+        <x:v>需覆盖空冲、接近点、击杀占位和未击杀停前格</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="32" customHeight="1">
@@ -1316,28 +1316,28 @@
         <x:v>A-032</x:v>
       </x:c>
       <x:c r="B37" s="8" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C37" s="8" t="str">
-        <x:v>当前棋子信息卡</x:v>
+        <x:v>车｜冲击延伸升级</x:v>
       </x:c>
       <x:c r="D37" s="8" t="str">
-        <x:v>1套</x:v>
+        <x:v>1套／等级变化</x:v>
       </x:c>
       <x:c r="E37" s="8" t="str">
-        <x:v>属性、AP、等级、SP</x:v>
+        <x:v>冲击距离 +1</x:v>
       </x:c>
       <x:c r="F37" s="8" t="str">
-        <x:v>CSS 信息卡＋文字</x:v>
+        <x:v>仅技能按钮和距离数值刷新</x:v>
       </x:c>
       <x:c r="G37" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H37" s="8" t="str">
-        <x:v>web/index.html:12,27</x:v>
+        <x:v>web/js/app.js:51; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I37" s="8" t="str">
-        <x:v>状态层级 TBD</x:v>
+        <x:v>最高 7 格；与疾行升级使用不同辨识</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="32" customHeight="1">
@@ -1345,28 +1345,28 @@
         <x:v>A-033</x:v>
       </x:c>
       <x:c r="B38" s="8" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C38" s="8" t="str">
-        <x:v>技能条目与禁用状态</x:v>
+        <x:v>车｜震退解锁</x:v>
       </x:c>
       <x:c r="D38" s="8" t="str">
         <x:v>1套</x:v>
       </x:c>
       <x:c r="E38" s="8" t="str">
-        <x:v>升级、转职、方向和扩散</x:v>
+        <x:v>花费 2 SP 解锁震退</x:v>
       </x:c>
       <x:c r="F38" s="8" t="str">
-        <x:v>CSS 按钮＋文字</x:v>
+        <x:v>仅按钮状态与文字刷新</x:v>
       </x:c>
       <x:c r="G38" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H38" s="8" t="str">
-        <x:v>web/index.html:13; web/js/app.js:42-56</x:v>
+        <x:v>web/js/app.js:52; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>各技能专属图标 TBD</x:v>
+        <x:v>表现永久解锁，不能误解为一次性攻击</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="32" customHeight="1">
@@ -1374,28 +1374,28 @@
         <x:v>A-034</x:v>
       </x:c>
       <x:c r="B39" s="8" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C39" s="8" t="str">
-        <x:v>方向与车模式按钮</x:v>
+        <x:v>车｜震退命中</x:v>
       </x:c>
       <x:c r="D39" s="8" t="str">
-        <x:v>2组</x:v>
+        <x:v>成功／受阻4态</x:v>
       </x:c>
       <x:c r="E39" s="8" t="str">
-        <x:v>弓枪四向；车移动／冲击</x:v>
+        <x:v>冲击命中存活目标后推 1 格</x:v>
       </x:c>
       <x:c r="F39" s="8" t="str">
-        <x:v>CSS 按钮＋选中描边</x:v>
+        <x:v>仅位置变化与文字结果</x:v>
       </x:c>
       <x:c r="G39" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H39" s="8" t="str">
-        <x:v>web/index.html:13; web/js/app.js:58</x:v>
+        <x:v>web/js/app.js:64; web/js/rules.js:42-46</x:v>
       </x:c>
       <x:c r="I39" s="8" t="str">
-        <x:v>交互态样式 TBD</x:v>
+        <x:v>区分成功、出界、宫界和占位受阻</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="32" customHeight="1">
@@ -1403,28 +1403,28 @@
         <x:v>A-035</x:v>
       </x:c>
       <x:c r="B40" s="8" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C40" s="8" t="str">
-        <x:v>敌方意图列表与序号</x:v>
+        <x:v>炮｜基础炮击</x:v>
       </x:c>
       <x:c r="D40" s="8" t="str">
-        <x:v>1套</x:v>
+        <x:v>横竖4方向</x:v>
       </x:c>
       <x:c r="E40" s="8" t="str">
-        <x:v>敌方行动顺序和状态</x:v>
+        <x:v>隔恰好一个炮架攻击单目标</x:v>
       </x:c>
       <x:c r="F40" s="8" t="str">
-        <x:v>CSS 圆序号＋文字</x:v>
+        <x:v>路径、炮架、目标圆点与文字预览</x:v>
       </x:c>
       <x:c r="G40" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H40" s="8" t="str">
-        <x:v>web/index.html:13; web/js/app.js:60</x:v>
+        <x:v>web/js/app.js:64; docs/us/US-001-cannon-fix.md:20-25</x:v>
       </x:c>
       <x:c r="I40" s="8" t="str">
-        <x:v>窄屏展开态已支持</x:v>
+        <x:v>需表现发射、越过炮架、命中和 2 点伤害</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="32" customHeight="1">
@@ -1432,28 +1432,28 @@
         <x:v>A-036</x:v>
       </x:c>
       <x:c r="B41" s="8" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C41" s="8" t="str">
-        <x:v>动作预览与受击警告</x:v>
+        <x:v>炮｜炮架充能／弹道</x:v>
       </x:c>
       <x:c r="D41" s="8" t="str">
-        <x:v>1套</x:v>
+        <x:v>敌友炮架2态</x:v>
       </x:c>
       <x:c r="E41" s="8" t="str">
-        <x:v>路径、伤害、友伤、威胁</x:v>
+        <x:v>炮击前识别唯一炮架</x:v>
       </x:c>
       <x:c r="F41" s="8" t="str">
-        <x:v>CSS 信息卡＋警告色</x:v>
+        <x:v>紫色炮架点＋黄色路径点</x:v>
       </x:c>
       <x:c r="G41" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H41" s="8" t="str">
-        <x:v>web/index.html:13; web/js/app.js:63</x:v>
+        <x:v>web/js/app.js:34,64</x:v>
       </x:c>
       <x:c r="I41" s="8" t="str">
-        <x:v>友军误伤须醒目</x:v>
+        <x:v>友军与敌军均可作炮架；不要表现为炮架受益</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="32" customHeight="1">
@@ -1461,28 +1461,28 @@
         <x:v>A-037</x:v>
       </x:c>
       <x:c r="B42" s="8" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C42" s="8" t="str">
-        <x:v>底部操作按钮</x:v>
+        <x:v>炮｜扩散解锁</x:v>
       </x:c>
       <x:c r="D42" s="8" t="str">
-        <x:v>4种</x:v>
+        <x:v>8方向变体</x:v>
       </x:c>
       <x:c r="E42" s="8" t="str">
-        <x:v>执行、取消、结束回合、暂停</x:v>
+        <x:v>逐个解锁目标邻格 N／NE／E／SE／S／SW／W／NW</x:v>
       </x:c>
       <x:c r="F42" s="8" t="str">
-        <x:v>CSS 按钮</x:v>
+        <x:v>仅技能按钮和扩散计数刷新</x:v>
       </x:c>
       <x:c r="G42" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H42" s="8" t="str">
-        <x:v>web/index.html:14,32</x:v>
+        <x:v>web/js/app.js:53-54; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I42" s="8" t="str">
-        <x:v>含禁用／悬停态</x:v>
+        <x:v>固定朝向、不随开炮方向旋转；每格 1 SP</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="32" customHeight="1">
@@ -1490,28 +1490,28 @@
         <x:v>A-038</x:v>
       </x:c>
       <x:c r="B43" s="8" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C43" s="8" t="str">
-        <x:v>结束回合确认弹窗</x:v>
+        <x:v>炮｜扩散命中</x:v>
       </x:c>
       <x:c r="D43" s="8" t="str">
-        <x:v>1套</x:v>
+        <x:v>主目标＋最多8邻格</x:v>
       </x:c>
       <x:c r="E43" s="8" t="str">
-        <x:v>提交敌方阶段前确认</x:v>
+        <x:v>炮击时对已解锁邻格同时造成伤害</x:v>
       </x:c>
       <x:c r="F43" s="8" t="str">
-        <x:v>CSS 遮罩＋对话框</x:v>
+        <x:v>预览列出命中；无范围爆炸特效资产</x:v>
       </x:c>
       <x:c r="G43" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H43" s="8" t="str">
-        <x:v>web/index.html:15,34</x:v>
+        <x:v>web/js/app.js:64; web/js/rules.js:45</x:v>
       </x:c>
       <x:c r="I43" s="8" t="str">
-        <x:v>正式插画需求 TBD</x:v>
+        <x:v>包含友伤和边界裁切；主目标与扩散命中需分层</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="32" customHeight="1">
@@ -1519,28 +1519,28 @@
         <x:v>A-039</x:v>
       </x:c>
       <x:c r="B44" s="8" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C44" s="8" t="str">
-        <x:v>暂停弹窗</x:v>
+        <x:v>兵｜连动升级</x:v>
       </x:c>
       <x:c r="D44" s="8" t="str">
-        <x:v>1套</x:v>
+        <x:v>1套／可重复</x:v>
       </x:c>
       <x:c r="E44" s="8" t="str">
-        <x:v>继续和重新开始</x:v>
+        <x:v>花费 2 SP，使下回合 AP 上限 +1</x:v>
       </x:c>
       <x:c r="F44" s="8" t="str">
-        <x:v>CSS 遮罩＋对话框</x:v>
+        <x:v>仅技能按钮和数值刷新</x:v>
       </x:c>
       <x:c r="G44" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H44" s="8" t="str">
-        <x:v>web/index.html:15,35</x:v>
+        <x:v>web/js/app.js:46; web/js/rules.js:19,53</x:v>
       </x:c>
       <x:c r="I44" s="8" t="str">
-        <x:v>正式插画需求 TBD</x:v>
+        <x:v>升级时与下回合实际生效时分别反馈</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="32" customHeight="1">
@@ -1548,28 +1548,28 @@
         <x:v>A-040</x:v>
       </x:c>
       <x:c r="B45" s="11" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C45" s="11" t="str">
-        <x:v>商店与马／炮商品卡</x:v>
+        <x:v>兵｜额外行动激活</x:v>
       </x:c>
       <x:c r="D45" s="11" t="str">
-        <x:v>1套＋2商品</x:v>
+        <x:v>1套／层数变化</x:v>
       </x:c>
       <x:c r="E45" s="11" t="str">
-        <x:v>首波结束后选购</x:v>
+        <x:v>连动在下一回合增加可用 AP</x:v>
       </x:c>
       <x:c r="F45" s="11" t="str">
-        <x:v>CSS 对话框＋文字商品卡</x:v>
+        <x:v>仅 AP 数字变化</x:v>
       </x:c>
       <x:c r="G45" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H45" s="11" t="str">
-        <x:v>web/index.html:15,36</x:v>
+        <x:v>web/js/rules.js:19</x:v>
       </x:c>
       <x:c r="I45" s="11" t="str">
-        <x:v>商品形象可复用棋子资产</x:v>
+        <x:v>需显示新增行动次数和已消耗层次</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="32" customHeight="1">
@@ -1577,28 +1577,28 @@
         <x:v>A-041</x:v>
       </x:c>
       <x:c r="B46" s="11" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C46" s="11" t="str">
-        <x:v>终局弹窗</x:v>
+        <x:v>兵｜转职弓兵</x:v>
       </x:c>
       <x:c r="D46" s="11" t="str">
-        <x:v>胜／阵亡／将死</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E46" s="11" t="str">
-        <x:v>最终结果</x:v>
+        <x:v>花费 2 SP，兵变为弓兵并获得攻击加成</x:v>
       </x:c>
       <x:c r="F46" s="11" t="str">
-        <x:v>CSS 对话框＋状态文字</x:v>
+        <x:v>棋子字样与属性瞬时变化</x:v>
       </x:c>
       <x:c r="G46" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H46" s="11" t="str">
-        <x:v>web/index.html:15,37</x:v>
+        <x:v>web/js/app.js:44; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I46" s="11" t="str">
-        <x:v>结果插画需求 TBD</x:v>
+        <x:v>保留原棋子身份、伤势和剩余 AP</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="32" customHeight="1">
@@ -1606,28 +1606,28 @@
         <x:v>A-042</x:v>
       </x:c>
       <x:c r="B47" s="11" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C47" s="11" t="str">
-        <x:v>短提示与危险提示</x:v>
+        <x:v>兵｜转职枪兵</x:v>
       </x:c>
       <x:c r="D47" s="11" t="str">
         <x:v>1套</x:v>
       </x:c>
       <x:c r="E47" s="11" t="str">
-        <x:v>购买、重开、操作失败</x:v>
+        <x:v>花费 2 SP，兵变为枪兵并获得 HP</x:v>
       </x:c>
       <x:c r="F47" s="11" t="str">
-        <x:v>CSS 横幅＋文字</x:v>
+        <x:v>棋子字样与属性瞬时变化</x:v>
       </x:c>
       <x:c r="G47" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H47" s="11" t="str">
-        <x:v>web/index.html:14,24; web/js/app.js:69</x:v>
+        <x:v>web/js/app.js:45; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
-        <x:v>信息可读性优先</x:v>
+        <x:v>保留原棋子身份、伤势和剩余 AP</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="32" customHeight="1">
@@ -1635,34 +1635,730 @@
         <x:v>A-043</x:v>
       </x:c>
       <x:c r="B48" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C48" s="11" t="str">
+        <x:v>弓兵｜四向射击</x:v>
+      </x:c>
+      <x:c r="D48" s="11" t="str">
+        <x:v>前／右／后／左</x:v>
+      </x:c>
+      <x:c r="E48" s="11" t="str">
+        <x:v>选一个方向，命中范围内首个敌人</x:v>
+      </x:c>
+      <x:c r="F48" s="11" t="str">
+        <x:v>黄色范围点和命中预览；无箭矢特效资产</x:v>
+      </x:c>
+      <x:c r="G48" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H48" s="11" t="str">
+        <x:v>web/js/app.js:59,64; web/js/rules.js:35</x:v>
+      </x:c>
+      <x:c r="I48" s="11" t="str">
+        <x:v>友军阻挡；需表现首个目标和 2 点伤害</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="32" customHeight="1">
+      <x:c r="A49" s="10" t="str">
+        <x:v>A-044</x:v>
+      </x:c>
+      <x:c r="B49" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C49" s="11" t="str">
+        <x:v>弓兵｜方向射程升级</x:v>
+      </x:c>
+      <x:c r="D49" s="11" t="str">
+        <x:v>4方向×6级</x:v>
+      </x:c>
+      <x:c r="E49" s="11" t="str">
+        <x:v>单方向每次 +1 格，最高 Lv.8／7格</x:v>
+      </x:c>
+      <x:c r="F49" s="11" t="str">
+        <x:v>仅方向按钮等级和距离文字刷新</x:v>
+      </x:c>
+      <x:c r="G49" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H49" s="11" t="str">
+        <x:v>web/js/app.js:47-48; web/js/rules.js:53</x:v>
+      </x:c>
+      <x:c r="I49" s="11" t="str">
+        <x:v>四方向独立，升级反馈须标明具体方向</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="32" customHeight="1">
+      <x:c r="A50" s="10" t="str">
+        <x:v>A-045</x:v>
+      </x:c>
+      <x:c r="B50" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C50" s="11" t="str">
+        <x:v>枪兵｜四向贯穿攻击</x:v>
+      </x:c>
+      <x:c r="D50" s="11" t="str">
+        <x:v>前／右／后／左</x:v>
+      </x:c>
+      <x:c r="E50" s="11" t="str">
+        <x:v>选一个方向，命中线内所有敌人</x:v>
+      </x:c>
+      <x:c r="F50" s="11" t="str">
+        <x:v>黄色范围点和命中列表；无枪击特效资产</x:v>
+      </x:c>
+      <x:c r="G50" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H50" s="11" t="str">
+        <x:v>web/js/app.js:59,64; web/js/rules.js:35</x:v>
+      </x:c>
+      <x:c r="I50" s="11" t="str">
+        <x:v>空格和敌人不中断，友军阻断；各目标 1 点伤害</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="32" customHeight="1">
+      <x:c r="A51" s="10" t="str">
+        <x:v>A-046</x:v>
+      </x:c>
+      <x:c r="B51" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C51" s="11" t="str">
+        <x:v>枪兵｜方向范围升级</x:v>
+      </x:c>
+      <x:c r="D51" s="11" t="str">
+        <x:v>4方向×6级</x:v>
+      </x:c>
+      <x:c r="E51" s="11" t="str">
+        <x:v>单方向每次 +1 格，最高 Lv.8／7格</x:v>
+      </x:c>
+      <x:c r="F51" s="11" t="str">
+        <x:v>仅方向按钮等级和距离文字刷新</x:v>
+      </x:c>
+      <x:c r="G51" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H51" s="11" t="str">
+        <x:v>web/js/app.js:47-48; web/js/rules.js:53</x:v>
+      </x:c>
+      <x:c r="I51" s="11" t="str">
+        <x:v>四方向独立；与弓兵升级可共用框架但视觉需可辨识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="32" customHeight="1">
+      <x:c r="A52" s="10" t="str">
+        <x:v>A-047</x:v>
+      </x:c>
+      <x:c r="B52" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C52" s="11" t="str">
+        <x:v>当前选中棋位</x:v>
+      </x:c>
+      <x:c r="D52" s="11" t="str">
+        <x:v>1种</x:v>
+      </x:c>
+      <x:c r="E52" s="11" t="str">
+        <x:v>选棋后标记起点</x:v>
+      </x:c>
+      <x:c r="F52" s="11" t="str">
+        <x:v>黄色半透明圆点</x:v>
+      </x:c>
+      <x:c r="G52" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H52" s="11" t="str">
+        <x:v>web/js/app.js:33-34</x:v>
+      </x:c>
+      <x:c r="I52" s="11" t="str">
+        <x:v>需与其他标记可区分</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="32" customHeight="1">
+      <x:c r="A53" s="10" t="str">
+        <x:v>A-048</x:v>
+      </x:c>
+      <x:c r="B53" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C53" s="11" t="str">
+        <x:v>合法移动落点</x:v>
+      </x:c>
+      <x:c r="D53" s="11" t="str">
+        <x:v>1种</x:v>
+      </x:c>
+      <x:c r="E53" s="11" t="str">
+        <x:v>移动选择</x:v>
+      </x:c>
+      <x:c r="F53" s="11" t="str">
+        <x:v>蓝色半透明圆点</x:v>
+      </x:c>
+      <x:c r="G53" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H53" s="11" t="str">
+        <x:v>web/js/app.js:33-34</x:v>
+      </x:c>
+      <x:c r="I53" s="11" t="str">
+        <x:v>需兼顾窄屏识别</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="32" customHeight="1">
+      <x:c r="A54" s="10" t="str">
+        <x:v>A-049</x:v>
+      </x:c>
+      <x:c r="B54" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C54" s="11" t="str">
+        <x:v>攻击与冲击目标</x:v>
+      </x:c>
+      <x:c r="D54" s="11" t="str">
+        <x:v>1种</x:v>
+      </x:c>
+      <x:c r="E54" s="11" t="str">
+        <x:v>攻击或车冲击</x:v>
+      </x:c>
+      <x:c r="F54" s="11" t="str">
+        <x:v>红色半透明圆点</x:v>
+      </x:c>
+      <x:c r="G54" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H54" s="11" t="str">
+        <x:v>web/js/app.js:33-34</x:v>
+      </x:c>
+      <x:c r="I54" s="11" t="str">
+        <x:v>需与移动落点可区分</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="32" customHeight="1">
+      <x:c r="A55" s="10" t="str">
+        <x:v>A-050</x:v>
+      </x:c>
+      <x:c r="B55" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C55" s="11" t="str">
+        <x:v>方向攻击范围</x:v>
+      </x:c>
+      <x:c r="D55" s="11" t="str">
+        <x:v>1种</x:v>
+      </x:c>
+      <x:c r="E55" s="11" t="str">
+        <x:v>弓／枪四向预览</x:v>
+      </x:c>
+      <x:c r="F55" s="11" t="str">
+        <x:v>黄色路径圆点</x:v>
+      </x:c>
+      <x:c r="G55" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H55" s="11" t="str">
+        <x:v>web/js/app.js:59</x:v>
+      </x:c>
+      <x:c r="I55" s="11" t="str">
+        <x:v>正式范围表现 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="32" customHeight="1">
+      <x:c r="A56" s="10" t="str">
+        <x:v>A-051</x:v>
+      </x:c>
+      <x:c r="B56" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C56" s="11" t="str">
+        <x:v>炮击路径与炮架</x:v>
+      </x:c>
+      <x:c r="D56" s="11" t="str">
+        <x:v>2种</x:v>
+      </x:c>
+      <x:c r="E56" s="11" t="str">
+        <x:v>炮击预览</x:v>
+      </x:c>
+      <x:c r="F56" s="11" t="str">
+        <x:v>黄色路径点＋紫色炮架点</x:v>
+      </x:c>
+      <x:c r="G56" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H56" s="11" t="str">
+        <x:v>web/js/app.js:34</x:v>
+      </x:c>
+      <x:c r="I56" s="11" t="str">
+        <x:v>必须辨识炮架与主目标</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="32" customHeight="1">
+      <x:c r="A57" s="10" t="str">
+        <x:v>A-052</x:v>
+      </x:c>
+      <x:c r="B57" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C57" s="11" t="str">
+        <x:v>炮主目标</x:v>
+      </x:c>
+      <x:c r="D57" s="11" t="str">
+        <x:v>1种</x:v>
+      </x:c>
+      <x:c r="E57" s="11" t="str">
+        <x:v>炮击预览</x:v>
+      </x:c>
+      <x:c r="F57" s="11" t="str">
+        <x:v>红色目标点</x:v>
+      </x:c>
+      <x:c r="G57" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H57" s="11" t="str">
+        <x:v>web/js/app.js:34</x:v>
+      </x:c>
+      <x:c r="I57" s="11" t="str">
+        <x:v>扩散格视觉表现 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="32" customHeight="1">
+      <x:c r="A58" s="10" t="str">
+        <x:v>A-053</x:v>
+      </x:c>
+      <x:c r="B58" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C58" s="11" t="str">
+        <x:v>战斗背景与主布局</x:v>
+      </x:c>
+      <x:c r="D58" s="11" t="str">
+        <x:v>桌面／窄屏</x:v>
+      </x:c>
+      <x:c r="E58" s="11" t="str">
+        <x:v>棋盘外背景与分区</x:v>
+      </x:c>
+      <x:c r="F58" s="11" t="str">
+        <x:v>CSS 纯色与响应式布局</x:v>
+      </x:c>
+      <x:c r="G58" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H58" s="11" t="str">
+        <x:v>web/index.html:8-14</x:v>
+      </x:c>
+      <x:c r="I58" s="11" t="str">
+        <x:v>正式背景、装饰 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="32" customHeight="1">
+      <x:c r="A59" s="10" t="str">
+        <x:v>A-054</x:v>
+      </x:c>
+      <x:c r="B59" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C59" s="11" t="str">
+        <x:v>顶部状态栏</x:v>
+      </x:c>
+      <x:c r="D59" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E59" s="11" t="str">
+        <x:v>波次、回合、HP、金币、击杀</x:v>
+      </x:c>
+      <x:c r="F59" s="11" t="str">
+        <x:v>CSS 卡片＋文字</x:v>
+      </x:c>
+      <x:c r="G59" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H59" s="11" t="str">
+        <x:v>web/index.html:11,23</x:v>
+      </x:c>
+      <x:c r="I59" s="11" t="str">
+        <x:v>图标需求 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="32" customHeight="1">
+      <x:c r="A60" s="10" t="str">
+        <x:v>A-055</x:v>
+      </x:c>
+      <x:c r="B60" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C60" s="11" t="str">
+        <x:v>我方单位列表与棋子徽记</x:v>
+      </x:c>
+      <x:c r="D60" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E60" s="11" t="str">
+        <x:v>选棋及单位状态</x:v>
+      </x:c>
+      <x:c r="F60" s="11" t="str">
+        <x:v>CSS 卡片＋汉字徽记</x:v>
+      </x:c>
+      <x:c r="G60" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H60" s="11" t="str">
+        <x:v>web/index.html:12,26; web/js/app.js:37</x:v>
+      </x:c>
+      <x:c r="I60" s="11" t="str">
+        <x:v>沿用棋子识别系统</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="32" customHeight="1">
+      <x:c r="A61" s="10" t="str">
+        <x:v>A-056</x:v>
+      </x:c>
+      <x:c r="B61" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C61" s="11" t="str">
+        <x:v>当前棋子信息卡</x:v>
+      </x:c>
+      <x:c r="D61" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E61" s="11" t="str">
+        <x:v>属性、AP、等级、SP</x:v>
+      </x:c>
+      <x:c r="F61" s="11" t="str">
+        <x:v>CSS 信息卡＋文字</x:v>
+      </x:c>
+      <x:c r="G61" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H61" s="11" t="str">
+        <x:v>web/index.html:12,27</x:v>
+      </x:c>
+      <x:c r="I61" s="11" t="str">
+        <x:v>状态层级 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="32" customHeight="1">
+      <x:c r="A62" s="10" t="str">
+        <x:v>A-057</x:v>
+      </x:c>
+      <x:c r="B62" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C62" s="11" t="str">
+        <x:v>技能条目与禁用状态</x:v>
+      </x:c>
+      <x:c r="D62" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E62" s="11" t="str">
+        <x:v>升级、转职、方向和扩散</x:v>
+      </x:c>
+      <x:c r="F62" s="11" t="str">
+        <x:v>CSS 按钮＋文字</x:v>
+      </x:c>
+      <x:c r="G62" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H62" s="11" t="str">
+        <x:v>web/index.html:13; web/js/app.js:42-56</x:v>
+      </x:c>
+      <x:c r="I62" s="11" t="str">
+        <x:v>各技能专属图标 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="32" customHeight="1">
+      <x:c r="A63" s="10" t="str">
+        <x:v>A-058</x:v>
+      </x:c>
+      <x:c r="B63" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C63" s="11" t="str">
+        <x:v>方向与车模式按钮</x:v>
+      </x:c>
+      <x:c r="D63" s="11" t="str">
+        <x:v>2组</x:v>
+      </x:c>
+      <x:c r="E63" s="11" t="str">
+        <x:v>弓枪四向；车移动／冲击</x:v>
+      </x:c>
+      <x:c r="F63" s="11" t="str">
+        <x:v>CSS 按钮＋选中描边</x:v>
+      </x:c>
+      <x:c r="G63" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H63" s="11" t="str">
+        <x:v>web/index.html:13; web/js/app.js:58</x:v>
+      </x:c>
+      <x:c r="I63" s="11" t="str">
+        <x:v>交互态样式 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="32" customHeight="1">
+      <x:c r="A64" s="10" t="str">
+        <x:v>A-059</x:v>
+      </x:c>
+      <x:c r="B64" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C64" s="11" t="str">
+        <x:v>敌方意图列表与序号</x:v>
+      </x:c>
+      <x:c r="D64" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E64" s="11" t="str">
+        <x:v>敌方行动顺序和状态</x:v>
+      </x:c>
+      <x:c r="F64" s="11" t="str">
+        <x:v>CSS 圆序号＋文字</x:v>
+      </x:c>
+      <x:c r="G64" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H64" s="11" t="str">
+        <x:v>web/index.html:13; web/js/app.js:60</x:v>
+      </x:c>
+      <x:c r="I64" s="11" t="str">
+        <x:v>窄屏展开态已支持</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="32" customHeight="1">
+      <x:c r="A65" s="10" t="str">
+        <x:v>A-060</x:v>
+      </x:c>
+      <x:c r="B65" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C65" s="11" t="str">
+        <x:v>动作预览与受击警告</x:v>
+      </x:c>
+      <x:c r="D65" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E65" s="11" t="str">
+        <x:v>路径、伤害、友伤、威胁</x:v>
+      </x:c>
+      <x:c r="F65" s="11" t="str">
+        <x:v>CSS 信息卡＋警告色</x:v>
+      </x:c>
+      <x:c r="G65" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H65" s="11" t="str">
+        <x:v>web/index.html:13; web/js/app.js:63</x:v>
+      </x:c>
+      <x:c r="I65" s="11" t="str">
+        <x:v>友军误伤须醒目</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="32" customHeight="1">
+      <x:c r="A66" s="10" t="str">
+        <x:v>A-061</x:v>
+      </x:c>
+      <x:c r="B66" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C66" s="11" t="str">
+        <x:v>底部操作按钮</x:v>
+      </x:c>
+      <x:c r="D66" s="11" t="str">
+        <x:v>4种</x:v>
+      </x:c>
+      <x:c r="E66" s="11" t="str">
+        <x:v>执行、取消、结束回合、暂停</x:v>
+      </x:c>
+      <x:c r="F66" s="11" t="str">
+        <x:v>CSS 按钮</x:v>
+      </x:c>
+      <x:c r="G66" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H66" s="11" t="str">
+        <x:v>web/index.html:14,32</x:v>
+      </x:c>
+      <x:c r="I66" s="11" t="str">
+        <x:v>含禁用／悬停态</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="32" customHeight="1">
+      <x:c r="A67" s="10" t="str">
+        <x:v>A-062</x:v>
+      </x:c>
+      <x:c r="B67" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C67" s="11" t="str">
+        <x:v>结束回合确认弹窗</x:v>
+      </x:c>
+      <x:c r="D67" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E67" s="11" t="str">
+        <x:v>提交敌方阶段前确认</x:v>
+      </x:c>
+      <x:c r="F67" s="11" t="str">
+        <x:v>CSS 遮罩＋对话框</x:v>
+      </x:c>
+      <x:c r="G67" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H67" s="11" t="str">
+        <x:v>web/index.html:15,34</x:v>
+      </x:c>
+      <x:c r="I67" s="11" t="str">
+        <x:v>正式插画需求 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="32" customHeight="1">
+      <x:c r="A68" s="10" t="str">
+        <x:v>A-063</x:v>
+      </x:c>
+      <x:c r="B68" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C68" s="11" t="str">
+        <x:v>暂停弹窗</x:v>
+      </x:c>
+      <x:c r="D68" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E68" s="11" t="str">
+        <x:v>继续和重新开始</x:v>
+      </x:c>
+      <x:c r="F68" s="11" t="str">
+        <x:v>CSS 遮罩＋对话框</x:v>
+      </x:c>
+      <x:c r="G68" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H68" s="11" t="str">
+        <x:v>web/index.html:15,35</x:v>
+      </x:c>
+      <x:c r="I68" s="11" t="str">
+        <x:v>正式插画需求 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="32" customHeight="1">
+      <x:c r="A69" s="10" t="str">
+        <x:v>A-064</x:v>
+      </x:c>
+      <x:c r="B69" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C69" s="11" t="str">
+        <x:v>商店与马／炮商品卡</x:v>
+      </x:c>
+      <x:c r="D69" s="11" t="str">
+        <x:v>1套＋2商品</x:v>
+      </x:c>
+      <x:c r="E69" s="11" t="str">
+        <x:v>首波结束后选购</x:v>
+      </x:c>
+      <x:c r="F69" s="11" t="str">
+        <x:v>CSS 对话框＋文字商品卡</x:v>
+      </x:c>
+      <x:c r="G69" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H69" s="11" t="str">
+        <x:v>web/index.html:15,36</x:v>
+      </x:c>
+      <x:c r="I69" s="11" t="str">
+        <x:v>商品形象可复用棋子资产</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="32" customHeight="1">
+      <x:c r="A70" s="10" t="str">
+        <x:v>A-065</x:v>
+      </x:c>
+      <x:c r="B70" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C70" s="11" t="str">
+        <x:v>终局弹窗</x:v>
+      </x:c>
+      <x:c r="D70" s="11" t="str">
+        <x:v>胜／阵亡／将死</x:v>
+      </x:c>
+      <x:c r="E70" s="11" t="str">
+        <x:v>最终结果</x:v>
+      </x:c>
+      <x:c r="F70" s="11" t="str">
+        <x:v>CSS 对话框＋状态文字</x:v>
+      </x:c>
+      <x:c r="G70" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H70" s="11" t="str">
+        <x:v>web/index.html:15,37</x:v>
+      </x:c>
+      <x:c r="I70" s="11" t="str">
+        <x:v>结果插画需求 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="32" customHeight="1">
+      <x:c r="A71" s="10" t="str">
+        <x:v>A-066</x:v>
+      </x:c>
+      <x:c r="B71" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C71" s="11" t="str">
+        <x:v>短提示与危险提示</x:v>
+      </x:c>
+      <x:c r="D71" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E71" s="11" t="str">
+        <x:v>购买、重开、操作失败</x:v>
+      </x:c>
+      <x:c r="F71" s="11" t="str">
+        <x:v>CSS 横幅＋文字</x:v>
+      </x:c>
+      <x:c r="G71" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H71" s="11" t="str">
+        <x:v>web/index.html:14,24; web/js/app.js:69</x:v>
+      </x:c>
+      <x:c r="I71" s="11" t="str">
+        <x:v>信息可读性优先</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="32" customHeight="1">
+      <x:c r="A72" s="10" t="str">
+        <x:v>A-067</x:v>
+      </x:c>
+      <x:c r="B72" s="11" t="str">
         <x:v>旧目录素材</x:v>
       </x:c>
-      <x:c r="C48" s="11" t="str">
+      <x:c r="C72" s="11" t="str">
         <x:v>僵尸角色图</x:v>
       </x:c>
-      <x:c r="D48" s="11" t="str">
+      <x:c r="D72" s="11" t="str">
         <x:v>1张</x:v>
       </x:c>
-      <x:c r="E48" s="11" t="str">
+      <x:c r="E72" s="11" t="str">
         <x:v>旧目录参考；网页未使用</x:v>
       </x:c>
-      <x:c r="F48" s="11" t="str">
+      <x:c r="F72" s="11" t="str">
         <x:v>PNG，像素风角色</x:v>
       </x:c>
-      <x:c r="G48" s="11" t="str">
+      <x:c r="G72" s="11" t="str">
         <x:v>已有文件未接入</x:v>
       </x:c>
-      <x:c r="H48" s="11" t="str">
+      <x:c r="H72" s="11" t="str">
         <x:v>m0-zyf/assets/art/jiangshi.png</x:v>
       </x:c>
-      <x:c r="I48" s="11" t="str">
+      <x:c r="I72" s="11" t="str">
         <x:v>与当前象棋题材的用途 TBD</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ea38fa6f82849ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra54246ffb3d7452c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1808,7 +2504,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49c538fcc5f34ae9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raecb7483895d4100"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore(assets): add terrain assets and correct board size in art list
</commit_message>
<xml_diff>
--- a/outputs/01a0bf14-7f85-7282-bb8d-672064556a58/美术资产清单.xlsx
+++ b/outputs/01a0bf14-7f85-7282-bb8d-672064556a58/美术资产清单.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="美术资产清单" sheetId="1" r:id="Ra513a2f0424f4cd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="源文件盘点" sheetId="2" r:id="R5db7b97349564186"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="美术资产清单" sheetId="1" r:id="R735b1bd6142b491f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="源文件盘点" sheetId="2" r:id="R5d8b2065cfac41f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VisualAssets" displayName="VisualAssets" ref="A5:I72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VisualAssets" displayName="VisualAssets" ref="A5:I91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="分类"/>
@@ -348,7 +348,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>范围：当前网页原型及工作区源素材；传统棋子按敌我分列，技能效果只预留己方，敌方按被动单位处理。</x:v>
+        <x:v>范围：当前主原型、独立地形实验及工作区源素材；地形资产来自 terrain-wave 实验，尚未合入主原型。</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -361,7 +361,7 @@
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>共 67 项视觉元素；传统棋子 14 款，项目转职 2 款；己方技能效果预留 24 项；旧目录源图片 1 个。</x:v>
+        <x:v>共 86 项视觉元素；传统棋子 14 款，项目转职 2 款；己方技能效果预留 24 项；地形资产与效果 19 项；旧目录源图片 1 个。</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -413,7 +413,7 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
-      <x:c r="A6" s="7" t="str">
+      <x:c r="A6" s="8" t="str">
         <x:v>A-001</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
@@ -442,7 +442,7 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="32" customHeight="1">
-      <x:c r="A7" s="7" t="str">
+      <x:c r="A7" s="8" t="str">
         <x:v>A-002</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">
@@ -471,65 +471,65 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
-      <x:c r="A8" s="7" t="str">
+      <x:c r="A8" s="8" t="str">
         <x:v>A-003</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
         <x:v>棋盘场景</x:v>
       </x:c>
       <x:c r="C8" s="8" t="str">
-        <x:v>8×8 网格线</x:v>
+        <x:v>9×9 网格线</x:v>
       </x:c>
       <x:c r="D8" s="8" t="str">
         <x:v>1套</x:v>
       </x:c>
       <x:c r="E8" s="8" t="str">
-        <x:v>64 个棋位</x:v>
+        <x:v>81 个棋位</x:v>
       </x:c>
       <x:c r="F8" s="8" t="str">
-        <x:v>Canvas 绘制</x:v>
+        <x:v>Canvas 线框绘制</x:v>
       </x:c>
       <x:c r="G8" s="8" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H8" s="8" t="str">
-        <x:v>web/js/app.js:22-23</x:v>
+        <x:v>web/js/app.js:22-27；web/js/rules.js:4</x:v>
       </x:c>
       <x:c r="I8" s="8" t="str">
         <x:v>线宽与正式样式 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
-      <x:c r="A9" s="7" t="str">
+      <x:c r="A9" s="8" t="str">
         <x:v>A-004</x:v>
       </x:c>
       <x:c r="B9" s="8" t="str">
         <x:v>棋盘场景</x:v>
       </x:c>
       <x:c r="C9" s="8" t="str">
-        <x:v>河界与文字</x:v>
+        <x:v>中央河道与文字</x:v>
       </x:c>
       <x:c r="D9" s="8" t="str">
         <x:v>1套</x:v>
       </x:c>
       <x:c r="E9" s="8" t="str">
-        <x:v>y=3/4 分界</x:v>
+        <x:v>第 5 行／y=4</x:v>
       </x:c>
       <x:c r="F9" s="8" t="str">
-        <x:v>Canvas 绘制</x:v>
+        <x:v>Canvas 色带与文字</x:v>
       </x:c>
       <x:c r="G9" s="8" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H9" s="8" t="str">
-        <x:v>web/js/app.js:24</x:v>
+        <x:v>web/js/app.js:24-25；web/js/rules.js:4</x:v>
       </x:c>
       <x:c r="I9" s="8" t="str">
-        <x:v>正式字样与样式 TBD</x:v>
+        <x:v>主原型为可通行河道；独立地形实验将其中 6 格设为水、3 格设为桥</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32" customHeight="1">
-      <x:c r="A10" s="7" t="str">
+      <x:c r="A10" s="8" t="str">
         <x:v>A-005</x:v>
       </x:c>
       <x:c r="B10" s="8" t="str">
@@ -551,14 +551,14 @@
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H10" s="8" t="str">
-        <x:v>web/js/app.js:25-26</x:v>
+        <x:v>web/js/app.js:26-27</x:v>
       </x:c>
       <x:c r="I10" s="8" t="str">
         <x:v>必须保留可辨识宫界</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="32" customHeight="1">
-      <x:c r="A11" s="7" t="str">
+      <x:c r="A11" s="8" t="str">
         <x:v>A-006</x:v>
       </x:c>
       <x:c r="B11" s="8" t="str">
@@ -568,10 +568,10 @@
         <x:v>棋位坐标字</x:v>
       </x:c>
       <x:c r="D11" s="8" t="str">
-        <x:v>64处</x:v>
+        <x:v>81处</x:v>
       </x:c>
       <x:c r="E11" s="8" t="str">
-        <x:v>开发定位辅助</x:v>
+        <x:v>9×9 棋位坐标</x:v>
       </x:c>
       <x:c r="F11" s="8" t="str">
         <x:v>Canvas 文字</x:v>
@@ -580,1785 +580,2340 @@
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H11" s="8" t="str">
-        <x:v>web/js/app.js:26</x:v>
+        <x:v>web/js/app.js:27</x:v>
       </x:c>
       <x:c r="I11" s="8" t="str">
-        <x:v>正式版是否显示 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="32" customHeight="1">
-      <x:c r="A12" s="7" t="str">
+        <x:v>调试信息；正式版本是否保留 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="38" customHeight="1">
+      <x:c r="A12" s="8" t="str">
         <x:v>A-007</x:v>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形资产</x:v>
       </x:c>
       <x:c r="C12" s="8" t="str">
-        <x:v>己方帅</x:v>
+        <x:v>普通陆地格</x:v>
       </x:c>
       <x:c r="D12" s="8" t="str">
-        <x:v>1款／标准1枚</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E12" s="8" t="str">
-        <x:v>己方主帅</x:v>
+        <x:v>基础可通行棋位</x:v>
       </x:c>
       <x:c r="F12" s="8" t="str">
-        <x:v>红色圆柱＋“帅”字</x:v>
+        <x:v>菱形草绿色地块；编辑器为方格</x:v>
       </x:c>
       <x:c r="G12" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>代码占位（独立实验）</x:v>
       </x:c>
       <x:c r="H12" s="8" t="str">
-        <x:v>web/js/app.js:4-6,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/style.css:1；app.js:99-116</x:v>
       </x:c>
       <x:c r="I12" s="8" t="str">
-        <x:v>中国象棋红方棋种；正式形象 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="32" customHeight="1">
-      <x:c r="A13" s="7" t="str">
+        <x:v>需兼容对局菱形与编辑器方格视图；正式纹理 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="38" customHeight="1">
+      <x:c r="A13" s="8" t="str">
         <x:v>A-008</x:v>
       </x:c>
       <x:c r="B13" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形资产</x:v>
       </x:c>
       <x:c r="C13" s="8" t="str">
-        <x:v>己方仕</x:v>
+        <x:v>水域格</x:v>
       </x:c>
       <x:c r="D13" s="8" t="str">
-        <x:v>1款／标准2枚</x:v>
+        <x:v>1套／默认6格</x:v>
       </x:c>
       <x:c r="E13" s="8" t="str">
-        <x:v>完整中国象棋红方名录</x:v>
+        <x:v>河道非桥棋位</x:v>
       </x:c>
       <x:c r="F13" s="8" t="str">
-        <x:v>无（当前未配置）</x:v>
+        <x:v>蓝绿色地块＋“≈”符号</x:v>
       </x:c>
       <x:c r="G13" s="8" t="str">
-        <x:v>未实现</x:v>
+        <x:v>代码占位（独立实验）</x:v>
       </x:c>
       <x:c r="H13" s="8" t="str">
-        <x:v>中国象棋棋种；用户补充</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:224-227；style.css:1</x:v>
       </x:c>
       <x:c r="I13" s="8" t="str">
-        <x:v>当前网页无己方仕；规则与造型 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="32" customHeight="1">
-      <x:c r="A14" s="7" t="str">
+        <x:v>默认第 5 行第 1、3、4、6、7、9 列；正式水面动画 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="38" customHeight="1">
+      <x:c r="A14" s="8" t="str">
         <x:v>A-009</x:v>
       </x:c>
       <x:c r="B14" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形资产</x:v>
       </x:c>
       <x:c r="C14" s="8" t="str">
-        <x:v>己方相</x:v>
+        <x:v>陆地桥格</x:v>
       </x:c>
       <x:c r="D14" s="8" t="str">
-        <x:v>1款／标准2枚</x:v>
+        <x:v>1套／默认3格</x:v>
       </x:c>
       <x:c r="E14" s="8" t="str">
-        <x:v>完整中国象棋红方名录</x:v>
+        <x:v>河道可通行桥位</x:v>
       </x:c>
       <x:c r="F14" s="8" t="str">
-        <x:v>无（当前未配置）</x:v>
+        <x:v>棕色木纹条带</x:v>
       </x:c>
       <x:c r="G14" s="8" t="str">
-        <x:v>未实现</x:v>
+        <x:v>代码占位（独立实验）</x:v>
       </x:c>
       <x:c r="H14" s="8" t="str">
-        <x:v>中国象棋棋种；用户补充</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:224-227；style.css:1</x:v>
       </x:c>
       <x:c r="I14" s="8" t="str">
-        <x:v>当前网页无相；规则与造型 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="32" customHeight="1">
-      <x:c r="A15" s="7" t="str">
+        <x:v>默认第 5 行第 2、5、8 列；桥体结构与栏杆 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="38" customHeight="1">
+      <x:c r="A15" s="8" t="str">
         <x:v>A-010</x:v>
       </x:c>
       <x:c r="B15" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形资产</x:v>
       </x:c>
       <x:c r="C15" s="8" t="str">
-        <x:v>己方马</x:v>
+        <x:v>完整山体</x:v>
       </x:c>
       <x:c r="D15" s="8" t="str">
-        <x:v>1款／标准2枚</x:v>
+        <x:v>1套／默认4座</x:v>
       </x:c>
       <x:c r="E15" s="8" t="str">
-        <x:v>首波商店购买</x:v>
+        <x:v>不可通行、可被攻击的障碍物</x:v>
       </x:c>
       <x:c r="F15" s="8" t="str">
-        <x:v>红色圆柱＋“马”字</x:v>
+        <x:v>灰色地块＋“▲”符号</x:v>
       </x:c>
       <x:c r="G15" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>代码占位（独立实验）</x:v>
       </x:c>
       <x:c r="H15" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:120-125,226；style.css:1</x:v>
       </x:c>
       <x:c r="I15" s="8" t="str">
-        <x:v>原型最多购买一枚；标准整副为两枚</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="32" customHeight="1">
-      <x:c r="A16" s="7" t="str">
+        <x:v>完整山体可承受第 1 次有效命中；体量与遮挡高度 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="38" customHeight="1">
+      <x:c r="A16" s="8" t="str">
         <x:v>A-011</x:v>
       </x:c>
       <x:c r="B16" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形资产</x:v>
       </x:c>
       <x:c r="C16" s="8" t="str">
-        <x:v>己方车</x:v>
+        <x:v>开裂山体</x:v>
       </x:c>
       <x:c r="D16" s="8" t="str">
-        <x:v>1款／标准2枚</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E16" s="8" t="str">
-        <x:v>初始队伍</x:v>
+        <x:v>山体受到 1 次有效命中后</x:v>
       </x:c>
       <x:c r="F16" s="8" t="str">
-        <x:v>红色圆柱＋“车”字</x:v>
+        <x:v>灰色地块＋“◭”符号</x:v>
       </x:c>
       <x:c r="G16" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>代码占位（独立实验）</x:v>
       </x:c>
       <x:c r="H16" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:120-125；style.css:1</x:v>
       </x:c>
       <x:c r="I16" s="8" t="str">
-        <x:v>原型初始一枚；标准整副为两枚</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="32" customHeight="1">
-      <x:c r="A17" s="7" t="str">
+        <x:v>再受 1 次有效命中后坍塌；裂纹形态 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="38" customHeight="1">
+      <x:c r="A17" s="8" t="str">
         <x:v>A-012</x:v>
       </x:c>
       <x:c r="B17" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形资产</x:v>
       </x:c>
       <x:c r="C17" s="8" t="str">
-        <x:v>己方炮</x:v>
+        <x:v>坍塌陆地／碎石</x:v>
       </x:c>
       <x:c r="D17" s="8" t="str">
-        <x:v>1款／标准2枚</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E17" s="8" t="str">
-        <x:v>首波商店购买</x:v>
+        <x:v>山体第 2 次有效命中后</x:v>
       </x:c>
       <x:c r="F17" s="8" t="str">
-        <x:v>红色圆柱＋“炮”字</x:v>
+        <x:v>褐色碎石地块＋“·”符号</x:v>
       </x:c>
       <x:c r="G17" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>代码占位（独立实验）</x:v>
       </x:c>
       <x:c r="H17" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:120-125；style.css:1</x:v>
       </x:c>
       <x:c r="I17" s="8" t="str">
-        <x:v>原型最多购买一枚；标准整副为两枚</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="32" customHeight="1">
-      <x:c r="A18" s="7" t="str">
+        <x:v>坍塌后恢复为可通行陆地；碎石密度与消散方式 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="38" customHeight="1">
+      <x:c r="A18" s="8" t="str">
         <x:v>A-013</x:v>
       </x:c>
       <x:c r="B18" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形资产</x:v>
       </x:c>
       <x:c r="C18" s="8" t="str">
-        <x:v>己方兵</x:v>
+        <x:v>树林格</x:v>
       </x:c>
       <x:c r="D18" s="8" t="str">
-        <x:v>1款／标准5枚</x:v>
+        <x:v>1套／默认5格</x:v>
       </x:c>
       <x:c r="E18" s="8" t="str">
-        <x:v>P1 等测试夹具</x:v>
+        <x:v>提供一定概率闪避的可通行棋位</x:v>
       </x:c>
       <x:c r="F18" s="8" t="str">
-        <x:v>红色圆柱＋“兵”字</x:v>
+        <x:v>深绿色地块＋“♠”符号</x:v>
       </x:c>
       <x:c r="G18" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>代码占位（独立实验）</x:v>
       </x:c>
       <x:c r="H18" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:174,227；style.css:1</x:v>
       </x:c>
       <x:c r="I18" s="8" t="str">
-        <x:v>正式局未提供招募；标准整副为五枚</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="32" customHeight="1">
-      <x:c r="A19" s="7" t="str">
+        <x:v>界面只表达“有一定概率闪避”，不显示 30% 或预告本次结果</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="38" customHeight="1">
+      <x:c r="A19" s="8" t="str">
         <x:v>A-014</x:v>
       </x:c>
       <x:c r="B19" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形效果</x:v>
       </x:c>
       <x:c r="C19" s="8" t="str">
-        <x:v>敌方将</x:v>
+        <x:v>入水波纹／溅水</x:v>
       </x:c>
       <x:c r="D19" s="8" t="str">
-        <x:v>1款／标准1枚</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E19" s="8" t="str">
-        <x:v>两波敌将</x:v>
+        <x:v>棋子进入或经过水域</x:v>
       </x:c>
       <x:c r="F19" s="8" t="str">
-        <x:v>蓝色方块＋“将”字</x:v>
+        <x:v>无独立特效</x:v>
       </x:c>
       <x:c r="G19" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H19" s="8" t="str">
-        <x:v>web/js/app.js:4-6,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:49,54</x:v>
       </x:c>
       <x:c r="I19" s="8" t="str">
-        <x:v>中国象棋黑方棋种；正式形象 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="32" customHeight="1">
-      <x:c r="A20" s="7" t="str">
+        <x:v>区分快速经过、停留和阵亡三种节奏 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="38" customHeight="1">
+      <x:c r="A20" s="8" t="str">
         <x:v>A-015</x:v>
       </x:c>
       <x:c r="B20" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形效果</x:v>
       </x:c>
       <x:c r="C20" s="8" t="str">
-        <x:v>敌方士</x:v>
+        <x:v>入水阵亡</x:v>
       </x:c>
       <x:c r="D20" s="8" t="str">
-        <x:v>1款／标准2枚</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E20" s="8" t="str">
-        <x:v>两波敌阵</x:v>
+        <x:v>兵／弓／枪／炮进入水域立即阵亡</x:v>
       </x:c>
       <x:c r="F20" s="8" t="str">
-        <x:v>蓝色方块＋“士”字</x:v>
+        <x:v>棋子直接移除＋战报文字</x:v>
       </x:c>
       <x:c r="G20" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H20" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:49,54</x:v>
       </x:c>
       <x:c r="I20" s="8" t="str">
-        <x:v>当前每波两枚；正式形象 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="32" customHeight="1">
-      <x:c r="A21" s="7" t="str">
+        <x:v>需包含棋子沉没、消散与击杀归属反馈；表现规格 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="38" customHeight="1">
+      <x:c r="A21" s="8" t="str">
         <x:v>A-016</x:v>
       </x:c>
       <x:c r="B21" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形效果</x:v>
       </x:c>
       <x:c r="C21" s="8" t="str">
-        <x:v>敌方象</x:v>
+        <x:v>水中禁攻状态</x:v>
       </x:c>
       <x:c r="D21" s="8" t="str">
-        <x:v>1款／标准2枚</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E21" s="8" t="str">
-        <x:v>完整中国象棋黑方名录</x:v>
+        <x:v>马或车停留水域时</x:v>
       </x:c>
       <x:c r="F21" s="8" t="str">
-        <x:v>无（当前未配置）</x:v>
+        <x:v>状态栏文字提示</x:v>
       </x:c>
       <x:c r="G21" s="8" t="str">
-        <x:v>未实现</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H21" s="8" t="str">
-        <x:v>中国象棋棋种；用户补充</x:v>
+        <x:v>web/experiments/terrain-wave/app.js:125-128；rules.js:94</x:v>
       </x:c>
       <x:c r="I21" s="8" t="str">
-        <x:v>当前网页无象；规则与造型 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="32" customHeight="1">
-      <x:c r="A22" s="7" t="str">
+        <x:v>建议棋子脚底或头像状态标识；正式形式 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="38" customHeight="1">
+      <x:c r="A22" s="8" t="str">
         <x:v>A-017</x:v>
       </x:c>
       <x:c r="B22" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形效果</x:v>
       </x:c>
       <x:c r="C22" s="8" t="str">
-        <x:v>敌方马</x:v>
+        <x:v>冲击遇水中断</x:v>
       </x:c>
       <x:c r="D22" s="8" t="str">
-        <x:v>1款／标准2枚</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E22" s="8" t="str">
-        <x:v>完整中国象棋黑方名录</x:v>
+        <x:v>车冲锋首次进入水域</x:v>
       </x:c>
       <x:c r="F22" s="8" t="str">
-        <x:v>通用棋子绘制可显示“马”字；未编队</x:v>
+        <x:v>棋子停在首个水格＋战报文字</x:v>
       </x:c>
       <x:c r="G22" s="8" t="str">
-        <x:v>未编队</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H22" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30; web/js/rules.js:8-9</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:112</x:v>
       </x:c>
       <x:c r="I22" s="8" t="str">
-        <x:v>当前两波敌阵均无马</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="32" customHeight="1">
-      <x:c r="A23" s="7" t="str">
+        <x:v>需要速度骤停、浪花和未造成伤害的清晰反馈</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="38" customHeight="1">
+      <x:c r="A23" s="8" t="str">
         <x:v>A-018</x:v>
       </x:c>
       <x:c r="B23" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形效果</x:v>
       </x:c>
       <x:c r="C23" s="8" t="str">
-        <x:v>敌方车</x:v>
+        <x:v>推水环境击杀</x:v>
       </x:c>
       <x:c r="D23" s="8" t="str">
-        <x:v>1款／标准2枚</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E23" s="8" t="str">
-        <x:v>两波敌阵</x:v>
+        <x:v>目标被推入水域并阵亡</x:v>
       </x:c>
       <x:c r="F23" s="8" t="str">
-        <x:v>蓝色方块＋“车”字</x:v>
+        <x:v>目标移除＋战报文字</x:v>
       </x:c>
       <x:c r="G23" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H23" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:54</x:v>
       </x:c>
       <x:c r="I23" s="8" t="str">
-        <x:v>原型每波一枚；标准整副为两枚</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="32" customHeight="1">
-      <x:c r="A24" s="7" t="str">
+        <x:v>与普通入水阵亡共用主体，补充推动方向与击杀归属</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="38" customHeight="1">
+      <x:c r="A24" s="8" t="str">
         <x:v>A-019</x:v>
       </x:c>
       <x:c r="B24" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形效果</x:v>
       </x:c>
       <x:c r="C24" s="8" t="str">
-        <x:v>敌方炮</x:v>
+        <x:v>山体受击</x:v>
       </x:c>
       <x:c r="D24" s="8" t="str">
-        <x:v>1款／标准2枚</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E24" s="8" t="str">
-        <x:v>两波敌阵</x:v>
+        <x:v>攻击命中山体</x:v>
       </x:c>
       <x:c r="F24" s="8" t="str">
-        <x:v>蓝色方块＋“炮”字</x:v>
+        <x:v>山体状态即时切换</x:v>
       </x:c>
       <x:c r="G24" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H24" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:120-125</x:v>
       </x:c>
       <x:c r="I24" s="8" t="str">
-        <x:v>原型每波一枚；标准整副为两枚</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="32" customHeight="1">
-      <x:c r="A25" s="7" t="str">
+        <x:v>命中伤害数值不影响阶段推进；尘屑与震动强度 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="38" customHeight="1">
+      <x:c r="A25" s="8" t="str">
         <x:v>A-020</x:v>
       </x:c>
       <x:c r="B25" s="8" t="str">
-        <x:v>棋子</x:v>
+        <x:v>地形效果</x:v>
       </x:c>
       <x:c r="C25" s="8" t="str">
-        <x:v>敌方卒</x:v>
+        <x:v>山体开裂</x:v>
       </x:c>
       <x:c r="D25" s="8" t="str">
-        <x:v>1款／标准5枚</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E25" s="8" t="str">
-        <x:v>两波敌阵</x:v>
+        <x:v>完整山体首次有效受击</x:v>
       </x:c>
       <x:c r="F25" s="8" t="str">
-        <x:v>蓝色方块＋“兵”字</x:v>
+        <x:v>▲ 切换为 ◭</x:v>
       </x:c>
       <x:c r="G25" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H25" s="8" t="str">
-        <x:v>web/js/app.js:4-6,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:120-125</x:v>
       </x:c>
       <x:c r="I25" s="8" t="str">
-        <x:v>标准黑方称“卒”；当前网页仍显示“兵”</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="32" customHeight="1">
-      <x:c r="A26" s="7" t="str">
+        <x:v>需要裂纹扩散或掉石过渡；持续时间 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="38" customHeight="1">
+      <x:c r="A26" s="8" t="str">
         <x:v>A-021</x:v>
       </x:c>
       <x:c r="B26" s="8" t="str">
-        <x:v>扩展棋子</x:v>
+        <x:v>地形效果</x:v>
       </x:c>
       <x:c r="C26" s="8" t="str">
-        <x:v>己方弓兵</x:v>
+        <x:v>山体坍塌</x:v>
       </x:c>
       <x:c r="D26" s="8" t="str">
-        <x:v>1种</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E26" s="8" t="str">
-        <x:v>兵转职；测试夹具</x:v>
+        <x:v>开裂山体再次有效受击</x:v>
       </x:c>
       <x:c r="F26" s="8" t="str">
-        <x:v>红色圆柱＋“弓”字</x:v>
+        <x:v>◭ 切换为碎石陆地</x:v>
       </x:c>
       <x:c r="G26" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H26" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:120-125</x:v>
       </x:c>
       <x:c r="I26" s="8" t="str">
-        <x:v>项目特有转职，不计入传统七类</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="32" customHeight="1">
-      <x:c r="A27" s="7" t="str">
+        <x:v>需要明确表现地形已可通行；扬尘范围与时长 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="38" customHeight="1">
+      <x:c r="A27" s="8" t="str">
         <x:v>A-022</x:v>
       </x:c>
       <x:c r="B27" s="8" t="str">
-        <x:v>扩展棋子</x:v>
+        <x:v>地形效果</x:v>
       </x:c>
       <x:c r="C27" s="8" t="str">
-        <x:v>己方枪兵</x:v>
+        <x:v>山体炮架高亮</x:v>
       </x:c>
       <x:c r="D27" s="8" t="str">
-        <x:v>1种</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E27" s="8" t="str">
-        <x:v>兵转职；测试夹具</x:v>
+        <x:v>炮攻击预览与结算</x:v>
       </x:c>
       <x:c r="F27" s="8" t="str">
-        <x:v>红色圆柱＋“枪”字</x:v>
+        <x:v>仅规则判定，无独立视觉</x:v>
       </x:c>
       <x:c r="G27" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H27" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:120-125</x:v>
       </x:c>
       <x:c r="I27" s="8" t="str">
-        <x:v>项目特有转职，不计入传统七类</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="32" customHeight="1">
-      <x:c r="A28" s="7" t="str">
+        <x:v>山可作为一个炮架；用于提示炮线中的架点，正式样式 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="38" customHeight="1">
+      <x:c r="A28" s="8" t="str">
         <x:v>A-023</x:v>
       </x:c>
       <x:c r="B28" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>地形效果</x:v>
       </x:c>
       <x:c r="C28" s="8" t="str">
-        <x:v>全体｜击杀成长反馈</x:v>
+        <x:v>树林掩护状态</x:v>
       </x:c>
       <x:c r="D28" s="8" t="str">
-        <x:v>9棋种通用</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E28" s="8" t="str">
-        <x:v>己方棋子击杀后 Lv、SP 与击杀数增加</x:v>
+        <x:v>棋子位于树林内</x:v>
       </x:c>
       <x:c r="F28" s="8" t="str">
-        <x:v>仅数值文字刷新；无独立特效资产</x:v>
+        <x:v>状态栏文字提示</x:v>
       </x:c>
       <x:c r="G28" s="8" t="str">
         <x:v>待制作</x:v>
       </x:c>
       <x:c r="H28" s="8" t="str">
-        <x:v>web/js/rules.js:38; web/js/app.js:37-40</x:v>
+        <x:v>web/experiments/terrain-wave/app.js:125-128；rules.js:174</x:v>
       </x:c>
       <x:c r="I28" s="8" t="str">
-        <x:v>建议包含棋子归属、等级提升和 SP 获得反馈</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="32" customHeight="1">
-      <x:c r="A29" s="7" t="str">
+        <x:v>所有攻击类型均适用；需要持续但不遮挡棋子的环境反馈</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="38" customHeight="1">
+      <x:c r="A29" s="8" t="str">
         <x:v>A-024</x:v>
       </x:c>
       <x:c r="B29" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>地形效果</x:v>
       </x:c>
       <x:c r="C29" s="8" t="str">
-        <x:v>全体｜强健升级</x:v>
+        <x:v>树林闪避／MISS</x:v>
       </x:c>
       <x:c r="D29" s="8" t="str">
-        <x:v>9棋种通用</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E29" s="8" t="str">
-        <x:v>己方存活棋子当前／最大 HP +1</x:v>
+        <x:v>树林闪避判定成功</x:v>
       </x:c>
       <x:c r="F29" s="8" t="str">
-        <x:v>仅按钮和 HP 数值刷新</x:v>
+        <x:v>战报文字；伤害与推动取消</x:v>
       </x:c>
       <x:c r="G29" s="8" t="str">
         <x:v>待制作</x:v>
       </x:c>
       <x:c r="H29" s="8" t="str">
-        <x:v>web/js/app.js:42; web/js/rules.js:53</x:v>
+        <x:v>web/experiments/terrain-wave/rules.js:174</x:v>
       </x:c>
       <x:c r="I29" s="8" t="str">
-        <x:v>帅、仕、相、马、车、炮、兵、弓兵、枪兵共用；仕／相规则仍 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="32" customHeight="1">
-      <x:c r="A30" s="7" t="str">
+        <x:v>结算后再揭示结果；可包含残影、落叶或 MISS 字样，正式方案 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="38" customHeight="1">
+      <x:c r="A30" s="8" t="str">
         <x:v>A-025</x:v>
       </x:c>
       <x:c r="B30" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>地形界面</x:v>
       </x:c>
       <x:c r="C30" s="8" t="str">
-        <x:v>帅｜专属技能效果预留</x:v>
+        <x:v>地图编辑地形画笔图标</x:v>
       </x:c>
       <x:c r="D30" s="8" t="str">
-        <x:v>1槽</x:v>
+        <x:v>6款</x:v>
       </x:c>
       <x:c r="E30" s="8" t="str">
-        <x:v>己方帅未来专属技能</x:v>
+        <x:v>陆地／水／桥／山／开裂山／树林画笔</x:v>
       </x:c>
       <x:c r="F30" s="8" t="str">
-        <x:v>无</x:v>
+        <x:v>字符图标：▧／≈／▰／▲／◭／♠</x:v>
       </x:c>
       <x:c r="G30" s="8" t="str">
-        <x:v>预留（规则TBD）</x:v>
+        <x:v>代码占位（独立实验）</x:v>
       </x:c>
       <x:c r="H30" s="8" t="str">
-        <x:v>用户要求预留所有己方棋子技能效果</x:v>
+        <x:v>web/experiments/terrain-wave/app.js:7</x:v>
       </x:c>
       <x:c r="I30" s="8" t="str">
-        <x:v>当前只有通用强健；技能名称、触发和表现 TBD</x:v>
+        <x:v>坍塌碎石为战斗状态，不作为当前画笔；正式图标 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="32" customHeight="1">
-      <x:c r="A31" s="7" t="str">
+      <x:c r="A31" s="8" t="str">
         <x:v>A-026</x:v>
       </x:c>
       <x:c r="B31" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C31" s="8" t="str">
-        <x:v>仕｜专属技能效果预留</x:v>
+        <x:v>己方帅</x:v>
       </x:c>
       <x:c r="D31" s="8" t="str">
-        <x:v>1槽</x:v>
+        <x:v>1款／标准1枚</x:v>
       </x:c>
       <x:c r="E31" s="8" t="str">
-        <x:v>己方仕未来专属技能</x:v>
+        <x:v>己方主帅</x:v>
       </x:c>
       <x:c r="F31" s="8" t="str">
-        <x:v>无</x:v>
+        <x:v>红色圆柱＋“帅”字</x:v>
       </x:c>
       <x:c r="G31" s="8" t="str">
-        <x:v>预留（规则TBD）</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H31" s="8" t="str">
-        <x:v>用户要求预留所有己方棋子技能效果</x:v>
+        <x:v>web/js/app.js:4-6,29-30</x:v>
       </x:c>
       <x:c r="I31" s="8" t="str">
-        <x:v>己方仕尚未进入规则；技能名称、触发和表现 TBD</x:v>
+        <x:v>中国象棋红方棋种；正式形象 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="32" customHeight="1">
-      <x:c r="A32" s="7" t="str">
+      <x:c r="A32" s="8" t="str">
         <x:v>A-027</x:v>
       </x:c>
       <x:c r="B32" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C32" s="8" t="str">
-        <x:v>相｜专属技能效果预留</x:v>
+        <x:v>己方仕</x:v>
       </x:c>
       <x:c r="D32" s="8" t="str">
-        <x:v>1槽</x:v>
+        <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E32" s="8" t="str">
-        <x:v>己方相未来专属技能</x:v>
+        <x:v>完整中国象棋红方名录</x:v>
       </x:c>
       <x:c r="F32" s="8" t="str">
-        <x:v>无</x:v>
+        <x:v>无（当前未配置）</x:v>
       </x:c>
       <x:c r="G32" s="8" t="str">
-        <x:v>预留（规则TBD）</x:v>
+        <x:v>未实现</x:v>
       </x:c>
       <x:c r="H32" s="8" t="str">
-        <x:v>用户要求预留所有己方棋子技能效果</x:v>
+        <x:v>中国象棋棋种；用户补充</x:v>
       </x:c>
       <x:c r="I32" s="8" t="str">
-        <x:v>己方相尚未进入规则；技能名称、触发和表现 TBD</x:v>
+        <x:v>当前网页无己方仕；规则与造型 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="32" customHeight="1">
-      <x:c r="A33" s="7" t="str">
+      <x:c r="A33" s="8" t="str">
         <x:v>A-028</x:v>
       </x:c>
       <x:c r="B33" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C33" s="8" t="str">
-        <x:v>马｜专属技能效果预留</x:v>
+        <x:v>己方相</x:v>
       </x:c>
       <x:c r="D33" s="8" t="str">
-        <x:v>1槽</x:v>
+        <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E33" s="8" t="str">
-        <x:v>己方马未来专属技能</x:v>
+        <x:v>完整中国象棋红方名录</x:v>
       </x:c>
       <x:c r="F33" s="8" t="str">
-        <x:v>无</x:v>
+        <x:v>无（当前未配置）</x:v>
       </x:c>
       <x:c r="G33" s="8" t="str">
-        <x:v>预留（规则TBD）</x:v>
+        <x:v>未实现</x:v>
       </x:c>
       <x:c r="H33" s="8" t="str">
-        <x:v>docs/us/US-001-m0-player-skills.md:2.2</x:v>
+        <x:v>中国象棋棋种；用户补充</x:v>
       </x:c>
       <x:c r="I33" s="8" t="str">
-        <x:v>当前马只有基础走法和通用强健；专属技能 TBD</x:v>
+        <x:v>当前网页无相；规则与造型 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="32" customHeight="1">
-      <x:c r="A34" s="7" t="str">
+      <x:c r="A34" s="8" t="str">
         <x:v>A-029</x:v>
       </x:c>
       <x:c r="B34" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C34" s="8" t="str">
-        <x:v>车｜疾行移动</x:v>
+        <x:v>己方马</x:v>
       </x:c>
       <x:c r="D34" s="8" t="str">
-        <x:v>直线4方向</x:v>
+        <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E34" s="8" t="str">
-        <x:v>执行独立普通移动</x:v>
+        <x:v>首波商店购买</x:v>
       </x:c>
       <x:c r="F34" s="8" t="str">
-        <x:v>棋位圆点与瞬时位移；无移动特效资产</x:v>
+        <x:v>红色圆柱＋“马”字</x:v>
       </x:c>
       <x:c r="G34" s="8" t="str">
-        <x:v>待制作</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H34" s="8" t="str">
-        <x:v>web/js/app.js:59,64; web/js/rules.js:31,43</x:v>
+        <x:v>web/js/app.js:4-5,29-30</x:v>
       </x:c>
       <x:c r="I34" s="8" t="str">
-        <x:v>表现起点、路径、终点和剩余移动额度</x:v>
+        <x:v>原型最多购买一枚；标准整副为两枚</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="32" customHeight="1">
-      <x:c r="A35" s="7" t="str">
+      <x:c r="A35" s="8" t="str">
         <x:v>A-030</x:v>
       </x:c>
       <x:c r="B35" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C35" s="8" t="str">
-        <x:v>车｜疾行升级</x:v>
+        <x:v>己方车</x:v>
       </x:c>
       <x:c r="D35" s="8" t="str">
-        <x:v>1套／等级变化</x:v>
+        <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E35" s="8" t="str">
-        <x:v>普通移动距离 +1</x:v>
+        <x:v>初始队伍</x:v>
       </x:c>
       <x:c r="F35" s="8" t="str">
-        <x:v>仅技能按钮和距离数值刷新</x:v>
+        <x:v>红色圆柱＋“车”字</x:v>
       </x:c>
       <x:c r="G35" s="8" t="str">
-        <x:v>待制作</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H35" s="8" t="str">
-        <x:v>web/js/app.js:50; web/js/rules.js:53</x:v>
+        <x:v>web/js/app.js:4-5,29-30</x:v>
       </x:c>
       <x:c r="I35" s="8" t="str">
-        <x:v>最高 7 格；升级反馈需区别于实际移动</x:v>
+        <x:v>原型初始一枚；标准整副为两枚</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="32" customHeight="1">
-      <x:c r="A36" s="7" t="str">
+      <x:c r="A36" s="8" t="str">
         <x:v>A-031</x:v>
       </x:c>
       <x:c r="B36" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C36" s="8" t="str">
-        <x:v>车｜冲击</x:v>
+        <x:v>己方炮</x:v>
       </x:c>
       <x:c r="D36" s="8" t="str">
-        <x:v>直线4方向</x:v>
+        <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E36" s="8" t="str">
-        <x:v>冲向空格或敌人</x:v>
+        <x:v>首波商店购买</x:v>
       </x:c>
       <x:c r="F36" s="8" t="str">
-        <x:v>目标圆点和文字预览；无冲击特效资产</x:v>
+        <x:v>红色圆柱＋“炮”字</x:v>
       </x:c>
       <x:c r="G36" s="8" t="str">
-        <x:v>待制作</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H36" s="8" t="str">
-        <x:v>web/js/app.js:59,64; web/js/rules.js:42-46</x:v>
+        <x:v>web/js/app.js:4-5,29-30</x:v>
       </x:c>
       <x:c r="I36" s="8" t="str">
-        <x:v>需覆盖空冲、接近点、击杀占位和未击杀停前格</x:v>
+        <x:v>原型最多购买一枚；标准整副为两枚</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="32" customHeight="1">
-      <x:c r="A37" s="7" t="str">
+      <x:c r="A37" s="8" t="str">
         <x:v>A-032</x:v>
       </x:c>
       <x:c r="B37" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C37" s="8" t="str">
-        <x:v>车｜冲击延伸升级</x:v>
+        <x:v>己方兵</x:v>
       </x:c>
       <x:c r="D37" s="8" t="str">
-        <x:v>1套／等级变化</x:v>
+        <x:v>1款／标准5枚</x:v>
       </x:c>
       <x:c r="E37" s="8" t="str">
-        <x:v>冲击距离 +1</x:v>
+        <x:v>P1 等测试夹具</x:v>
       </x:c>
       <x:c r="F37" s="8" t="str">
-        <x:v>仅技能按钮和距离数值刷新</x:v>
+        <x:v>红色圆柱＋“兵”字</x:v>
       </x:c>
       <x:c r="G37" s="8" t="str">
-        <x:v>待制作</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H37" s="8" t="str">
-        <x:v>web/js/app.js:51; web/js/rules.js:53</x:v>
+        <x:v>web/js/app.js:4-5,29-30</x:v>
       </x:c>
       <x:c r="I37" s="8" t="str">
-        <x:v>最高 7 格；与疾行升级使用不同辨识</x:v>
+        <x:v>正式局未提供招募；标准整副为五枚</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="32" customHeight="1">
-      <x:c r="A38" s="7" t="str">
+      <x:c r="A38" s="8" t="str">
         <x:v>A-033</x:v>
       </x:c>
       <x:c r="B38" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C38" s="8" t="str">
-        <x:v>车｜震退解锁</x:v>
+        <x:v>敌方将</x:v>
       </x:c>
       <x:c r="D38" s="8" t="str">
-        <x:v>1套</x:v>
+        <x:v>1款／标准1枚</x:v>
       </x:c>
       <x:c r="E38" s="8" t="str">
-        <x:v>花费 2 SP 解锁震退</x:v>
+        <x:v>两波敌将</x:v>
       </x:c>
       <x:c r="F38" s="8" t="str">
-        <x:v>仅按钮状态与文字刷新</x:v>
+        <x:v>蓝色方块＋“将”字</x:v>
       </x:c>
       <x:c r="G38" s="8" t="str">
-        <x:v>待制作</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H38" s="8" t="str">
-        <x:v>web/js/app.js:52; web/js/rules.js:53</x:v>
+        <x:v>web/js/app.js:4-6,29-30</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>表现永久解锁，不能误解为一次性攻击</x:v>
+        <x:v>中国象棋黑方棋种；正式形象 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="32" customHeight="1">
-      <x:c r="A39" s="7" t="str">
+      <x:c r="A39" s="8" t="str">
         <x:v>A-034</x:v>
       </x:c>
       <x:c r="B39" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C39" s="8" t="str">
-        <x:v>车｜震退命中</x:v>
+        <x:v>敌方士</x:v>
       </x:c>
       <x:c r="D39" s="8" t="str">
-        <x:v>成功／受阻4态</x:v>
+        <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E39" s="8" t="str">
-        <x:v>冲击命中存活目标后推 1 格</x:v>
+        <x:v>两波敌阵</x:v>
       </x:c>
       <x:c r="F39" s="8" t="str">
-        <x:v>仅位置变化与文字结果</x:v>
+        <x:v>蓝色方块＋“士”字</x:v>
       </x:c>
       <x:c r="G39" s="8" t="str">
-        <x:v>待制作</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H39" s="8" t="str">
-        <x:v>web/js/app.js:64; web/js/rules.js:42-46</x:v>
+        <x:v>web/js/app.js:4-5,29-30</x:v>
       </x:c>
       <x:c r="I39" s="8" t="str">
-        <x:v>区分成功、出界、宫界和占位受阻</x:v>
+        <x:v>当前每波两枚；正式形象 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="32" customHeight="1">
-      <x:c r="A40" s="7" t="str">
+      <x:c r="A40" s="8" t="str">
         <x:v>A-035</x:v>
       </x:c>
       <x:c r="B40" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C40" s="8" t="str">
-        <x:v>炮｜基础炮击</x:v>
+        <x:v>敌方象</x:v>
       </x:c>
       <x:c r="D40" s="8" t="str">
-        <x:v>横竖4方向</x:v>
+        <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E40" s="8" t="str">
-        <x:v>隔恰好一个炮架攻击单目标</x:v>
+        <x:v>完整中国象棋黑方名录</x:v>
       </x:c>
       <x:c r="F40" s="8" t="str">
-        <x:v>路径、炮架、目标圆点与文字预览</x:v>
+        <x:v>无（当前未配置）</x:v>
       </x:c>
       <x:c r="G40" s="8" t="str">
-        <x:v>待制作</x:v>
+        <x:v>未实现</x:v>
       </x:c>
       <x:c r="H40" s="8" t="str">
-        <x:v>web/js/app.js:64; docs/us/US-001-cannon-fix.md:20-25</x:v>
+        <x:v>中国象棋棋种；用户补充</x:v>
       </x:c>
       <x:c r="I40" s="8" t="str">
-        <x:v>需表现发射、越过炮架、命中和 2 点伤害</x:v>
+        <x:v>当前网页无象；规则与造型 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="32" customHeight="1">
-      <x:c r="A41" s="7" t="str">
+      <x:c r="A41" s="8" t="str">
         <x:v>A-036</x:v>
       </x:c>
       <x:c r="B41" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C41" s="8" t="str">
-        <x:v>炮｜炮架充能／弹道</x:v>
+        <x:v>敌方马</x:v>
       </x:c>
       <x:c r="D41" s="8" t="str">
-        <x:v>敌友炮架2态</x:v>
+        <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E41" s="8" t="str">
-        <x:v>炮击前识别唯一炮架</x:v>
+        <x:v>完整中国象棋黑方名录</x:v>
       </x:c>
       <x:c r="F41" s="8" t="str">
-        <x:v>紫色炮架点＋黄色路径点</x:v>
+        <x:v>通用棋子绘制可显示“马”字；未编队</x:v>
       </x:c>
       <x:c r="G41" s="8" t="str">
-        <x:v>待制作</x:v>
+        <x:v>未编队</x:v>
       </x:c>
       <x:c r="H41" s="8" t="str">
-        <x:v>web/js/app.js:34,64</x:v>
+        <x:v>web/js/app.js:4-5,29-30; web/js/rules.js:8-9</x:v>
       </x:c>
       <x:c r="I41" s="8" t="str">
-        <x:v>友军与敌军均可作炮架；不要表现为炮架受益</x:v>
+        <x:v>当前两波敌阵均无马</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="32" customHeight="1">
-      <x:c r="A42" s="7" t="str">
+      <x:c r="A42" s="8" t="str">
         <x:v>A-037</x:v>
       </x:c>
       <x:c r="B42" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C42" s="8" t="str">
-        <x:v>炮｜扩散解锁</x:v>
+        <x:v>敌方车</x:v>
       </x:c>
       <x:c r="D42" s="8" t="str">
-        <x:v>8方向变体</x:v>
+        <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E42" s="8" t="str">
-        <x:v>逐个解锁目标邻格 N／NE／E／SE／S／SW／W／NW</x:v>
+        <x:v>两波敌阵</x:v>
       </x:c>
       <x:c r="F42" s="8" t="str">
-        <x:v>仅技能按钮和扩散计数刷新</x:v>
+        <x:v>蓝色方块＋“车”字</x:v>
       </x:c>
       <x:c r="G42" s="8" t="str">
-        <x:v>待制作</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H42" s="8" t="str">
-        <x:v>web/js/app.js:53-54; web/js/rules.js:53</x:v>
+        <x:v>web/js/app.js:4-5,29-30</x:v>
       </x:c>
       <x:c r="I42" s="8" t="str">
-        <x:v>固定朝向、不随开炮方向旋转；每格 1 SP</x:v>
+        <x:v>原型每波一枚；标准整副为两枚</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="32" customHeight="1">
-      <x:c r="A43" s="7" t="str">
+      <x:c r="A43" s="8" t="str">
         <x:v>A-038</x:v>
       </x:c>
       <x:c r="B43" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C43" s="8" t="str">
-        <x:v>炮｜扩散命中</x:v>
+        <x:v>敌方炮</x:v>
       </x:c>
       <x:c r="D43" s="8" t="str">
-        <x:v>主目标＋最多8邻格</x:v>
+        <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E43" s="8" t="str">
-        <x:v>炮击时对已解锁邻格同时造成伤害</x:v>
+        <x:v>两波敌阵</x:v>
       </x:c>
       <x:c r="F43" s="8" t="str">
-        <x:v>预览列出命中；无范围爆炸特效资产</x:v>
+        <x:v>蓝色方块＋“炮”字</x:v>
       </x:c>
       <x:c r="G43" s="8" t="str">
-        <x:v>待制作</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H43" s="8" t="str">
-        <x:v>web/js/app.js:64; web/js/rules.js:45</x:v>
+        <x:v>web/js/app.js:4-5,29-30</x:v>
       </x:c>
       <x:c r="I43" s="8" t="str">
-        <x:v>包含友伤和边界裁切；主目标与扩散命中需分层</x:v>
+        <x:v>原型每波一枚；标准整副为两枚</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="32" customHeight="1">
-      <x:c r="A44" s="7" t="str">
+      <x:c r="A44" s="8" t="str">
         <x:v>A-039</x:v>
       </x:c>
       <x:c r="B44" s="8" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>棋子</x:v>
       </x:c>
       <x:c r="C44" s="8" t="str">
-        <x:v>兵｜连动升级</x:v>
+        <x:v>敌方卒</x:v>
       </x:c>
       <x:c r="D44" s="8" t="str">
-        <x:v>1套／可重复</x:v>
+        <x:v>1款／标准5枚</x:v>
       </x:c>
       <x:c r="E44" s="8" t="str">
-        <x:v>花费 2 SP，使下回合 AP 上限 +1</x:v>
+        <x:v>两波敌阵</x:v>
       </x:c>
       <x:c r="F44" s="8" t="str">
-        <x:v>仅技能按钮和数值刷新</x:v>
+        <x:v>蓝色方块＋“兵”字</x:v>
       </x:c>
       <x:c r="G44" s="8" t="str">
-        <x:v>待制作</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H44" s="8" t="str">
-        <x:v>web/js/app.js:46; web/js/rules.js:19,53</x:v>
+        <x:v>web/js/app.js:4-6,29-30</x:v>
       </x:c>
       <x:c r="I44" s="8" t="str">
-        <x:v>升级时与下回合实际生效时分别反馈</x:v>
+        <x:v>标准黑方称“卒”；当前网页仍显示“兵”</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="32" customHeight="1">
-      <x:c r="A45" s="10" t="str">
+      <x:c r="A45" s="11" t="str">
         <x:v>A-040</x:v>
       </x:c>
       <x:c r="B45" s="11" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>扩展棋子</x:v>
       </x:c>
       <x:c r="C45" s="11" t="str">
-        <x:v>兵｜额外行动激活</x:v>
+        <x:v>己方弓兵</x:v>
       </x:c>
       <x:c r="D45" s="11" t="str">
-        <x:v>1套／层数变化</x:v>
+        <x:v>1种</x:v>
       </x:c>
       <x:c r="E45" s="11" t="str">
-        <x:v>连动在下一回合增加可用 AP</x:v>
+        <x:v>兵转职；测试夹具</x:v>
       </x:c>
       <x:c r="F45" s="11" t="str">
-        <x:v>仅 AP 数字变化</x:v>
+        <x:v>红色圆柱＋“弓”字</x:v>
       </x:c>
       <x:c r="G45" s="11" t="str">
-        <x:v>待制作</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H45" s="11" t="str">
-        <x:v>web/js/rules.js:19</x:v>
+        <x:v>web/js/app.js:4-5,29-30</x:v>
       </x:c>
       <x:c r="I45" s="11" t="str">
-        <x:v>需显示新增行动次数和已消耗层次</x:v>
+        <x:v>项目特有转职，不计入传统七类</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="32" customHeight="1">
-      <x:c r="A46" s="10" t="str">
+      <x:c r="A46" s="11" t="str">
         <x:v>A-041</x:v>
       </x:c>
       <x:c r="B46" s="11" t="str">
-        <x:v>己方技能效果</x:v>
+        <x:v>扩展棋子</x:v>
       </x:c>
       <x:c r="C46" s="11" t="str">
-        <x:v>兵｜转职弓兵</x:v>
+        <x:v>己方枪兵</x:v>
       </x:c>
       <x:c r="D46" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>1种</x:v>
       </x:c>
       <x:c r="E46" s="11" t="str">
-        <x:v>花费 2 SP，兵变为弓兵并获得攻击加成</x:v>
+        <x:v>兵转职；测试夹具</x:v>
       </x:c>
       <x:c r="F46" s="11" t="str">
-        <x:v>棋子字样与属性瞬时变化</x:v>
+        <x:v>红色圆柱＋“枪”字</x:v>
       </x:c>
       <x:c r="G46" s="11" t="str">
-        <x:v>待制作</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H46" s="11" t="str">
-        <x:v>web/js/app.js:44; web/js/rules.js:53</x:v>
+        <x:v>web/js/app.js:4-5,29-30</x:v>
       </x:c>
       <x:c r="I46" s="11" t="str">
-        <x:v>保留原棋子身份、伤势和剩余 AP</x:v>
+        <x:v>项目特有转职，不计入传统七类</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="32" customHeight="1">
-      <x:c r="A47" s="10" t="str">
+      <x:c r="A47" s="11" t="str">
         <x:v>A-042</x:v>
       </x:c>
       <x:c r="B47" s="11" t="str">
         <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C47" s="11" t="str">
-        <x:v>兵｜转职枪兵</x:v>
+        <x:v>全体｜击杀成长反馈</x:v>
       </x:c>
       <x:c r="D47" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>9棋种通用</x:v>
       </x:c>
       <x:c r="E47" s="11" t="str">
-        <x:v>花费 2 SP，兵变为枪兵并获得 HP</x:v>
+        <x:v>己方棋子击杀后 Lv、SP 与击杀数增加</x:v>
       </x:c>
       <x:c r="F47" s="11" t="str">
-        <x:v>棋子字样与属性瞬时变化</x:v>
+        <x:v>仅数值文字刷新；无独立特效资产</x:v>
       </x:c>
       <x:c r="G47" s="11" t="str">
         <x:v>待制作</x:v>
       </x:c>
       <x:c r="H47" s="11" t="str">
-        <x:v>web/js/app.js:45; web/js/rules.js:53</x:v>
+        <x:v>web/js/rules.js:38; web/js/app.js:37-40</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
-        <x:v>保留原棋子身份、伤势和剩余 AP</x:v>
+        <x:v>建议包含棋子归属、等级提升和 SP 获得反馈</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="32" customHeight="1">
-      <x:c r="A48" s="10" t="str">
+      <x:c r="A48" s="11" t="str">
         <x:v>A-043</x:v>
       </x:c>
       <x:c r="B48" s="11" t="str">
         <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C48" s="11" t="str">
-        <x:v>弓兵｜四向射击</x:v>
+        <x:v>全体｜强健升级</x:v>
       </x:c>
       <x:c r="D48" s="11" t="str">
-        <x:v>前／右／后／左</x:v>
+        <x:v>9棋种通用</x:v>
       </x:c>
       <x:c r="E48" s="11" t="str">
-        <x:v>选一个方向，命中范围内首个敌人</x:v>
+        <x:v>己方存活棋子当前／最大 HP +1</x:v>
       </x:c>
       <x:c r="F48" s="11" t="str">
-        <x:v>黄色范围点和命中预览；无箭矢特效资产</x:v>
+        <x:v>仅按钮和 HP 数值刷新</x:v>
       </x:c>
       <x:c r="G48" s="11" t="str">
         <x:v>待制作</x:v>
       </x:c>
       <x:c r="H48" s="11" t="str">
-        <x:v>web/js/app.js:59,64; web/js/rules.js:35</x:v>
+        <x:v>web/js/app.js:42; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I48" s="11" t="str">
-        <x:v>友军阻挡；需表现首个目标和 2 点伤害</x:v>
+        <x:v>帅、仕、相、马、车、炮、兵、弓兵、枪兵共用；仕／相规则仍 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="32" customHeight="1">
-      <x:c r="A49" s="10" t="str">
+      <x:c r="A49" s="11" t="str">
         <x:v>A-044</x:v>
       </x:c>
       <x:c r="B49" s="11" t="str">
         <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C49" s="11" t="str">
-        <x:v>弓兵｜方向射程升级</x:v>
+        <x:v>帅｜专属技能效果预留</x:v>
       </x:c>
       <x:c r="D49" s="11" t="str">
-        <x:v>4方向×6级</x:v>
+        <x:v>1槽</x:v>
       </x:c>
       <x:c r="E49" s="11" t="str">
-        <x:v>单方向每次 +1 格，最高 Lv.8／7格</x:v>
+        <x:v>己方帅未来专属技能</x:v>
       </x:c>
       <x:c r="F49" s="11" t="str">
-        <x:v>仅方向按钮等级和距离文字刷新</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="G49" s="11" t="str">
-        <x:v>待制作</x:v>
+        <x:v>预留（规则TBD）</x:v>
       </x:c>
       <x:c r="H49" s="11" t="str">
-        <x:v>web/js/app.js:47-48; web/js/rules.js:53</x:v>
+        <x:v>用户要求预留所有己方棋子技能效果</x:v>
       </x:c>
       <x:c r="I49" s="11" t="str">
-        <x:v>四方向独立，升级反馈须标明具体方向</x:v>
+        <x:v>当前只有通用强健；技能名称、触发和表现 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="32" customHeight="1">
-      <x:c r="A50" s="10" t="str">
+      <x:c r="A50" s="11" t="str">
         <x:v>A-045</x:v>
       </x:c>
       <x:c r="B50" s="11" t="str">
         <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C50" s="11" t="str">
-        <x:v>枪兵｜四向贯穿攻击</x:v>
+        <x:v>仕｜专属技能效果预留</x:v>
       </x:c>
       <x:c r="D50" s="11" t="str">
-        <x:v>前／右／后／左</x:v>
+        <x:v>1槽</x:v>
       </x:c>
       <x:c r="E50" s="11" t="str">
-        <x:v>选一个方向，命中线内所有敌人</x:v>
+        <x:v>己方仕未来专属技能</x:v>
       </x:c>
       <x:c r="F50" s="11" t="str">
-        <x:v>黄色范围点和命中列表；无枪击特效资产</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="G50" s="11" t="str">
-        <x:v>待制作</x:v>
+        <x:v>预留（规则TBD）</x:v>
       </x:c>
       <x:c r="H50" s="11" t="str">
-        <x:v>web/js/app.js:59,64; web/js/rules.js:35</x:v>
+        <x:v>用户要求预留所有己方棋子技能效果</x:v>
       </x:c>
       <x:c r="I50" s="11" t="str">
-        <x:v>空格和敌人不中断，友军阻断；各目标 1 点伤害</x:v>
+        <x:v>己方仕尚未进入规则；技能名称、触发和表现 TBD</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="32" customHeight="1">
-      <x:c r="A51" s="10" t="str">
+      <x:c r="A51" s="11" t="str">
         <x:v>A-046</x:v>
       </x:c>
       <x:c r="B51" s="11" t="str">
         <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C51" s="11" t="str">
-        <x:v>枪兵｜方向范围升级</x:v>
+        <x:v>相｜专属技能效果预留</x:v>
       </x:c>
       <x:c r="D51" s="11" t="str">
-        <x:v>4方向×6级</x:v>
+        <x:v>1槽</x:v>
       </x:c>
       <x:c r="E51" s="11" t="str">
-        <x:v>单方向每次 +1 格，最高 Lv.8／7格</x:v>
+        <x:v>己方相未来专属技能</x:v>
       </x:c>
       <x:c r="F51" s="11" t="str">
-        <x:v>仅方向按钮等级和距离文字刷新</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="G51" s="11" t="str">
+        <x:v>预留（规则TBD）</x:v>
+      </x:c>
+      <x:c r="H51" s="11" t="str">
+        <x:v>用户要求预留所有己方棋子技能效果</x:v>
+      </x:c>
+      <x:c r="I51" s="11" t="str">
+        <x:v>己方相尚未进入规则；技能名称、触发和表现 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="32" customHeight="1">
+      <x:c r="A52" s="11" t="str">
+        <x:v>A-047</x:v>
+      </x:c>
+      <x:c r="B52" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C52" s="11" t="str">
+        <x:v>马｜专属技能效果预留</x:v>
+      </x:c>
+      <x:c r="D52" s="11" t="str">
+        <x:v>1槽</x:v>
+      </x:c>
+      <x:c r="E52" s="11" t="str">
+        <x:v>己方马未来专属技能</x:v>
+      </x:c>
+      <x:c r="F52" s="11" t="str">
+        <x:v>无</x:v>
+      </x:c>
+      <x:c r="G52" s="11" t="str">
+        <x:v>预留（规则TBD）</x:v>
+      </x:c>
+      <x:c r="H52" s="11" t="str">
+        <x:v>docs/us/US-001-m0-player-skills.md:2.2</x:v>
+      </x:c>
+      <x:c r="I52" s="11" t="str">
+        <x:v>当前马只有基础走法和通用强健；专属技能 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="32" customHeight="1">
+      <x:c r="A53" s="11" t="str">
+        <x:v>A-048</x:v>
+      </x:c>
+      <x:c r="B53" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C53" s="11" t="str">
+        <x:v>车｜疾行移动</x:v>
+      </x:c>
+      <x:c r="D53" s="11" t="str">
+        <x:v>直线4方向</x:v>
+      </x:c>
+      <x:c r="E53" s="11" t="str">
+        <x:v>执行独立普通移动</x:v>
+      </x:c>
+      <x:c r="F53" s="11" t="str">
+        <x:v>棋位圆点与瞬时位移；无移动特效资产</x:v>
+      </x:c>
+      <x:c r="G53" s="11" t="str">
         <x:v>待制作</x:v>
       </x:c>
-      <x:c r="H51" s="11" t="str">
-        <x:v>web/js/app.js:47-48; web/js/rules.js:53</x:v>
-      </x:c>
-      <x:c r="I51" s="11" t="str">
-        <x:v>四方向独立；与弓兵升级可共用框架但视觉需可辨识</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="32" customHeight="1">
-      <x:c r="A52" s="10" t="str">
-        <x:v>A-047</x:v>
-      </x:c>
-      <x:c r="B52" s="11" t="str">
-        <x:v>操作标记</x:v>
-      </x:c>
-      <x:c r="C52" s="11" t="str">
-        <x:v>当前选中棋位</x:v>
-      </x:c>
-      <x:c r="D52" s="11" t="str">
-        <x:v>1种</x:v>
-      </x:c>
-      <x:c r="E52" s="11" t="str">
-        <x:v>选棋后标记起点</x:v>
-      </x:c>
-      <x:c r="F52" s="11" t="str">
-        <x:v>黄色半透明圆点</x:v>
-      </x:c>
-      <x:c r="G52" s="11" t="str">
-        <x:v>代码占位</x:v>
-      </x:c>
-      <x:c r="H52" s="11" t="str">
-        <x:v>web/js/app.js:33-34</x:v>
-      </x:c>
-      <x:c r="I52" s="11" t="str">
-        <x:v>需与其他标记可区分</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="32" customHeight="1">
-      <x:c r="A53" s="10" t="str">
-        <x:v>A-048</x:v>
-      </x:c>
-      <x:c r="B53" s="11" t="str">
-        <x:v>操作标记</x:v>
-      </x:c>
-      <x:c r="C53" s="11" t="str">
-        <x:v>合法移动落点</x:v>
-      </x:c>
-      <x:c r="D53" s="11" t="str">
-        <x:v>1种</x:v>
-      </x:c>
-      <x:c r="E53" s="11" t="str">
-        <x:v>移动选择</x:v>
-      </x:c>
-      <x:c r="F53" s="11" t="str">
-        <x:v>蓝色半透明圆点</x:v>
-      </x:c>
-      <x:c r="G53" s="11" t="str">
-        <x:v>代码占位</x:v>
-      </x:c>
       <x:c r="H53" s="11" t="str">
-        <x:v>web/js/app.js:33-34</x:v>
+        <x:v>web/js/app.js:59,64; web/js/rules.js:31,43</x:v>
       </x:c>
       <x:c r="I53" s="11" t="str">
-        <x:v>需兼顾窄屏识别</x:v>
+        <x:v>表现起点、路径、终点和剩余移动额度</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="32" customHeight="1">
-      <x:c r="A54" s="10" t="str">
+      <x:c r="A54" s="11" t="str">
         <x:v>A-049</x:v>
       </x:c>
       <x:c r="B54" s="11" t="str">
-        <x:v>操作标记</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C54" s="11" t="str">
-        <x:v>攻击与冲击目标</x:v>
+        <x:v>车｜疾行升级</x:v>
       </x:c>
       <x:c r="D54" s="11" t="str">
-        <x:v>1种</x:v>
+        <x:v>1套／等级变化</x:v>
       </x:c>
       <x:c r="E54" s="11" t="str">
-        <x:v>攻击或车冲击</x:v>
+        <x:v>普通移动距离 +1</x:v>
       </x:c>
       <x:c r="F54" s="11" t="str">
-        <x:v>红色半透明圆点</x:v>
+        <x:v>仅技能按钮和距离数值刷新</x:v>
       </x:c>
       <x:c r="G54" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H54" s="11" t="str">
-        <x:v>web/js/app.js:33-34</x:v>
+        <x:v>web/js/app.js:50; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I54" s="11" t="str">
-        <x:v>需与移动落点可区分</x:v>
+        <x:v>最高 7 格；升级反馈需区别于实际移动</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="32" customHeight="1">
-      <x:c r="A55" s="10" t="str">
+      <x:c r="A55" s="11" t="str">
         <x:v>A-050</x:v>
       </x:c>
       <x:c r="B55" s="11" t="str">
-        <x:v>操作标记</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C55" s="11" t="str">
-        <x:v>方向攻击范围</x:v>
+        <x:v>车｜冲击</x:v>
       </x:c>
       <x:c r="D55" s="11" t="str">
-        <x:v>1种</x:v>
+        <x:v>直线4方向</x:v>
       </x:c>
       <x:c r="E55" s="11" t="str">
-        <x:v>弓／枪四向预览</x:v>
+        <x:v>冲向空格或敌人</x:v>
       </x:c>
       <x:c r="F55" s="11" t="str">
-        <x:v>黄色路径圆点</x:v>
+        <x:v>目标圆点和文字预览；无冲击特效资产</x:v>
       </x:c>
       <x:c r="G55" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H55" s="11" t="str">
-        <x:v>web/js/app.js:59</x:v>
+        <x:v>web/js/app.js:59,64; web/js/rules.js:42-46</x:v>
       </x:c>
       <x:c r="I55" s="11" t="str">
-        <x:v>正式范围表现 TBD</x:v>
+        <x:v>需覆盖空冲、接近点、击杀占位和未击杀停前格</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="32" customHeight="1">
-      <x:c r="A56" s="10" t="str">
+      <x:c r="A56" s="11" t="str">
         <x:v>A-051</x:v>
       </x:c>
       <x:c r="B56" s="11" t="str">
-        <x:v>操作标记</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C56" s="11" t="str">
-        <x:v>炮击路径与炮架</x:v>
+        <x:v>车｜冲击延伸升级</x:v>
       </x:c>
       <x:c r="D56" s="11" t="str">
-        <x:v>2种</x:v>
+        <x:v>1套／等级变化</x:v>
       </x:c>
       <x:c r="E56" s="11" t="str">
-        <x:v>炮击预览</x:v>
+        <x:v>冲击距离 +1</x:v>
       </x:c>
       <x:c r="F56" s="11" t="str">
-        <x:v>黄色路径点＋紫色炮架点</x:v>
+        <x:v>仅技能按钮和距离数值刷新</x:v>
       </x:c>
       <x:c r="G56" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H56" s="11" t="str">
-        <x:v>web/js/app.js:34</x:v>
+        <x:v>web/js/app.js:51; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I56" s="11" t="str">
-        <x:v>必须辨识炮架与主目标</x:v>
+        <x:v>最高 7 格；与疾行升级使用不同辨识</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="32" customHeight="1">
-      <x:c r="A57" s="10" t="str">
+      <x:c r="A57" s="11" t="str">
         <x:v>A-052</x:v>
       </x:c>
       <x:c r="B57" s="11" t="str">
-        <x:v>操作标记</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C57" s="11" t="str">
-        <x:v>炮主目标</x:v>
+        <x:v>车｜震退解锁</x:v>
       </x:c>
       <x:c r="D57" s="11" t="str">
-        <x:v>1种</x:v>
+        <x:v>1套</x:v>
       </x:c>
       <x:c r="E57" s="11" t="str">
-        <x:v>炮击预览</x:v>
+        <x:v>花费 2 SP 解锁震退</x:v>
       </x:c>
       <x:c r="F57" s="11" t="str">
-        <x:v>红色目标点</x:v>
+        <x:v>仅按钮状态与文字刷新</x:v>
       </x:c>
       <x:c r="G57" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H57" s="11" t="str">
-        <x:v>web/js/app.js:34</x:v>
+        <x:v>web/js/app.js:52; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I57" s="11" t="str">
-        <x:v>扩散格视觉表现 TBD</x:v>
+        <x:v>表现永久解锁，不能误解为一次性攻击</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="32" customHeight="1">
-      <x:c r="A58" s="10" t="str">
+      <x:c r="A58" s="11" t="str">
         <x:v>A-053</x:v>
       </x:c>
       <x:c r="B58" s="11" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C58" s="11" t="str">
-        <x:v>战斗背景与主布局</x:v>
+        <x:v>车｜震退命中</x:v>
       </x:c>
       <x:c r="D58" s="11" t="str">
-        <x:v>桌面／窄屏</x:v>
+        <x:v>成功／受阻4态</x:v>
       </x:c>
       <x:c r="E58" s="11" t="str">
-        <x:v>棋盘外背景与分区</x:v>
+        <x:v>冲击命中存活目标后推 1 格</x:v>
       </x:c>
       <x:c r="F58" s="11" t="str">
-        <x:v>CSS 纯色与响应式布局</x:v>
+        <x:v>仅位置变化与文字结果</x:v>
       </x:c>
       <x:c r="G58" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H58" s="11" t="str">
-        <x:v>web/index.html:8-14</x:v>
+        <x:v>web/js/app.js:64; web/js/rules.js:42-46</x:v>
       </x:c>
       <x:c r="I58" s="11" t="str">
-        <x:v>正式背景、装饰 TBD</x:v>
+        <x:v>区分成功、出界、宫界和占位受阻</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="32" customHeight="1">
-      <x:c r="A59" s="10" t="str">
+      <x:c r="A59" s="11" t="str">
         <x:v>A-054</x:v>
       </x:c>
       <x:c r="B59" s="11" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C59" s="11" t="str">
-        <x:v>顶部状态栏</x:v>
+        <x:v>炮｜基础炮击</x:v>
       </x:c>
       <x:c r="D59" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>横竖4方向</x:v>
       </x:c>
       <x:c r="E59" s="11" t="str">
-        <x:v>波次、回合、HP、金币、击杀</x:v>
+        <x:v>隔恰好一个炮架攻击单目标</x:v>
       </x:c>
       <x:c r="F59" s="11" t="str">
-        <x:v>CSS 卡片＋文字</x:v>
+        <x:v>路径、炮架、目标圆点与文字预览</x:v>
       </x:c>
       <x:c r="G59" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H59" s="11" t="str">
-        <x:v>web/index.html:11,23</x:v>
+        <x:v>web/js/app.js:64; docs/us/US-001-cannon-fix.md:20-25</x:v>
       </x:c>
       <x:c r="I59" s="11" t="str">
-        <x:v>图标需求 TBD</x:v>
+        <x:v>需表现发射、越过炮架、命中和 2 点伤害</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="32" customHeight="1">
-      <x:c r="A60" s="10" t="str">
+      <x:c r="A60" s="11" t="str">
         <x:v>A-055</x:v>
       </x:c>
       <x:c r="B60" s="11" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C60" s="11" t="str">
-        <x:v>我方单位列表与棋子徽记</x:v>
+        <x:v>炮｜炮架充能／弹道</x:v>
       </x:c>
       <x:c r="D60" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>敌友炮架2态</x:v>
       </x:c>
       <x:c r="E60" s="11" t="str">
-        <x:v>选棋及单位状态</x:v>
+        <x:v>炮击前识别唯一炮架</x:v>
       </x:c>
       <x:c r="F60" s="11" t="str">
-        <x:v>CSS 卡片＋汉字徽记</x:v>
+        <x:v>紫色炮架点＋黄色路径点</x:v>
       </x:c>
       <x:c r="G60" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H60" s="11" t="str">
-        <x:v>web/index.html:12,26; web/js/app.js:37</x:v>
+        <x:v>web/js/app.js:34,64</x:v>
       </x:c>
       <x:c r="I60" s="11" t="str">
-        <x:v>沿用棋子识别系统</x:v>
+        <x:v>友军与敌军均可作炮架；不要表现为炮架受益</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="32" customHeight="1">
-      <x:c r="A61" s="10" t="str">
+      <x:c r="A61" s="11" t="str">
         <x:v>A-056</x:v>
       </x:c>
       <x:c r="B61" s="11" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C61" s="11" t="str">
-        <x:v>当前棋子信息卡</x:v>
+        <x:v>炮｜扩散解锁</x:v>
       </x:c>
       <x:c r="D61" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>8方向变体</x:v>
       </x:c>
       <x:c r="E61" s="11" t="str">
-        <x:v>属性、AP、等级、SP</x:v>
+        <x:v>逐个解锁目标邻格 N／NE／E／SE／S／SW／W／NW</x:v>
       </x:c>
       <x:c r="F61" s="11" t="str">
-        <x:v>CSS 信息卡＋文字</x:v>
+        <x:v>仅技能按钮和扩散计数刷新</x:v>
       </x:c>
       <x:c r="G61" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H61" s="11" t="str">
-        <x:v>web/index.html:12,27</x:v>
+        <x:v>web/js/app.js:53-54; web/js/rules.js:53</x:v>
       </x:c>
       <x:c r="I61" s="11" t="str">
-        <x:v>状态层级 TBD</x:v>
+        <x:v>固定朝向、不随开炮方向旋转；每格 1 SP</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="32" customHeight="1">
-      <x:c r="A62" s="10" t="str">
+      <x:c r="A62" s="11" t="str">
         <x:v>A-057</x:v>
       </x:c>
       <x:c r="B62" s="11" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C62" s="11" t="str">
-        <x:v>技能条目与禁用状态</x:v>
+        <x:v>炮｜扩散命中</x:v>
       </x:c>
       <x:c r="D62" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>主目标＋最多8邻格</x:v>
       </x:c>
       <x:c r="E62" s="11" t="str">
-        <x:v>升级、转职、方向和扩散</x:v>
+        <x:v>炮击时对已解锁邻格同时造成伤害</x:v>
       </x:c>
       <x:c r="F62" s="11" t="str">
-        <x:v>CSS 按钮＋文字</x:v>
+        <x:v>预览列出命中；无范围爆炸特效资产</x:v>
       </x:c>
       <x:c r="G62" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H62" s="11" t="str">
-        <x:v>web/index.html:13; web/js/app.js:42-56</x:v>
+        <x:v>web/js/app.js:64; web/js/rules.js:45</x:v>
       </x:c>
       <x:c r="I62" s="11" t="str">
-        <x:v>各技能专属图标 TBD</x:v>
+        <x:v>包含友伤和边界裁切；主目标与扩散命中需分层</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="32" customHeight="1">
-      <x:c r="A63" s="10" t="str">
+      <x:c r="A63" s="11" t="str">
         <x:v>A-058</x:v>
       </x:c>
       <x:c r="B63" s="11" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C63" s="11" t="str">
-        <x:v>方向与车模式按钮</x:v>
+        <x:v>兵｜连动升级</x:v>
       </x:c>
       <x:c r="D63" s="11" t="str">
-        <x:v>2组</x:v>
+        <x:v>1套／可重复</x:v>
       </x:c>
       <x:c r="E63" s="11" t="str">
-        <x:v>弓枪四向；车移动／冲击</x:v>
+        <x:v>花费 2 SP，使下回合 AP 上限 +1</x:v>
       </x:c>
       <x:c r="F63" s="11" t="str">
-        <x:v>CSS 按钮＋选中描边</x:v>
+        <x:v>仅技能按钮和数值刷新</x:v>
       </x:c>
       <x:c r="G63" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H63" s="11" t="str">
-        <x:v>web/index.html:13; web/js/app.js:58</x:v>
+        <x:v>web/js/app.js:46; web/js/rules.js:19,53</x:v>
       </x:c>
       <x:c r="I63" s="11" t="str">
-        <x:v>交互态样式 TBD</x:v>
+        <x:v>升级时与下回合实际生效时分别反馈</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="32" customHeight="1">
-      <x:c r="A64" s="10" t="str">
+      <x:c r="A64" s="11" t="str">
         <x:v>A-059</x:v>
       </x:c>
       <x:c r="B64" s="11" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C64" s="11" t="str">
-        <x:v>敌方意图列表与序号</x:v>
+        <x:v>兵｜额外行动激活</x:v>
       </x:c>
       <x:c r="D64" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>1套／层数变化</x:v>
       </x:c>
       <x:c r="E64" s="11" t="str">
-        <x:v>敌方行动顺序和状态</x:v>
+        <x:v>连动在下一回合增加可用 AP</x:v>
       </x:c>
       <x:c r="F64" s="11" t="str">
-        <x:v>CSS 圆序号＋文字</x:v>
+        <x:v>仅 AP 数字变化</x:v>
       </x:c>
       <x:c r="G64" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H64" s="11" t="str">
-        <x:v>web/index.html:13; web/js/app.js:60</x:v>
+        <x:v>web/js/rules.js:19</x:v>
       </x:c>
       <x:c r="I64" s="11" t="str">
-        <x:v>窄屏展开态已支持</x:v>
+        <x:v>需显示新增行动次数和已消耗层次</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="32" customHeight="1">
-      <x:c r="A65" s="10" t="str">
+      <x:c r="A65" s="11" t="str">
         <x:v>A-060</x:v>
       </x:c>
       <x:c r="B65" s="11" t="str">
-        <x:v>界面</x:v>
+        <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C65" s="11" t="str">
-        <x:v>动作预览与受击警告</x:v>
+        <x:v>兵｜转职弓兵</x:v>
       </x:c>
       <x:c r="D65" s="11" t="str">
         <x:v>1套</x:v>
       </x:c>
       <x:c r="E65" s="11" t="str">
+        <x:v>花费 2 SP，兵变为弓兵并获得攻击加成</x:v>
+      </x:c>
+      <x:c r="F65" s="11" t="str">
+        <x:v>棋子字样与属性瞬时变化</x:v>
+      </x:c>
+      <x:c r="G65" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H65" s="11" t="str">
+        <x:v>web/js/app.js:44; web/js/rules.js:53</x:v>
+      </x:c>
+      <x:c r="I65" s="11" t="str">
+        <x:v>保留原棋子身份、伤势和剩余 AP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="32" customHeight="1">
+      <x:c r="A66" s="11" t="str">
+        <x:v>A-061</x:v>
+      </x:c>
+      <x:c r="B66" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C66" s="11" t="str">
+        <x:v>兵｜转职枪兵</x:v>
+      </x:c>
+      <x:c r="D66" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E66" s="11" t="str">
+        <x:v>花费 2 SP，兵变为枪兵并获得 HP</x:v>
+      </x:c>
+      <x:c r="F66" s="11" t="str">
+        <x:v>棋子字样与属性瞬时变化</x:v>
+      </x:c>
+      <x:c r="G66" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H66" s="11" t="str">
+        <x:v>web/js/app.js:45; web/js/rules.js:53</x:v>
+      </x:c>
+      <x:c r="I66" s="11" t="str">
+        <x:v>保留原棋子身份、伤势和剩余 AP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="32" customHeight="1">
+      <x:c r="A67" s="11" t="str">
+        <x:v>A-062</x:v>
+      </x:c>
+      <x:c r="B67" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C67" s="11" t="str">
+        <x:v>弓兵｜四向射击</x:v>
+      </x:c>
+      <x:c r="D67" s="11" t="str">
+        <x:v>前／右／后／左</x:v>
+      </x:c>
+      <x:c r="E67" s="11" t="str">
+        <x:v>选一个方向，命中范围内首个敌人</x:v>
+      </x:c>
+      <x:c r="F67" s="11" t="str">
+        <x:v>黄色范围点和命中预览；无箭矢特效资产</x:v>
+      </x:c>
+      <x:c r="G67" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H67" s="11" t="str">
+        <x:v>web/js/app.js:59,64; web/js/rules.js:35</x:v>
+      </x:c>
+      <x:c r="I67" s="11" t="str">
+        <x:v>友军阻挡；需表现首个目标和 2 点伤害</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="32" customHeight="1">
+      <x:c r="A68" s="11" t="str">
+        <x:v>A-063</x:v>
+      </x:c>
+      <x:c r="B68" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C68" s="11" t="str">
+        <x:v>弓兵｜方向射程升级</x:v>
+      </x:c>
+      <x:c r="D68" s="11" t="str">
+        <x:v>4方向×6级</x:v>
+      </x:c>
+      <x:c r="E68" s="11" t="str">
+        <x:v>单方向每次 +1 格，最高 Lv.8／7格</x:v>
+      </x:c>
+      <x:c r="F68" s="11" t="str">
+        <x:v>仅方向按钮等级和距离文字刷新</x:v>
+      </x:c>
+      <x:c r="G68" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H68" s="11" t="str">
+        <x:v>web/js/app.js:47-48; web/js/rules.js:53</x:v>
+      </x:c>
+      <x:c r="I68" s="11" t="str">
+        <x:v>四方向独立，升级反馈须标明具体方向</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="32" customHeight="1">
+      <x:c r="A69" s="11" t="str">
+        <x:v>A-064</x:v>
+      </x:c>
+      <x:c r="B69" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C69" s="11" t="str">
+        <x:v>枪兵｜四向贯穿攻击</x:v>
+      </x:c>
+      <x:c r="D69" s="11" t="str">
+        <x:v>前／右／后／左</x:v>
+      </x:c>
+      <x:c r="E69" s="11" t="str">
+        <x:v>选一个方向，命中线内所有敌人</x:v>
+      </x:c>
+      <x:c r="F69" s="11" t="str">
+        <x:v>黄色范围点和命中列表；无枪击特效资产</x:v>
+      </x:c>
+      <x:c r="G69" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H69" s="11" t="str">
+        <x:v>web/js/app.js:59,64; web/js/rules.js:35</x:v>
+      </x:c>
+      <x:c r="I69" s="11" t="str">
+        <x:v>空格和敌人不中断，友军阻断；各目标 1 点伤害</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="32" customHeight="1">
+      <x:c r="A70" s="11" t="str">
+        <x:v>A-065</x:v>
+      </x:c>
+      <x:c r="B70" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C70" s="11" t="str">
+        <x:v>枪兵｜方向范围升级</x:v>
+      </x:c>
+      <x:c r="D70" s="11" t="str">
+        <x:v>4方向×6级</x:v>
+      </x:c>
+      <x:c r="E70" s="11" t="str">
+        <x:v>单方向每次 +1 格，最高 Lv.8／7格</x:v>
+      </x:c>
+      <x:c r="F70" s="11" t="str">
+        <x:v>仅方向按钮等级和距离文字刷新</x:v>
+      </x:c>
+      <x:c r="G70" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H70" s="11" t="str">
+        <x:v>web/js/app.js:47-48; web/js/rules.js:53</x:v>
+      </x:c>
+      <x:c r="I70" s="11" t="str">
+        <x:v>四方向独立；与弓兵升级可共用框架但视觉需可辨识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="32" customHeight="1">
+      <x:c r="A71" s="11" t="str">
+        <x:v>A-066</x:v>
+      </x:c>
+      <x:c r="B71" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C71" s="11" t="str">
+        <x:v>当前选中棋位</x:v>
+      </x:c>
+      <x:c r="D71" s="11" t="str">
+        <x:v>1种</x:v>
+      </x:c>
+      <x:c r="E71" s="11" t="str">
+        <x:v>选棋后标记起点</x:v>
+      </x:c>
+      <x:c r="F71" s="11" t="str">
+        <x:v>黄色半透明圆点</x:v>
+      </x:c>
+      <x:c r="G71" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H71" s="11" t="str">
+        <x:v>web/js/app.js:33-34</x:v>
+      </x:c>
+      <x:c r="I71" s="11" t="str">
+        <x:v>需与其他标记可区分</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="32" customHeight="1">
+      <x:c r="A72" s="11" t="str">
+        <x:v>A-067</x:v>
+      </x:c>
+      <x:c r="B72" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C72" s="11" t="str">
+        <x:v>合法移动落点</x:v>
+      </x:c>
+      <x:c r="D72" s="11" t="str">
+        <x:v>1种</x:v>
+      </x:c>
+      <x:c r="E72" s="11" t="str">
+        <x:v>移动选择</x:v>
+      </x:c>
+      <x:c r="F72" s="11" t="str">
+        <x:v>蓝色半透明圆点</x:v>
+      </x:c>
+      <x:c r="G72" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H72" s="11" t="str">
+        <x:v>web/js/app.js:33-34</x:v>
+      </x:c>
+      <x:c r="I72" s="11" t="str">
+        <x:v>需兼顾窄屏识别</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="32" customHeight="1">
+      <x:c r="A73" s="11" t="str">
+        <x:v>A-068</x:v>
+      </x:c>
+      <x:c r="B73" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C73" s="11" t="str">
+        <x:v>攻击与冲击目标</x:v>
+      </x:c>
+      <x:c r="D73" s="11" t="str">
+        <x:v>1种</x:v>
+      </x:c>
+      <x:c r="E73" s="11" t="str">
+        <x:v>攻击或车冲击</x:v>
+      </x:c>
+      <x:c r="F73" s="11" t="str">
+        <x:v>红色半透明圆点</x:v>
+      </x:c>
+      <x:c r="G73" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H73" s="11" t="str">
+        <x:v>web/js/app.js:33-34</x:v>
+      </x:c>
+      <x:c r="I73" s="11" t="str">
+        <x:v>需与移动落点可区分</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="32" customHeight="1">
+      <x:c r="A74" s="11" t="str">
+        <x:v>A-069</x:v>
+      </x:c>
+      <x:c r="B74" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C74" s="11" t="str">
+        <x:v>方向攻击范围</x:v>
+      </x:c>
+      <x:c r="D74" s="11" t="str">
+        <x:v>1种</x:v>
+      </x:c>
+      <x:c r="E74" s="11" t="str">
+        <x:v>弓／枪四向预览</x:v>
+      </x:c>
+      <x:c r="F74" s="11" t="str">
+        <x:v>黄色路径圆点</x:v>
+      </x:c>
+      <x:c r="G74" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H74" s="11" t="str">
+        <x:v>web/js/app.js:59</x:v>
+      </x:c>
+      <x:c r="I74" s="11" t="str">
+        <x:v>正式范围表现 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="32" customHeight="1">
+      <x:c r="A75" s="11" t="str">
+        <x:v>A-070</x:v>
+      </x:c>
+      <x:c r="B75" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C75" s="11" t="str">
+        <x:v>炮击路径与炮架</x:v>
+      </x:c>
+      <x:c r="D75" s="11" t="str">
+        <x:v>2种</x:v>
+      </x:c>
+      <x:c r="E75" s="11" t="str">
+        <x:v>炮击预览</x:v>
+      </x:c>
+      <x:c r="F75" s="11" t="str">
+        <x:v>黄色路径点＋紫色炮架点</x:v>
+      </x:c>
+      <x:c r="G75" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H75" s="11" t="str">
+        <x:v>web/js/app.js:34</x:v>
+      </x:c>
+      <x:c r="I75" s="11" t="str">
+        <x:v>必须辨识炮架与主目标</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="32" customHeight="1">
+      <x:c r="A76" s="11" t="str">
+        <x:v>A-071</x:v>
+      </x:c>
+      <x:c r="B76" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C76" s="11" t="str">
+        <x:v>炮主目标</x:v>
+      </x:c>
+      <x:c r="D76" s="11" t="str">
+        <x:v>1种</x:v>
+      </x:c>
+      <x:c r="E76" s="11" t="str">
+        <x:v>炮击预览</x:v>
+      </x:c>
+      <x:c r="F76" s="11" t="str">
+        <x:v>红色目标点</x:v>
+      </x:c>
+      <x:c r="G76" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H76" s="11" t="str">
+        <x:v>web/js/app.js:34</x:v>
+      </x:c>
+      <x:c r="I76" s="11" t="str">
+        <x:v>扩散格视觉表现 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="32" customHeight="1">
+      <x:c r="A77" s="11" t="str">
+        <x:v>A-072</x:v>
+      </x:c>
+      <x:c r="B77" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C77" s="11" t="str">
+        <x:v>战斗背景与主布局</x:v>
+      </x:c>
+      <x:c r="D77" s="11" t="str">
+        <x:v>桌面／窄屏</x:v>
+      </x:c>
+      <x:c r="E77" s="11" t="str">
+        <x:v>棋盘外背景与分区</x:v>
+      </x:c>
+      <x:c r="F77" s="11" t="str">
+        <x:v>CSS 纯色与响应式布局</x:v>
+      </x:c>
+      <x:c r="G77" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H77" s="11" t="str">
+        <x:v>web/index.html:8-14</x:v>
+      </x:c>
+      <x:c r="I77" s="11" t="str">
+        <x:v>正式背景、装饰 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="32" customHeight="1">
+      <x:c r="A78" s="11" t="str">
+        <x:v>A-073</x:v>
+      </x:c>
+      <x:c r="B78" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C78" s="11" t="str">
+        <x:v>顶部状态栏</x:v>
+      </x:c>
+      <x:c r="D78" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E78" s="11" t="str">
+        <x:v>波次、回合、HP、金币、击杀</x:v>
+      </x:c>
+      <x:c r="F78" s="11" t="str">
+        <x:v>CSS 卡片＋文字</x:v>
+      </x:c>
+      <x:c r="G78" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H78" s="11" t="str">
+        <x:v>web/index.html:11,23</x:v>
+      </x:c>
+      <x:c r="I78" s="11" t="str">
+        <x:v>图标需求 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="32" customHeight="1">
+      <x:c r="A79" s="11" t="str">
+        <x:v>A-074</x:v>
+      </x:c>
+      <x:c r="B79" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C79" s="11" t="str">
+        <x:v>我方单位列表与棋子徽记</x:v>
+      </x:c>
+      <x:c r="D79" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E79" s="11" t="str">
+        <x:v>选棋及单位状态</x:v>
+      </x:c>
+      <x:c r="F79" s="11" t="str">
+        <x:v>CSS 卡片＋汉字徽记</x:v>
+      </x:c>
+      <x:c r="G79" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H79" s="11" t="str">
+        <x:v>web/index.html:12,26; web/js/app.js:37</x:v>
+      </x:c>
+      <x:c r="I79" s="11" t="str">
+        <x:v>沿用棋子识别系统</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="32" customHeight="1">
+      <x:c r="A80" s="11" t="str">
+        <x:v>A-075</x:v>
+      </x:c>
+      <x:c r="B80" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C80" s="11" t="str">
+        <x:v>当前棋子信息卡</x:v>
+      </x:c>
+      <x:c r="D80" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E80" s="11" t="str">
+        <x:v>属性、AP、等级、SP</x:v>
+      </x:c>
+      <x:c r="F80" s="11" t="str">
+        <x:v>CSS 信息卡＋文字</x:v>
+      </x:c>
+      <x:c r="G80" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H80" s="11" t="str">
+        <x:v>web/index.html:12,27</x:v>
+      </x:c>
+      <x:c r="I80" s="11" t="str">
+        <x:v>状态层级 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="32" customHeight="1">
+      <x:c r="A81" s="11" t="str">
+        <x:v>A-076</x:v>
+      </x:c>
+      <x:c r="B81" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C81" s="11" t="str">
+        <x:v>技能条目与禁用状态</x:v>
+      </x:c>
+      <x:c r="D81" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E81" s="11" t="str">
+        <x:v>升级、转职、方向和扩散</x:v>
+      </x:c>
+      <x:c r="F81" s="11" t="str">
+        <x:v>CSS 按钮＋文字</x:v>
+      </x:c>
+      <x:c r="G81" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H81" s="11" t="str">
+        <x:v>web/index.html:13; web/js/app.js:42-56</x:v>
+      </x:c>
+      <x:c r="I81" s="11" t="str">
+        <x:v>各技能专属图标 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="32" customHeight="1">
+      <x:c r="A82" s="11" t="str">
+        <x:v>A-077</x:v>
+      </x:c>
+      <x:c r="B82" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C82" s="11" t="str">
+        <x:v>方向与车模式按钮</x:v>
+      </x:c>
+      <x:c r="D82" s="11" t="str">
+        <x:v>2组</x:v>
+      </x:c>
+      <x:c r="E82" s="11" t="str">
+        <x:v>弓枪四向；车移动／冲击</x:v>
+      </x:c>
+      <x:c r="F82" s="11" t="str">
+        <x:v>CSS 按钮＋选中描边</x:v>
+      </x:c>
+      <x:c r="G82" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H82" s="11" t="str">
+        <x:v>web/index.html:13; web/js/app.js:58</x:v>
+      </x:c>
+      <x:c r="I82" s="11" t="str">
+        <x:v>交互态样式 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="32" customHeight="1">
+      <x:c r="A83" s="11" t="str">
+        <x:v>A-078</x:v>
+      </x:c>
+      <x:c r="B83" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C83" s="11" t="str">
+        <x:v>敌方意图列表与序号</x:v>
+      </x:c>
+      <x:c r="D83" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E83" s="11" t="str">
+        <x:v>敌方行动顺序和状态</x:v>
+      </x:c>
+      <x:c r="F83" s="11" t="str">
+        <x:v>CSS 圆序号＋文字</x:v>
+      </x:c>
+      <x:c r="G83" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H83" s="11" t="str">
+        <x:v>web/index.html:13; web/js/app.js:60</x:v>
+      </x:c>
+      <x:c r="I83" s="11" t="str">
+        <x:v>窄屏展开态已支持</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="32" customHeight="1">
+      <x:c r="A84" s="11" t="str">
+        <x:v>A-079</x:v>
+      </x:c>
+      <x:c r="B84" s="11" t="str">
+        <x:v>界面</x:v>
+      </x:c>
+      <x:c r="C84" s="11" t="str">
+        <x:v>动作预览与受击警告</x:v>
+      </x:c>
+      <x:c r="D84" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E84" s="11" t="str">
         <x:v>路径、伤害、友伤、威胁</x:v>
       </x:c>
-      <x:c r="F65" s="11" t="str">
+      <x:c r="F84" s="11" t="str">
         <x:v>CSS 信息卡＋警告色</x:v>
       </x:c>
-      <x:c r="G65" s="11" t="str">
-        <x:v>代码占位</x:v>
-      </x:c>
-      <x:c r="H65" s="11" t="str">
+      <x:c r="G84" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H84" s="11" t="str">
         <x:v>web/index.html:13; web/js/app.js:63</x:v>
       </x:c>
-      <x:c r="I65" s="11" t="str">
+      <x:c r="I84" s="11" t="str">
         <x:v>友军误伤须醒目</x:v>
       </x:c>
     </x:row>
-    <x:row r="66" ht="32" customHeight="1">
-      <x:c r="A66" s="10" t="str">
-        <x:v>A-061</x:v>
-      </x:c>
-      <x:c r="B66" s="11" t="str">
+    <x:row r="85" ht="32" customHeight="1">
+      <x:c r="A85" s="11" t="str">
+        <x:v>A-080</x:v>
+      </x:c>
+      <x:c r="B85" s="11" t="str">
         <x:v>界面</x:v>
       </x:c>
-      <x:c r="C66" s="11" t="str">
+      <x:c r="C85" s="11" t="str">
         <x:v>底部操作按钮</x:v>
       </x:c>
-      <x:c r="D66" s="11" t="str">
+      <x:c r="D85" s="11" t="str">
         <x:v>4种</x:v>
       </x:c>
-      <x:c r="E66" s="11" t="str">
+      <x:c r="E85" s="11" t="str">
         <x:v>执行、取消、结束回合、暂停</x:v>
       </x:c>
-      <x:c r="F66" s="11" t="str">
+      <x:c r="F85" s="11" t="str">
         <x:v>CSS 按钮</x:v>
       </x:c>
-      <x:c r="G66" s="11" t="str">
-        <x:v>代码占位</x:v>
-      </x:c>
-      <x:c r="H66" s="11" t="str">
+      <x:c r="G85" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H85" s="11" t="str">
         <x:v>web/index.html:14,32</x:v>
       </x:c>
-      <x:c r="I66" s="11" t="str">
+      <x:c r="I85" s="11" t="str">
         <x:v>含禁用／悬停态</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" ht="32" customHeight="1">
-      <x:c r="A67" s="10" t="str">
-        <x:v>A-062</x:v>
-      </x:c>
-      <x:c r="B67" s="11" t="str">
+    <x:row r="86" ht="32" customHeight="1">
+      <x:c r="A86" s="11" t="str">
+        <x:v>A-081</x:v>
+      </x:c>
+      <x:c r="B86" s="11" t="str">
         <x:v>界面</x:v>
       </x:c>
-      <x:c r="C67" s="11" t="str">
+      <x:c r="C86" s="11" t="str">
         <x:v>结束回合确认弹窗</x:v>
       </x:c>
-      <x:c r="D67" s="11" t="str">
+      <x:c r="D86" s="11" t="str">
         <x:v>1套</x:v>
       </x:c>
-      <x:c r="E67" s="11" t="str">
+      <x:c r="E86" s="11" t="str">
         <x:v>提交敌方阶段前确认</x:v>
       </x:c>
-      <x:c r="F67" s="11" t="str">
+      <x:c r="F86" s="11" t="str">
         <x:v>CSS 遮罩＋对话框</x:v>
       </x:c>
-      <x:c r="G67" s="11" t="str">
-        <x:v>代码占位</x:v>
-      </x:c>
-      <x:c r="H67" s="11" t="str">
+      <x:c r="G86" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H86" s="11" t="str">
         <x:v>web/index.html:15,34</x:v>
       </x:c>
-      <x:c r="I67" s="11" t="str">
+      <x:c r="I86" s="11" t="str">
         <x:v>正式插画需求 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="32" customHeight="1">
-      <x:c r="A68" s="10" t="str">
-        <x:v>A-063</x:v>
-      </x:c>
-      <x:c r="B68" s="11" t="str">
+    <x:row r="87" ht="32" customHeight="1">
+      <x:c r="A87" s="11" t="str">
+        <x:v>A-082</x:v>
+      </x:c>
+      <x:c r="B87" s="11" t="str">
         <x:v>界面</x:v>
       </x:c>
-      <x:c r="C68" s="11" t="str">
+      <x:c r="C87" s="11" t="str">
         <x:v>暂停弹窗</x:v>
       </x:c>
-      <x:c r="D68" s="11" t="str">
+      <x:c r="D87" s="11" t="str">
         <x:v>1套</x:v>
       </x:c>
-      <x:c r="E68" s="11" t="str">
+      <x:c r="E87" s="11" t="str">
         <x:v>继续和重新开始</x:v>
       </x:c>
-      <x:c r="F68" s="11" t="str">
+      <x:c r="F87" s="11" t="str">
         <x:v>CSS 遮罩＋对话框</x:v>
       </x:c>
-      <x:c r="G68" s="11" t="str">
-        <x:v>代码占位</x:v>
-      </x:c>
-      <x:c r="H68" s="11" t="str">
+      <x:c r="G87" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H87" s="11" t="str">
         <x:v>web/index.html:15,35</x:v>
       </x:c>
-      <x:c r="I68" s="11" t="str">
+      <x:c r="I87" s="11" t="str">
         <x:v>正式插画需求 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="69" ht="32" customHeight="1">
-      <x:c r="A69" s="10" t="str">
-        <x:v>A-064</x:v>
-      </x:c>
-      <x:c r="B69" s="11" t="str">
+    <x:row r="88" ht="32" customHeight="1">
+      <x:c r="A88" s="11" t="str">
+        <x:v>A-083</x:v>
+      </x:c>
+      <x:c r="B88" s="11" t="str">
         <x:v>界面</x:v>
       </x:c>
-      <x:c r="C69" s="11" t="str">
+      <x:c r="C88" s="11" t="str">
         <x:v>商店与马／炮商品卡</x:v>
       </x:c>
-      <x:c r="D69" s="11" t="str">
+      <x:c r="D88" s="11" t="str">
         <x:v>1套＋2商品</x:v>
       </x:c>
-      <x:c r="E69" s="11" t="str">
+      <x:c r="E88" s="11" t="str">
         <x:v>首波结束后选购</x:v>
       </x:c>
-      <x:c r="F69" s="11" t="str">
+      <x:c r="F88" s="11" t="str">
         <x:v>CSS 对话框＋文字商品卡</x:v>
       </x:c>
-      <x:c r="G69" s="11" t="str">
-        <x:v>代码占位</x:v>
-      </x:c>
-      <x:c r="H69" s="11" t="str">
+      <x:c r="G88" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H88" s="11" t="str">
         <x:v>web/index.html:15,36</x:v>
       </x:c>
-      <x:c r="I69" s="11" t="str">
+      <x:c r="I88" s="11" t="str">
         <x:v>商品形象可复用棋子资产</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" ht="32" customHeight="1">
-      <x:c r="A70" s="10" t="str">
-        <x:v>A-065</x:v>
-      </x:c>
-      <x:c r="B70" s="11" t="str">
+    <x:row r="89" ht="32" customHeight="1">
+      <x:c r="A89" s="11" t="str">
+        <x:v>A-084</x:v>
+      </x:c>
+      <x:c r="B89" s="11" t="str">
         <x:v>界面</x:v>
       </x:c>
-      <x:c r="C70" s="11" t="str">
+      <x:c r="C89" s="11" t="str">
         <x:v>终局弹窗</x:v>
       </x:c>
-      <x:c r="D70" s="11" t="str">
+      <x:c r="D89" s="11" t="str">
         <x:v>胜／阵亡／将死</x:v>
       </x:c>
-      <x:c r="E70" s="11" t="str">
+      <x:c r="E89" s="11" t="str">
         <x:v>最终结果</x:v>
       </x:c>
-      <x:c r="F70" s="11" t="str">
+      <x:c r="F89" s="11" t="str">
         <x:v>CSS 对话框＋状态文字</x:v>
       </x:c>
-      <x:c r="G70" s="11" t="str">
-        <x:v>代码占位</x:v>
-      </x:c>
-      <x:c r="H70" s="11" t="str">
+      <x:c r="G89" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H89" s="11" t="str">
         <x:v>web/index.html:15,37</x:v>
       </x:c>
-      <x:c r="I70" s="11" t="str">
+      <x:c r="I89" s="11" t="str">
         <x:v>结果插画需求 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="32" customHeight="1">
-      <x:c r="A71" s="10" t="str">
-        <x:v>A-066</x:v>
-      </x:c>
-      <x:c r="B71" s="11" t="str">
+    <x:row r="90" ht="32" customHeight="1">
+      <x:c r="A90" s="11" t="str">
+        <x:v>A-085</x:v>
+      </x:c>
+      <x:c r="B90" s="11" t="str">
         <x:v>界面</x:v>
       </x:c>
-      <x:c r="C71" s="11" t="str">
+      <x:c r="C90" s="11" t="str">
         <x:v>短提示与危险提示</x:v>
       </x:c>
-      <x:c r="D71" s="11" t="str">
+      <x:c r="D90" s="11" t="str">
         <x:v>1套</x:v>
       </x:c>
-      <x:c r="E71" s="11" t="str">
+      <x:c r="E90" s="11" t="str">
         <x:v>购买、重开、操作失败</x:v>
       </x:c>
-      <x:c r="F71" s="11" t="str">
+      <x:c r="F90" s="11" t="str">
         <x:v>CSS 横幅＋文字</x:v>
       </x:c>
-      <x:c r="G71" s="11" t="str">
-        <x:v>代码占位</x:v>
-      </x:c>
-      <x:c r="H71" s="11" t="str">
+      <x:c r="G90" s="11" t="str">
+        <x:v>代码占位</x:v>
+      </x:c>
+      <x:c r="H90" s="11" t="str">
         <x:v>web/index.html:14,24; web/js/app.js:69</x:v>
       </x:c>
-      <x:c r="I71" s="11" t="str">
+      <x:c r="I90" s="11" t="str">
         <x:v>信息可读性优先</x:v>
       </x:c>
     </x:row>
-    <x:row r="72" ht="32" customHeight="1">
-      <x:c r="A72" s="10" t="str">
-        <x:v>A-067</x:v>
-      </x:c>
-      <x:c r="B72" s="11" t="str">
+    <x:row r="91" ht="32" customHeight="1">
+      <x:c r="A91" s="11" t="str">
+        <x:v>A-086</x:v>
+      </x:c>
+      <x:c r="B91" s="11" t="str">
         <x:v>旧目录素材</x:v>
       </x:c>
-      <x:c r="C72" s="11" t="str">
+      <x:c r="C91" s="11" t="str">
         <x:v>僵尸角色图</x:v>
       </x:c>
-      <x:c r="D72" s="11" t="str">
+      <x:c r="D91" s="11" t="str">
         <x:v>1张</x:v>
       </x:c>
-      <x:c r="E72" s="11" t="str">
+      <x:c r="E91" s="11" t="str">
         <x:v>旧目录参考；网页未使用</x:v>
       </x:c>
-      <x:c r="F72" s="11" t="str">
+      <x:c r="F91" s="11" t="str">
         <x:v>PNG，像素风角色</x:v>
       </x:c>
-      <x:c r="G72" s="11" t="str">
+      <x:c r="G91" s="11" t="str">
         <x:v>已有文件未接入</x:v>
       </x:c>
-      <x:c r="H72" s="11" t="str">
+      <x:c r="H91" s="11" t="str">
         <x:v>m0-zyf/assets/art/jiangshi.png</x:v>
       </x:c>
-      <x:c r="I72" s="11" t="str">
+      <x:c r="I91" s="11" t="str">
         <x:v>与当前象棋题材的用途 TBD</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:I2"/>
+    <x:mergeCell ref="A3:I3"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra54246ffb3d7452c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd18c32eec5642d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2504,7 +3059,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raecb7483895d4100"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a0cfd5789394cb6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore(assets): update art asset list
</commit_message>
<xml_diff>
--- a/outputs/01a0bf14-7f85-7282-bb8d-672064556a58/美术资产清单.xlsx
+++ b/outputs/01a0bf14-7f85-7282-bb8d-672064556a58/美术资产清单.xlsx
@@ -2,8 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="美术资产清单" sheetId="1" r:id="R735b1bd6142b491f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="源文件盘点" sheetId="2" r:id="R5d8b2065cfac41f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="美术资产清单" sheetId="1" r:id="Rf0261a8c855d4fcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="源文件盘点" sheetId="2" r:id="Re40b2ce53eb44b92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="界面规格" sheetId="3" r:id="Rb9ecb261437b495c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图分区" sheetId="4" r:id="R867d38e4eaad4961"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="5">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0"/>
+  </x:numFmts>
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -42,8 +47,29 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="18"/>
+      <x:color rgb="FF18364D"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF526471"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -55,6 +81,16 @@
         <x:fgColor rgb="FF233347"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF183E5A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF4F8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -62,7 +98,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="12">
+  <x:cellXfs count="22">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -87,6 +123,32 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -95,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VisualAssets" displayName="VisualAssets" ref="A5:I91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VisualAssets" displayName="VisualAssets" ref="A5:I136" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="分类"/>
@@ -122,6 +184,40 @@
     <x:tableColumn id="6" name="透明通道"/>
     <x:tableColumn id="7" name="网页使用"/>
     <x:tableColumn id="8" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="UiSpecs" displayName="UiSpecs" ref="A5:I64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="编号"/>
+    <x:tableColumn id="2" name="资源/组件"/>
+    <x:tableColumn id="3" name="替换槽位名"/>
+    <x:tableColumn id="4" name="建议尺寸 px"/>
+    <x:tableColumn id="5" name="格式与切图"/>
+    <x:tableColumn id="6" name="交互状态"/>
+    <x:tableColumn id="7" name="使用位置"/>
+    <x:tableColumn id="8" name="数量/变体"/>
+    <x:tableColumn id="9" name="交付说明"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="MapRegions" displayName="MapRegions" ref="A5:I8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="关卡"/>
+    <x:tableColumn id="2" name="暂定区域名"/>
+    <x:tableColumn id="3" name="区域槽位"/>
+    <x:tableColumn id="4" name="构图位置"/>
+    <x:tableColumn id="5" name="视觉主题"/>
+    <x:tableColumn id="6" name="重点资源"/>
+    <x:tableColumn id="7" name="状态预留"/>
+    <x:tableColumn id="8" name="玩法接入"/>
+    <x:tableColumn id="9" name="参考与说明"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -348,7 +444,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>范围：当前主原型、独立地形实验及工作区源素材；地形资产来自 terrain-wave 实验，尚未合入主原型。</x:v>
+        <x:v>范围：主原型、独立地形实验、Loading/主菜单/三关地图美术占位；三关规则与流程接入 TBD。</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -361,7 +457,7 @@
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>共 86 项视觉元素；传统棋子 14 款，项目转职 2 款；己方技能效果预留 24 项；地形资产与效果 19 项；旧目录源图片 1 个。</x:v>
+        <x:v>共 131 项视觉元素/组件记录；本次新增 45 项。传统棋子14款、扩展棋子2款、己方技能效果24项、地形19项保留。UI交付规格详见“界面规格”。</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -2482,22 +2578,22 @@
         <x:v>战斗背景与主布局</x:v>
       </x:c>
       <x:c r="D77" s="11" t="str">
-        <x:v>桌面／窄屏</x:v>
+        <x:v>桌面／手机2套</x:v>
       </x:c>
       <x:c r="E77" s="11" t="str">
-        <x:v>棋盘外背景与分区</x:v>
+        <x:v>桌面菱形棋盘四角HUD；手机一屏布局</x:v>
       </x:c>
       <x:c r="F77" s="11" t="str">
-        <x:v>CSS 纯色与响应式布局</x:v>
+        <x:v>CSS响应式布局</x:v>
       </x:c>
       <x:c r="G77" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H77" s="11" t="str">
-        <x:v>web/index.html:8-14</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I77" s="11" t="str">
-        <x:v>正式背景、装饰 TBD</x:v>
+        <x:v>组件总项；面板切图复用A-109起通用资源，桌面1920×1080、手机1344×2772</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="32" customHeight="1">
@@ -2508,25 +2604,25 @@
         <x:v>界面</x:v>
       </x:c>
       <x:c r="C78" s="11" t="str">
-        <x:v>顶部状态栏</x:v>
+        <x:v>战斗状态栏</x:v>
       </x:c>
       <x:c r="D78" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>桌面／手机2套</x:v>
       </x:c>
       <x:c r="E78" s="11" t="str">
-        <x:v>波次、回合、HP、金币、击杀</x:v>
+        <x:v>波次、回合、主帅HP、金币、击杀</x:v>
       </x:c>
       <x:c r="F78" s="11" t="str">
-        <x:v>CSS 卡片＋文字</x:v>
+        <x:v>CSS卡片＋文字</x:v>
       </x:c>
       <x:c r="G78" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H78" s="11" t="str">
-        <x:v>web/index.html:11,23</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I78" s="11" t="str">
-        <x:v>图标需求 TBD</x:v>
+        <x:v>桌面左上；手机仅保留紧凑主要数值，完整状态折叠</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="32" customHeight="1">
@@ -2540,22 +2636,22 @@
         <x:v>我方单位列表与棋子徽记</x:v>
       </x:c>
       <x:c r="D79" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>敌我可区分，己方9棋种槽位</x:v>
       </x:c>
       <x:c r="E79" s="11" t="str">
-        <x:v>选棋及单位状态</x:v>
+        <x:v>选棋与单位状态</x:v>
       </x:c>
       <x:c r="F79" s="11" t="str">
-        <x:v>CSS 卡片＋汉字徽记</x:v>
+        <x:v>CSS卡片＋汉字徽记</x:v>
       </x:c>
       <x:c r="G79" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H79" s="11" t="str">
-        <x:v>web/index.html:12,26; web/js/app.js:37</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I79" s="11" t="str">
-        <x:v>沿用棋子识别系统</x:v>
+        <x:v>徽记复用棋子；默认/选中/行动耗尽；未实现棋种仍仅预留</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="32" customHeight="1">
@@ -2569,22 +2665,22 @@
         <x:v>当前棋子信息卡</x:v>
       </x:c>
       <x:c r="D80" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>桌面详情／手机摘要</x:v>
       </x:c>
       <x:c r="E80" s="11" t="str">
-        <x:v>属性、AP、等级、SP</x:v>
+        <x:v>属性、行动余量、等级、SP</x:v>
       </x:c>
       <x:c r="F80" s="11" t="str">
-        <x:v>CSS 信息卡＋文字</x:v>
+        <x:v>CSS信息卡＋文字</x:v>
       </x:c>
       <x:c r="G80" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H80" s="11" t="str">
-        <x:v>web/index.html:12,27</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I80" s="11" t="str">
-        <x:v>状态层级 TBD</x:v>
+        <x:v>长说明可展开，动态数值不烘焙</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="32" customHeight="1">
@@ -2598,22 +2694,22 @@
         <x:v>技能条目与禁用状态</x:v>
       </x:c>
       <x:c r="D81" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>1套＋图标槽位</x:v>
       </x:c>
       <x:c r="E81" s="11" t="str">
-        <x:v>升级、转职、方向和扩散</x:v>
+        <x:v>升级、转职、方向和炮扩散</x:v>
       </x:c>
       <x:c r="F81" s="11" t="str">
-        <x:v>CSS 按钮＋文字</x:v>
+        <x:v>CSS按钮＋文字</x:v>
       </x:c>
       <x:c r="G81" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H81" s="11" t="str">
-        <x:v>web/index.html:13; web/js/app.js:42-56</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I81" s="11" t="str">
-        <x:v>各技能专属图标 TBD</x:v>
+        <x:v>可购买/已解锁/缺SP/当前阶段不可购买；专属技能仍为己方</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="32" customHeight="1">
@@ -2627,22 +2723,22 @@
         <x:v>方向与车模式按钮</x:v>
       </x:c>
       <x:c r="D82" s="11" t="str">
-        <x:v>2组</x:v>
+        <x:v>四方向＋移动/冲锋/牵引</x:v>
       </x:c>
       <x:c r="E82" s="11" t="str">
-        <x:v>弓枪四向；车移动／冲击</x:v>
+        <x:v>弓枪方向；车职业模式</x:v>
       </x:c>
       <x:c r="F82" s="11" t="str">
-        <x:v>CSS 按钮＋选中描边</x:v>
+        <x:v>CSS按钮＋选中描边</x:v>
       </x:c>
       <x:c r="G82" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H82" s="11" t="str">
-        <x:v>web/index.html:13; web/js/app.js:58</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I82" s="11" t="str">
-        <x:v>交互态样式 TBD</x:v>
+        <x:v>默认/选中/禁用；手机触控面积至少44逻辑像素</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="32" customHeight="1">
@@ -2659,19 +2755,19 @@
         <x:v>1套</x:v>
       </x:c>
       <x:c r="E83" s="11" t="str">
-        <x:v>敌方行动顺序和状态</x:v>
+        <x:v>敌方行动顺序和预期状态</x:v>
       </x:c>
       <x:c r="F83" s="11" t="str">
-        <x:v>CSS 圆序号＋文字</x:v>
+        <x:v>折叠列表＋序号</x:v>
       </x:c>
       <x:c r="G83" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H83" s="11" t="str">
-        <x:v>web/index.html:13; web/js/app.js:60</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I83" s="11" t="str">
-        <x:v>窄屏展开态已支持</x:v>
+        <x:v>成功/失效/落空/已移除/待机需区分</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="32" customHeight="1">
@@ -2685,22 +2781,22 @@
         <x:v>动作预览与受击警告</x:v>
       </x:c>
       <x:c r="D84" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>桌面详情／手机摘要</x:v>
       </x:c>
       <x:c r="E84" s="11" t="str">
-        <x:v>路径、伤害、友伤、威胁</x:v>
+        <x:v>路径、伤害、友伤、主帅威胁</x:v>
       </x:c>
       <x:c r="F84" s="11" t="str">
-        <x:v>CSS 信息卡＋警告色</x:v>
+        <x:v>信息卡＋棋盘标记</x:v>
       </x:c>
       <x:c r="G84" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H84" s="11" t="str">
-        <x:v>web/index.html:13; web/js/app.js:63</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I84" s="11" t="str">
-        <x:v>友军误伤须醒目</x:v>
+        <x:v>友伤醒目；桌面点目标直接攻击，手机保留执行确认</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="32" customHeight="1">
@@ -2711,25 +2807,25 @@
         <x:v>界面</x:v>
       </x:c>
       <x:c r="C85" s="11" t="str">
-        <x:v>底部操作按钮</x:v>
+        <x:v>战斗操作按钮</x:v>
       </x:c>
       <x:c r="D85" s="11" t="str">
-        <x:v>4种</x:v>
+        <x:v>执行/取消/撤销/结束回合/暂停</x:v>
       </x:c>
       <x:c r="E85" s="11" t="str">
-        <x:v>执行、取消、结束回合、暂停</x:v>
+        <x:v>桌面左上与手机底部</x:v>
       </x:c>
       <x:c r="F85" s="11" t="str">
-        <x:v>CSS 按钮</x:v>
+        <x:v>CSS按钮</x:v>
       </x:c>
       <x:c r="G85" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H85" s="11" t="str">
-        <x:v>web/index.html:14,32</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I85" s="11" t="str">
-        <x:v>含禁用／悬停态</x:v>
+        <x:v>桌面隐藏执行按钮；底板共用通用按钮皮肤</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="32" customHeight="1">
@@ -2746,19 +2842,19 @@
         <x:v>1套</x:v>
       </x:c>
       <x:c r="E86" s="11" t="str">
-        <x:v>提交敌方阶段前确认</x:v>
+        <x:v>结算敌方阶段前确认</x:v>
       </x:c>
       <x:c r="F86" s="11" t="str">
-        <x:v>CSS 遮罩＋对话框</x:v>
+        <x:v>遮罩＋对话框</x:v>
       </x:c>
       <x:c r="G86" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H86" s="11" t="str">
-        <x:v>web/index.html:15,34</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I86" s="11" t="str">
-        <x:v>正式插画需求 TBD</x:v>
+        <x:v>确认/继续行动；未行动名单为独立悬停组件</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="32" customHeight="1">
@@ -2775,19 +2871,19 @@
         <x:v>1套</x:v>
       </x:c>
       <x:c r="E87" s="11" t="str">
-        <x:v>继续和重新开始</x:v>
+        <x:v>继续/重新开始</x:v>
       </x:c>
       <x:c r="F87" s="11" t="str">
-        <x:v>CSS 遮罩＋对话框</x:v>
+        <x:v>遮罩＋对话框</x:v>
       </x:c>
       <x:c r="G87" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H87" s="11" t="str">
-        <x:v>web/index.html:15,35</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I87" s="11" t="str">
-        <x:v>正式插画需求 TBD</x:v>
+        <x:v>复用面板、遮罩、主次按钮</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="32" customHeight="1">
@@ -2798,25 +2894,25 @@
         <x:v>界面</x:v>
       </x:c>
       <x:c r="C88" s="11" t="str">
-        <x:v>商店与马／炮商品卡</x:v>
+        <x:v>商店与商品卡</x:v>
       </x:c>
       <x:c r="D88" s="11" t="str">
-        <x:v>1套＋2商品</x:v>
+        <x:v>兵/车/马/炮4类</x:v>
       </x:c>
       <x:c r="E88" s="11" t="str">
-        <x:v>首波结束后选购</x:v>
+        <x:v>关间整备与上阵后备</x:v>
       </x:c>
       <x:c r="F88" s="11" t="str">
-        <x:v>CSS 对话框＋文字商品卡</x:v>
+        <x:v>对话框＋商品卡＋队伍列表</x:v>
       </x:c>
       <x:c r="G88" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H88" s="11" t="str">
-        <x:v>web/index.html:15,36</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I88" s="11" t="str">
-        <x:v>商品形象可复用棋子资产</x:v>
+        <x:v>商品像复用棋子；价格、阵容容量实时文字</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="32" customHeight="1">
@@ -2830,22 +2926,22 @@
         <x:v>终局弹窗</x:v>
       </x:c>
       <x:c r="D89" s="11" t="str">
-        <x:v>胜／阵亡／将死</x:v>
+        <x:v>胜利/阵亡/将死3态</x:v>
       </x:c>
       <x:c r="E89" s="11" t="str">
-        <x:v>最终结果</x:v>
+        <x:v>战斗结果</x:v>
       </x:c>
       <x:c r="F89" s="11" t="str">
-        <x:v>CSS 对话框＋状态文字</x:v>
+        <x:v>对话框＋状态文字</x:v>
       </x:c>
       <x:c r="G89" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H89" s="11" t="str">
-        <x:v>web/index.html:15,37</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I89" s="11" t="str">
-        <x:v>结果插画需求 TBD</x:v>
+        <x:v>独立结果标题装饰详见新增条目；统计数字实时文字</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="32" customHeight="1">
@@ -2859,22 +2955,22 @@
         <x:v>短提示与危险提示</x:v>
       </x:c>
       <x:c r="D90" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>普通/成功/警告3态</x:v>
       </x:c>
       <x:c r="E90" s="11" t="str">
-        <x:v>购买、重开、操作失败</x:v>
+        <x:v>购买、重开、操作失败、危险反馈</x:v>
       </x:c>
       <x:c r="F90" s="11" t="str">
-        <x:v>CSS 横幅＋文字</x:v>
+        <x:v>短提示横幅＋文字</x:v>
       </x:c>
       <x:c r="G90" s="11" t="str">
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H90" s="11" t="str">
-        <x:v>web/index.html:14,24; web/js/app.js:69</x:v>
+        <x:v>2026-10-05 当前UI核对</x:v>
       </x:c>
       <x:c r="I90" s="11" t="str">
-        <x:v>信息可读性优先</x:v>
+        <x:v>底板复用；提示色必须同时有文字或图标辨识</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="32" customHeight="1">
@@ -2904,6 +3000,1311 @@
       </x:c>
       <x:c r="I91" s="11" t="str">
         <x:v>与当前象棋题材的用途 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="60" customHeight="1">
+      <x:c r="A92" s="11" t="str">
+        <x:v>A-087</x:v>
+      </x:c>
+      <x:c r="B92" s="11" t="str">
+        <x:v>启动界面</x:v>
+      </x:c>
+      <x:c r="C92" s="11" t="str">
+        <x:v>Loading 背景</x:v>
+      </x:c>
+      <x:c r="D92" s="11" t="str">
+        <x:v>横竖2版</x:v>
+      </x:c>
+      <x:c r="E92" s="11" t="str">
+        <x:v>全屏背景</x:v>
+      </x:c>
+      <x:c r="F92" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G92" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H92" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I92" s="11" t="str">
+        <x:v>重要主体留在中央安全区；横竖单独构图</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="60" customHeight="1">
+      <x:c r="A93" s="11" t="str">
+        <x:v>A-088</x:v>
+      </x:c>
+      <x:c r="B93" s="11" t="str">
+        <x:v>启动界面</x:v>
+      </x:c>
+      <x:c r="C93" s="11" t="str">
+        <x:v>游戏标志与题字</x:v>
+      </x:c>
+      <x:c r="D93" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E93" s="11" t="str">
+        <x:v>Loading/主菜单共用</x:v>
+      </x:c>
+      <x:c r="F93" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G93" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H93" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I93" s="11" t="str">
+        <x:v>暂用九格战阵文字；正式标志 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="60" customHeight="1">
+      <x:c r="A94" s="11" t="str">
+        <x:v>A-089</x:v>
+      </x:c>
+      <x:c r="B94" s="11" t="str">
+        <x:v>启动界面</x:v>
+      </x:c>
+      <x:c r="C94" s="11" t="str">
+        <x:v>加载进度条底框</x:v>
+      </x:c>
+      <x:c r="D94" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E94" s="11" t="str">
+        <x:v>Loading 底部</x:v>
+      </x:c>
+      <x:c r="F94" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G94" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H94" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I94" s="11" t="str">
+        <x:v>底框与填充分离，长度由程序控制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="60" customHeight="1">
+      <x:c r="A95" s="11" t="str">
+        <x:v>A-090</x:v>
+      </x:c>
+      <x:c r="B95" s="11" t="str">
+        <x:v>启动界面</x:v>
+      </x:c>
+      <x:c r="C95" s="11" t="str">
+        <x:v>加载进度条填充</x:v>
+      </x:c>
+      <x:c r="D95" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E95" s="11" t="str">
+        <x:v>Loading 进度</x:v>
+      </x:c>
+      <x:c r="F95" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G95" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H95" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I95" s="11" t="str">
+        <x:v>不把百分比烘焙到图片</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="60" customHeight="1">
+      <x:c r="A96" s="11" t="str">
+        <x:v>A-091</x:v>
+      </x:c>
+      <x:c r="B96" s="11" t="str">
+        <x:v>启动界面</x:v>
+      </x:c>
+      <x:c r="C96" s="11" t="str">
+        <x:v>加载提示框与装饰</x:v>
+      </x:c>
+      <x:c r="D96" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E96" s="11" t="str">
+        <x:v>Loading 文案区域</x:v>
+      </x:c>
+      <x:c r="F96" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G96" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H96" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I96" s="11" t="str">
+        <x:v>文案用实时文字；字体需可商用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="60" customHeight="1">
+      <x:c r="A97" s="11" t="str">
+        <x:v>A-092</x:v>
+      </x:c>
+      <x:c r="B97" s="11" t="str">
+        <x:v>启动界面</x:v>
+      </x:c>
+      <x:c r="C97" s="11" t="str">
+        <x:v>加载旋转标识</x:v>
+      </x:c>
+      <x:c r="D97" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E97" s="11" t="str">
+        <x:v>Loading 等待状态</x:v>
+      </x:c>
+      <x:c r="F97" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G97" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H97" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I97" s="11" t="str">
+        <x:v>代码旋转即可；不强制逐帧动画</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="60" customHeight="1">
+      <x:c r="A98" s="11" t="str">
+        <x:v>A-093</x:v>
+      </x:c>
+      <x:c r="B98" s="11" t="str">
+        <x:v>启动界面</x:v>
+      </x:c>
+      <x:c r="C98" s="11" t="str">
+        <x:v>加载失败与重试提示</x:v>
+      </x:c>
+      <x:c r="D98" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E98" s="11" t="str">
+        <x:v>Loading 异常态</x:v>
+      </x:c>
+      <x:c r="F98" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G98" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H98" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I98" s="11" t="str">
+        <x:v>预留视觉状态，样稿不模拟网络异常</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="60" customHeight="1">
+      <x:c r="A99" s="11" t="str">
+        <x:v>A-094</x:v>
+      </x:c>
+      <x:c r="B99" s="11" t="str">
+        <x:v>菜单界面</x:v>
+      </x:c>
+      <x:c r="C99" s="11" t="str">
+        <x:v>主菜单背景</x:v>
+      </x:c>
+      <x:c r="D99" s="11" t="str">
+        <x:v>横竖2版</x:v>
+      </x:c>
+      <x:c r="E99" s="11" t="str">
+        <x:v>主菜单全屏</x:v>
+      </x:c>
+      <x:c r="F99" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G99" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H99" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I99" s="11" t="str">
+        <x:v>文字与按钮独立，不烘焙</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="60" customHeight="1">
+      <x:c r="A100" s="11" t="str">
+        <x:v>A-095</x:v>
+      </x:c>
+      <x:c r="B100" s="11" t="str">
+        <x:v>菜单界面</x:v>
+      </x:c>
+      <x:c r="C100" s="11" t="str">
+        <x:v>主菜单主按钮</x:v>
+      </x:c>
+      <x:c r="D100" s="11" t="str">
+        <x:v>4态</x:v>
+      </x:c>
+      <x:c r="E100" s="11" t="str">
+        <x:v>开始游戏/继续游戏</x:v>
+      </x:c>
+      <x:c r="F100" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G100" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H100" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I100" s="11" t="str">
+        <x:v>两个功能共用按钮皮肤，继续游戏规则 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="60" customHeight="1">
+      <x:c r="A101" s="11" t="str">
+        <x:v>A-096</x:v>
+      </x:c>
+      <x:c r="B101" s="11" t="str">
+        <x:v>菜单界面</x:v>
+      </x:c>
+      <x:c r="C101" s="11" t="str">
+        <x:v>主菜单次按钮</x:v>
+      </x:c>
+      <x:c r="D101" s="11" t="str">
+        <x:v>4态</x:v>
+      </x:c>
+      <x:c r="E101" s="11" t="str">
+        <x:v>设置/制作人员/返回</x:v>
+      </x:c>
+      <x:c r="F101" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G101" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H101" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I101" s="11" t="str">
+        <x:v>按钮文字独立</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="60" customHeight="1">
+      <x:c r="A102" s="11" t="str">
+        <x:v>A-097</x:v>
+      </x:c>
+      <x:c r="B102" s="11" t="str">
+        <x:v>菜单界面</x:v>
+      </x:c>
+      <x:c r="C102" s="11" t="str">
+        <x:v>菜单装饰前景</x:v>
+      </x:c>
+      <x:c r="D102" s="11" t="str">
+        <x:v>横竖2版</x:v>
+      </x:c>
+      <x:c r="E102" s="11" t="str">
+        <x:v>主菜单边角</x:v>
+      </x:c>
+      <x:c r="F102" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G102" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H102" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I102" s="11" t="str">
+        <x:v>可用棋子/兵旗/印章；不遮挡按钮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="60" customHeight="1">
+      <x:c r="A103" s="11" t="str">
+        <x:v>A-098</x:v>
+      </x:c>
+      <x:c r="B103" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C103" s="11" t="str">
+        <x:v>战国题材地图底图</x:v>
+      </x:c>
+      <x:c r="D103" s="11" t="str">
+        <x:v>横竖2版</x:v>
+      </x:c>
+      <x:c r="E103" s="11" t="str">
+        <x:v>开始游戏后的选关页</x:v>
+      </x:c>
+      <x:c r="F103" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G103" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H103" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I103" s="11" t="str">
+        <x:v>三分区为玩法草案；历史边界和时代年份 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="60" customHeight="1">
+      <x:c r="A104" s="11" t="str">
+        <x:v>A-099</x:v>
+      </x:c>
+      <x:c r="B104" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C104" s="11" t="str">
+        <x:v>第1关区域 关中</x:v>
+      </x:c>
+      <x:c r="D104" s="11" t="str">
+        <x:v>3态</x:v>
+      </x:c>
+      <x:c r="E104" s="11" t="str">
+        <x:v>西部关卡区域</x:v>
+      </x:c>
+      <x:c r="F104" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G104" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H104" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I104" s="11" t="str">
+        <x:v>西部关中主题；山隘/城塞视觉；区域范围与关名 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="60" customHeight="1">
+      <x:c r="A105" s="11" t="str">
+        <x:v>A-100</x:v>
+      </x:c>
+      <x:c r="B105" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C105" s="11" t="str">
+        <x:v>第2关区域 中原</x:v>
+      </x:c>
+      <x:c r="D105" s="11" t="str">
+        <x:v>3态</x:v>
+      </x:c>
+      <x:c r="E105" s="11" t="str">
+        <x:v>中央关卡区域</x:v>
+      </x:c>
+      <x:c r="F105" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G105" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H105" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I105" s="11" t="str">
+        <x:v>中央平原主题；河流/城邑视觉；区域范围与关名 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="60" customHeight="1">
+      <x:c r="A106" s="11" t="str">
+        <x:v>A-101</x:v>
+      </x:c>
+      <x:c r="B106" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C106" s="11" t="str">
+        <x:v>第3关区域 江淮</x:v>
+      </x:c>
+      <x:c r="D106" s="11" t="str">
+        <x:v>3态</x:v>
+      </x:c>
+      <x:c r="E106" s="11" t="str">
+        <x:v>东南关卡区域</x:v>
+      </x:c>
+      <x:c r="F106" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G106" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H106" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I106" s="11" t="str">
+        <x:v>东南水网主题；水泽/林地视觉；区域范围与关名 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="60" customHeight="1">
+      <x:c r="A107" s="11" t="str">
+        <x:v>A-102</x:v>
+      </x:c>
+      <x:c r="B107" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C107" s="11" t="str">
+        <x:v>区域分界描边</x:v>
+      </x:c>
+      <x:c r="D107" s="11" t="str">
+        <x:v>1套3区域</x:v>
+      </x:c>
+      <x:c r="E107" s="11" t="str">
+        <x:v>地图分区</x:v>
+      </x:c>
+      <x:c r="F107" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G107" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H107" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I107" s="11" t="str">
+        <x:v>三个区域共边不得出现缝隙；非真实国界</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="60" customHeight="1">
+      <x:c r="A108" s="11" t="str">
+        <x:v>A-103</x:v>
+      </x:c>
+      <x:c r="B108" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C108" s="11" t="str">
+        <x:v>关卡节点徽章</x:v>
+      </x:c>
+      <x:c r="D108" s="11" t="str">
+        <x:v>3编号×4态</x:v>
+      </x:c>
+      <x:c r="E108" s="11" t="str">
+        <x:v>三个关卡入口</x:v>
+      </x:c>
+      <x:c r="F108" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G108" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H108" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I108" s="11" t="str">
+        <x:v>美术预留4态；解锁条件 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="60" customHeight="1">
+      <x:c r="A109" s="11" t="str">
+        <x:v>A-104</x:v>
+      </x:c>
+      <x:c r="B109" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C109" s="11" t="str">
+        <x:v>行军路线与箭头</x:v>
+      </x:c>
+      <x:c r="D109" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E109" s="11" t="str">
+        <x:v>1→2→3区域连接</x:v>
+      </x:c>
+      <x:c r="F109" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G109" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H109" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I109" s="11" t="str">
+        <x:v>路线仅为叙事顺序草案，不代表已实现进度</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="60" customHeight="1">
+      <x:c r="A110" s="11" t="str">
+        <x:v>A-105</x:v>
+      </x:c>
+      <x:c r="B110" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C110" s="11" t="str">
+        <x:v>地图山川城邑装饰</x:v>
+      </x:c>
+      <x:c r="D110" s="11" t="str">
+        <x:v>山/河/城/林4类</x:v>
+      </x:c>
+      <x:c r="E110" s="11" t="str">
+        <x:v>地图地貌</x:v>
+      </x:c>
+      <x:c r="F110" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G110" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H110" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I110" s="11" t="str">
+        <x:v>与战斗格地形资产不同，不能混作棋盘素材</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="60" customHeight="1">
+      <x:c r="A111" s="11" t="str">
+        <x:v>A-106</x:v>
+      </x:c>
+      <x:c r="B111" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C111" s="11" t="str">
+        <x:v>关卡介绍插画</x:v>
+      </x:c>
+      <x:c r="D111" s="11" t="str">
+        <x:v>3张</x:v>
+      </x:c>
+      <x:c r="E111" s="11" t="str">
+        <x:v>选关详情卡</x:v>
+      </x:c>
+      <x:c r="F111" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G111" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H111" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I111" s="11" t="str">
+        <x:v>依次山隘、平原城邑、水网；最终题材 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="60" customHeight="1">
+      <x:c r="A112" s="11" t="str">
+        <x:v>A-107</x:v>
+      </x:c>
+      <x:c r="B112" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C112" s="11" t="str">
+        <x:v>选关详情卡底板</x:v>
+      </x:c>
+      <x:c r="D112" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E112" s="11" t="str">
+        <x:v>关卡说明与进入按钮</x:v>
+      </x:c>
+      <x:c r="F112" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G112" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H112" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I112" s="11" t="str">
+        <x:v>标题、难度、奖励用文字；玩法参数 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="60" customHeight="1">
+      <x:c r="A113" s="11" t="str">
+        <x:v>A-108</x:v>
+      </x:c>
+      <x:c r="B113" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C113" s="11" t="str">
+        <x:v>未解锁与通关印章</x:v>
+      </x:c>
+      <x:c r="D113" s="11" t="str">
+        <x:v>2款</x:v>
+      </x:c>
+      <x:c r="E113" s="11" t="str">
+        <x:v>地图节点及介绍卡</x:v>
+      </x:c>
+      <x:c r="F113" s="11" t="str">
+        <x:v>独立美术样稿中预留</x:v>
+      </x:c>
+      <x:c r="G113" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H113" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I113" s="11" t="str">
+        <x:v>不能仅依靠颜色区分状态</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="60" customHeight="1">
+      <x:c r="A114" s="11" t="str">
+        <x:v>A-109</x:v>
+      </x:c>
+      <x:c r="B114" s="11" t="str">
+        <x:v>通用UI</x:v>
+      </x:c>
+      <x:c r="C114" s="11" t="str">
+        <x:v>通用面板底板与边框</x:v>
+      </x:c>
+      <x:c r="D114" s="11" t="str">
+        <x:v>普通/强调2套</x:v>
+      </x:c>
+      <x:c r="E114" s="11" t="str">
+        <x:v>战斗卡片与弹窗</x:v>
+      </x:c>
+      <x:c r="F114" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G114" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H114" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I114" s="11" t="str">
+        <x:v>保留四角，中心可拉伸；复用A-072至A-085容器</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="60" customHeight="1">
+      <x:c r="A115" s="11" t="str">
+        <x:v>A-110</x:v>
+      </x:c>
+      <x:c r="B115" s="11" t="str">
+        <x:v>通用UI</x:v>
+      </x:c>
+      <x:c r="C115" s="11" t="str">
+        <x:v>通用按钮皮肤</x:v>
+      </x:c>
+      <x:c r="D115" s="11" t="str">
+        <x:v>主/次/危险3类×4态</x:v>
+      </x:c>
+      <x:c r="E115" s="11" t="str">
+        <x:v>战斗与弹窗按钮</x:v>
+      </x:c>
+      <x:c r="F115" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G115" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H115" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I115" s="11" t="str">
+        <x:v>结束回合、撤销、暂停、取消、确认共用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="60" customHeight="1">
+      <x:c r="A116" s="11" t="str">
+        <x:v>A-111</x:v>
+      </x:c>
+      <x:c r="B116" s="11" t="str">
+        <x:v>通用UI</x:v>
+      </x:c>
+      <x:c r="C116" s="11" t="str">
+        <x:v>通用功能图标</x:v>
+      </x:c>
+      <x:c r="D116" s="11" t="str">
+        <x:v>8款</x:v>
+      </x:c>
+      <x:c r="E116" s="11" t="str">
+        <x:v>返回/关闭/设置/暂停/继续/重试/收起/展开</x:v>
+      </x:c>
+      <x:c r="F116" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G116" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H116" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I116" s="11" t="str">
+        <x:v>点击区域由程序保持至少44逻辑像素</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="60" customHeight="1">
+      <x:c r="A117" s="11" t="str">
+        <x:v>A-112</x:v>
+      </x:c>
+      <x:c r="B117" s="11" t="str">
+        <x:v>通用UI</x:v>
+      </x:c>
+      <x:c r="C117" s="11" t="str">
+        <x:v>资源属性图标</x:v>
+      </x:c>
+      <x:c r="D117" s="11" t="str">
+        <x:v>7款</x:v>
+      </x:c>
+      <x:c r="E117" s="11" t="str">
+        <x:v>HP/AP/SP/金币/回合/击杀/等级</x:v>
+      </x:c>
+      <x:c r="F117" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G117" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H117" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I117" s="11" t="str">
+        <x:v>保留数值文字，避免仅靠图标猜测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="60" customHeight="1">
+      <x:c r="A118" s="11" t="str">
+        <x:v>A-113</x:v>
+      </x:c>
+      <x:c r="B118" s="11" t="str">
+        <x:v>通用UI</x:v>
+      </x:c>
+      <x:c r="C118" s="11" t="str">
+        <x:v>提示浮层底板</x:v>
+      </x:c>
+      <x:c r="D118" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E118" s="11" t="str">
+        <x:v>未行动名单、说明、悬停信息</x:v>
+      </x:c>
+      <x:c r="F118" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G118" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H118" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I118" s="11" t="str">
+        <x:v>长名单自动伸展；复用通用文本</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="60" customHeight="1">
+      <x:c r="A119" s="11" t="str">
+        <x:v>A-114</x:v>
+      </x:c>
+      <x:c r="B119" s="11" t="str">
+        <x:v>通用UI</x:v>
+      </x:c>
+      <x:c r="C119" s="11" t="str">
+        <x:v>弹窗遮罩</x:v>
+      </x:c>
+      <x:c r="D119" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E119" s="11" t="str">
+        <x:v>暂停/确认/成长等模态层</x:v>
+      </x:c>
+      <x:c r="F119" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G119" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H119" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I119" s="11" t="str">
+        <x:v>透明度由代码配置；不计单独美术图片</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="60" customHeight="1">
+      <x:c r="A120" s="11" t="str">
+        <x:v>A-115</x:v>
+      </x:c>
+      <x:c r="B120" s="11" t="str">
+        <x:v>通用UI</x:v>
+      </x:c>
+      <x:c r="C120" s="11" t="str">
+        <x:v>滚动条与分页页签</x:v>
+      </x:c>
+      <x:c r="D120" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E120" s="11" t="str">
+        <x:v>技能/敌情/手机面板</x:v>
+      </x:c>
+      <x:c r="F120" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G120" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H120" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I120" s="11" t="str">
+        <x:v>文字实时排版；手机保持可触控</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="60" customHeight="1">
+      <x:c r="A121" s="11" t="str">
+        <x:v>A-116</x:v>
+      </x:c>
+      <x:c r="B121" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C121" s="11" t="str">
+        <x:v>棋子头顶血条底框与填充</x:v>
+      </x:c>
+      <x:c r="D121" s="11" t="str">
+        <x:v>敌我2套</x:v>
+      </x:c>
+      <x:c r="E121" s="11" t="str">
+        <x:v>每枚存活棋子上方</x:v>
+      </x:c>
+      <x:c r="F121" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G121" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H121" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I121" s="11" t="str">
+        <x:v>当前数字HP保留；阵营颜色及形状需区分</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="60" customHeight="1">
+      <x:c r="A122" s="11" t="str">
+        <x:v>A-117</x:v>
+      </x:c>
+      <x:c r="B122" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C122" s="11" t="str">
+        <x:v>伤害数字与击杀标记</x:v>
+      </x:c>
+      <x:c r="D122" s="11" t="str">
+        <x:v>普通/友伤/致命3态</x:v>
+      </x:c>
+      <x:c r="E122" s="11" t="str">
+        <x:v>棋盘攻击预览和结算</x:v>
+      </x:c>
+      <x:c r="F122" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G122" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H122" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I122" s="11" t="str">
+        <x:v>不逐个数字切图；与己方技能效果素材分开</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="60" customHeight="1">
+      <x:c r="A123" s="11" t="str">
+        <x:v>A-118</x:v>
+      </x:c>
+      <x:c r="B123" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C123" s="11" t="str">
+        <x:v>攻击与位移方向箭头</x:v>
+      </x:c>
+      <x:c r="D123" s="11" t="str">
+        <x:v>攻击/推/拉3款</x:v>
+      </x:c>
+      <x:c r="E123" s="11" t="str">
+        <x:v>棋盘路径预览</x:v>
+      </x:c>
+      <x:c r="F123" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G123" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H123" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I123" s="11" t="str">
+        <x:v>方向由程序旋转，颜色外保留形状区分</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="60" customHeight="1">
+      <x:c r="A124" s="11" t="str">
+        <x:v>A-119</x:v>
+      </x:c>
+      <x:c r="B124" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C124" s="11" t="str">
+        <x:v>敌方出生预告标记</x:v>
+      </x:c>
+      <x:c r="D124" s="11" t="str">
+        <x:v>3态</x:v>
+      </x:c>
+      <x:c r="E124" s="11" t="str">
+        <x:v>援军出生格</x:v>
+      </x:c>
+      <x:c r="F124" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G124" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H124" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I124" s="11" t="str">
+        <x:v>只表达规则已揭示的信息</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="60" customHeight="1">
+      <x:c r="A125" s="11" t="str">
+        <x:v>A-120</x:v>
+      </x:c>
+      <x:c r="B125" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C125" s="11" t="str">
+        <x:v>主帅增益选择卡</x:v>
+      </x:c>
+      <x:c r="D125" s="11" t="str">
+        <x:v>3款</x:v>
+      </x:c>
+      <x:c r="E125" s="11" t="str">
+        <x:v>坚守/疾行/救援</x:v>
+      </x:c>
+      <x:c r="F125" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G125" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H125" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I125" s="11" t="str">
+        <x:v>不烘焙技能描述和数值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="60" customHeight="1">
+      <x:c r="A126" s="11" t="str">
+        <x:v>A-121</x:v>
+      </x:c>
+      <x:c r="B126" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C126" s="11" t="str">
+        <x:v>技能图标合集</x:v>
+      </x:c>
+      <x:c r="D126" s="11" t="str">
+        <x:v>通用1套＋己方9棋种槽位</x:v>
+      </x:c>
+      <x:c r="E126" s="11" t="str">
+        <x:v>升级/转职/方向/扩散</x:v>
+      </x:c>
+      <x:c r="F126" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G126" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H126" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I126" s="11" t="str">
+        <x:v>与A-042至A-065技能特效分开；敌方不新增主动技能</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="60" customHeight="1">
+      <x:c r="A127" s="11" t="str">
+        <x:v>A-122</x:v>
+      </x:c>
+      <x:c r="B127" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C127" s="11" t="str">
+        <x:v>关卡目标卡与阶段标签</x:v>
+      </x:c>
+      <x:c r="D127" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E127" s="11" t="str">
+        <x:v>保护主帅/回合阶段</x:v>
+      </x:c>
+      <x:c r="F127" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G127" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H127" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I127" s="11" t="str">
+        <x:v>目标文案来自规则，不能写死为图片</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="60" customHeight="1">
+      <x:c r="A128" s="11" t="str">
+        <x:v>A-123</x:v>
+      </x:c>
+      <x:c r="B128" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C128" s="11" t="str">
+        <x:v>结束回合未行动提醒</x:v>
+      </x:c>
+      <x:c r="D128" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E128" s="11" t="str">
+        <x:v>结束回合悬停</x:v>
+      </x:c>
+      <x:c r="F128" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G128" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H128" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I128" s="11" t="str">
+        <x:v>列棋名及坐标；预留未行动徽记96×96</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="60" customHeight="1">
+      <x:c r="A129" s="11" t="str">
+        <x:v>A-124</x:v>
+      </x:c>
+      <x:c r="B129" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C129" s="11" t="str">
+        <x:v>布阵与上阵后备标记</x:v>
+      </x:c>
+      <x:c r="D129" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E129" s="11" t="str">
+        <x:v>布阵/商店队伍管理</x:v>
+      </x:c>
+      <x:c r="F129" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G129" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H129" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I129" s="11" t="str">
+        <x:v>头像复用己方棋子资源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="60" customHeight="1">
+      <x:c r="A130" s="11" t="str">
+        <x:v>A-125</x:v>
+      </x:c>
+      <x:c r="B130" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C130" s="11" t="str">
+        <x:v>救援角色卡与恢复标记</x:v>
+      </x:c>
+      <x:c r="D130" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E130" s="11" t="str">
+        <x:v>第6回合救援</x:v>
+      </x:c>
+      <x:c r="F130" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G130" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H130" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I130" s="11" t="str">
+        <x:v>人物形象复用棋子；恢复表现关联技能通用效果</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="60" customHeight="1">
+      <x:c r="A131" s="11" t="str">
+        <x:v>A-126</x:v>
+      </x:c>
+      <x:c r="B131" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C131" s="11" t="str">
+        <x:v>商店商品与价格标签</x:v>
+      </x:c>
+      <x:c r="D131" s="11" t="str">
+        <x:v>兵/车/马/炮4类</x:v>
+      </x:c>
+      <x:c r="E131" s="11" t="str">
+        <x:v>关间整备</x:v>
+      </x:c>
+      <x:c r="F131" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G131" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H131" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I131" s="11" t="str">
+        <x:v>棋子像复用，价格由程序写入</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="60" customHeight="1">
+      <x:c r="A132" s="11" t="str">
+        <x:v>A-127</x:v>
+      </x:c>
+      <x:c r="B132" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C132" s="11" t="str">
+        <x:v>胜败结果标题与装饰</x:v>
+      </x:c>
+      <x:c r="D132" s="11" t="str">
+        <x:v>胜利/主帅阵亡/将死3款</x:v>
+      </x:c>
+      <x:c r="E132" s="11" t="str">
+        <x:v>结果界面</x:v>
+      </x:c>
+      <x:c r="F132" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G132" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H132" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I132" s="11" t="str">
+        <x:v>统计数字和操作按钮独立</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="60" customHeight="1">
+      <x:c r="A133" s="11" t="str">
+        <x:v>A-128</x:v>
+      </x:c>
+      <x:c r="B133" s="11" t="str">
+        <x:v>手机UI</x:v>
+      </x:c>
+      <x:c r="C133" s="11" t="str">
+        <x:v>底部信息导航图标</x:v>
+      </x:c>
+      <x:c r="D133" s="11" t="str">
+        <x:v>4款</x:v>
+      </x:c>
+      <x:c r="E133" s="11" t="str">
+        <x:v>队伍/技能/敌情/更多</x:v>
+      </x:c>
+      <x:c r="F133" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G133" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H133" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I133" s="11" t="str">
+        <x:v>448×924逻辑视口，3倍参考导出；保持一屏</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="60" customHeight="1">
+      <x:c r="A134" s="11" t="str">
+        <x:v>A-129</x:v>
+      </x:c>
+      <x:c r="B134" s="11" t="str">
+        <x:v>手机UI</x:v>
+      </x:c>
+      <x:c r="C134" s="11" t="str">
+        <x:v>信息展开面板与抓手</x:v>
+      </x:c>
+      <x:c r="D134" s="11" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="E134" s="11" t="str">
+        <x:v>完整详情、敌情、战况记录</x:v>
+      </x:c>
+      <x:c r="F134" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G134" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H134" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I134" s="11" t="str">
+        <x:v>内容可内部滚动，主战斗页不滚动</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="60" customHeight="1">
+      <x:c r="A135" s="11" t="str">
+        <x:v>A-130</x:v>
+      </x:c>
+      <x:c r="B135" s="11" t="str">
+        <x:v>手机UI</x:v>
+      </x:c>
+      <x:c r="C135" s="11" t="str">
+        <x:v>紧凑棋子与预览卡</x:v>
+      </x:c>
+      <x:c r="D135" s="11" t="str">
+        <x:v>2套</x:v>
+      </x:c>
+      <x:c r="E135" s="11" t="str">
+        <x:v>棋盘下方摘要</x:v>
+      </x:c>
+      <x:c r="F135" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G135" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H135" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I135" s="11" t="str">
+        <x:v>与桌面信息同源，文本不烘焙</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="60" customHeight="1">
+      <x:c r="A136" s="11" t="str">
+        <x:v>A-131</x:v>
+      </x:c>
+      <x:c r="B136" s="11" t="str">
+        <x:v>通用UI</x:v>
+      </x:c>
+      <x:c r="C136" s="11" t="str">
+        <x:v>字体与排版规范</x:v>
+      </x:c>
+      <x:c r="D136" s="11" t="str">
+        <x:v>标题/正文/数字3用途</x:v>
+      </x:c>
+      <x:c r="E136" s="11" t="str">
+        <x:v>全部页面</x:v>
+      </x:c>
+      <x:c r="F136" s="11" t="str">
+        <x:v>现有HTML/CSS或资源规格预留</x:v>
+      </x:c>
+      <x:c r="G136" s="11" t="str">
+        <x:v>预留／待制作</x:v>
+      </x:c>
+      <x:c r="H136" s="11" t="str">
+        <x:v>2026-10-05 美术需求</x:v>
+      </x:c>
+      <x:c r="I136" s="11" t="str">
+        <x:v>字体授权 TBD；资源尺寸为制作建议，最终风格待确认</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2913,7 +4314,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd18c32eec5642d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6c06b4ef505437e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3030,7 +4431,7 @@
     </x:row>
     <x:row r="7" ht="29" customHeight="1">
       <x:c r="A7" s="1" t="str">
-        <x:v>当前网页没有独立图片、模型或字体文件。棋盘、棋子、标记由 web/js/app.js 绘制；界面由 web/index.html 的 HTML/CSS 呈现。</x:v>
+        <x:v>新增的Loading、菜单和三关地图为HTML/CSS/SVG占位，尚无正式插画或切图。资源预留清单已建立；独立地形实验和旧源图片保留。</x:v>
       </x:c>
       <x:c r="B7" s="1"/>
       <x:c r="C7" s="1"/>
@@ -3059,7 +4460,1973 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a0cfd5789394cb6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35e0ce456f4f4c07"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="29" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="27" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="53" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>UI 美术交付规格</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="13" t="str">
+        <x:v>尺寸为建议制作像素。手机参考布局448×924，资源按3倍制作；桌面1920×1080并支持缩放。编号与主清单一一对应，组件总项和子资源不能简单相加为图片数。最终风格、历史疆界、动画和功能接入待确认。</x:v>
+      </x:c>
+      <x:c r="B2" s="13"/>
+      <x:c r="C2" s="13"/>
+      <x:c r="D2" s="13"/>
+      <x:c r="E2" s="13"/>
+      <x:c r="F2" s="13"/>
+      <x:c r="G2" s="13"/>
+      <x:c r="H2" s="13"/>
+      <x:c r="I2" s="13"/>
+    </x:row>
+    <x:row r="3" ht="25" customHeight="1">
+      <x:c r="A3" s="13"/>
+      <x:c r="B3" s="13"/>
+      <x:c r="C3" s="13"/>
+      <x:c r="D3" s="13"/>
+      <x:c r="E3" s="13"/>
+      <x:c r="F3" s="13"/>
+      <x:c r="G3" s="13"/>
+      <x:c r="H3" s="13"/>
+      <x:c r="I3" s="13"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="18" t="str">
+        <x:v>编号</x:v>
+      </x:c>
+      <x:c r="B5" s="18" t="str">
+        <x:v>资源/组件</x:v>
+      </x:c>
+      <x:c r="C5" s="18" t="str">
+        <x:v>替换槽位名</x:v>
+      </x:c>
+      <x:c r="D5" s="18" t="str">
+        <x:v>建议尺寸 px</x:v>
+      </x:c>
+      <x:c r="E5" s="18" t="str">
+        <x:v>格式与切图</x:v>
+      </x:c>
+      <x:c r="F5" s="18" t="str">
+        <x:v>交互状态</x:v>
+      </x:c>
+      <x:c r="G5" s="18" t="str">
+        <x:v>使用位置</x:v>
+      </x:c>
+      <x:c r="H5" s="18" t="str">
+        <x:v>数量/变体</x:v>
+      </x:c>
+      <x:c r="I5" s="18" t="str">
+        <x:v>交付说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="76" customHeight="1">
+      <x:c r="A6" s="19" t="str">
+        <x:v>A-072</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="str">
+        <x:v>战斗背景与主布局</x:v>
+      </x:c>
+      <x:c r="C6" s="19" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D6" s="19" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E6" s="19" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F6" s="19" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G6" s="19" t="str">
+        <x:v>桌面菱形棋盘四角HUD；手机一屏布局</x:v>
+      </x:c>
+      <x:c r="H6" s="19" t="str">
+        <x:v>桌面／手机2套</x:v>
+      </x:c>
+      <x:c r="I6" s="19" t="str">
+        <x:v>组件总项；面板切图复用A-109起通用资源，桌面1920×1080、手机1344×2772</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="76" customHeight="1">
+      <x:c r="A7" s="16" t="str">
+        <x:v>A-073</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="str">
+        <x:v>战斗状态栏</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F7" s="16" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="str">
+        <x:v>波次、回合、主帅HP、金币、击杀</x:v>
+      </x:c>
+      <x:c r="H7" s="16" t="str">
+        <x:v>桌面／手机2套</x:v>
+      </x:c>
+      <x:c r="I7" s="16" t="str">
+        <x:v>桌面左上；手机仅保留紧凑主要数值，完整状态折叠</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="76" customHeight="1">
+      <x:c r="A8" s="19" t="str">
+        <x:v>A-074</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
+        <x:v>我方单位列表与棋子徽记</x:v>
+      </x:c>
+      <x:c r="C8" s="19" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D8" s="19" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E8" s="19" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F8" s="19" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G8" s="19" t="str">
+        <x:v>选棋与单位状态</x:v>
+      </x:c>
+      <x:c r="H8" s="19" t="str">
+        <x:v>敌我可区分，己方9棋种槽位</x:v>
+      </x:c>
+      <x:c r="I8" s="19" t="str">
+        <x:v>徽记复用棋子；默认/选中/行动耗尽；未实现棋种仍仅预留</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="76" customHeight="1">
+      <x:c r="A9" s="16" t="str">
+        <x:v>A-075</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="str">
+        <x:v>当前棋子信息卡</x:v>
+      </x:c>
+      <x:c r="C9" s="16" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D9" s="16" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E9" s="16" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F9" s="16" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="str">
+        <x:v>属性、行动余量、等级、SP</x:v>
+      </x:c>
+      <x:c r="H9" s="16" t="str">
+        <x:v>桌面详情／手机摘要</x:v>
+      </x:c>
+      <x:c r="I9" s="16" t="str">
+        <x:v>长说明可展开，动态数值不烘焙</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="76" customHeight="1">
+      <x:c r="A10" s="19" t="str">
+        <x:v>A-076</x:v>
+      </x:c>
+      <x:c r="B10" s="19" t="str">
+        <x:v>技能条目与禁用状态</x:v>
+      </x:c>
+      <x:c r="C10" s="19" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D10" s="19" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E10" s="19" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F10" s="19" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G10" s="19" t="str">
+        <x:v>升级、转职、方向和炮扩散</x:v>
+      </x:c>
+      <x:c r="H10" s="19" t="str">
+        <x:v>1套＋图标槽位</x:v>
+      </x:c>
+      <x:c r="I10" s="19" t="str">
+        <x:v>可购买/已解锁/缺SP/当前阶段不可购买；专属技能仍为己方</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="76" customHeight="1">
+      <x:c r="A11" s="16" t="str">
+        <x:v>A-077</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>方向与车模式按钮</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D11" s="16" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E11" s="16" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F11" s="16" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str">
+        <x:v>弓枪方向；车职业模式</x:v>
+      </x:c>
+      <x:c r="H11" s="16" t="str">
+        <x:v>四方向＋移动/冲锋/牵引</x:v>
+      </x:c>
+      <x:c r="I11" s="16" t="str">
+        <x:v>默认/选中/禁用；手机触控面积至少44逻辑像素</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="76" customHeight="1">
+      <x:c r="A12" s="19" t="str">
+        <x:v>A-078</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
+        <x:v>敌方意图列表与序号</x:v>
+      </x:c>
+      <x:c r="C12" s="19" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D12" s="19" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E12" s="19" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F12" s="19" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G12" s="19" t="str">
+        <x:v>敌方行动顺序和预期状态</x:v>
+      </x:c>
+      <x:c r="H12" s="19" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I12" s="19" t="str">
+        <x:v>成功/失效/落空/已移除/待机需区分</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="76" customHeight="1">
+      <x:c r="A13" s="16" t="str">
+        <x:v>A-079</x:v>
+      </x:c>
+      <x:c r="B13" s="16" t="str">
+        <x:v>动作预览与受击警告</x:v>
+      </x:c>
+      <x:c r="C13" s="16" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D13" s="16" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E13" s="16" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F13" s="16" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G13" s="16" t="str">
+        <x:v>路径、伤害、友伤、主帅威胁</x:v>
+      </x:c>
+      <x:c r="H13" s="16" t="str">
+        <x:v>桌面详情／手机摘要</x:v>
+      </x:c>
+      <x:c r="I13" s="16" t="str">
+        <x:v>友伤醒目；桌面点目标直接攻击，手机保留执行确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="76" customHeight="1">
+      <x:c r="A14" s="19" t="str">
+        <x:v>A-080</x:v>
+      </x:c>
+      <x:c r="B14" s="19" t="str">
+        <x:v>战斗操作按钮</x:v>
+      </x:c>
+      <x:c r="C14" s="19" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D14" s="19" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E14" s="19" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F14" s="19" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G14" s="19" t="str">
+        <x:v>桌面左上与手机底部</x:v>
+      </x:c>
+      <x:c r="H14" s="19" t="str">
+        <x:v>执行/取消/撤销/结束回合/暂停</x:v>
+      </x:c>
+      <x:c r="I14" s="19" t="str">
+        <x:v>桌面隐藏执行按钮；底板共用通用按钮皮肤</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="76" customHeight="1">
+      <x:c r="A15" s="16" t="str">
+        <x:v>A-081</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="str">
+        <x:v>结束回合确认弹窗</x:v>
+      </x:c>
+      <x:c r="C15" s="16" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D15" s="16" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E15" s="16" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F15" s="16" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G15" s="16" t="str">
+        <x:v>结算敌方阶段前确认</x:v>
+      </x:c>
+      <x:c r="H15" s="16" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I15" s="16" t="str">
+        <x:v>确认/继续行动；未行动名单为独立悬停组件</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="76" customHeight="1">
+      <x:c r="A16" s="19" t="str">
+        <x:v>A-082</x:v>
+      </x:c>
+      <x:c r="B16" s="19" t="str">
+        <x:v>暂停弹窗</x:v>
+      </x:c>
+      <x:c r="C16" s="19" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D16" s="19" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E16" s="19" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F16" s="19" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G16" s="19" t="str">
+        <x:v>继续/重新开始</x:v>
+      </x:c>
+      <x:c r="H16" s="19" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I16" s="19" t="str">
+        <x:v>复用面板、遮罩、主次按钮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="76" customHeight="1">
+      <x:c r="A17" s="16" t="str">
+        <x:v>A-083</x:v>
+      </x:c>
+      <x:c r="B17" s="16" t="str">
+        <x:v>商店与商品卡</x:v>
+      </x:c>
+      <x:c r="C17" s="16" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D17" s="16" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E17" s="16" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F17" s="16" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G17" s="16" t="str">
+        <x:v>关间整备与上阵后备</x:v>
+      </x:c>
+      <x:c r="H17" s="16" t="str">
+        <x:v>兵/车/马/炮4类</x:v>
+      </x:c>
+      <x:c r="I17" s="16" t="str">
+        <x:v>商品像复用棋子；价格、阵容容量实时文字</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="76" customHeight="1">
+      <x:c r="A18" s="19" t="str">
+        <x:v>A-084</x:v>
+      </x:c>
+      <x:c r="B18" s="19" t="str">
+        <x:v>终局弹窗</x:v>
+      </x:c>
+      <x:c r="C18" s="19" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D18" s="19" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E18" s="19" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F18" s="19" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G18" s="19" t="str">
+        <x:v>战斗结果</x:v>
+      </x:c>
+      <x:c r="H18" s="19" t="str">
+        <x:v>胜利/阵亡/将死3态</x:v>
+      </x:c>
+      <x:c r="I18" s="19" t="str">
+        <x:v>独立结果标题装饰详见新增条目；统计数字实时文字</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="76" customHeight="1">
+      <x:c r="A19" s="16" t="str">
+        <x:v>A-085</x:v>
+      </x:c>
+      <x:c r="B19" s="16" t="str">
+        <x:v>短提示与危险提示</x:v>
+      </x:c>
+      <x:c r="C19" s="16" t="str">
+        <x:v>现有组件总项；复用通用资源</x:v>
+      </x:c>
+      <x:c r="D19" s="16" t="str">
+        <x:v>桌面1920×1080；手机1344×2772</x:v>
+      </x:c>
+      <x:c r="E19" s="16" t="str">
+        <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
+      </x:c>
+      <x:c r="F19" s="16" t="str">
+        <x:v>详见用途与主清单</x:v>
+      </x:c>
+      <x:c r="G19" s="16" t="str">
+        <x:v>购买、重开、操作失败、危险反馈</x:v>
+      </x:c>
+      <x:c r="H19" s="16" t="str">
+        <x:v>普通/成功/警告3态</x:v>
+      </x:c>
+      <x:c r="I19" s="16" t="str">
+        <x:v>底板复用；提示色必须同时有文字或图标辨识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="76" customHeight="1">
+      <x:c r="A20" s="19" t="str">
+        <x:v>A-087</x:v>
+      </x:c>
+      <x:c r="B20" s="19" t="str">
+        <x:v>Loading 背景</x:v>
+      </x:c>
+      <x:c r="C20" s="19" t="str">
+        <x:v>loading-bg</x:v>
+      </x:c>
+      <x:c r="D20" s="19" t="str">
+        <x:v>1920×1080 / 1344×2772</x:v>
+      </x:c>
+      <x:c r="E20" s="19" t="str">
+        <x:v>WebP/JPG，不透明</x:v>
+      </x:c>
+      <x:c r="F20" s="19" t="str">
+        <x:v>加载静态背景</x:v>
+      </x:c>
+      <x:c r="G20" s="19" t="str">
+        <x:v>全屏背景</x:v>
+      </x:c>
+      <x:c r="H20" s="19" t="str">
+        <x:v>横竖2版</x:v>
+      </x:c>
+      <x:c r="I20" s="19" t="str">
+        <x:v>重要主体留在中央安全区；横竖单独构图</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="76" customHeight="1">
+      <x:c r="A21" s="16" t="str">
+        <x:v>A-088</x:v>
+      </x:c>
+      <x:c r="B21" s="16" t="str">
+        <x:v>游戏标志与题字</x:v>
+      </x:c>
+      <x:c r="C21" s="16" t="str">
+        <x:v>game-logo</x:v>
+      </x:c>
+      <x:c r="D21" s="16" t="str">
+        <x:v>横版640×240 / 竖版900×360</x:v>
+      </x:c>
+      <x:c r="E21" s="16" t="str">
+        <x:v>PNG/SVG，透明</x:v>
+      </x:c>
+      <x:c r="F21" s="16" t="str">
+        <x:v>正常</x:v>
+      </x:c>
+      <x:c r="G21" s="16" t="str">
+        <x:v>Loading/主菜单共用</x:v>
+      </x:c>
+      <x:c r="H21" s="16" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I21" s="16" t="str">
+        <x:v>暂用九格战阵文字；正式标志 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="76" customHeight="1">
+      <x:c r="A22" s="19" t="str">
+        <x:v>A-089</x:v>
+      </x:c>
+      <x:c r="B22" s="19" t="str">
+        <x:v>加载进度条底框</x:v>
+      </x:c>
+      <x:c r="C22" s="19" t="str">
+        <x:v>loading-track</x:v>
+      </x:c>
+      <x:c r="D22" s="19" t="str">
+        <x:v>800×40</x:v>
+      </x:c>
+      <x:c r="E22" s="19" t="str">
+        <x:v>PNG，透明，横向九宫格</x:v>
+      </x:c>
+      <x:c r="F22" s="19" t="str">
+        <x:v>正常</x:v>
+      </x:c>
+      <x:c r="G22" s="19" t="str">
+        <x:v>Loading 底部</x:v>
+      </x:c>
+      <x:c r="H22" s="19" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I22" s="19" t="str">
+        <x:v>底框与填充分离，长度由程序控制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="76" customHeight="1">
+      <x:c r="A23" s="16" t="str">
+        <x:v>A-090</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="str">
+        <x:v>加载进度条填充</x:v>
+      </x:c>
+      <x:c r="C23" s="16" t="str">
+        <x:v>loading-fill</x:v>
+      </x:c>
+      <x:c r="D23" s="16" t="str">
+        <x:v>760×24</x:v>
+      </x:c>
+      <x:c r="E23" s="16" t="str">
+        <x:v>PNG，透明，可平铺</x:v>
+      </x:c>
+      <x:c r="F23" s="16" t="str">
+        <x:v>0%至100%由代码裁切</x:v>
+      </x:c>
+      <x:c r="G23" s="16" t="str">
+        <x:v>Loading 进度</x:v>
+      </x:c>
+      <x:c r="H23" s="16" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I23" s="16" t="str">
+        <x:v>不把百分比烘焙到图片</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="76" customHeight="1">
+      <x:c r="A24" s="19" t="str">
+        <x:v>A-091</x:v>
+      </x:c>
+      <x:c r="B24" s="19" t="str">
+        <x:v>加载提示框与装饰</x:v>
+      </x:c>
+      <x:c r="C24" s="19" t="str">
+        <x:v>loading-tip</x:v>
+      </x:c>
+      <x:c r="D24" s="19" t="str">
+        <x:v>1000×120</x:v>
+      </x:c>
+      <x:c r="E24" s="19" t="str">
+        <x:v>PNG，透明，九宫格</x:v>
+      </x:c>
+      <x:c r="F24" s="19" t="str">
+        <x:v>正常</x:v>
+      </x:c>
+      <x:c r="G24" s="19" t="str">
+        <x:v>Loading 文案区域</x:v>
+      </x:c>
+      <x:c r="H24" s="19" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I24" s="19" t="str">
+        <x:v>文案用实时文字；字体需可商用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="76" customHeight="1">
+      <x:c r="A25" s="16" t="str">
+        <x:v>A-092</x:v>
+      </x:c>
+      <x:c r="B25" s="16" t="str">
+        <x:v>加载旋转标识</x:v>
+      </x:c>
+      <x:c r="C25" s="16" t="str">
+        <x:v>loading-spinner</x:v>
+      </x:c>
+      <x:c r="D25" s="16" t="str">
+        <x:v>128×128</x:v>
+      </x:c>
+      <x:c r="E25" s="16" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F25" s="16" t="str">
+        <x:v>循环旋转</x:v>
+      </x:c>
+      <x:c r="G25" s="16" t="str">
+        <x:v>Loading 等待状态</x:v>
+      </x:c>
+      <x:c r="H25" s="16" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I25" s="16" t="str">
+        <x:v>代码旋转即可；不强制逐帧动画</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="76" customHeight="1">
+      <x:c r="A26" s="19" t="str">
+        <x:v>A-093</x:v>
+      </x:c>
+      <x:c r="B26" s="19" t="str">
+        <x:v>加载失败与重试提示</x:v>
+      </x:c>
+      <x:c r="C26" s="19" t="str">
+        <x:v>loading-error</x:v>
+      </x:c>
+      <x:c r="D26" s="19" t="str">
+        <x:v>图标96×96；框复用通用弹窗</x:v>
+      </x:c>
+      <x:c r="E26" s="19" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F26" s="19" t="str">
+        <x:v>失败/重试</x:v>
+      </x:c>
+      <x:c r="G26" s="19" t="str">
+        <x:v>Loading 异常态</x:v>
+      </x:c>
+      <x:c r="H26" s="19" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I26" s="19" t="str">
+        <x:v>预留视觉状态，样稿不模拟网络异常</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="76" customHeight="1">
+      <x:c r="A27" s="16" t="str">
+        <x:v>A-094</x:v>
+      </x:c>
+      <x:c r="B27" s="16" t="str">
+        <x:v>主菜单背景</x:v>
+      </x:c>
+      <x:c r="C27" s="16" t="str">
+        <x:v>menu-bg</x:v>
+      </x:c>
+      <x:c r="D27" s="16" t="str">
+        <x:v>1920×1080 / 1344×2772</x:v>
+      </x:c>
+      <x:c r="E27" s="16" t="str">
+        <x:v>WebP/JPG，不透明</x:v>
+      </x:c>
+      <x:c r="F27" s="16" t="str">
+        <x:v>正常</x:v>
+      </x:c>
+      <x:c r="G27" s="16" t="str">
+        <x:v>主菜单全屏</x:v>
+      </x:c>
+      <x:c r="H27" s="16" t="str">
+        <x:v>横竖2版</x:v>
+      </x:c>
+      <x:c r="I27" s="16" t="str">
+        <x:v>文字与按钮独立，不烘焙</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="76" customHeight="1">
+      <x:c r="A28" s="19" t="str">
+        <x:v>A-095</x:v>
+      </x:c>
+      <x:c r="B28" s="19" t="str">
+        <x:v>主菜单主按钮</x:v>
+      </x:c>
+      <x:c r="C28" s="19" t="str">
+        <x:v>menu-primary</x:v>
+      </x:c>
+      <x:c r="D28" s="19" t="str">
+        <x:v>480×96</x:v>
+      </x:c>
+      <x:c r="E28" s="19" t="str">
+        <x:v>PNG，透明，九宫格</x:v>
+      </x:c>
+      <x:c r="F28" s="19" t="str">
+        <x:v>默认/悬停/按下/禁用</x:v>
+      </x:c>
+      <x:c r="G28" s="19" t="str">
+        <x:v>开始游戏/继续游戏</x:v>
+      </x:c>
+      <x:c r="H28" s="19" t="str">
+        <x:v>4态</x:v>
+      </x:c>
+      <x:c r="I28" s="19" t="str">
+        <x:v>两个功能共用按钮皮肤，继续游戏规则 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="76" customHeight="1">
+      <x:c r="A29" s="16" t="str">
+        <x:v>A-096</x:v>
+      </x:c>
+      <x:c r="B29" s="16" t="str">
+        <x:v>主菜单次按钮</x:v>
+      </x:c>
+      <x:c r="C29" s="16" t="str">
+        <x:v>menu-secondary</x:v>
+      </x:c>
+      <x:c r="D29" s="16" t="str">
+        <x:v>360×72</x:v>
+      </x:c>
+      <x:c r="E29" s="16" t="str">
+        <x:v>PNG，透明，九宫格</x:v>
+      </x:c>
+      <x:c r="F29" s="16" t="str">
+        <x:v>默认/悬停/按下/禁用</x:v>
+      </x:c>
+      <x:c r="G29" s="16" t="str">
+        <x:v>设置/制作人员/返回</x:v>
+      </x:c>
+      <x:c r="H29" s="16" t="str">
+        <x:v>4态</x:v>
+      </x:c>
+      <x:c r="I29" s="16" t="str">
+        <x:v>按钮文字独立</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="76" customHeight="1">
+      <x:c r="A30" s="19" t="str">
+        <x:v>A-097</x:v>
+      </x:c>
+      <x:c r="B30" s="19" t="str">
+        <x:v>菜单装饰前景</x:v>
+      </x:c>
+      <x:c r="C30" s="19" t="str">
+        <x:v>menu-ornament</x:v>
+      </x:c>
+      <x:c r="D30" s="19" t="str">
+        <x:v>1920×1080 / 1344×2772</x:v>
+      </x:c>
+      <x:c r="E30" s="19" t="str">
+        <x:v>PNG/WebP，透明</x:v>
+      </x:c>
+      <x:c r="F30" s="19" t="str">
+        <x:v>静态</x:v>
+      </x:c>
+      <x:c r="G30" s="19" t="str">
+        <x:v>主菜单边角</x:v>
+      </x:c>
+      <x:c r="H30" s="19" t="str">
+        <x:v>横竖2版</x:v>
+      </x:c>
+      <x:c r="I30" s="19" t="str">
+        <x:v>可用棋子/兵旗/印章；不遮挡按钮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="76" customHeight="1">
+      <x:c r="A31" s="16" t="str">
+        <x:v>A-098</x:v>
+      </x:c>
+      <x:c r="B31" s="16" t="str">
+        <x:v>战国题材地图底图</x:v>
+      </x:c>
+      <x:c r="C31" s="16" t="str">
+        <x:v>campaign-map</x:v>
+      </x:c>
+      <x:c r="D31" s="16" t="str">
+        <x:v>1920×1080 / 1344×2772</x:v>
+      </x:c>
+      <x:c r="E31" s="16" t="str">
+        <x:v>WebP/PNG；另交分层源文件</x:v>
+      </x:c>
+      <x:c r="F31" s="16" t="str">
+        <x:v>无选中态底图</x:v>
+      </x:c>
+      <x:c r="G31" s="16" t="str">
+        <x:v>开始游戏后的选关页</x:v>
+      </x:c>
+      <x:c r="H31" s="16" t="str">
+        <x:v>横竖2版</x:v>
+      </x:c>
+      <x:c r="I31" s="16" t="str">
+        <x:v>三分区为玩法草案；历史边界和时代年份 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="76" customHeight="1">
+      <x:c r="A32" s="19" t="str">
+        <x:v>A-099</x:v>
+      </x:c>
+      <x:c r="B32" s="19" t="str">
+        <x:v>第1关区域 关中</x:v>
+      </x:c>
+      <x:c r="C32" s="19" t="str">
+        <x:v>region-01</x:v>
+      </x:c>
+      <x:c r="D32" s="19" t="str">
+        <x:v>统一地图画布，按底图同坐标导出</x:v>
+      </x:c>
+      <x:c r="E32" s="19" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F32" s="19" t="str">
+        <x:v>默认/悬停/选中</x:v>
+      </x:c>
+      <x:c r="G32" s="19" t="str">
+        <x:v>西部关卡区域</x:v>
+      </x:c>
+      <x:c r="H32" s="19" t="str">
+        <x:v>3态</x:v>
+      </x:c>
+      <x:c r="I32" s="19" t="str">
+        <x:v>西部关中主题；山隘/城塞视觉；区域范围与关名 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="76" customHeight="1">
+      <x:c r="A33" s="16" t="str">
+        <x:v>A-100</x:v>
+      </x:c>
+      <x:c r="B33" s="16" t="str">
+        <x:v>第2关区域 中原</x:v>
+      </x:c>
+      <x:c r="C33" s="16" t="str">
+        <x:v>region-02</x:v>
+      </x:c>
+      <x:c r="D33" s="16" t="str">
+        <x:v>统一地图画布，按底图同坐标导出</x:v>
+      </x:c>
+      <x:c r="E33" s="16" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F33" s="16" t="str">
+        <x:v>默认/悬停/选中</x:v>
+      </x:c>
+      <x:c r="G33" s="16" t="str">
+        <x:v>中央关卡区域</x:v>
+      </x:c>
+      <x:c r="H33" s="16" t="str">
+        <x:v>3态</x:v>
+      </x:c>
+      <x:c r="I33" s="16" t="str">
+        <x:v>中央平原主题；河流/城邑视觉；区域范围与关名 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="76" customHeight="1">
+      <x:c r="A34" s="19" t="str">
+        <x:v>A-101</x:v>
+      </x:c>
+      <x:c r="B34" s="19" t="str">
+        <x:v>第3关区域 江淮</x:v>
+      </x:c>
+      <x:c r="C34" s="19" t="str">
+        <x:v>region-03</x:v>
+      </x:c>
+      <x:c r="D34" s="19" t="str">
+        <x:v>统一地图画布，按底图同坐标导出</x:v>
+      </x:c>
+      <x:c r="E34" s="19" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F34" s="19" t="str">
+        <x:v>默认/悬停/选中</x:v>
+      </x:c>
+      <x:c r="G34" s="19" t="str">
+        <x:v>东南关卡区域</x:v>
+      </x:c>
+      <x:c r="H34" s="19" t="str">
+        <x:v>3态</x:v>
+      </x:c>
+      <x:c r="I34" s="19" t="str">
+        <x:v>东南水网主题；水泽/林地视觉；区域范围与关名 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="76" customHeight="1">
+      <x:c r="A35" s="16" t="str">
+        <x:v>A-102</x:v>
+      </x:c>
+      <x:c r="B35" s="16" t="str">
+        <x:v>区域分界描边</x:v>
+      </x:c>
+      <x:c r="C35" s="16" t="str">
+        <x:v>region-border</x:v>
+      </x:c>
+      <x:c r="D35" s="16" t="str">
+        <x:v>与地图画布一致</x:v>
+      </x:c>
+      <x:c r="E35" s="16" t="str">
+        <x:v>SVG优先，透明</x:v>
+      </x:c>
+      <x:c r="F35" s="16" t="str">
+        <x:v>常态/选中加粗</x:v>
+      </x:c>
+      <x:c r="G35" s="16" t="str">
+        <x:v>地图分区</x:v>
+      </x:c>
+      <x:c r="H35" s="16" t="str">
+        <x:v>1套3区域</x:v>
+      </x:c>
+      <x:c r="I35" s="16" t="str">
+        <x:v>三个区域共边不得出现缝隙；非真实国界</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="76" customHeight="1">
+      <x:c r="A36" s="19" t="str">
+        <x:v>A-103</x:v>
+      </x:c>
+      <x:c r="B36" s="19" t="str">
+        <x:v>关卡节点徽章</x:v>
+      </x:c>
+      <x:c r="C36" s="19" t="str">
+        <x:v>level-node</x:v>
+      </x:c>
+      <x:c r="D36" s="19" t="str">
+        <x:v>192×192</x:v>
+      </x:c>
+      <x:c r="E36" s="19" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F36" s="19" t="str">
+        <x:v>未解锁/可挑战/当前选择/已通关</x:v>
+      </x:c>
+      <x:c r="G36" s="19" t="str">
+        <x:v>三个关卡入口</x:v>
+      </x:c>
+      <x:c r="H36" s="19" t="str">
+        <x:v>3编号×4态</x:v>
+      </x:c>
+      <x:c r="I36" s="19" t="str">
+        <x:v>美术预留4态；解锁条件 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="76" customHeight="1">
+      <x:c r="A37" s="16" t="str">
+        <x:v>A-104</x:v>
+      </x:c>
+      <x:c r="B37" s="16" t="str">
+        <x:v>行军路线与箭头</x:v>
+      </x:c>
+      <x:c r="C37" s="16" t="str">
+        <x:v>campaign-route</x:v>
+      </x:c>
+      <x:c r="D37" s="16" t="str">
+        <x:v>24px线宽；端点64×64</x:v>
+      </x:c>
+      <x:c r="E37" s="16" t="str">
+        <x:v>SVG，透明</x:v>
+      </x:c>
+      <x:c r="F37" s="16" t="str">
+        <x:v>未推进/已推进</x:v>
+      </x:c>
+      <x:c r="G37" s="16" t="str">
+        <x:v>1→2→3区域连接</x:v>
+      </x:c>
+      <x:c r="H37" s="16" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I37" s="16" t="str">
+        <x:v>路线仅为叙事顺序草案，不代表已实现进度</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="76" customHeight="1">
+      <x:c r="A38" s="19" t="str">
+        <x:v>A-105</x:v>
+      </x:c>
+      <x:c r="B38" s="19" t="str">
+        <x:v>地图山川城邑装饰</x:v>
+      </x:c>
+      <x:c r="C38" s="19" t="str">
+        <x:v>map-landmarks</x:v>
+      </x:c>
+      <x:c r="D38" s="19" t="str">
+        <x:v>256×256图标或底图独立图层</x:v>
+      </x:c>
+      <x:c r="E38" s="19" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F38" s="19" t="str">
+        <x:v>静态</x:v>
+      </x:c>
+      <x:c r="G38" s="19" t="str">
+        <x:v>地图地貌</x:v>
+      </x:c>
+      <x:c r="H38" s="19" t="str">
+        <x:v>山/河/城/林4类</x:v>
+      </x:c>
+      <x:c r="I38" s="19" t="str">
+        <x:v>与战斗格地形资产不同，不能混作棋盘素材</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="76" customHeight="1">
+      <x:c r="A39" s="16" t="str">
+        <x:v>A-106</x:v>
+      </x:c>
+      <x:c r="B39" s="16" t="str">
+        <x:v>关卡介绍插画</x:v>
+      </x:c>
+      <x:c r="C39" s="16" t="str">
+        <x:v>level-art</x:v>
+      </x:c>
+      <x:c r="D39" s="16" t="str">
+        <x:v>640×360 / 900×600</x:v>
+      </x:c>
+      <x:c r="E39" s="16" t="str">
+        <x:v>WebP/JPG，不透明</x:v>
+      </x:c>
+      <x:c r="F39" s="16" t="str">
+        <x:v>每关1张</x:v>
+      </x:c>
+      <x:c r="G39" s="16" t="str">
+        <x:v>选关详情卡</x:v>
+      </x:c>
+      <x:c r="H39" s="16" t="str">
+        <x:v>3张</x:v>
+      </x:c>
+      <x:c r="I39" s="16" t="str">
+        <x:v>依次山隘、平原城邑、水网；最终题材 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="76" customHeight="1">
+      <x:c r="A40" s="19" t="str">
+        <x:v>A-107</x:v>
+      </x:c>
+      <x:c r="B40" s="19" t="str">
+        <x:v>选关详情卡底板</x:v>
+      </x:c>
+      <x:c r="C40" s="19" t="str">
+        <x:v>level-panel</x:v>
+      </x:c>
+      <x:c r="D40" s="19" t="str">
+        <x:v>600×420 / 1200×600</x:v>
+      </x:c>
+      <x:c r="E40" s="19" t="str">
+        <x:v>PNG，透明，九宫格</x:v>
+      </x:c>
+      <x:c r="F40" s="19" t="str">
+        <x:v>默认</x:v>
+      </x:c>
+      <x:c r="G40" s="19" t="str">
+        <x:v>关卡说明与进入按钮</x:v>
+      </x:c>
+      <x:c r="H40" s="19" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I40" s="19" t="str">
+        <x:v>标题、难度、奖励用文字；玩法参数 TBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="76" customHeight="1">
+      <x:c r="A41" s="16" t="str">
+        <x:v>A-108</x:v>
+      </x:c>
+      <x:c r="B41" s="16" t="str">
+        <x:v>未解锁与通关印章</x:v>
+      </x:c>
+      <x:c r="C41" s="16" t="str">
+        <x:v>level-status</x:v>
+      </x:c>
+      <x:c r="D41" s="16" t="str">
+        <x:v>160×160</x:v>
+      </x:c>
+      <x:c r="E41" s="16" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F41" s="16" t="str">
+        <x:v>锁定/通关</x:v>
+      </x:c>
+      <x:c r="G41" s="16" t="str">
+        <x:v>地图节点及介绍卡</x:v>
+      </x:c>
+      <x:c r="H41" s="16" t="str">
+        <x:v>2款</x:v>
+      </x:c>
+      <x:c r="I41" s="16" t="str">
+        <x:v>不能仅依靠颜色区分状态</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="76" customHeight="1">
+      <x:c r="A42" s="19" t="str">
+        <x:v>A-109</x:v>
+      </x:c>
+      <x:c r="B42" s="19" t="str">
+        <x:v>通用面板底板与边框</x:v>
+      </x:c>
+      <x:c r="C42" s="19" t="str">
+        <x:v>ui-panel</x:v>
+      </x:c>
+      <x:c r="D42" s="19" t="str">
+        <x:v>256×256</x:v>
+      </x:c>
+      <x:c r="E42" s="19" t="str">
+        <x:v>PNG，透明，九宫格</x:v>
+      </x:c>
+      <x:c r="F42" s="19" t="str">
+        <x:v>常态/强调</x:v>
+      </x:c>
+      <x:c r="G42" s="19" t="str">
+        <x:v>战斗卡片与弹窗</x:v>
+      </x:c>
+      <x:c r="H42" s="19" t="str">
+        <x:v>普通/强调2套</x:v>
+      </x:c>
+      <x:c r="I42" s="19" t="str">
+        <x:v>保留四角，中心可拉伸；复用A-072至A-085容器</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="76" customHeight="1">
+      <x:c r="A43" s="16" t="str">
+        <x:v>A-110</x:v>
+      </x:c>
+      <x:c r="B43" s="16" t="str">
+        <x:v>通用按钮皮肤</x:v>
+      </x:c>
+      <x:c r="C43" s="16" t="str">
+        <x:v>ui-button</x:v>
+      </x:c>
+      <x:c r="D43" s="16" t="str">
+        <x:v>256×80</x:v>
+      </x:c>
+      <x:c r="E43" s="16" t="str">
+        <x:v>PNG，透明，九宫格</x:v>
+      </x:c>
+      <x:c r="F43" s="16" t="str">
+        <x:v>默认/悬停/按下/禁用</x:v>
+      </x:c>
+      <x:c r="G43" s="16" t="str">
+        <x:v>战斗与弹窗按钮</x:v>
+      </x:c>
+      <x:c r="H43" s="16" t="str">
+        <x:v>主/次/危险3类×4态</x:v>
+      </x:c>
+      <x:c r="I43" s="16" t="str">
+        <x:v>结束回合、撤销、暂停、取消、确认共用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="76" customHeight="1">
+      <x:c r="A44" s="19" t="str">
+        <x:v>A-111</x:v>
+      </x:c>
+      <x:c r="B44" s="19" t="str">
+        <x:v>通用功能图标</x:v>
+      </x:c>
+      <x:c r="C44" s="19" t="str">
+        <x:v>ui-icons</x:v>
+      </x:c>
+      <x:c r="D44" s="19" t="str">
+        <x:v>96×96</x:v>
+      </x:c>
+      <x:c r="E44" s="19" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F44" s="19" t="str">
+        <x:v>默认/禁用/选中按需</x:v>
+      </x:c>
+      <x:c r="G44" s="19" t="str">
+        <x:v>返回/关闭/设置/暂停/继续/重试/收起/展开</x:v>
+      </x:c>
+      <x:c r="H44" s="19" t="str">
+        <x:v>8款</x:v>
+      </x:c>
+      <x:c r="I44" s="19" t="str">
+        <x:v>点击区域由程序保持至少44逻辑像素</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="76" customHeight="1">
+      <x:c r="A45" s="16" t="str">
+        <x:v>A-112</x:v>
+      </x:c>
+      <x:c r="B45" s="16" t="str">
+        <x:v>资源属性图标</x:v>
+      </x:c>
+      <x:c r="C45" s="16" t="str">
+        <x:v>ui-stats</x:v>
+      </x:c>
+      <x:c r="D45" s="16" t="str">
+        <x:v>96×96</x:v>
+      </x:c>
+      <x:c r="E45" s="16" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F45" s="16" t="str">
+        <x:v>常态</x:v>
+      </x:c>
+      <x:c r="G45" s="16" t="str">
+        <x:v>HP/AP/SP/金币/回合/击杀/等级</x:v>
+      </x:c>
+      <x:c r="H45" s="16" t="str">
+        <x:v>7款</x:v>
+      </x:c>
+      <x:c r="I45" s="16" t="str">
+        <x:v>保留数值文字，避免仅靠图标猜测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="76" customHeight="1">
+      <x:c r="A46" s="19" t="str">
+        <x:v>A-113</x:v>
+      </x:c>
+      <x:c r="B46" s="19" t="str">
+        <x:v>提示浮层底板</x:v>
+      </x:c>
+      <x:c r="C46" s="19" t="str">
+        <x:v>ui-tooltip</x:v>
+      </x:c>
+      <x:c r="D46" s="19" t="str">
+        <x:v>320×240</x:v>
+      </x:c>
+      <x:c r="E46" s="19" t="str">
+        <x:v>PNG，透明，九宫格</x:v>
+      </x:c>
+      <x:c r="F46" s="19" t="str">
+        <x:v>普通/警告</x:v>
+      </x:c>
+      <x:c r="G46" s="19" t="str">
+        <x:v>未行动名单、说明、悬停信息</x:v>
+      </x:c>
+      <x:c r="H46" s="19" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I46" s="19" t="str">
+        <x:v>长名单自动伸展；复用通用文本</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="76" customHeight="1">
+      <x:c r="A47" s="16" t="str">
+        <x:v>A-114</x:v>
+      </x:c>
+      <x:c r="B47" s="16" t="str">
+        <x:v>弹窗遮罩</x:v>
+      </x:c>
+      <x:c r="C47" s="16" t="str">
+        <x:v>ui-scrim</x:v>
+      </x:c>
+      <x:c r="D47" s="16" t="str">
+        <x:v>全屏自适应</x:v>
+      </x:c>
+      <x:c r="E47" s="16" t="str">
+        <x:v>程序半透明纯色，无需切图</x:v>
+      </x:c>
+      <x:c r="F47" s="16" t="str">
+        <x:v>显示/隐藏</x:v>
+      </x:c>
+      <x:c r="G47" s="16" t="str">
+        <x:v>暂停/确认/成长等模态层</x:v>
+      </x:c>
+      <x:c r="H47" s="16" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I47" s="16" t="str">
+        <x:v>透明度由代码配置；不计单独美术图片</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="76" customHeight="1">
+      <x:c r="A48" s="19" t="str">
+        <x:v>A-115</x:v>
+      </x:c>
+      <x:c r="B48" s="19" t="str">
+        <x:v>滚动条与分页页签</x:v>
+      </x:c>
+      <x:c r="C48" s="19" t="str">
+        <x:v>ui-tabs-scroll</x:v>
+      </x:c>
+      <x:c r="D48" s="19" t="str">
+        <x:v>64×128滚动条；240×64页签</x:v>
+      </x:c>
+      <x:c r="E48" s="19" t="str">
+        <x:v>PNG九宫格或CSS</x:v>
+      </x:c>
+      <x:c r="F48" s="19" t="str">
+        <x:v>默认/悬停/选中/禁用</x:v>
+      </x:c>
+      <x:c r="G48" s="19" t="str">
+        <x:v>技能/敌情/手机面板</x:v>
+      </x:c>
+      <x:c r="H48" s="19" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I48" s="19" t="str">
+        <x:v>文字实时排版；手机保持可触控</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="76" customHeight="1">
+      <x:c r="A49" s="16" t="str">
+        <x:v>A-116</x:v>
+      </x:c>
+      <x:c r="B49" s="16" t="str">
+        <x:v>棋子头顶血条底框与填充</x:v>
+      </x:c>
+      <x:c r="C49" s="16" t="str">
+        <x:v>unit-hp</x:v>
+      </x:c>
+      <x:c r="D49" s="16" t="str">
+        <x:v>240×48</x:v>
+      </x:c>
+      <x:c r="E49" s="16" t="str">
+        <x:v>SVG/PNG，透明，填充分离</x:v>
+      </x:c>
+      <x:c r="F49" s="16" t="str">
+        <x:v>满血/残血/濒危</x:v>
+      </x:c>
+      <x:c r="G49" s="16" t="str">
+        <x:v>每枚存活棋子上方</x:v>
+      </x:c>
+      <x:c r="H49" s="16" t="str">
+        <x:v>敌我2套</x:v>
+      </x:c>
+      <x:c r="I49" s="16" t="str">
+        <x:v>当前数字HP保留；阵营颜色及形状需区分</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="76" customHeight="1">
+      <x:c r="A50" s="19" t="str">
+        <x:v>A-117</x:v>
+      </x:c>
+      <x:c r="B50" s="19" t="str">
+        <x:v>伤害数字与击杀标记</x:v>
+      </x:c>
+      <x:c r="C50" s="19" t="str">
+        <x:v>damage-label</x:v>
+      </x:c>
+      <x:c r="D50" s="19" t="str">
+        <x:v>字高64；标记96×96</x:v>
+      </x:c>
+      <x:c r="E50" s="19" t="str">
+        <x:v>数字代码文字；标记SVG/PNG</x:v>
+      </x:c>
+      <x:c r="F50" s="19" t="str">
+        <x:v>预览/实际伤害区分</x:v>
+      </x:c>
+      <x:c r="G50" s="19" t="str">
+        <x:v>棋盘攻击预览和结算</x:v>
+      </x:c>
+      <x:c r="H50" s="19" t="str">
+        <x:v>普通/友伤/致命3态</x:v>
+      </x:c>
+      <x:c r="I50" s="19" t="str">
+        <x:v>不逐个数字切图；与己方技能效果素材分开</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="76" customHeight="1">
+      <x:c r="A51" s="16" t="str">
+        <x:v>A-118</x:v>
+      </x:c>
+      <x:c r="B51" s="16" t="str">
+        <x:v>攻击与位移方向箭头</x:v>
+      </x:c>
+      <x:c r="C51" s="16" t="str">
+        <x:v>action-arrow</x:v>
+      </x:c>
+      <x:c r="D51" s="16" t="str">
+        <x:v>端点128×128；线条可伸缩</x:v>
+      </x:c>
+      <x:c r="E51" s="16" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F51" s="16" t="str">
+        <x:v>可执行/受阻</x:v>
+      </x:c>
+      <x:c r="G51" s="16" t="str">
+        <x:v>棋盘路径预览</x:v>
+      </x:c>
+      <x:c r="H51" s="16" t="str">
+        <x:v>攻击/推/拉3款</x:v>
+      </x:c>
+      <x:c r="I51" s="16" t="str">
+        <x:v>方向由程序旋转，颜色外保留形状区分</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="76" customHeight="1">
+      <x:c r="A52" s="19" t="str">
+        <x:v>A-119</x:v>
+      </x:c>
+      <x:c r="B52" s="19" t="str">
+        <x:v>敌方出生预告标记</x:v>
+      </x:c>
+      <x:c r="C52" s="19" t="str">
+        <x:v>spawn-marker</x:v>
+      </x:c>
+      <x:c r="D52" s="19" t="str">
+        <x:v>256×256</x:v>
+      </x:c>
+      <x:c r="E52" s="19" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F52" s="19" t="str">
+        <x:v>预告/受阻/等待重试</x:v>
+      </x:c>
+      <x:c r="G52" s="19" t="str">
+        <x:v>援军出生格</x:v>
+      </x:c>
+      <x:c r="H52" s="19" t="str">
+        <x:v>3态</x:v>
+      </x:c>
+      <x:c r="I52" s="19" t="str">
+        <x:v>只表达规则已揭示的信息</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="76" customHeight="1">
+      <x:c r="A53" s="16" t="str">
+        <x:v>A-120</x:v>
+      </x:c>
+      <x:c r="B53" s="16" t="str">
+        <x:v>主帅增益选择卡</x:v>
+      </x:c>
+      <x:c r="C53" s="16" t="str">
+        <x:v>commander-card</x:v>
+      </x:c>
+      <x:c r="D53" s="16" t="str">
+        <x:v>插画384×384；卡底复用通用面板</x:v>
+      </x:c>
+      <x:c r="E53" s="16" t="str">
+        <x:v>PNG/WebP，透明插画</x:v>
+      </x:c>
+      <x:c r="F53" s="16" t="str">
+        <x:v>默认/悬停/选中</x:v>
+      </x:c>
+      <x:c r="G53" s="16" t="str">
+        <x:v>坚守/疾行/救援</x:v>
+      </x:c>
+      <x:c r="H53" s="16" t="str">
+        <x:v>3款</x:v>
+      </x:c>
+      <x:c r="I53" s="16" t="str">
+        <x:v>不烘焙技能描述和数值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="76" customHeight="1">
+      <x:c r="A54" s="19" t="str">
+        <x:v>A-121</x:v>
+      </x:c>
+      <x:c r="B54" s="19" t="str">
+        <x:v>技能图标合集</x:v>
+      </x:c>
+      <x:c r="C54" s="19" t="str">
+        <x:v>skill-icons</x:v>
+      </x:c>
+      <x:c r="D54" s="19" t="str">
+        <x:v>128×128</x:v>
+      </x:c>
+      <x:c r="E54" s="19" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F54" s="19" t="str">
+        <x:v>可购买/已解锁/不可购买</x:v>
+      </x:c>
+      <x:c r="G54" s="19" t="str">
+        <x:v>升级/转职/方向/扩散</x:v>
+      </x:c>
+      <x:c r="H54" s="19" t="str">
+        <x:v>通用1套＋己方9棋种槽位</x:v>
+      </x:c>
+      <x:c r="I54" s="19" t="str">
+        <x:v>与A-042至A-065技能特效分开；敌方不新增主动技能</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="76" customHeight="1">
+      <x:c r="A55" s="16" t="str">
+        <x:v>A-122</x:v>
+      </x:c>
+      <x:c r="B55" s="16" t="str">
+        <x:v>关卡目标卡与阶段标签</x:v>
+      </x:c>
+      <x:c r="C55" s="16" t="str">
+        <x:v>objective-panel</x:v>
+      </x:c>
+      <x:c r="D55" s="16" t="str">
+        <x:v>480×240；标签240×64</x:v>
+      </x:c>
+      <x:c r="E55" s="16" t="str">
+        <x:v>PNG，透明，九宫格</x:v>
+      </x:c>
+      <x:c r="F55" s="16" t="str">
+        <x:v>我方/敌方/布阵/结束</x:v>
+      </x:c>
+      <x:c r="G55" s="16" t="str">
+        <x:v>保护主帅/回合阶段</x:v>
+      </x:c>
+      <x:c r="H55" s="16" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I55" s="16" t="str">
+        <x:v>目标文案来自规则，不能写死为图片</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="76" customHeight="1">
+      <x:c r="A56" s="19" t="str">
+        <x:v>A-123</x:v>
+      </x:c>
+      <x:c r="B56" s="19" t="str">
+        <x:v>结束回合未行动提醒</x:v>
+      </x:c>
+      <x:c r="C56" s="19" t="str">
+        <x:v>end-turn-reminder</x:v>
+      </x:c>
+      <x:c r="D56" s="19" t="str">
+        <x:v>复用ui-tooltip</x:v>
+      </x:c>
+      <x:c r="E56" s="19" t="str">
+        <x:v>无需独立图片，布局组件</x:v>
+      </x:c>
+      <x:c r="F56" s="19" t="str">
+        <x:v>有未行动棋子/全部已行动</x:v>
+      </x:c>
+      <x:c r="G56" s="19" t="str">
+        <x:v>结束回合悬停</x:v>
+      </x:c>
+      <x:c r="H56" s="19" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I56" s="19" t="str">
+        <x:v>列棋名及坐标；预留未行动徽记96×96</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="76" customHeight="1">
+      <x:c r="A57" s="16" t="str">
+        <x:v>A-124</x:v>
+      </x:c>
+      <x:c r="B57" s="16" t="str">
+        <x:v>布阵与上阵后备标记</x:v>
+      </x:c>
+      <x:c r="C57" s="16" t="str">
+        <x:v>deployment-marker</x:v>
+      </x:c>
+      <x:c r="D57" s="16" t="str">
+        <x:v>标记96×96；格框256×256</x:v>
+      </x:c>
+      <x:c r="E57" s="16" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F57" s="16" t="str">
+        <x:v>已上阵/后备/选中/不可放置</x:v>
+      </x:c>
+      <x:c r="G57" s="16" t="str">
+        <x:v>布阵/商店队伍管理</x:v>
+      </x:c>
+      <x:c r="H57" s="16" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I57" s="16" t="str">
+        <x:v>头像复用己方棋子资源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="76" customHeight="1">
+      <x:c r="A58" s="19" t="str">
+        <x:v>A-125</x:v>
+      </x:c>
+      <x:c r="B58" s="19" t="str">
+        <x:v>救援角色卡与恢复标记</x:v>
+      </x:c>
+      <x:c r="C58" s="19" t="str">
+        <x:v>rescue-card</x:v>
+      </x:c>
+      <x:c r="D58" s="19" t="str">
+        <x:v>卡底320×420；标记128×128</x:v>
+      </x:c>
+      <x:c r="E58" s="19" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F58" s="19" t="str">
+        <x:v>回血/复活/不可选</x:v>
+      </x:c>
+      <x:c r="G58" s="19" t="str">
+        <x:v>第6回合救援</x:v>
+      </x:c>
+      <x:c r="H58" s="19" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I58" s="19" t="str">
+        <x:v>人物形象复用棋子；恢复表现关联技能通用效果</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="76" customHeight="1">
+      <x:c r="A59" s="16" t="str">
+        <x:v>A-126</x:v>
+      </x:c>
+      <x:c r="B59" s="16" t="str">
+        <x:v>商店商品与价格标签</x:v>
+      </x:c>
+      <x:c r="C59" s="16" t="str">
+        <x:v>shop-card</x:v>
+      </x:c>
+      <x:c r="D59" s="16" t="str">
+        <x:v>商品像256×256；价签240×72</x:v>
+      </x:c>
+      <x:c r="E59" s="16" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F59" s="16" t="str">
+        <x:v>可购买/金币不足/容量受限</x:v>
+      </x:c>
+      <x:c r="G59" s="16" t="str">
+        <x:v>关间整备</x:v>
+      </x:c>
+      <x:c r="H59" s="16" t="str">
+        <x:v>兵/车/马/炮4类</x:v>
+      </x:c>
+      <x:c r="I59" s="16" t="str">
+        <x:v>棋子像复用，价格由程序写入</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="76" customHeight="1">
+      <x:c r="A60" s="19" t="str">
+        <x:v>A-127</x:v>
+      </x:c>
+      <x:c r="B60" s="19" t="str">
+        <x:v>胜败结果标题与装饰</x:v>
+      </x:c>
+      <x:c r="C60" s="19" t="str">
+        <x:v>result-art</x:v>
+      </x:c>
+      <x:c r="D60" s="19" t="str">
+        <x:v>960×360 / 1100×440</x:v>
+      </x:c>
+      <x:c r="E60" s="19" t="str">
+        <x:v>PNG，透明</x:v>
+      </x:c>
+      <x:c r="F60" s="19" t="str">
+        <x:v>3种结果</x:v>
+      </x:c>
+      <x:c r="G60" s="19" t="str">
+        <x:v>结果界面</x:v>
+      </x:c>
+      <x:c r="H60" s="19" t="str">
+        <x:v>胜利/主帅阵亡/将死3款</x:v>
+      </x:c>
+      <x:c r="I60" s="19" t="str">
+        <x:v>统计数字和操作按钮独立</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="76" customHeight="1">
+      <x:c r="A61" s="16" t="str">
+        <x:v>A-128</x:v>
+      </x:c>
+      <x:c r="B61" s="16" t="str">
+        <x:v>底部信息导航图标</x:v>
+      </x:c>
+      <x:c r="C61" s="16" t="str">
+        <x:v>mobile-nav</x:v>
+      </x:c>
+      <x:c r="D61" s="16" t="str">
+        <x:v>96×96</x:v>
+      </x:c>
+      <x:c r="E61" s="16" t="str">
+        <x:v>SVG/PNG，透明</x:v>
+      </x:c>
+      <x:c r="F61" s="16" t="str">
+        <x:v>默认/选中/提示</x:v>
+      </x:c>
+      <x:c r="G61" s="16" t="str">
+        <x:v>队伍/技能/敌情/更多</x:v>
+      </x:c>
+      <x:c r="H61" s="16" t="str">
+        <x:v>4款</x:v>
+      </x:c>
+      <x:c r="I61" s="16" t="str">
+        <x:v>448×924逻辑视口，3倍参考导出；保持一屏</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="76" customHeight="1">
+      <x:c r="A62" s="19" t="str">
+        <x:v>A-129</x:v>
+      </x:c>
+      <x:c r="B62" s="19" t="str">
+        <x:v>信息展开面板与抓手</x:v>
+      </x:c>
+      <x:c r="C62" s="19" t="str">
+        <x:v>mobile-sheet</x:v>
+      </x:c>
+      <x:c r="D62" s="19" t="str">
+        <x:v>宽1344，高度自适应；抓手144×12</x:v>
+      </x:c>
+      <x:c r="E62" s="19" t="str">
+        <x:v>PNG九宫格或CSS</x:v>
+      </x:c>
+      <x:c r="F62" s="19" t="str">
+        <x:v>展开/收起</x:v>
+      </x:c>
+      <x:c r="G62" s="19" t="str">
+        <x:v>完整详情、敌情、战况记录</x:v>
+      </x:c>
+      <x:c r="H62" s="19" t="str">
+        <x:v>1套</x:v>
+      </x:c>
+      <x:c r="I62" s="19" t="str">
+        <x:v>内容可内部滚动，主战斗页不滚动</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="76" customHeight="1">
+      <x:c r="A63" s="16" t="str">
+        <x:v>A-130</x:v>
+      </x:c>
+      <x:c r="B63" s="16" t="str">
+        <x:v>紧凑棋子与预览卡</x:v>
+      </x:c>
+      <x:c r="C63" s="16" t="str">
+        <x:v>mobile-summary</x:v>
+      </x:c>
+      <x:c r="D63" s="16" t="str">
+        <x:v>1296×312参考</x:v>
+      </x:c>
+      <x:c r="E63" s="16" t="str">
+        <x:v>PNG九宫格或CSS</x:v>
+      </x:c>
+      <x:c r="F63" s="16" t="str">
+        <x:v>常态/警告/无选择</x:v>
+      </x:c>
+      <x:c r="G63" s="16" t="str">
+        <x:v>棋盘下方摘要</x:v>
+      </x:c>
+      <x:c r="H63" s="16" t="str">
+        <x:v>2套</x:v>
+      </x:c>
+      <x:c r="I63" s="16" t="str">
+        <x:v>与桌面信息同源，文本不烘焙</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="76" customHeight="1">
+      <x:c r="A64" s="19" t="str">
+        <x:v>A-131</x:v>
+      </x:c>
+      <x:c r="B64" s="19" t="str">
+        <x:v>字体与排版规范</x:v>
+      </x:c>
+      <x:c r="C64" s="19" t="str">
+        <x:v>ui-type</x:v>
+      </x:c>
+      <x:c r="D64" s="19" t="str">
+        <x:v>标题32-64；正文14-18逻辑px</x:v>
+      </x:c>
+      <x:c r="E64" s="19" t="str">
+        <x:v>可商用字体授权或系统字体</x:v>
+      </x:c>
+      <x:c r="F64" s="19" t="str">
+        <x:v>常态/强调/警告</x:v>
+      </x:c>
+      <x:c r="G64" s="19" t="str">
+        <x:v>全部页面</x:v>
+      </x:c>
+      <x:c r="H64" s="19" t="str">
+        <x:v>标题/正文/数字3用途</x:v>
+      </x:c>
+      <x:c r="I64" s="19" t="str">
+        <x:v>字体授权 TBD；资源尺寸为制作建议，最终风格待确认</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:I3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5846739d9be04a9e"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="33" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="33" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="37" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="65" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>三关地图美术分区</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="13" t="str">
+        <x:v>三关是新的美术预留，不等同于战斗内的两波敌军。示意图只表达西→中→东南的关卡构图，不是战国七国疆界复原。三关敌阵、解锁方式、具体疆界与年代均 TBD。</x:v>
+      </x:c>
+      <x:c r="B2" s="13"/>
+      <x:c r="C2" s="13"/>
+      <x:c r="D2" s="13"/>
+      <x:c r="E2" s="13"/>
+      <x:c r="F2" s="13"/>
+      <x:c r="G2" s="13"/>
+      <x:c r="H2" s="13"/>
+      <x:c r="I2" s="13"/>
+    </x:row>
+    <x:row r="3" ht="25" customHeight="1">
+      <x:c r="A3" s="13"/>
+      <x:c r="B3" s="13"/>
+      <x:c r="C3" s="13"/>
+      <x:c r="D3" s="13"/>
+      <x:c r="E3" s="13"/>
+      <x:c r="F3" s="13"/>
+      <x:c r="G3" s="13"/>
+      <x:c r="H3" s="13"/>
+      <x:c r="I3" s="13"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="18" t="str">
+        <x:v>关卡</x:v>
+      </x:c>
+      <x:c r="B5" s="18" t="str">
+        <x:v>暂定区域名</x:v>
+      </x:c>
+      <x:c r="C5" s="18" t="str">
+        <x:v>区域槽位</x:v>
+      </x:c>
+      <x:c r="D5" s="18" t="str">
+        <x:v>构图位置</x:v>
+      </x:c>
+      <x:c r="E5" s="18" t="str">
+        <x:v>视觉主题</x:v>
+      </x:c>
+      <x:c r="F5" s="18" t="str">
+        <x:v>重点资源</x:v>
+      </x:c>
+      <x:c r="G5" s="18" t="str">
+        <x:v>状态预留</x:v>
+      </x:c>
+      <x:c r="H5" s="18" t="str">
+        <x:v>玩法接入</x:v>
+      </x:c>
+      <x:c r="I5" s="18" t="str">
+        <x:v>参考与说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="76" customHeight="1">
+      <x:c r="A6" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="str">
+        <x:v>关中</x:v>
+      </x:c>
+      <x:c r="C6" s="19" t="str">
+        <x:v>region-01</x:v>
+      </x:c>
+      <x:c r="D6" s="19" t="str">
+        <x:v>西部</x:v>
+      </x:c>
+      <x:c r="E6" s="19" t="str">
+        <x:v>山隘、城塞、土黄色</x:v>
+      </x:c>
+      <x:c r="F6" s="19" t="str">
+        <x:v>区域高亮、节点、山隘插画</x:v>
+      </x:c>
+      <x:c r="G6" s="19" t="str">
+        <x:v>未解锁/可挑战/选中/通关</x:v>
+      </x:c>
+      <x:c r="H6" s="19" t="str">
+        <x:v>TBD，美术样稿未接入战斗</x:v>
+      </x:c>
+      <x:c r="I6" s="19" t="str">
+        <x:v>地理题材参考；关卡边界为设计草案。https://commons.wikimedia.org/wiki/File:ZH-战国七雄地图.jpg</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="76" customHeight="1">
+      <x:c r="A7" s="21" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="str">
+        <x:v>中原</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="str">
+        <x:v>region-02</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>中央</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="str">
+        <x:v>平原、河流、城邑、青绿</x:v>
+      </x:c>
+      <x:c r="F7" s="16" t="str">
+        <x:v>区域高亮、节点、城邑插画</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="str">
+        <x:v>未解锁/可挑战/选中/通关</x:v>
+      </x:c>
+      <x:c r="H7" s="16" t="str">
+        <x:v>TBD，美术样稿未接入战斗</x:v>
+      </x:c>
+      <x:c r="I7" s="16" t="str">
+        <x:v>国别归属、地图年代不作精确标注。https://commons.wikimedia.org/wiki/File:ZH-战国七雄地图.jpg</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="76" customHeight="1">
+      <x:c r="A8" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
+        <x:v>江淮</x:v>
+      </x:c>
+      <x:c r="C8" s="19" t="str">
+        <x:v>region-03</x:v>
+      </x:c>
+      <x:c r="D8" s="19" t="str">
+        <x:v>东南</x:v>
+      </x:c>
+      <x:c r="E8" s="19" t="str">
+        <x:v>水网、林地、蓝绿</x:v>
+      </x:c>
+      <x:c r="F8" s="19" t="str">
+        <x:v>区域高亮、节点、水泽插画</x:v>
+      </x:c>
+      <x:c r="G8" s="19" t="str">
+        <x:v>未解锁/可挑战/选中/通关</x:v>
+      </x:c>
+      <x:c r="H8" s="19" t="str">
+        <x:v>TBD，美术样稿未接入战斗</x:v>
+      </x:c>
+      <x:c r="I8" s="19" t="str">
+        <x:v>战国题材局部地图，非现代全国行政图。https://commons.wikimedia.org/wiki/File:ZH-战国七雄地图.jpg</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:I3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a7e71c6ab774eb1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore(assets): refresh art asset list and inspect dump
</commit_message>
<xml_diff>
--- a/outputs/01a0bf14-7f85-7282-bb8d-672064556a58/美术资产清单.xlsx
+++ b/outputs/01a0bf14-7f85-7282-bb8d-672064556a58/美术资产清单.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="美术资产清单" sheetId="1" r:id="Rf0261a8c855d4fcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="源文件盘点" sheetId="2" r:id="Re40b2ce53eb44b92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="界面规格" sheetId="3" r:id="Rb9ecb261437b495c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图分区" sheetId="4" r:id="R867d38e4eaad4961"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="美术资产清单" sheetId="1" r:id="Rb64142bda47a4737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="源文件盘点" sheetId="2" r:id="R59cc77f368894bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="界面规格" sheetId="3" r:id="R508fa4bc3ad94343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图分区" sheetId="4" r:id="Rb92de17ffe5742f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Microsoft YaHei"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -91,6 +91,11 @@
         <x:fgColor rgb="FFEDF4F8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -98,7 +103,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="22">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -149,6 +154,9 @@
     <x:xf numFmtId="200" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -157,7 +165,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VisualAssets" displayName="VisualAssets" ref="A5:I136" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VisualAssets" displayName="VisualAssets" ref="A5:I167" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="分类"/>
@@ -190,7 +198,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="UiSpecs" displayName="UiSpecs" ref="A5:I64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="UiSpecs" displayName="UiSpecs" ref="A5:I95" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="资源/组件"/>
@@ -442,9 +450,9 @@
       <x:c r="H1" s="1"/>
       <x:c r="I1" s="1"/>
     </x:row>
-    <x:row r="2" ht="25" customHeight="1">
+    <x:row r="2" ht="35" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>范围：主原型、独立地形实验、Loading/主菜单/三关地图美术占位；三关规则与流程接入 TBD。</x:v>
+        <x:v>核对日期：2026-10-22。范围：主原型、三关地图、第0关教学、主营地、公共SP、仕防御塔、主帅辅助与马跳跃技能；WIP另标。</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -455,9 +463,9 @@
       <x:c r="H2" s="1"/>
       <x:c r="I2" s="1"/>
     </x:row>
-    <x:row r="3" ht="25" customHeight="1">
+    <x:row r="3" ht="35" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>共 131 项视觉元素/组件记录；本次新增 45 项。传统棋子14款、扩展棋子2款、己方技能效果24项、地形19项保留。UI交付规格详见“界面规格”。</x:v>
+        <x:v>共162项组件/视觉记录；本次新增31项（A-132～A-162），修订42项。总项与子资源存在复用，不等于图片张数；详细交付见“界面规格”。</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -595,7 +603,7 @@
         <x:v>线宽与正式样式 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="32" customHeight="1">
+    <x:row r="9" ht="100" customHeight="1">
       <x:c r="A9" s="8" t="str">
         <x:v>A-004</x:v>
       </x:c>
@@ -603,25 +611,25 @@
         <x:v>棋盘场景</x:v>
       </x:c>
       <x:c r="C9" s="8" t="str">
-        <x:v>中央河道与文字</x:v>
+        <x:v>河道与桥位整体构图</x:v>
       </x:c>
       <x:c r="D9" s="8" t="str">
-        <x:v>1套</x:v>
+        <x:v>随关卡配置</x:v>
       </x:c>
       <x:c r="E9" s="8" t="str">
-        <x:v>第 5 行／y=4</x:v>
+        <x:v>主战斗及关卡预览</x:v>
       </x:c>
       <x:c r="F9" s="8" t="str">
-        <x:v>Canvas 色带与文字</x:v>
+        <x:v>代码格子/文字占位</x:v>
       </x:c>
       <x:c r="G9" s="8" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>待制作</x:v>
       </x:c>
       <x:c r="H9" s="8" t="str">
-        <x:v>web/js/app.js:24-25；web/js/rules.js:4</x:v>
+        <x:v>docs/us/US-020-main-camp.md R08；US007/009/011</x:v>
       </x:c>
       <x:c r="I9" s="8" t="str">
-        <x:v>主原型为可通行河道；独立地形实验将其中 6 格设为水、3 格设为桥</x:v>
+        <x:v>地形已接入主原型；位置读取有效关卡配置，不把旧固定河道作为全部关卡规格。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32" customHeight="1">
@@ -711,7 +719,7 @@
         <x:v>需兼容对局菱形与编辑器方格视图；正式纹理 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="38" customHeight="1">
+    <x:row r="13" ht="100" customHeight="1">
       <x:c r="A13" s="8" t="str">
         <x:v>A-008</x:v>
       </x:c>
@@ -725,7 +733,7 @@
         <x:v>1套／默认6格</x:v>
       </x:c>
       <x:c r="E13" s="8" t="str">
-        <x:v>河道非桥棋位</x:v>
+        <x:v>关卡配置中的水域格</x:v>
       </x:c>
       <x:c r="F13" s="8" t="str">
         <x:v>蓝绿色地块＋“≈”符号</x:v>
@@ -734,13 +742,13 @@
         <x:v>代码占位（独立实验）</x:v>
       </x:c>
       <x:c r="H13" s="8" t="str">
-        <x:v>web/experiments/terrain-wave/rules.js:224-227；style.css:1</x:v>
+        <x:v>US007/009/011；US020 R08</x:v>
       </x:c>
       <x:c r="I13" s="8" t="str">
-        <x:v>默认第 5 行第 1、3、4、6、7、9 列；正式水面动画 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="38" customHeight="1">
+        <x:v>水位以有效地图为准；地图预览与实战共用配置。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="100" customHeight="1">
       <x:c r="A14" s="8" t="str">
         <x:v>A-009</x:v>
       </x:c>
@@ -754,7 +762,7 @@
         <x:v>1套／默认3格</x:v>
       </x:c>
       <x:c r="E14" s="8" t="str">
-        <x:v>河道可通行桥位</x:v>
+        <x:v>关卡配置中的桥位</x:v>
       </x:c>
       <x:c r="F14" s="8" t="str">
         <x:v>棕色木纹条带</x:v>
@@ -763,10 +771,10 @@
         <x:v>代码占位（独立实验）</x:v>
       </x:c>
       <x:c r="H14" s="8" t="str">
-        <x:v>web/experiments/terrain-wave/rules.js:224-227；style.css:1</x:v>
+        <x:v>US007/009/011；US020 R08</x:v>
       </x:c>
       <x:c r="I14" s="8" t="str">
-        <x:v>默认第 5 行第 2、5、8 列；桥体结构与栏杆 TBD</x:v>
+        <x:v>桥按陆地通行；桥位以有效地图为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="38" customHeight="1">
@@ -856,7 +864,7 @@
         <x:v>坍塌后恢复为可通行陆地；碎石密度与消散方式 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="38" customHeight="1">
+    <x:row r="18" ht="100" customHeight="1">
       <x:c r="A18" s="8" t="str">
         <x:v>A-013</x:v>
       </x:c>
@@ -879,10 +887,10 @@
         <x:v>代码占位（独立实验）</x:v>
       </x:c>
       <x:c r="H18" s="8" t="str">
-        <x:v>web/experiments/terrain-wave/rules.js:174,227；style.css:1</x:v>
+        <x:v>US007；US018；US021</x:v>
       </x:c>
       <x:c r="I18" s="8" t="str">
-        <x:v>界面只表达“有一定概率闪避”，不显示 30% 或预告本次结果</x:v>
+        <x:v>树林30%闪避为现行规则；预览表达条件结果，不预抽本次随机结果。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="38" customHeight="1">
@@ -914,7 +922,7 @@
         <x:v>区分快速经过、停留和阵亡三种节奏 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="38" customHeight="1">
+    <x:row r="20" ht="100" customHeight="1">
       <x:c r="A20" s="8" t="str">
         <x:v>A-015</x:v>
       </x:c>
@@ -928,7 +936,7 @@
         <x:v>1套</x:v>
       </x:c>
       <x:c r="E20" s="8" t="str">
-        <x:v>兵／弓／枪／炮进入水域立即阵亡</x:v>
+        <x:v>兵/弓/枪/炮入水及主帅被强制入水阵亡</x:v>
       </x:c>
       <x:c r="F20" s="8" t="str">
         <x:v>棋子直接移除＋战报文字</x:v>
@@ -937,10 +945,10 @@
         <x:v>待制作</x:v>
       </x:c>
       <x:c r="H20" s="8" t="str">
-        <x:v>web/experiments/terrain-wave/rules.js:49,54</x:v>
+        <x:v>docs/us/US-019-commander-support-movement.md</x:v>
       </x:c>
       <x:c r="I20" s="8" t="str">
-        <x:v>需包含棋子沉没、消散与击杀归属反馈；表现规格 TBD</x:v>
+        <x:v>主帅不能主动入水，强制入水立即失败；复用沉没主体并保留主帅失败反馈。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="38" customHeight="1">
@@ -1233,7 +1241,7 @@
         <x:v>坍塌碎石为战斗状态，不作为当前画笔；正式图标 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="32" customHeight="1">
+    <x:row r="31" ht="100" customHeight="1">
       <x:c r="A31" s="8" t="str">
         <x:v>A-026</x:v>
       </x:c>
@@ -1247,7 +1255,7 @@
         <x:v>1款／标准1枚</x:v>
       </x:c>
       <x:c r="E31" s="8" t="str">
-        <x:v>己方主帅</x:v>
+        <x:v>正式旅程主帅，纯辅助与移动</x:v>
       </x:c>
       <x:c r="F31" s="8" t="str">
         <x:v>红色圆柱＋“帅”字</x:v>
@@ -1256,13 +1264,13 @@
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H31" s="8" t="str">
-        <x:v>web/js/app.js:4-6,29-30</x:v>
+        <x:v>docs/us/US-019-commander-support-movement.md</x:v>
       </x:c>
       <x:c r="I31" s="8" t="str">
-        <x:v>中国象棋红方棋种；正式形象 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="32" customHeight="1">
+        <x:v>无攻击、无个人升级；宫内米字线、宫外横竖一步；形象与敌方将区分。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="100" customHeight="1">
       <x:c r="A32" s="8" t="str">
         <x:v>A-027</x:v>
       </x:c>
@@ -1270,25 +1278,25 @@
         <x:v>棋子</x:v>
       </x:c>
       <x:c r="C32" s="8" t="str">
-        <x:v>己方仕</x:v>
+        <x:v>己方仕（固定防御塔）</x:v>
       </x:c>
       <x:c r="D32" s="8" t="str">
-        <x:v>1款／标准2枚</x:v>
+        <x:v>1套，可同时部署2座</x:v>
       </x:c>
       <x:c r="E32" s="8" t="str">
-        <x:v>完整中国象棋红方名录</x:v>
+        <x:v>主营地招募、九宫左右侧位</x:v>
       </x:c>
       <x:c r="F32" s="8" t="str">
-        <x:v>无（当前未配置）</x:v>
+        <x:v>汉字棋子/装置占位</x:v>
       </x:c>
       <x:c r="G32" s="8" t="str">
-        <x:v>未实现</x:v>
+        <x:v>规则已实现／美术待制作</x:v>
       </x:c>
       <x:c r="H32" s="8" t="str">
-        <x:v>中国象棋棋种；用户补充</x:v>
+        <x:v>docs/us/US-018-advisor-defense-tower.md；US020</x:v>
       </x:c>
       <x:c r="I32" s="8" t="str">
-        <x:v>当前网页无己方仕；规则与造型 TBD</x:v>
+        <x:v>固定(4,2)/(6,2)，2HP，不主动移动；普通敌方士不改成塔。残骸另见A-148。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="32" customHeight="1">
@@ -1320,7 +1328,7 @@
         <x:v>当前网页无相；规则与造型 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="32" customHeight="1">
+    <x:row r="34" ht="100" customHeight="1">
       <x:c r="A34" s="8" t="str">
         <x:v>A-029</x:v>
       </x:c>
@@ -1334,7 +1342,7 @@
         <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E34" s="8" t="str">
-        <x:v>首波商店购买</x:v>
+        <x:v>初始队伍1枚；主营地可招募</x:v>
       </x:c>
       <x:c r="F34" s="8" t="str">
         <x:v>红色圆柱＋“马”字</x:v>
@@ -1343,10 +1351,10 @@
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H34" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>US020 初始阵容；US021</x:v>
       </x:c>
       <x:c r="I34" s="8" t="str">
-        <x:v>原型最多购买一枚；标准整副为两枚</x:v>
+        <x:v>初始普通队友为兵2马1车1；马有日字移动及主动跳跃攻击，不再沿用旧普通攻击。</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="32" customHeight="1">
@@ -1378,7 +1386,7 @@
         <x:v>原型初始一枚；标准整副为两枚</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="32" customHeight="1">
+    <x:row r="36" ht="100" customHeight="1">
       <x:c r="A36" s="8" t="str">
         <x:v>A-031</x:v>
       </x:c>
@@ -1392,7 +1400,7 @@
         <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E36" s="8" t="str">
-        <x:v>首波商店购买</x:v>
+        <x:v>主营地8猫粮招募，无初始炮</x:v>
       </x:c>
       <x:c r="F36" s="8" t="str">
         <x:v>红色圆柱＋“炮”字</x:v>
@@ -1401,13 +1409,13 @@
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H36" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>US013；US020</x:v>
       </x:c>
       <x:c r="I36" s="8" t="str">
-        <x:v>原型最多购买一枚；标准整副为两枚</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="32" customHeight="1">
+        <x:v>不写死最多购买一枚；普通队友库存不限，部署人口另计。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="100" customHeight="1">
       <x:c r="A37" s="8" t="str">
         <x:v>A-032</x:v>
       </x:c>
@@ -1421,7 +1429,7 @@
         <x:v>1款／标准5枚</x:v>
       </x:c>
       <x:c r="E37" s="8" t="str">
-        <x:v>P1 等测试夹具</x:v>
+        <x:v>初始队伍2枚；主营地招募；转职</x:v>
       </x:c>
       <x:c r="F37" s="8" t="str">
         <x:v>红色圆柱＋“兵”字</x:v>
@@ -1430,10 +1438,10 @@
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H37" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30</x:v>
+        <x:v>US020 初始阵容及R04</x:v>
       </x:c>
       <x:c r="I37" s="8" t="str">
-        <x:v>正式局未提供招募；标准整副为五枚</x:v>
+        <x:v>两枚兵共用美术但身份独立；可各自转职弓兵/枪兵，不需两套皮肤。</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="32" customHeight="1">
@@ -1523,7 +1531,7 @@
         <x:v>当前网页无象；规则与造型 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="32" customHeight="1">
+    <x:row r="41" ht="100" customHeight="1">
       <x:c r="A41" s="8" t="str">
         <x:v>A-036</x:v>
       </x:c>
@@ -1537,7 +1545,7 @@
         <x:v>1款／标准2枚</x:v>
       </x:c>
       <x:c r="E41" s="8" t="str">
-        <x:v>完整中国象棋黑方名录</x:v>
+        <x:v>敌方马棋种预留，按实际关卡/编辑器配置</x:v>
       </x:c>
       <x:c r="F41" s="8" t="str">
         <x:v>通用棋子绘制可显示“马”字；未编队</x:v>
@@ -1546,10 +1554,10 @@
         <x:v>未编队</x:v>
       </x:c>
       <x:c r="H41" s="8" t="str">
-        <x:v>web/js/app.js:4-5,29-30; web/js/rules.js:8-9</x:v>
+        <x:v>US011；US021</x:v>
       </x:c>
       <x:c r="I41" s="8" t="str">
-        <x:v>当前两波敌阵均无马</x:v>
+        <x:v>敌方马规则不随我方跳跃技能变更；不新增敌方主动技能特效。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="32" customHeight="1">
@@ -1697,7 +1705,7 @@
         <x:v>项目特有转职，不计入传统七类</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="32" customHeight="1">
+    <x:row r="47" ht="100" customHeight="1">
       <x:c r="A47" s="11" t="str">
         <x:v>A-042</x:v>
       </x:c>
@@ -1711,7 +1719,7 @@
         <x:v>9棋种通用</x:v>
       </x:c>
       <x:c r="E47" s="11" t="str">
-        <x:v>己方棋子击杀后 Lv、SP 与击杀数增加</x:v>
+        <x:v>有效击杀的个人等级/击杀及全队公共SP增长</x:v>
       </x:c>
       <x:c r="F47" s="11" t="str">
         <x:v>仅数值文字刷新；无独立特效资产</x:v>
@@ -1720,13 +1728,13 @@
         <x:v>待制作</x:v>
       </x:c>
       <x:c r="H47" s="11" t="str">
-        <x:v>web/js/rules.js:38; web/js/app.js:37-40</x:v>
+        <x:v>US017；US021</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
-        <x:v>建议包含棋子归属、等级提升和 SP 获得反馈</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="32" customHeight="1">
+        <x:v>等级/击杀归个人，SP入全队唯一钱包；共享SP反馈见A-161，不为每枚棋子做个人钱包。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="100" customHeight="1">
       <x:c r="A48" s="11" t="str">
         <x:v>A-043</x:v>
       </x:c>
@@ -1737,10 +1745,10 @@
         <x:v>全体｜强健升级</x:v>
       </x:c>
       <x:c r="D48" s="11" t="str">
-        <x:v>9棋种通用</x:v>
+        <x:v>现有6类普通队友共用；相TBD</x:v>
       </x:c>
       <x:c r="E48" s="11" t="str">
-        <x:v>己方存活棋子当前／最大 HP +1</x:v>
+        <x:v>具备资格的普通队友强健升级</x:v>
       </x:c>
       <x:c r="F48" s="11" t="str">
         <x:v>仅按钮和 HP 数值刷新</x:v>
@@ -1749,13 +1757,13 @@
         <x:v>待制作</x:v>
       </x:c>
       <x:c r="H48" s="11" t="str">
-        <x:v>web/js/app.js:42; web/js/rules.js:53</x:v>
+        <x:v>US018；US019；US021</x:v>
       </x:c>
       <x:c r="I48" s="11" t="str">
-        <x:v>帅、仕、相、马、车、炮、兵、弓兵、枪兵共用；仕／相规则仍 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="32" customHeight="1">
+        <x:v>主帅、仕不得使用强健；相尚未实现，其资格TBD。马保留已有强健，与三项新升级并存。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="100" customHeight="1">
       <x:c r="A49" s="11" t="str">
         <x:v>A-044</x:v>
       </x:c>
@@ -1763,28 +1771,28 @@
         <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C49" s="11" t="str">
-        <x:v>帅｜专属技能效果预留</x:v>
+        <x:v>帅｜团队旅程增益表现</x:v>
       </x:c>
       <x:c r="D49" s="11" t="str">
-        <x:v>1槽</x:v>
+        <x:v>坚守/疾行/救援3款</x:v>
       </x:c>
       <x:c r="E49" s="11" t="str">
-        <x:v>己方帅未来专属技能</x:v>
+        <x:v>主营地解锁及战斗增益状态</x:v>
       </x:c>
       <x:c r="F49" s="11" t="str">
-        <x:v>无</x:v>
+        <x:v>文字/按钮占位</x:v>
       </x:c>
       <x:c r="G49" s="11" t="str">
-        <x:v>预留（规则TBD）</x:v>
+        <x:v>规则已确认／美术待制作</x:v>
       </x:c>
       <x:c r="H49" s="11" t="str">
-        <x:v>用户要求预留所有己方棋子技能效果</x:v>
+        <x:v>US019；US020 R05</x:v>
       </x:c>
       <x:c r="I49" s="11" t="str">
-        <x:v>当前只有通用强健；技能名称、触发和表现 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="32" customHeight="1">
+        <x:v>替代旧专属攻击/个人强健占位；不是范围光环。普通队友受益，主帅和仕排除。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="100" customHeight="1">
       <x:c r="A50" s="11" t="str">
         <x:v>A-045</x:v>
       </x:c>
@@ -1792,25 +1800,25 @@
         <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C50" s="11" t="str">
-        <x:v>仕｜专属技能效果预留</x:v>
+        <x:v>仕｜自动开火效果总项</x:v>
       </x:c>
       <x:c r="D50" s="11" t="str">
-        <x:v>1槽</x:v>
+        <x:v>弹道/命中/冷却/预览</x:v>
       </x:c>
       <x:c r="E50" s="11" t="str">
-        <x:v>己方仕未来专属技能</x:v>
+        <x:v>我方结束回合后、敌攻前自动开火</x:v>
       </x:c>
       <x:c r="F50" s="11" t="str">
-        <x:v>无</x:v>
+        <x:v>规则和连线占位</x:v>
       </x:c>
       <x:c r="G50" s="11" t="str">
-        <x:v>预留（规则TBD）</x:v>
+        <x:v>规则已实现／美术待制作</x:v>
       </x:c>
       <x:c r="H50" s="11" t="str">
-        <x:v>用户要求预留所有己方棋子技能效果</x:v>
+        <x:v>US018</x:v>
       </x:c>
       <x:c r="I50" s="11" t="str">
-        <x:v>己方仕尚未进入规则；技能名称、触发和表现 TBD</x:v>
+        <x:v>固定塔八邻格单目标攻击；子资源A-148～153，按复用关系制作，不增加主动技能。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="32" customHeight="1">
@@ -1842,7 +1850,7 @@
         <x:v>己方相尚未进入规则；技能名称、触发和表现 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="32" customHeight="1">
+    <x:row r="52" ht="100" customHeight="1">
       <x:c r="A52" s="11" t="str">
         <x:v>A-047</x:v>
       </x:c>
@@ -1850,25 +1858,25 @@
         <x:v>己方技能效果</x:v>
       </x:c>
       <x:c r="C52" s="11" t="str">
-        <x:v>马｜专属技能效果预留</x:v>
+        <x:v>马｜跳跃攻击效果总项</x:v>
       </x:c>
       <x:c r="D52" s="11" t="str">
-        <x:v>1槽</x:v>
+        <x:v>跳跃/落地四邻伤害/推动</x:v>
       </x:c>
       <x:c r="E52" s="11" t="str">
-        <x:v>己方马未来专属技能</x:v>
+        <x:v>我方马主动技能</x:v>
       </x:c>
       <x:c r="F52" s="11" t="str">
-        <x:v>无</x:v>
+        <x:v>规则及棋盘标记占位</x:v>
       </x:c>
       <x:c r="G52" s="11" t="str">
-        <x:v>预留（规则TBD）</x:v>
+        <x:v>桌面功能已交付／美术待制作</x:v>
       </x:c>
       <x:c r="H52" s="11" t="str">
-        <x:v>docs/us/US-001-m0-player-skills.md:2.2</x:v>
+        <x:v>US021（2026-10-22）</x:v>
       </x:c>
       <x:c r="I52" s="11" t="str">
-        <x:v>当前马只有基础走法和通用强健；专属技能 TBD</x:v>
+        <x:v>替代旧“专属技能TBD”。直线空格落点1～2格，强化最高4格；四邻伤害含友军；子资源A-154～159。手机横版布局仍未通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="32" customHeight="1">
@@ -2016,7 +2024,7 @@
         <x:v>表现永久解锁，不能误解为一次性攻击</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="32" customHeight="1">
+    <x:row r="58" ht="100" customHeight="1">
       <x:c r="A58" s="11" t="str">
         <x:v>A-053</x:v>
       </x:c>
@@ -2039,10 +2047,10 @@
         <x:v>待制作</x:v>
       </x:c>
       <x:c r="H58" s="11" t="str">
-        <x:v>web/js/app.js:64; web/js/rules.js:42-46</x:v>
+        <x:v>US010；US019</x:v>
       </x:c>
       <x:c r="I58" s="11" t="str">
-        <x:v>区分成功、出界、宫界和占位受阻</x:v>
+        <x:v>区分推动成功、出界和占位阻挡；主帅可被推出宫，不能把宫界统一绘成禁止位移。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="32" customHeight="1">
@@ -2596,7 +2604,7 @@
         <x:v>组件总项；面板切图复用A-109起通用资源，桌面1920×1080、手机1344×2772</x:v>
       </x:c>
     </x:row>
-    <x:row r="78" ht="32" customHeight="1">
+    <x:row r="78" ht="100" customHeight="1">
       <x:c r="A78" s="11" t="str">
         <x:v>A-073</x:v>
       </x:c>
@@ -2607,22 +2615,22 @@
         <x:v>战斗状态栏</x:v>
       </x:c>
       <x:c r="D78" s="11" t="str">
-        <x:v>桌面／手机2套</x:v>
+        <x:v>桌面/手机</x:v>
       </x:c>
       <x:c r="E78" s="11" t="str">
-        <x:v>波次、回合、主帅HP、金币、击杀</x:v>
+        <x:v>波次、回合、双方主帅HP、猫粮、公共SP、击杀、旅程增益</x:v>
       </x:c>
       <x:c r="F78" s="11" t="str">
-        <x:v>CSS卡片＋文字</x:v>
+        <x:v>HTML/CSS动态文字</x:v>
       </x:c>
       <x:c r="G78" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>代码占位／美术待制作</x:v>
       </x:c>
       <x:c r="H78" s="11" t="str">
-        <x:v>2026-10-05 当前UI核对</x:v>
+        <x:v>US017；US020</x:v>
       </x:c>
       <x:c r="I78" s="11" t="str">
-        <x:v>桌面左上；手机仅保留紧凑主要数值，完整状态折叠</x:v>
+        <x:v>猫粮替代金币，SP为全队余额；增益允许多项同时生效。</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="32" customHeight="1">
@@ -2654,7 +2662,7 @@
         <x:v>徽记复用棋子；默认/选中/行动耗尽；未实现棋种仍仅预留</x:v>
       </x:c>
     </x:row>
-    <x:row r="80" ht="32" customHeight="1">
+    <x:row r="80" ht="100" customHeight="1">
       <x:c r="A80" s="11" t="str">
         <x:v>A-075</x:v>
       </x:c>
@@ -2668,7 +2676,7 @@
         <x:v>桌面详情／手机摘要</x:v>
       </x:c>
       <x:c r="E80" s="11" t="str">
-        <x:v>属性、行动余量、等级、SP</x:v>
+        <x:v>属性、行动余量、个人等级/击杀、公共SP消费资格</x:v>
       </x:c>
       <x:c r="F80" s="11" t="str">
         <x:v>CSS信息卡＋文字</x:v>
@@ -2677,13 +2685,13 @@
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H80" s="11" t="str">
-        <x:v>2026-10-05 当前UI核对</x:v>
+        <x:v>US017；US018；US019；US021</x:v>
       </x:c>
       <x:c r="I80" s="11" t="str">
-        <x:v>长说明可展开，动态数值不烘焙</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="81" ht="32" customHeight="1">
+        <x:v>不显示个人SP钱包；帅无升级，仕有冷却，马区分普通移动与跳跃攻击。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="100" customHeight="1">
       <x:c r="A81" s="11" t="str">
         <x:v>A-076</x:v>
       </x:c>
@@ -2697,7 +2705,7 @@
         <x:v>1套＋图标槽位</x:v>
       </x:c>
       <x:c r="E81" s="11" t="str">
-        <x:v>升级、转职、方向和炮扩散</x:v>
+        <x:v>公共SP升级、转职、方向强化、炮扩散、仕间隔及马三项强化</x:v>
       </x:c>
       <x:c r="F81" s="11" t="str">
         <x:v>CSS按钮＋文字</x:v>
@@ -2706,13 +2714,13 @@
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H81" s="11" t="str">
-        <x:v>2026-10-05 当前UI核对</x:v>
+        <x:v>US017～021</x:v>
       </x:c>
       <x:c r="I81" s="11" t="str">
-        <x:v>可购买/已解锁/缺SP/当前阶段不可购买；专属技能仍为己方</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="82" ht="32" customHeight="1">
+        <x:v>技能资格按棋种；马推动2SP、距离每次1SP、伤害每次2SP独立购买，主帅无个人升级。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="100" customHeight="1">
       <x:c r="A82" s="11" t="str">
         <x:v>A-077</x:v>
       </x:c>
@@ -2720,13 +2728,13 @@
         <x:v>界面</x:v>
       </x:c>
       <x:c r="C82" s="11" t="str">
-        <x:v>方向与车模式按钮</x:v>
+        <x:v>方向及车/马操作模式按钮</x:v>
       </x:c>
       <x:c r="D82" s="11" t="str">
-        <x:v>四方向＋移动/冲锋/牵引</x:v>
+        <x:v>四方向＋车模式＋马双模式</x:v>
       </x:c>
       <x:c r="E82" s="11" t="str">
-        <x:v>弓枪方向；车职业模式</x:v>
+        <x:v>弓枪方向、车操作、马普通移动/跳跃攻击</x:v>
       </x:c>
       <x:c r="F82" s="11" t="str">
         <x:v>CSS按钮＋选中描边</x:v>
@@ -2735,10 +2743,10 @@
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H82" s="11" t="str">
-        <x:v>2026-10-05 当前UI核对</x:v>
+        <x:v>US021</x:v>
       </x:c>
       <x:c r="I82" s="11" t="str">
-        <x:v>默认/选中/禁用；手机触控面积至少44逻辑像素</x:v>
+        <x:v>马仅普通移动和跳跃攻击两个入口，不保留旧普通攻击；手机横版改造待另行授权。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="32" customHeight="1">
@@ -2770,7 +2778,7 @@
         <x:v>成功/失效/落空/已移除/待机需区分</x:v>
       </x:c>
     </x:row>
-    <x:row r="84" ht="32" customHeight="1">
+    <x:row r="84" ht="100" customHeight="1">
       <x:c r="A84" s="11" t="str">
         <x:v>A-079</x:v>
       </x:c>
@@ -2784,7 +2792,7 @@
         <x:v>桌面详情／手机摘要</x:v>
       </x:c>
       <x:c r="E84" s="11" t="str">
-        <x:v>路径、伤害、友伤、主帅威胁</x:v>
+        <x:v>路径、伤害、友伤、主帅威胁、仕自动攻击及马落点四邻</x:v>
       </x:c>
       <x:c r="F84" s="11" t="str">
         <x:v>信息卡＋棋盘标记</x:v>
@@ -2793,10 +2801,10 @@
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H84" s="11" t="str">
-        <x:v>2026-10-05 当前UI核对</x:v>
+        <x:v>US018；US019；US021</x:v>
       </x:c>
       <x:c r="I84" s="11" t="str">
-        <x:v>友伤醒目；桌面点目标直接攻击，手机保留执行确认</x:v>
+        <x:v>友伤、推动/碰撞与树林条件结果可辨；桌面点目标直接攻击，手机保留执行确认。</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="32" customHeight="1">
@@ -2886,7 +2894,7 @@
         <x:v>复用面板、遮罩、主次按钮</x:v>
       </x:c>
     </x:row>
-    <x:row r="88" ht="32" customHeight="1">
+    <x:row r="88" ht="100" customHeight="1">
       <x:c r="A88" s="11" t="str">
         <x:v>A-083</x:v>
       </x:c>
@@ -2894,28 +2902,28 @@
         <x:v>界面</x:v>
       </x:c>
       <x:c r="C88" s="11" t="str">
-        <x:v>商店与商品卡</x:v>
+        <x:v>主营地与招募商品卡（原关间商店）</x:v>
       </x:c>
       <x:c r="D88" s="11" t="str">
-        <x:v>兵/车/马/炮4类</x:v>
+        <x:v>兵/车/马/炮/仕</x:v>
       </x:c>
       <x:c r="E88" s="11" t="str">
-        <x:v>关间整备与上阵后备</x:v>
+        <x:v>首次教学后及非最终关胜利后整备</x:v>
       </x:c>
       <x:c r="F88" s="11" t="str">
-        <x:v>对话框＋商品卡＋队伍列表</x:v>
+        <x:v>camp页面及动态卡片占位</x:v>
       </x:c>
       <x:c r="G88" s="11" t="str">
-        <x:v>代码占位</x:v>
+        <x:v>功能已接入／美术待制作</x:v>
       </x:c>
       <x:c r="H88" s="11" t="str">
-        <x:v>2026-10-05 当前UI核对</x:v>
+        <x:v>US020；US018</x:v>
       </x:c>
       <x:c r="I88" s="11" t="str">
-        <x:v>商品像复用棋子；价格、阵容容量实时文字</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="89" ht="32" customHeight="1">
+        <x:v>总项复用商品皮肤；猫粮价格、部署上限、队友总数和后备数实时显示，主帅与仕单列。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="100" customHeight="1">
       <x:c r="A89" s="11" t="str">
         <x:v>A-084</x:v>
       </x:c>
@@ -2926,7 +2934,7 @@
         <x:v>终局弹窗</x:v>
       </x:c>
       <x:c r="D89" s="11" t="str">
-        <x:v>胜利/阵亡/将死3态</x:v>
+        <x:v>胜利/主帅阵亡失败/三关通关</x:v>
       </x:c>
       <x:c r="E89" s="11" t="str">
         <x:v>战斗结果</x:v>
@@ -2938,10 +2946,10 @@
         <x:v>代码占位</x:v>
       </x:c>
       <x:c r="H89" s="11" t="str">
-        <x:v>2026-10-05 当前UI核对</x:v>
+        <x:v>US019；US020</x:v>
       </x:c>
       <x:c r="I89" s="11" t="str">
-        <x:v>独立结果标题装饰详见新增条目；统计数字实时文字</x:v>
+        <x:v>不以搜索将死作为现行失败条件；教学结果另列A-143。</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="32" customHeight="1">
@@ -3234,7 +3242,7 @@
         <x:v>文字与按钮独立，不烘焙</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" ht="60" customHeight="1">
+    <x:row r="100" ht="100" customHeight="1">
       <x:c r="A100" s="11" t="str">
         <x:v>A-095</x:v>
       </x:c>
@@ -3257,10 +3265,10 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H100" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US020 R09</x:v>
       </x:c>
       <x:c r="I100" s="11" t="str">
-        <x:v>两个功能共用按钮皮肤，继续游戏规则 TBD</x:v>
+        <x:v>已有本地旅程时可继续；重开旅程需确认，实时显示存档状态，不把按钮可用态烘焙。</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="60" customHeight="1">
@@ -3321,7 +3329,7 @@
         <x:v>可用棋子/兵旗/印章；不遮挡按钮</x:v>
       </x:c>
     </x:row>
-    <x:row r="103" ht="60" customHeight="1">
+    <x:row r="103" ht="100" customHeight="1">
       <x:c r="A103" s="11" t="str">
         <x:v>A-098</x:v>
       </x:c>
@@ -3335,7 +3343,7 @@
         <x:v>横竖2版</x:v>
       </x:c>
       <x:c r="E103" s="11" t="str">
-        <x:v>开始游戏后的选关页</x:v>
+        <x:v>主营地出发后的选关地图</x:v>
       </x:c>
       <x:c r="F103" s="11" t="str">
         <x:v>独立美术样稿中预留</x:v>
@@ -3344,13 +3352,13 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H103" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US020 R02/R08</x:v>
       </x:c>
       <x:c r="I103" s="11" t="str">
-        <x:v>三分区为玩法草案；历史边界和时代年份 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="104" ht="60" customHeight="1">
+        <x:v>1→2→3顺序解锁；三关都可预览。演武场独立地图地区仍属US016 WIP。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="100" customHeight="1">
       <x:c r="A104" s="11" t="str">
         <x:v>A-099</x:v>
       </x:c>
@@ -3373,13 +3381,13 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H104" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US012；US020 R08</x:v>
       </x:c>
       <x:c r="I104" s="11" t="str">
-        <x:v>西部关中主题；山隘/城塞视觉；区域范围与关名 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="105" ht="60" customHeight="1">
+        <x:v>关名已用于当前原型；美术边界、精确历史年代TBD，不据此复原真实疆界。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="100" customHeight="1">
       <x:c r="A105" s="11" t="str">
         <x:v>A-100</x:v>
       </x:c>
@@ -3402,13 +3410,13 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H105" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US012；US020 R08</x:v>
       </x:c>
       <x:c r="I105" s="11" t="str">
-        <x:v>中央平原主题；河流/城邑视觉；区域范围与关名 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="106" ht="60" customHeight="1">
+        <x:v>关名已用于当前原型；美术边界、精确历史年代TBD，不据此复原真实疆界。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="100" customHeight="1">
       <x:c r="A106" s="11" t="str">
         <x:v>A-101</x:v>
       </x:c>
@@ -3431,10 +3439,10 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H106" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US012；US020 R08</x:v>
       </x:c>
       <x:c r="I106" s="11" t="str">
-        <x:v>东南水网主题；水泽/林地视觉；区域范围与关名 TBD</x:v>
+        <x:v>关名已用于当前原型；美术边界、精确历史年代TBD，不据此复原真实疆界。</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="60" customHeight="1">
@@ -3466,7 +3474,7 @@
         <x:v>三个区域共边不得出现缝隙；非真实国界</x:v>
       </x:c>
     </x:row>
-    <x:row r="108" ht="60" customHeight="1">
+    <x:row r="108" ht="100" customHeight="1">
       <x:c r="A108" s="11" t="str">
         <x:v>A-103</x:v>
       </x:c>
@@ -3489,13 +3497,13 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H108" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US020 R08</x:v>
       </x:c>
       <x:c r="I108" s="11" t="str">
-        <x:v>美术预留4态；解锁条件 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="109" ht="60" customHeight="1">
+        <x:v>锁定/可挑战/选中/通关；锁定与已通关可预览，但不可跳关或重打。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="100" customHeight="1">
       <x:c r="A109" s="11" t="str">
         <x:v>A-104</x:v>
       </x:c>
@@ -3518,10 +3526,10 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H109" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US012；US020 R08</x:v>
       </x:c>
       <x:c r="I109" s="11" t="str">
-        <x:v>路线仅为叙事顺序草案，不代表已实现进度</x:v>
+        <x:v>正式顺序1→2→3已确认；路线不表示任意分支或可重打。</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="60" customHeight="1">
@@ -3582,7 +3590,7 @@
         <x:v>依次山隘、平原城邑、水网；最终题材 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="112" ht="60" customHeight="1">
+    <x:row r="112" ht="100" customHeight="1">
       <x:c r="A112" s="11" t="str">
         <x:v>A-107</x:v>
       </x:c>
@@ -3596,7 +3604,7 @@
         <x:v>1套</x:v>
       </x:c>
       <x:c r="E112" s="11" t="str">
-        <x:v>关卡说明与进入按钮</x:v>
+        <x:v>关卡说明、地形/首波预览与进入按钮</x:v>
       </x:c>
       <x:c r="F112" s="11" t="str">
         <x:v>独立美术样稿中预留</x:v>
@@ -3605,10 +3613,10 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H112" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US020 R08</x:v>
       </x:c>
       <x:c r="I112" s="11" t="str">
-        <x:v>标题、难度、奖励用文字；玩法参数 TBD</x:v>
+        <x:v>底板复用；第二波位置不提前显示；战术缩略图由程序生成，见A-139。</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="60" customHeight="1">
@@ -3698,7 +3706,7 @@
         <x:v>结束回合、撤销、暂停、取消、确认共用</x:v>
       </x:c>
     </x:row>
-    <x:row r="116" ht="60" customHeight="1">
+    <x:row r="116" ht="100" customHeight="1">
       <x:c r="A116" s="11" t="str">
         <x:v>A-111</x:v>
       </x:c>
@@ -3712,7 +3720,7 @@
         <x:v>8款</x:v>
       </x:c>
       <x:c r="E116" s="11" t="str">
-        <x:v>返回/关闭/设置/暂停/继续/重试/收起/展开</x:v>
+        <x:v>返回/关闭/设置/暂停/继续/重试/收起/展开/帮助/保存</x:v>
       </x:c>
       <x:c r="F116" s="11" t="str">
         <x:v>现有HTML/CSS或资源规格预留</x:v>
@@ -3721,13 +3729,13 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H116" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US015；US020</x:v>
       </x:c>
       <x:c r="I116" s="11" t="str">
-        <x:v>点击区域由程序保持至少44逻辑像素</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="117" ht="60" customHeight="1">
+        <x:v>复用通用图标；44逻辑像素为点击热区，不要求图标本身44像素。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="100" customHeight="1">
       <x:c r="A117" s="11" t="str">
         <x:v>A-112</x:v>
       </x:c>
@@ -3738,10 +3746,10 @@
         <x:v>资源属性图标</x:v>
       </x:c>
       <x:c r="D117" s="11" t="str">
-        <x:v>7款</x:v>
+        <x:v>HP/AP/公共SP/猫粮/回合/击杀/等级/部署上限</x:v>
       </x:c>
       <x:c r="E117" s="11" t="str">
-        <x:v>HP/AP/SP/金币/回合/击杀/等级</x:v>
+        <x:v>全部资源与属性栏</x:v>
       </x:c>
       <x:c r="F117" s="11" t="str">
         <x:v>现有HTML/CSS或资源规格预留</x:v>
@@ -3750,10 +3758,10 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H117" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US017；US020</x:v>
       </x:c>
       <x:c r="I117" s="11" t="str">
-        <x:v>保留数值文字，避免仅靠图标猜测</x:v>
+        <x:v>金币图标退役并替换猫粮A-160；公共SP仅一份钱包。实时数值不切图。</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="60" customHeight="1">
@@ -3959,7 +3967,7 @@
         <x:v>只表达规则已揭示的信息</x:v>
       </x:c>
     </x:row>
-    <x:row r="125" ht="60" customHeight="1">
+    <x:row r="125" ht="100" customHeight="1">
       <x:c r="A125" s="11" t="str">
         <x:v>A-120</x:v>
       </x:c>
@@ -3967,28 +3975,28 @@
         <x:v>战斗UI</x:v>
       </x:c>
       <x:c r="C125" s="11" t="str">
-        <x:v>主帅增益选择卡</x:v>
+        <x:v>主帅旅程增益卡（替代三选一）</x:v>
       </x:c>
       <x:c r="D125" s="11" t="str">
-        <x:v>3款</x:v>
+        <x:v>坚守/疾行/救援3款及状态</x:v>
       </x:c>
       <x:c r="E125" s="11" t="str">
-        <x:v>坚守/疾行/救援</x:v>
+        <x:v>主营地顺序解锁、战斗摘要</x:v>
       </x:c>
       <x:c r="F125" s="11" t="str">
-        <x:v>现有HTML/CSS或资源规格预留</x:v>
+        <x:v>动态卡片/文字占位</x:v>
       </x:c>
       <x:c r="G125" s="11" t="str">
-        <x:v>预留／待制作</x:v>
+        <x:v>功能已接入／美术待制作</x:v>
       </x:c>
       <x:c r="H125" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US020 R05</x:v>
       </x:c>
       <x:c r="I125" s="11" t="str">
-        <x:v>不烘焙技能描述和数值</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="126" ht="60" customHeight="1">
+        <x:v>首次入营免费坚守；疾行5猫粮、救援5猫粮，依次解锁、同时生效、跨关保留；不再制作互斥三选一。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="100" customHeight="1">
       <x:c r="A126" s="11" t="str">
         <x:v>A-121</x:v>
       </x:c>
@@ -4002,7 +4010,7 @@
         <x:v>通用1套＋己方9棋种槽位</x:v>
       </x:c>
       <x:c r="E126" s="11" t="str">
-        <x:v>升级/转职/方向/扩散</x:v>
+        <x:v>普通队友技能/转职/方向/扩散；仕间隔；马推动/距离/伤害</x:v>
       </x:c>
       <x:c r="F126" s="11" t="str">
         <x:v>现有HTML/CSS或资源规格预留</x:v>
@@ -4011,10 +4019,10 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H126" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US017～021</x:v>
       </x:c>
       <x:c r="I126" s="11" t="str">
-        <x:v>与A-042至A-065技能特效分开；敌方不新增主动技能</x:v>
+        <x:v>主帅无个人技能升级图标；与技能效果区分；敌方不新增主动技能。</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="60" customHeight="1">
@@ -4075,7 +4083,7 @@
         <x:v>列棋名及坐标；预留未行动徽记96×96</x:v>
       </x:c>
     </x:row>
-    <x:row r="129" ht="60" customHeight="1">
+    <x:row r="129" ht="100" customHeight="1">
       <x:c r="A129" s="11" t="str">
         <x:v>A-124</x:v>
       </x:c>
@@ -4089,7 +4097,7 @@
         <x:v>1套</x:v>
       </x:c>
       <x:c r="E129" s="11" t="str">
-        <x:v>布阵/商店队伍管理</x:v>
+        <x:v>主营地、布阵的上阵/后备及独立主帅/仕列表</x:v>
       </x:c>
       <x:c r="F129" s="11" t="str">
         <x:v>现有HTML/CSS或资源规格预留</x:v>
@@ -4098,13 +4106,13 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H129" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US020 R04</x:v>
       </x:c>
       <x:c r="I129" s="11" t="str">
-        <x:v>头像复用己方棋子资源</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="130" ht="60" customHeight="1">
+        <x:v>普通队友总数不限；部署人口初始4上限8。主帅和仕不占人口，仕无后备；共用棋子像。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="100" customHeight="1">
       <x:c r="A130" s="11" t="str">
         <x:v>A-125</x:v>
       </x:c>
@@ -4112,28 +4120,28 @@
         <x:v>战斗UI</x:v>
       </x:c>
       <x:c r="C130" s="11" t="str">
-        <x:v>救援角色卡与恢复标记</x:v>
+        <x:v>救援选择卡与恢复/复活标记</x:v>
       </x:c>
       <x:c r="D130" s="11" t="str">
-        <x:v>1套</x:v>
+        <x:v>受伤恢复/尸体复活/跳过</x:v>
       </x:c>
       <x:c r="E130" s="11" t="str">
-        <x:v>第6回合救援</x:v>
+        <x:v>已解锁救援后的第二波开始前</x:v>
       </x:c>
       <x:c r="F130" s="11" t="str">
-        <x:v>现有HTML/CSS或资源规格预留</x:v>
+        <x:v>名单与恢复占位</x:v>
       </x:c>
       <x:c r="G130" s="11" t="str">
-        <x:v>预留／待制作</x:v>
+        <x:v>功能已接入／美术待制作</x:v>
       </x:c>
       <x:c r="H130" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US020 R06</x:v>
       </x:c>
       <x:c r="I130" s="11" t="str">
-        <x:v>人物形象复用棋子；恢复表现关联技能通用效果</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="131" ht="60" customHeight="1">
+        <x:v>受伤普通队友回满血；有效尸体原位1HP复活；排除主帅、仕、已毁尸体、满血及后备。效果见A-162。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="100" customHeight="1">
       <x:c r="A131" s="11" t="str">
         <x:v>A-126</x:v>
       </x:c>
@@ -4141,13 +4149,13 @@
         <x:v>战斗UI</x:v>
       </x:c>
       <x:c r="C131" s="11" t="str">
-        <x:v>商店商品与价格标签</x:v>
+        <x:v>营地招募商品与猫粮价格标签</x:v>
       </x:c>
       <x:c r="D131" s="11" t="str">
-        <x:v>兵/车/马/炮4类</x:v>
+        <x:v>普通队友及仕商品</x:v>
       </x:c>
       <x:c r="E131" s="11" t="str">
-        <x:v>关间整备</x:v>
+        <x:v>主营地招募</x:v>
       </x:c>
       <x:c r="F131" s="11" t="str">
         <x:v>现有HTML/CSS或资源规格预留</x:v>
@@ -4156,10 +4164,10 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H131" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US020 R03/R04</x:v>
       </x:c>
       <x:c r="I131" s="11" t="str">
-        <x:v>棋子像复用，价格由程序写入</x:v>
+        <x:v>不足仅禁用且保留价格，不显示差额；部署满员仍可招募至后备，仕最多两座。</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="60" customHeight="1">
@@ -4191,7 +4199,7 @@
         <x:v>统计数字和操作按钮独立</x:v>
       </x:c>
     </x:row>
-    <x:row r="133" ht="60" customHeight="1">
+    <x:row r="133" ht="100" customHeight="1">
       <x:c r="A133" s="11" t="str">
         <x:v>A-128</x:v>
       </x:c>
@@ -4214,13 +4222,13 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H133" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US015；US020；US021</x:v>
       </x:c>
       <x:c r="I133" s="11" t="str">
-        <x:v>448×924逻辑视口，3倍参考导出；保持一屏</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="134" ht="60" customHeight="1">
+        <x:v>448×924逻辑视口，3倍参考导出；保持一屏；手机横版844×390存在棋盘不可辨问题，最终布局/切图规格TBD，不标全端通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="100" customHeight="1">
       <x:c r="A134" s="11" t="str">
         <x:v>A-129</x:v>
       </x:c>
@@ -4243,13 +4251,13 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H134" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US015；US020；US021</x:v>
       </x:c>
       <x:c r="I134" s="11" t="str">
-        <x:v>内容可内部滚动，主战斗页不滚动</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="135" ht="60" customHeight="1">
+        <x:v>内容可内部滚动，主战斗页不滚动；手机横版844×390存在棋盘不可辨问题，最终布局/切图规格TBD，不标全端通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="100" customHeight="1">
       <x:c r="A135" s="11" t="str">
         <x:v>A-130</x:v>
       </x:c>
@@ -4272,10 +4280,10 @@
         <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="H135" s="11" t="str">
-        <x:v>2026-10-05 美术需求</x:v>
+        <x:v>US015；US020；US021</x:v>
       </x:c>
       <x:c r="I135" s="11" t="str">
-        <x:v>与桌面信息同源，文本不烘焙</x:v>
+        <x:v>与桌面信息同源，文本不烘焙；手机横版844×390存在棋盘不可辨问题，最终布局/切图规格TBD，不标全端通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="60" customHeight="1">
@@ -4305,6 +4313,905 @@
       </x:c>
       <x:c r="I136" s="11" t="str">
         <x:v>字体授权 TBD；资源尺寸为制作建议，最终风格待确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="90" customHeight="1">
+      <x:c r="A137" s="11" t="str">
+        <x:v>A-132</x:v>
+      </x:c>
+      <x:c r="B137" s="11" t="str">
+        <x:v>营地UI</x:v>
+      </x:c>
+      <x:c r="C137" s="11" t="str">
+        <x:v>主营地背景</x:v>
+      </x:c>
+      <x:c r="D137" s="11" t="str">
+        <x:v>桌面/手机构图</x:v>
+      </x:c>
+      <x:c r="E137" s="11" t="str">
+        <x:v>主营地全屏</x:v>
+      </x:c>
+      <x:c r="F137" s="11" t="str">
+        <x:v>CSS面板占位</x:v>
+      </x:c>
+      <x:c r="G137" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H137" s="11" t="str">
+        <x:v>US020</x:v>
+      </x:c>
+      <x:c r="I137" s="11" t="str">
+        <x:v>营地氛围插画可复用菜单元素；视觉风格TBD。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="90" customHeight="1">
+      <x:c r="A138" s="11" t="str">
+        <x:v>A-133</x:v>
+      </x:c>
+      <x:c r="B138" s="11" t="str">
+        <x:v>营地UI</x:v>
+      </x:c>
+      <x:c r="C138" s="11" t="str">
+        <x:v>营地功能分区底板</x:v>
+      </x:c>
+      <x:c r="D138" s="11" t="str">
+        <x:v>资源/名单/招募/成长/技能5区</x:v>
+      </x:c>
+      <x:c r="E138" s="11" t="str">
+        <x:v>主营地布局</x:v>
+      </x:c>
+      <x:c r="F138" s="11" t="str">
+        <x:v>HTML/CSS卡片</x:v>
+      </x:c>
+      <x:c r="G138" s="11" t="str">
+        <x:v>复用／待制作</x:v>
+      </x:c>
+      <x:c r="H138" s="11" t="str">
+        <x:v>US020</x:v>
+      </x:c>
+      <x:c r="I138" s="11" t="str">
+        <x:v>复用A-109/110；分区标题为动态文字，不制作五套重复底板。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="90" customHeight="1">
+      <x:c r="A139" s="11" t="str">
+        <x:v>A-134</x:v>
+      </x:c>
+      <x:c r="B139" s="11" t="str">
+        <x:v>营地UI</x:v>
+      </x:c>
+      <x:c r="C139" s="11" t="str">
+        <x:v>队友总数与部署上限组件</x:v>
+      </x:c>
+      <x:c r="D139" s="11" t="str">
+        <x:v>总数/后备数/部署数/扩编状态</x:v>
+      </x:c>
+      <x:c r="E139" s="11" t="str">
+        <x:v>营地和布阵</x:v>
+      </x:c>
+      <x:c r="F139" s="11" t="str">
+        <x:v>动态文字及按钮</x:v>
+      </x:c>
+      <x:c r="G139" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H139" s="11" t="str">
+        <x:v>US020 R04（2026-10-21）</x:v>
+      </x:c>
+      <x:c r="I139" s="11" t="str">
+        <x:v>库存不限、部署4→8；主帅与仕单列；价格和人数不烘焙。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="90" customHeight="1">
+      <x:c r="A140" s="11" t="str">
+        <x:v>A-135</x:v>
+      </x:c>
+      <x:c r="B140" s="11" t="str">
+        <x:v>营地UI</x:v>
+      </x:c>
+      <x:c r="C140" s="11" t="str">
+        <x:v>旅程增益解锁顺序与状态连接</x:v>
+      </x:c>
+      <x:c r="D140" s="11" t="str">
+        <x:v>锁定/可购买/已解锁</x:v>
+      </x:c>
+      <x:c r="E140" s="11" t="str">
+        <x:v>主营地增益区</x:v>
+      </x:c>
+      <x:c r="F140" s="11" t="str">
+        <x:v>按钮与状态文字</x:v>
+      </x:c>
+      <x:c r="G140" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H140" s="11" t="str">
+        <x:v>US020 R05</x:v>
+      </x:c>
+      <x:c r="I140" s="11" t="str">
+        <x:v>坚守→疾行→救援；复用A-120三图标，增加前置关系及同时生效状态。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="90" customHeight="1">
+      <x:c r="A141" s="11" t="str">
+        <x:v>A-136</x:v>
+      </x:c>
+      <x:c r="B141" s="11" t="str">
+        <x:v>营地UI</x:v>
+      </x:c>
+      <x:c r="C141" s="11" t="str">
+        <x:v>主营地首次指引与帮助卡</x:v>
+      </x:c>
+      <x:c r="D141" s="11" t="str">
+        <x:v>首次/跳过/帮助重看</x:v>
+      </x:c>
+      <x:c r="E141" s="11" t="str">
+        <x:v>首次入营与帮助</x:v>
+      </x:c>
+      <x:c r="F141" s="11" t="str">
+        <x:v>现有说明弹窗</x:v>
+      </x:c>
+      <x:c r="G141" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H141" s="11" t="str">
+        <x:v>US020 R10</x:v>
+      </x:c>
+      <x:c r="I141" s="11" t="str">
+        <x:v>解释猫粮、库存/部署、招募、公共SP及增益顺序；复用通用弹窗，无新引导角色。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="90" customHeight="1">
+      <x:c r="A142" s="11" t="str">
+        <x:v>A-137</x:v>
+      </x:c>
+      <x:c r="B142" s="11" t="str">
+        <x:v>营地效果</x:v>
+      </x:c>
+      <x:c r="C142" s="11" t="str">
+        <x:v>回营恢复反馈</x:v>
+      </x:c>
+      <x:c r="D142" s="11" t="str">
+        <x:v>伤员恢复/普通队友与仕恢复</x:v>
+      </x:c>
+      <x:c r="E142" s="11" t="str">
+        <x:v>非最终关胜利回营</x:v>
+      </x:c>
+      <x:c r="F142" s="11" t="str">
+        <x:v>属性更新占位</x:v>
+      </x:c>
+      <x:c r="G142" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H142" s="11" t="str">
+        <x:v>US020 R07</x:v>
+      </x:c>
+      <x:c r="I142" s="11" t="str">
+        <x:v>复用治疗/复活主体，回营恢复不误表现为关内治疗仕。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="90" customHeight="1">
+      <x:c r="A143" s="11" t="str">
+        <x:v>A-138</x:v>
+      </x:c>
+      <x:c r="B143" s="11" t="str">
+        <x:v>通用UI</x:v>
+      </x:c>
+      <x:c r="C143" s="11" t="str">
+        <x:v>本地保存与保存失败反馈</x:v>
+      </x:c>
+      <x:c r="D143" s="11" t="str">
+        <x:v>已保存/失败/本次会话</x:v>
+      </x:c>
+      <x:c r="E143" s="11" t="str">
+        <x:v>营地消费、继续旅程和存储异常</x:v>
+      </x:c>
+      <x:c r="F143" s="11" t="str">
+        <x:v>动态提示文字</x:v>
+      </x:c>
+      <x:c r="G143" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H143" s="11" t="str">
+        <x:v>US020 R09</x:v>
+      </x:c>
+      <x:c r="I143" s="11" t="str">
+        <x:v>复用A-085/111，保存失败不能显示成功；不承诺云同步。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="90" customHeight="1">
+      <x:c r="A144" s="11" t="str">
+        <x:v>A-139</x:v>
+      </x:c>
+      <x:c r="B144" s="11" t="str">
+        <x:v>关卡地图</x:v>
+      </x:c>
+      <x:c r="C144" s="11" t="str">
+        <x:v>关卡战术缩略图及棋种图例</x:v>
+      </x:c>
+      <x:c r="D144" s="11" t="str">
+        <x:v>地形/首波敌方站位</x:v>
+      </x:c>
+      <x:c r="E144" s="11" t="str">
+        <x:v>三关选关详情</x:v>
+      </x:c>
+      <x:c r="F144" s="11" t="str">
+        <x:v>有效地图配置生成</x:v>
+      </x:c>
+      <x:c r="G144" s="11" t="str">
+        <x:v>复用／待制作</x:v>
+      </x:c>
+      <x:c r="H144" s="11" t="str">
+        <x:v>US020 R08</x:v>
+      </x:c>
+      <x:c r="I144" s="11" t="str">
+        <x:v>复用地形与敌方棋子缩略像；程序生成，不手绘三张易失真的战局图；不泄露第二波。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="90" customHeight="1">
+      <x:c r="A145" s="11" t="str">
+        <x:v>A-140</x:v>
+      </x:c>
+      <x:c r="B145" s="11" t="str">
+        <x:v>教学UI</x:v>
+      </x:c>
+      <x:c r="C145" s="11" t="str">
+        <x:v>第0关演武场入口卡</x:v>
+      </x:c>
+      <x:c r="D145" s="11" t="str">
+        <x:v>首次必修/曾完成可跳过</x:v>
+      </x:c>
+      <x:c r="E145" s="11" t="str">
+        <x:v>新旅程教学入口</x:v>
+      </x:c>
+      <x:c r="F145" s="11" t="str">
+        <x:v>教学入口已接入</x:v>
+      </x:c>
+      <x:c r="G145" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H145" s="11" t="str">
+        <x:v>US020 R01；US016内容</x:v>
+      </x:c>
+      <x:c r="I145" s="11" t="str">
+        <x:v>首次必须完成；曾完成才可跳过；完成/合法跳过先入营地，覆盖US016旧首次可跳过方案。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="90" customHeight="1">
+      <x:c r="A146" s="11" t="str">
+        <x:v>A-141</x:v>
+      </x:c>
+      <x:c r="B146" s="11" t="str">
+        <x:v>教学UI</x:v>
+      </x:c>
+      <x:c r="C146" s="11" t="str">
+        <x:v>教学步骤卡与进度</x:v>
+      </x:c>
+      <x:c r="D146" s="11" t="str">
+        <x:v>7步/当前/完成</x:v>
+      </x:c>
+      <x:c r="E146" s="11" t="str">
+        <x:v>教学战斗提示区</x:v>
+      </x:c>
+      <x:c r="F146" s="11" t="str">
+        <x:v>现有步骤标题与文字</x:v>
+      </x:c>
+      <x:c r="G146" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H146" s="11" t="str">
+        <x:v>US020；US016教学内容</x:v>
+      </x:c>
+      <x:c r="I146" s="11" t="str">
+        <x:v>进度由操作事件驱动；不把步骤文字烘焙到图内。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="90" customHeight="1">
+      <x:c r="A147" s="11" t="str">
+        <x:v>A-142</x:v>
+      </x:c>
+      <x:c r="B147" s="11" t="str">
+        <x:v>教学UI</x:v>
+      </x:c>
+      <x:c r="C147" s="11" t="str">
+        <x:v>教学聚焦框与指向箭头</x:v>
+      </x:c>
+      <x:c r="D147" s="11" t="str">
+        <x:v>棋子/格子/按钮高亮</x:v>
+      </x:c>
+      <x:c r="E147" s="11" t="str">
+        <x:v>教学指定操作目标</x:v>
+      </x:c>
+      <x:c r="F147" s="11" t="str">
+        <x:v>现有提示与标记占位</x:v>
+      </x:c>
+      <x:c r="G147" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H147" s="11" t="str">
+        <x:v>US016；US020</x:v>
+      </x:c>
+      <x:c r="I147" s="11" t="str">
+        <x:v>复用A-066～071/118；描边和文字共同提示，避免只靠颜色。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="90" customHeight="1">
+      <x:c r="A148" s="11" t="str">
+        <x:v>A-143</x:v>
+      </x:c>
+      <x:c r="B148" s="11" t="str">
+        <x:v>教学UI</x:v>
+      </x:c>
+      <x:c r="C148" s="11" t="str">
+        <x:v>教学完成与失败反馈</x:v>
+      </x:c>
+      <x:c r="D148" s="11" t="str">
+        <x:v>完成/重试/入营</x:v>
+      </x:c>
+      <x:c r="E148" s="11" t="str">
+        <x:v>教学结果层</x:v>
+      </x:c>
+      <x:c r="F148" s="11" t="str">
+        <x:v>教学结果弹窗</x:v>
+      </x:c>
+      <x:c r="G148" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H148" s="11" t="str">
+        <x:v>US020 R01</x:v>
+      </x:c>
+      <x:c r="I148" s="11" t="str">
+        <x:v>完成所得猫粮保留，教学技能/伤亡清空；失败只重试；复用A-127标题装饰。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="90" customHeight="1">
+      <x:c r="A149" s="11" t="str">
+        <x:v>A-144</x:v>
+      </x:c>
+      <x:c r="B149" s="11" t="str">
+        <x:v>教学UI</x:v>
+      </x:c>
+      <x:c r="C149" s="11" t="str">
+        <x:v>合法跳过教学确认弹窗</x:v>
+      </x:c>
+      <x:c r="D149" s="11" t="str">
+        <x:v>返回学习/确认跳过</x:v>
+      </x:c>
+      <x:c r="E149" s="11" t="str">
+        <x:v>曾完成教学的新旅程</x:v>
+      </x:c>
+      <x:c r="F149" s="11" t="str">
+        <x:v>现有确认弹窗</x:v>
+      </x:c>
+      <x:c r="G149" s="11" t="str">
+        <x:v>复用／待制作</x:v>
+      </x:c>
+      <x:c r="H149" s="11" t="str">
+        <x:v>US020 R01；US016</x:v>
+      </x:c>
+      <x:c r="I149" s="11" t="str">
+        <x:v>二次确认，仅曾完成者可用；跳过不给教学收益；复用A-109/110/114。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="90" customHeight="1">
+      <x:c r="A150" s="11" t="str">
+        <x:v>A-145</x:v>
+      </x:c>
+      <x:c r="B150" s="11" t="str">
+        <x:v>教学预留</x:v>
+      </x:c>
+      <x:c r="C150" s="11" t="str">
+        <x:v>演武场独立地图地区</x:v>
+      </x:c>
+      <x:c r="D150" s="11" t="str">
+        <x:v>区域/旗帜/选中描边</x:v>
+      </x:c>
+      <x:c r="E150" s="11" t="str">
+        <x:v>初始地图独立教学地区</x:v>
+      </x:c>
+      <x:c r="F150" s="11" t="str">
+        <x:v>独立地图入口尚未实现</x:v>
+      </x:c>
+      <x:c r="G150" s="22" t="str">
+        <x:v>WIP／仅预留</x:v>
+      </x:c>
+      <x:c r="H150" s="11" t="str">
+        <x:v>US016（US020未覆盖的草案）</x:v>
+      </x:c>
+      <x:c r="I150" s="11" t="str">
+        <x:v>第0关教学已接入不代表独立地图地区已实现；位置、入口关系和最终布局TBD。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="90" customHeight="1">
+      <x:c r="A151" s="11" t="str">
+        <x:v>A-146</x:v>
+      </x:c>
+      <x:c r="B151" s="11" t="str">
+        <x:v>教学预留</x:v>
+      </x:c>
+      <x:c r="C151" s="11" t="str">
+        <x:v>演武场地图状态徽记</x:v>
+      </x:c>
+      <x:c r="D151" s="11" t="str">
+        <x:v>待学习/已完成/已跳过</x:v>
+      </x:c>
+      <x:c r="E151" s="11" t="str">
+        <x:v>教学地图地区</x:v>
+      </x:c>
+      <x:c r="F151" s="11" t="str">
+        <x:v>方案预留</x:v>
+      </x:c>
+      <x:c r="G151" s="22" t="str">
+        <x:v>WIP／仅预留</x:v>
+      </x:c>
+      <x:c r="H151" s="11" t="str">
+        <x:v>US016</x:v>
+      </x:c>
+      <x:c r="I151" s="11" t="str">
+        <x:v>必须遵循首次必修的新规则；是否展示已跳过及重学去向TBD。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="90" customHeight="1">
+      <x:c r="A152" s="11" t="str">
+        <x:v>A-147</x:v>
+      </x:c>
+      <x:c r="B152" s="11" t="str">
+        <x:v>教学预留</x:v>
+      </x:c>
+      <x:c r="C152" s="11" t="str">
+        <x:v>正式流程首次规则提示</x:v>
+      </x:c>
+      <x:c r="D152" s="11" t="str">
+        <x:v>部署/地形/弓炮/SP/友伤等</x:v>
+      </x:c>
+      <x:c r="E152" s="11" t="str">
+        <x:v>首次遇到相关玩法</x:v>
+      </x:c>
+      <x:c r="F152" s="11" t="str">
+        <x:v>草案，非完整提示系统</x:v>
+      </x:c>
+      <x:c r="G152" s="22" t="str">
+        <x:v>WIP／仅预留</x:v>
+      </x:c>
+      <x:c r="H152" s="11" t="str">
+        <x:v>US016 §4</x:v>
+      </x:c>
+      <x:c r="I152" s="11" t="str">
+        <x:v>仅预留通用提示皮肤与小图；精确触发、频率、帮助入口TBD，复用现有图标。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="90" customHeight="1">
+      <x:c r="A153" s="11" t="str">
+        <x:v>A-148</x:v>
+      </x:c>
+      <x:c r="B153" s="11" t="str">
+        <x:v>棋子状态</x:v>
+      </x:c>
+      <x:c r="C153" s="11" t="str">
+        <x:v>仕｜被毁残骸</x:v>
+      </x:c>
+      <x:c r="D153" s="11" t="str">
+        <x:v>1套，双侧共用</x:v>
+      </x:c>
+      <x:c r="E153" s="11" t="str">
+        <x:v>仕阵亡占格</x:v>
+      </x:c>
+      <x:c r="F153" s="11" t="str">
+        <x:v>规则尸体/残骸占位</x:v>
+      </x:c>
+      <x:c r="G153" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H153" s="11" t="str">
+        <x:v>US018 §6</x:v>
+      </x:c>
+      <x:c r="I153" s="11" t="str">
+        <x:v>活塔不能移动，残骸可推动、作炮架、入水销毁；不能被关内救援。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="90" customHeight="1">
+      <x:c r="A154" s="11" t="str">
+        <x:v>A-149</x:v>
+      </x:c>
+      <x:c r="B154" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C154" s="11" t="str">
+        <x:v>仕｜自动射击弹道与命中</x:v>
+      </x:c>
+      <x:c r="D154" s="11" t="str">
+        <x:v>发射/命中/闪避</x:v>
+      </x:c>
+      <x:c r="E154" s="11" t="str">
+        <x:v>结束回合后敌攻前</x:v>
+      </x:c>
+      <x:c r="F154" s="11" t="str">
+        <x:v>连线/结算占位</x:v>
+      </x:c>
+      <x:c r="G154" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H154" s="11" t="str">
+        <x:v>US018 §3～4</x:v>
+      </x:c>
+      <x:c r="I154" s="11" t="str">
+        <x:v>八邻格选1敌人，双塔可同目标；动画顺序不改变同时锁定规则；复用A-117/024。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="90" customHeight="1">
+      <x:c r="A155" s="11" t="str">
+        <x:v>A-150</x:v>
+      </x:c>
+      <x:c r="B155" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C155" s="11" t="str">
+        <x:v>仕｜就绪与冷却标识</x:v>
+      </x:c>
+      <x:c r="D155" s="11" t="str">
+        <x:v>就绪有目标/就绪无目标/冷却</x:v>
+      </x:c>
+      <x:c r="E155" s="11" t="str">
+        <x:v>仕详情、棋盘、名单</x:v>
+      </x:c>
+      <x:c r="F155" s="11" t="str">
+        <x:v>动态文字占位</x:v>
+      </x:c>
+      <x:c r="G155" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H155" s="11" t="str">
+        <x:v>US018 §5/7</x:v>
+      </x:c>
+      <x:c r="I155" s="11" t="str">
+        <x:v>间隔3→2→1；剩余回合实时文字；0不表示点击即开火。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="90" customHeight="1">
+      <x:c r="A156" s="11" t="str">
+        <x:v>A-151</x:v>
+      </x:c>
+      <x:c r="B156" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C156" s="11" t="str">
+        <x:v>仕｜自动目标预览连线</x:v>
+      </x:c>
+      <x:c r="D156" s="11" t="str">
+        <x:v>候选目标/条件命中</x:v>
+      </x:c>
+      <x:c r="E156" s="11" t="str">
+        <x:v>当前局面的回合末预测</x:v>
+      </x:c>
+      <x:c r="F156" s="11" t="str">
+        <x:v>规则预览连线</x:v>
+      </x:c>
+      <x:c r="G156" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H156" s="11" t="str">
+        <x:v>US018 §7</x:v>
+      </x:c>
+      <x:c r="I156" s="11" t="str">
+        <x:v>与敌方锁定意图区分；玩家行动后可更新，树林结果为条件预览。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="90" customHeight="1">
+      <x:c r="A157" s="11" t="str">
+        <x:v>A-152</x:v>
+      </x:c>
+      <x:c r="B157" s="11" t="str">
+        <x:v>布阵UI</x:v>
+      </x:c>
+      <x:c r="C157" s="11" t="str">
+        <x:v>仕｜左右固定侧位与占用标记</x:v>
+      </x:c>
+      <x:c r="D157" s="11" t="str">
+        <x:v>左/右/空置/占用/冲突</x:v>
+      </x:c>
+      <x:c r="E157" s="11" t="str">
+        <x:v>仕布阵</x:v>
+      </x:c>
+      <x:c r="F157" s="11" t="str">
+        <x:v>侧位选择控件</x:v>
+      </x:c>
+      <x:c r="G157" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H157" s="11" t="str">
+        <x:v>US018；US020 R04</x:v>
+      </x:c>
+      <x:c r="I157" s="11" t="str">
+        <x:v>(4,2)/(6,2)；最多2座，不占部署人口且无装置后备；复用A-124。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="90" customHeight="1">
+      <x:c r="A158" s="11" t="str">
+        <x:v>A-153</x:v>
+      </x:c>
+      <x:c r="B158" s="11" t="str">
+        <x:v>技能UI</x:v>
+      </x:c>
+      <x:c r="C158" s="11" t="str">
+        <x:v>仕｜间隔升级图标与档位</x:v>
+      </x:c>
+      <x:c r="D158" s="11" t="str">
+        <x:v>3回合/2回合/1回合</x:v>
+      </x:c>
+      <x:c r="E158" s="11" t="str">
+        <x:v>营地/布阵/战斗技能栏</x:v>
+      </x:c>
+      <x:c r="F158" s="11" t="str">
+        <x:v>间隔升级按钮</x:v>
+      </x:c>
+      <x:c r="G158" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H158" s="11" t="str">
+        <x:v>US018 §5；US020</x:v>
+      </x:c>
+      <x:c r="I158" s="11" t="str">
+        <x:v>两座独立升级、共享SP，3/5SP；只升间隔，不暗示伤害或射程升级。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="90" customHeight="1">
+      <x:c r="A159" s="11" t="str">
+        <x:v>A-154</x:v>
+      </x:c>
+      <x:c r="B159" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C159" s="11" t="str">
+        <x:v>马｜起跳、越障与落地</x:v>
+      </x:c>
+      <x:c r="D159" s="11" t="str">
+        <x:v>起跳/空中/落地</x:v>
+      </x:c>
+      <x:c r="E159" s="11" t="str">
+        <x:v>主动跳跃攻击</x:v>
+      </x:c>
+      <x:c r="F159" s="11" t="str">
+        <x:v>棋位变化/标记占位</x:v>
+      </x:c>
+      <x:c r="G159" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H159" s="11" t="str">
+        <x:v>US021 §3</x:v>
+      </x:c>
+      <x:c r="I159" s="11" t="str">
+        <x:v>上下左右空格落点，基础2格、最高4格；不能把普通日字移动做成落地攻击。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="90" customHeight="1">
+      <x:c r="A160" s="11" t="str">
+        <x:v>A-155</x:v>
+      </x:c>
+      <x:c r="B160" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C160" s="11" t="str">
+        <x:v>马｜落点四邻冲击与友伤</x:v>
+      </x:c>
+      <x:c r="D160" s="11" t="str">
+        <x:v>1～3伤害档/边缘裁切</x:v>
+      </x:c>
+      <x:c r="E160" s="11" t="str">
+        <x:v>跳跃落地结算</x:v>
+      </x:c>
+      <x:c r="F160" s="11" t="str">
+        <x:v>规则及范围标记</x:v>
+      </x:c>
+      <x:c r="G160" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H160" s="11" t="str">
+        <x:v>US021 §3/5</x:v>
+      </x:c>
+      <x:c r="I160" s="11" t="str">
+        <x:v>只作用上下左右四邻；包含友军和山，非斜邻群伤；复用伤害数字、山体受击和树林闪避。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="90" customHeight="1">
+      <x:c r="A161" s="11" t="str">
+        <x:v>A-156</x:v>
+      </x:c>
+      <x:c r="B161" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C161" s="11" t="str">
+        <x:v>马｜推动与碰撞反馈</x:v>
+      </x:c>
+      <x:c r="D161" s="11" t="str">
+        <x:v>向外推/受阻/入水/尸体推动</x:v>
+      </x:c>
+      <x:c r="E161" s="11" t="str">
+        <x:v>解锁推动后的跳跃落地</x:v>
+      </x:c>
+      <x:c r="F161" s="11" t="str">
+        <x:v>规则位移占位</x:v>
+      </x:c>
+      <x:c r="G161" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H161" s="11" t="str">
+        <x:v>US021 §5</x:v>
+      </x:c>
+      <x:c r="I161" s="11" t="str">
+        <x:v>先四邻伤害再推动存活者与尸体；复用A-018/118及碰撞反馈，不另画四方向套图。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="90" customHeight="1">
+      <x:c r="A162" s="11" t="str">
+        <x:v>A-157</x:v>
+      </x:c>
+      <x:c r="B162" s="11" t="str">
+        <x:v>操作标记</x:v>
+      </x:c>
+      <x:c r="C162" s="11" t="str">
+        <x:v>马｜跳跃落点与四邻预览</x:v>
+      </x:c>
+      <x:c r="D162" s="11" t="str">
+        <x:v>合法落点/选中落点/伤害/推动/友伤</x:v>
+      </x:c>
+      <x:c r="E162" s="11" t="str">
+        <x:v>马技能预览</x:v>
+      </x:c>
+      <x:c r="F162" s="11" t="str">
+        <x:v>现有棋盘高亮</x:v>
+      </x:c>
+      <x:c r="G162" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H162" s="11" t="str">
+        <x:v>US021 H20</x:v>
+      </x:c>
+      <x:c r="I162" s="11" t="str">
+        <x:v>落点必须为空，落点不受伤；中心与四邻不同标记，明确友伤，边缘裁切。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="90" customHeight="1">
+      <x:c r="A163" s="11" t="str">
+        <x:v>A-158</x:v>
+      </x:c>
+      <x:c r="B163" s="11" t="str">
+        <x:v>技能UI</x:v>
+      </x:c>
+      <x:c r="C163" s="11" t="str">
+        <x:v>马｜三项独立升级图标</x:v>
+      </x:c>
+      <x:c r="D163" s="11" t="str">
+        <x:v>推动解除马腿/距离/伤害3款</x:v>
+      </x:c>
+      <x:c r="E163" s="11" t="str">
+        <x:v>营地、布阵和战斗技能区</x:v>
+      </x:c>
+      <x:c r="F163" s="11" t="str">
+        <x:v>升级按钮及档位</x:v>
+      </x:c>
+      <x:c r="G163" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H163" s="11" t="str">
+        <x:v>US021 §4</x:v>
+      </x:c>
+      <x:c r="I163" s="11" t="str">
+        <x:v>推动2SP一次；距离1SP/级至4格；伤害2SP/级至3；三项无相互前置，价格实时文字。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="90" customHeight="1">
+      <x:c r="A164" s="11" t="str">
+        <x:v>A-159</x:v>
+      </x:c>
+      <x:c r="B164" s="11" t="str">
+        <x:v>战斗UI</x:v>
+      </x:c>
+      <x:c r="C164" s="11" t="str">
+        <x:v>马｜双模式与独立行动额度</x:v>
+      </x:c>
+      <x:c r="D164" s="11" t="str">
+        <x:v>普通移动/跳跃攻击；可用/耗尽</x:v>
+      </x:c>
+      <x:c r="E164" s="11" t="str">
+        <x:v>马操作区、详情与名单</x:v>
+      </x:c>
+      <x:c r="F164" s="11" t="str">
+        <x:v>现有模式按钮</x:v>
+      </x:c>
+      <x:c r="G164" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H164" s="11" t="str">
+        <x:v>US021 §2/6</x:v>
+      </x:c>
+      <x:c r="I164" s="11" t="str">
+        <x:v>可移动后跳跃；跳跃后不能再移动。无旧普通攻击入口，升级不恢复行动；复用A-077。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="90" customHeight="1">
+      <x:c r="A165" s="11" t="str">
+        <x:v>A-160</x:v>
+      </x:c>
+      <x:c r="B165" s="11" t="str">
+        <x:v>通用UI</x:v>
+      </x:c>
+      <x:c r="C165" s="11" t="str">
+        <x:v>猫粮货币图标</x:v>
+      </x:c>
+      <x:c r="D165" s="11" t="str">
+        <x:v>普通/收入/支出/不足</x:v>
+      </x:c>
+      <x:c r="E165" s="11" t="str">
+        <x:v>营地、战斗、结算、教学</x:v>
+      </x:c>
+      <x:c r="F165" s="11" t="str">
+        <x:v>猫粮文字占位</x:v>
+      </x:c>
+      <x:c r="G165" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H165" s="11" t="str">
+        <x:v>US020 R03</x:v>
+      </x:c>
+      <x:c r="I165" s="11" t="str">
+        <x:v>替换金币图标，仍单钱包；数值与价格代码生成，不新增第二货币。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="90" customHeight="1">
+      <x:c r="A166" s="11" t="str">
+        <x:v>A-161</x:v>
+      </x:c>
+      <x:c r="B166" s="11" t="str">
+        <x:v>资源反馈</x:v>
+      </x:c>
+      <x:c r="C166" s="11" t="str">
+        <x:v>公共SP获得与消费反馈</x:v>
+      </x:c>
+      <x:c r="D166" s="11" t="str">
+        <x:v>获得/消费/不足/满级</x:v>
+      </x:c>
+      <x:c r="E166" s="11" t="str">
+        <x:v>击杀、营地及战斗升级</x:v>
+      </x:c>
+      <x:c r="F166" s="11" t="str">
+        <x:v>全队余额与提示</x:v>
+      </x:c>
+      <x:c r="G166" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H166" s="11" t="str">
+        <x:v>US017；US020；US021</x:v>
+      </x:c>
+      <x:c r="I166" s="11" t="str">
+        <x:v>指向唯一公共SP栏；个人等级/击杀仍独立，复用A-112和A-042。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="90" customHeight="1">
+      <x:c r="A167" s="11" t="str">
+        <x:v>A-162</x:v>
+      </x:c>
+      <x:c r="B167" s="11" t="str">
+        <x:v>己方技能效果</x:v>
+      </x:c>
+      <x:c r="C167" s="11" t="str">
+        <x:v>救援｜治疗与原位复活</x:v>
+      </x:c>
+      <x:c r="D167" s="11" t="str">
+        <x:v>伤员回满/尸体1HP复活</x:v>
+      </x:c>
+      <x:c r="E167" s="11" t="str">
+        <x:v>第二波开始前救援</x:v>
+      </x:c>
+      <x:c r="F167" s="11" t="str">
+        <x:v>HP与尸体状态变化</x:v>
+      </x:c>
+      <x:c r="G167" s="11" t="str">
+        <x:v>待制作</x:v>
+      </x:c>
+      <x:c r="H167" s="11" t="str">
+        <x:v>US020 R06</x:v>
+      </x:c>
+      <x:c r="I167" s="11" t="str">
+        <x:v>区别治疗和复活；复用A-125卡片，主帅/仕不适用，不表现异地传送。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4314,7 +5221,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6c06b4ef505437e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R467b196a737045b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4431,7 +5338,7 @@
     </x:row>
     <x:row r="7" ht="29" customHeight="1">
       <x:c r="A7" s="1" t="str">
-        <x:v>新增的Loading、菜单和三关地图为HTML/CSS/SVG占位，尚无正式插画或切图。资源预留清单已建立；独立地形实验和旧源图片保留。</x:v>
+        <x:v>2026-10-22：主流程、营地、教学及新增技能已有代码占位，尚未发现正式美术文件新增；本表“待制作”不等同功能未实现。旧目录图片仅作历史盘点。</x:v>
       </x:c>
       <x:c r="B7" s="1"/>
       <x:c r="C7" s="1"/>
@@ -4443,7 +5350,7 @@
     </x:row>
     <x:row r="8" ht="29" customHeight="1">
       <x:c r="A8" s="1" t="str">
-        <x:v>依据：web/js/app.js；web/index.html；docs/us/US-001-m0-player-skills.md。</x:v>
+        <x:v>需求依据：US013～US021，以US020营地/教学及US021马技能收口为准；代码静态核对web/index.html与web/assets。</x:v>
       </x:c>
       <x:c r="B8" s="1"/>
       <x:c r="C8" s="1"/>
@@ -4460,7 +5367,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35e0ce456f4f4c07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafbc18bfc2dc45bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4485,9 +5392,9 @@
         <x:v>UI 美术交付规格</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="25" customHeight="1">
+    <x:row r="2" ht="35" customHeight="1">
       <x:c r="A2" s="13" t="str">
-        <x:v>尺寸为建议制作像素。手机参考布局448×924，资源按3倍制作；桌面1920×1080并支持缩放。编号与主清单一一对应，组件总项和子资源不能简单相加为图片数。最终风格、历史疆界、动画和功能接入待确认。</x:v>
+        <x:v>2026-10-22更新。沿用桌面1920×1080、Mate40Pro竖版448×924逻辑/1344×2772制作参考。新图标96×96仅建议。手机横版844×390棋盘仍有既有问题，布局与最终切图TBD。总项与子资源复用；文字和数值由程序生成。</x:v>
       </x:c>
       <x:c r="B2" s="13"/>
       <x:c r="C2" s="13"/>
@@ -4498,7 +5405,7 @@
       <x:c r="H2" s="13"/>
       <x:c r="I2" s="13"/>
     </x:row>
-    <x:row r="3" ht="25" customHeight="1">
+    <x:row r="3" ht="35" customHeight="1">
       <x:c r="A3" s="13"/>
       <x:c r="B3" s="13"/>
       <x:c r="C3" s="13"/>
@@ -4567,7 +5474,7 @@
         <x:v>组件总项；面板切图复用A-109起通用资源，桌面1920×1080、手机1344×2772</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="76" customHeight="1">
+    <x:row r="7" ht="98" customHeight="1">
       <x:c r="A7" s="16" t="str">
         <x:v>A-073</x:v>
       </x:c>
@@ -4584,16 +5491,16 @@
         <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
       </x:c>
       <x:c r="F7" s="16" t="str">
-        <x:v>详见用途与主清单</x:v>
+        <x:v>代码占位／美术待制作</x:v>
       </x:c>
       <x:c r="G7" s="16" t="str">
-        <x:v>波次、回合、主帅HP、金币、击杀</x:v>
+        <x:v>波次、回合、双方主帅HP、猫粮、公共SP、击杀、旅程增益</x:v>
       </x:c>
       <x:c r="H7" s="16" t="str">
-        <x:v>桌面／手机2套</x:v>
+        <x:v>桌面/手机</x:v>
       </x:c>
       <x:c r="I7" s="16" t="str">
-        <x:v>桌面左上；手机仅保留紧凑主要数值，完整状态折叠</x:v>
+        <x:v>猫粮替代金币，SP为全队余额；增益允许多项同时生效。 来源：US017；US020</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="76" customHeight="1">
@@ -4625,7 +5532,7 @@
         <x:v>徽记复用棋子；默认/选中/行动耗尽；未实现棋种仍仅预留</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="76" customHeight="1">
+    <x:row r="9" ht="98" customHeight="1">
       <x:c r="A9" s="16" t="str">
         <x:v>A-075</x:v>
       </x:c>
@@ -4642,19 +5549,19 @@
         <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
       </x:c>
       <x:c r="F9" s="16" t="str">
-        <x:v>详见用途与主清单</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="G9" s="16" t="str">
-        <x:v>属性、行动余量、等级、SP</x:v>
+        <x:v>属性、行动余量、个人等级/击杀、公共SP消费资格</x:v>
       </x:c>
       <x:c r="H9" s="16" t="str">
         <x:v>桌面详情／手机摘要</x:v>
       </x:c>
       <x:c r="I9" s="16" t="str">
-        <x:v>长说明可展开，动态数值不烘焙</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="76" customHeight="1">
+        <x:v>不显示个人SP钱包；帅无升级，仕有冷却，马区分普通移动与跳跃攻击。 来源：US017；US018；US019；US021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="98" customHeight="1">
       <x:c r="A10" s="19" t="str">
         <x:v>A-076</x:v>
       </x:c>
@@ -4671,24 +5578,24 @@
         <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
       </x:c>
       <x:c r="F10" s="19" t="str">
-        <x:v>详见用途与主清单</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="G10" s="19" t="str">
-        <x:v>升级、转职、方向和炮扩散</x:v>
+        <x:v>公共SP升级、转职、方向强化、炮扩散、仕间隔及马三项强化</x:v>
       </x:c>
       <x:c r="H10" s="19" t="str">
         <x:v>1套＋图标槽位</x:v>
       </x:c>
       <x:c r="I10" s="19" t="str">
-        <x:v>可购买/已解锁/缺SP/当前阶段不可购买；专属技能仍为己方</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="76" customHeight="1">
+        <x:v>技能资格按棋种；马推动2SP、距离每次1SP、伤害每次2SP独立购买，主帅无个人升级。 来源：US017～021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="98" customHeight="1">
       <x:c r="A11" s="16" t="str">
         <x:v>A-077</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>方向与车模式按钮</x:v>
+        <x:v>方向及车/马操作模式按钮</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
         <x:v>现有组件总项；复用通用资源</x:v>
@@ -4700,16 +5607,16 @@
         <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
       </x:c>
       <x:c r="F11" s="16" t="str">
-        <x:v>详见用途与主清单</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="G11" s="16" t="str">
-        <x:v>弓枪方向；车职业模式</x:v>
+        <x:v>弓枪方向、车操作、马普通移动/跳跃攻击</x:v>
       </x:c>
       <x:c r="H11" s="16" t="str">
-        <x:v>四方向＋移动/冲锋/牵引</x:v>
+        <x:v>四方向＋车模式＋马双模式</x:v>
       </x:c>
       <x:c r="I11" s="16" t="str">
-        <x:v>默认/选中/禁用；手机触控面积至少44逻辑像素</x:v>
+        <x:v>马仅普通移动和跳跃攻击两个入口，不保留旧普通攻击；手机横版改造待另行授权。 来源：US021</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="76" customHeight="1">
@@ -4741,7 +5648,7 @@
         <x:v>成功/失效/落空/已移除/待机需区分</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="76" customHeight="1">
+    <x:row r="13" ht="98" customHeight="1">
       <x:c r="A13" s="16" t="str">
         <x:v>A-079</x:v>
       </x:c>
@@ -4758,16 +5665,16 @@
         <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
       </x:c>
       <x:c r="F13" s="16" t="str">
-        <x:v>详见用途与主清单</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="G13" s="16" t="str">
-        <x:v>路径、伤害、友伤、主帅威胁</x:v>
+        <x:v>路径、伤害、友伤、主帅威胁、仕自动攻击及马落点四邻</x:v>
       </x:c>
       <x:c r="H13" s="16" t="str">
         <x:v>桌面详情／手机摘要</x:v>
       </x:c>
       <x:c r="I13" s="16" t="str">
-        <x:v>友伤醒目；桌面点目标直接攻击，手机保留执行确认</x:v>
+        <x:v>友伤、推动/碰撞与树林条件结果可辨；桌面点目标直接攻击，手机保留执行确认。 来源：US018；US019；US021</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="76" customHeight="1">
@@ -4857,12 +5764,12 @@
         <x:v>复用面板、遮罩、主次按钮</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="76" customHeight="1">
+    <x:row r="17" ht="98" customHeight="1">
       <x:c r="A17" s="16" t="str">
         <x:v>A-083</x:v>
       </x:c>
       <x:c r="B17" s="16" t="str">
-        <x:v>商店与商品卡</x:v>
+        <x:v>主营地与招募商品卡（原关间商店）</x:v>
       </x:c>
       <x:c r="C17" s="16" t="str">
         <x:v>现有组件总项；复用通用资源</x:v>
@@ -4874,19 +5781,19 @@
         <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
       </x:c>
       <x:c r="F17" s="16" t="str">
-        <x:v>详见用途与主清单</x:v>
+        <x:v>功能已接入／美术待制作</x:v>
       </x:c>
       <x:c r="G17" s="16" t="str">
-        <x:v>关间整备与上阵后备</x:v>
+        <x:v>首次教学后及非最终关胜利后整备</x:v>
       </x:c>
       <x:c r="H17" s="16" t="str">
-        <x:v>兵/车/马/炮4类</x:v>
+        <x:v>兵/车/马/炮/仕</x:v>
       </x:c>
       <x:c r="I17" s="16" t="str">
-        <x:v>商品像复用棋子；价格、阵容容量实时文字</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="76" customHeight="1">
+        <x:v>总项复用商品皮肤；猫粮价格、部署上限、队友总数和后备数实时显示，主帅与仕单列。 来源：US020；US018</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="98" customHeight="1">
       <x:c r="A18" s="19" t="str">
         <x:v>A-084</x:v>
       </x:c>
@@ -4903,16 +5810,16 @@
         <x:v>容器PNG九宫格/图标SVG；文字由代码</x:v>
       </x:c>
       <x:c r="F18" s="19" t="str">
-        <x:v>详见用途与主清单</x:v>
+        <x:v>代码占位</x:v>
       </x:c>
       <x:c r="G18" s="19" t="str">
         <x:v>战斗结果</x:v>
       </x:c>
       <x:c r="H18" s="19" t="str">
-        <x:v>胜利/阵亡/将死3态</x:v>
+        <x:v>胜利/主帅阵亡失败/三关通关</x:v>
       </x:c>
       <x:c r="I18" s="19" t="str">
-        <x:v>独立结果标题装饰详见新增条目；统计数字实时文字</x:v>
+        <x:v>不以搜索将死作为现行失败条件；教学结果另列A-143。 来源：US019；US020</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="76" customHeight="1">
@@ -5176,7 +6083,7 @@
         <x:v>文字与按钮独立，不烘焙</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="76" customHeight="1">
+    <x:row r="28" ht="98" customHeight="1">
       <x:c r="A28" s="19" t="str">
         <x:v>A-095</x:v>
       </x:c>
@@ -5193,7 +6100,7 @@
         <x:v>PNG，透明，九宫格</x:v>
       </x:c>
       <x:c r="F28" s="19" t="str">
-        <x:v>默认/悬停/按下/禁用</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G28" s="19" t="str">
         <x:v>开始游戏/继续游戏</x:v>
@@ -5202,7 +6109,7 @@
         <x:v>4态</x:v>
       </x:c>
       <x:c r="I28" s="19" t="str">
-        <x:v>两个功能共用按钮皮肤，继续游戏规则 TBD</x:v>
+        <x:v>已有本地旅程时可继续；重开旅程需确认，实时显示存档状态，不把按钮可用态烘焙。 来源：US020 R09</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="76" customHeight="1">
@@ -5263,7 +6170,7 @@
         <x:v>可用棋子/兵旗/印章；不遮挡按钮</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="76" customHeight="1">
+    <x:row r="31" ht="98" customHeight="1">
       <x:c r="A31" s="16" t="str">
         <x:v>A-098</x:v>
       </x:c>
@@ -5280,19 +6187,19 @@
         <x:v>WebP/PNG；另交分层源文件</x:v>
       </x:c>
       <x:c r="F31" s="16" t="str">
-        <x:v>无选中态底图</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G31" s="16" t="str">
-        <x:v>开始游戏后的选关页</x:v>
+        <x:v>主营地出发后的选关地图</x:v>
       </x:c>
       <x:c r="H31" s="16" t="str">
         <x:v>横竖2版</x:v>
       </x:c>
       <x:c r="I31" s="16" t="str">
-        <x:v>三分区为玩法草案；历史边界和时代年份 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="76" customHeight="1">
+        <x:v>1→2→3顺序解锁；三关都可预览。演武场独立地图地区仍属US016 WIP。 来源：US020 R02/R08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="98" customHeight="1">
       <x:c r="A32" s="19" t="str">
         <x:v>A-099</x:v>
       </x:c>
@@ -5309,7 +6216,7 @@
         <x:v>SVG/PNG，透明</x:v>
       </x:c>
       <x:c r="F32" s="19" t="str">
-        <x:v>默认/悬停/选中</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G32" s="19" t="str">
         <x:v>西部关卡区域</x:v>
@@ -5318,10 +6225,10 @@
         <x:v>3态</x:v>
       </x:c>
       <x:c r="I32" s="19" t="str">
-        <x:v>西部关中主题；山隘/城塞视觉；区域范围与关名 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="76" customHeight="1">
+        <x:v>关名已用于当前原型；美术边界、精确历史年代TBD，不据此复原真实疆界。 来源：US012；US020 R08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="98" customHeight="1">
       <x:c r="A33" s="16" t="str">
         <x:v>A-100</x:v>
       </x:c>
@@ -5338,7 +6245,7 @@
         <x:v>SVG/PNG，透明</x:v>
       </x:c>
       <x:c r="F33" s="16" t="str">
-        <x:v>默认/悬停/选中</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G33" s="16" t="str">
         <x:v>中央关卡区域</x:v>
@@ -5347,10 +6254,10 @@
         <x:v>3态</x:v>
       </x:c>
       <x:c r="I33" s="16" t="str">
-        <x:v>中央平原主题；河流/城邑视觉；区域范围与关名 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="76" customHeight="1">
+        <x:v>关名已用于当前原型；美术边界、精确历史年代TBD，不据此复原真实疆界。 来源：US012；US020 R08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="98" customHeight="1">
       <x:c r="A34" s="19" t="str">
         <x:v>A-101</x:v>
       </x:c>
@@ -5367,7 +6274,7 @@
         <x:v>SVG/PNG，透明</x:v>
       </x:c>
       <x:c r="F34" s="19" t="str">
-        <x:v>默认/悬停/选中</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G34" s="19" t="str">
         <x:v>东南关卡区域</x:v>
@@ -5376,7 +6283,7 @@
         <x:v>3态</x:v>
       </x:c>
       <x:c r="I34" s="19" t="str">
-        <x:v>东南水网主题；水泽/林地视觉；区域范围与关名 TBD</x:v>
+        <x:v>关名已用于当前原型；美术边界、精确历史年代TBD，不据此复原真实疆界。 来源：US012；US020 R08</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="76" customHeight="1">
@@ -5408,7 +6315,7 @@
         <x:v>三个区域共边不得出现缝隙；非真实国界</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="76" customHeight="1">
+    <x:row r="36" ht="98" customHeight="1">
       <x:c r="A36" s="19" t="str">
         <x:v>A-103</x:v>
       </x:c>
@@ -5425,7 +6332,7 @@
         <x:v>SVG/PNG，透明</x:v>
       </x:c>
       <x:c r="F36" s="19" t="str">
-        <x:v>未解锁/可挑战/当前选择/已通关</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G36" s="19" t="str">
         <x:v>三个关卡入口</x:v>
@@ -5434,10 +6341,10 @@
         <x:v>3编号×4态</x:v>
       </x:c>
       <x:c r="I36" s="19" t="str">
-        <x:v>美术预留4态；解锁条件 TBD</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="76" customHeight="1">
+        <x:v>锁定/可挑战/选中/通关；锁定与已通关可预览，但不可跳关或重打。 来源：US020 R08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="98" customHeight="1">
       <x:c r="A37" s="16" t="str">
         <x:v>A-104</x:v>
       </x:c>
@@ -5454,7 +6361,7 @@
         <x:v>SVG，透明</x:v>
       </x:c>
       <x:c r="F37" s="16" t="str">
-        <x:v>未推进/已推进</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G37" s="16" t="str">
         <x:v>1→2→3区域连接</x:v>
@@ -5463,7 +6370,7 @@
         <x:v>1套</x:v>
       </x:c>
       <x:c r="I37" s="16" t="str">
-        <x:v>路线仅为叙事顺序草案，不代表已实现进度</x:v>
+        <x:v>正式顺序1→2→3已确认；路线不表示任意分支或可重打。 来源：US012；US020 R08</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="76" customHeight="1">
@@ -5524,7 +6431,7 @@
         <x:v>依次山隘、平原城邑、水网；最终题材 TBD</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="76" customHeight="1">
+    <x:row r="40" ht="98" customHeight="1">
       <x:c r="A40" s="19" t="str">
         <x:v>A-107</x:v>
       </x:c>
@@ -5541,16 +6448,16 @@
         <x:v>PNG，透明，九宫格</x:v>
       </x:c>
       <x:c r="F40" s="19" t="str">
-        <x:v>默认</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G40" s="19" t="str">
-        <x:v>关卡说明与进入按钮</x:v>
+        <x:v>关卡说明、地形/首波预览与进入按钮</x:v>
       </x:c>
       <x:c r="H40" s="19" t="str">
         <x:v>1套</x:v>
       </x:c>
       <x:c r="I40" s="19" t="str">
-        <x:v>标题、难度、奖励用文字；玩法参数 TBD</x:v>
+        <x:v>底板复用；第二波位置不提前显示；战术缩略图由程序生成，见A-139。 来源：US020 R08</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="76" customHeight="1">
@@ -5640,7 +6547,7 @@
         <x:v>结束回合、撤销、暂停、取消、确认共用</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="76" customHeight="1">
+    <x:row r="44" ht="98" customHeight="1">
       <x:c r="A44" s="19" t="str">
         <x:v>A-111</x:v>
       </x:c>
@@ -5657,19 +6564,19 @@
         <x:v>SVG/PNG，透明</x:v>
       </x:c>
       <x:c r="F44" s="19" t="str">
-        <x:v>默认/禁用/选中按需</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G44" s="19" t="str">
-        <x:v>返回/关闭/设置/暂停/继续/重试/收起/展开</x:v>
+        <x:v>返回/关闭/设置/暂停/继续/重试/收起/展开/帮助/保存</x:v>
       </x:c>
       <x:c r="H44" s="19" t="str">
         <x:v>8款</x:v>
       </x:c>
       <x:c r="I44" s="19" t="str">
-        <x:v>点击区域由程序保持至少44逻辑像素</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="76" customHeight="1">
+        <x:v>复用通用图标；44逻辑像素为点击热区，不要求图标本身44像素。 来源：US015；US020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="98" customHeight="1">
       <x:c r="A45" s="16" t="str">
         <x:v>A-112</x:v>
       </x:c>
@@ -5686,16 +6593,16 @@
         <x:v>SVG/PNG，透明</x:v>
       </x:c>
       <x:c r="F45" s="16" t="str">
-        <x:v>常态</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G45" s="16" t="str">
-        <x:v>HP/AP/SP/金币/回合/击杀/等级</x:v>
+        <x:v>全部资源与属性栏</x:v>
       </x:c>
       <x:c r="H45" s="16" t="str">
-        <x:v>7款</x:v>
+        <x:v>HP/AP/公共SP/猫粮/回合/击杀/等级/部署上限</x:v>
       </x:c>
       <x:c r="I45" s="16" t="str">
-        <x:v>保留数值文字，避免仅靠图标猜测</x:v>
+        <x:v>金币图标退役并替换猫粮A-160；公共SP仅一份钱包。实时数值不切图。 来源：US017；US020</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="76" customHeight="1">
@@ -5901,12 +6808,12 @@
         <x:v>只表达规则已揭示的信息</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="76" customHeight="1">
+    <x:row r="53" ht="98" customHeight="1">
       <x:c r="A53" s="16" t="str">
         <x:v>A-120</x:v>
       </x:c>
       <x:c r="B53" s="16" t="str">
-        <x:v>主帅增益选择卡</x:v>
+        <x:v>主帅旅程增益卡（替代三选一）</x:v>
       </x:c>
       <x:c r="C53" s="16" t="str">
         <x:v>commander-card</x:v>
@@ -5918,19 +6825,19 @@
         <x:v>PNG/WebP，透明插画</x:v>
       </x:c>
       <x:c r="F53" s="16" t="str">
-        <x:v>默认/悬停/选中</x:v>
+        <x:v>功能已接入／美术待制作</x:v>
       </x:c>
       <x:c r="G53" s="16" t="str">
-        <x:v>坚守/疾行/救援</x:v>
+        <x:v>主营地顺序解锁、战斗摘要</x:v>
       </x:c>
       <x:c r="H53" s="16" t="str">
-        <x:v>3款</x:v>
+        <x:v>坚守/疾行/救援3款及状态</x:v>
       </x:c>
       <x:c r="I53" s="16" t="str">
-        <x:v>不烘焙技能描述和数值</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="76" customHeight="1">
+        <x:v>首次入营免费坚守；疾行5猫粮、救援5猫粮，依次解锁、同时生效、跨关保留；不再制作互斥三选一。 来源：US020 R05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="98" customHeight="1">
       <x:c r="A54" s="19" t="str">
         <x:v>A-121</x:v>
       </x:c>
@@ -5947,16 +6854,16 @@
         <x:v>SVG/PNG，透明</x:v>
       </x:c>
       <x:c r="F54" s="19" t="str">
-        <x:v>可购买/已解锁/不可购买</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G54" s="19" t="str">
-        <x:v>升级/转职/方向/扩散</x:v>
+        <x:v>普通队友技能/转职/方向/扩散；仕间隔；马推动/距离/伤害</x:v>
       </x:c>
       <x:c r="H54" s="19" t="str">
         <x:v>通用1套＋己方9棋种槽位</x:v>
       </x:c>
       <x:c r="I54" s="19" t="str">
-        <x:v>与A-042至A-065技能特效分开；敌方不新增主动技能</x:v>
+        <x:v>主帅无个人技能升级图标；与技能效果区分；敌方不新增主动技能。 来源：US017～021</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="76" customHeight="1">
@@ -6017,7 +6924,7 @@
         <x:v>列棋名及坐标；预留未行动徽记96×96</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="76" customHeight="1">
+    <x:row r="57" ht="98" customHeight="1">
       <x:c r="A57" s="16" t="str">
         <x:v>A-124</x:v>
       </x:c>
@@ -6034,24 +6941,24 @@
         <x:v>SVG/PNG，透明</x:v>
       </x:c>
       <x:c r="F57" s="16" t="str">
-        <x:v>已上阵/后备/选中/不可放置</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G57" s="16" t="str">
-        <x:v>布阵/商店队伍管理</x:v>
+        <x:v>主营地、布阵的上阵/后备及独立主帅/仕列表</x:v>
       </x:c>
       <x:c r="H57" s="16" t="str">
         <x:v>1套</x:v>
       </x:c>
       <x:c r="I57" s="16" t="str">
-        <x:v>头像复用己方棋子资源</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58" ht="76" customHeight="1">
+        <x:v>普通队友总数不限；部署人口初始4上限8。主帅和仕不占人口，仕无后备；共用棋子像。 来源：US020 R04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="98" customHeight="1">
       <x:c r="A58" s="19" t="str">
         <x:v>A-125</x:v>
       </x:c>
       <x:c r="B58" s="19" t="str">
-        <x:v>救援角色卡与恢复标记</x:v>
+        <x:v>救援选择卡与恢复/复活标记</x:v>
       </x:c>
       <x:c r="C58" s="19" t="str">
         <x:v>rescue-card</x:v>
@@ -6063,24 +6970,24 @@
         <x:v>SVG/PNG，透明</x:v>
       </x:c>
       <x:c r="F58" s="19" t="str">
-        <x:v>回血/复活/不可选</x:v>
+        <x:v>功能已接入／美术待制作</x:v>
       </x:c>
       <x:c r="G58" s="19" t="str">
-        <x:v>第6回合救援</x:v>
+        <x:v>已解锁救援后的第二波开始前</x:v>
       </x:c>
       <x:c r="H58" s="19" t="str">
-        <x:v>1套</x:v>
+        <x:v>受伤恢复/尸体复活/跳过</x:v>
       </x:c>
       <x:c r="I58" s="19" t="str">
-        <x:v>人物形象复用棋子；恢复表现关联技能通用效果</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="76" customHeight="1">
+        <x:v>受伤普通队友回满血；有效尸体原位1HP复活；排除主帅、仕、已毁尸体、满血及后备。效果见A-162。 来源：US020 R06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="98" customHeight="1">
       <x:c r="A59" s="16" t="str">
         <x:v>A-126</x:v>
       </x:c>
       <x:c r="B59" s="16" t="str">
-        <x:v>商店商品与价格标签</x:v>
+        <x:v>营地招募商品与猫粮价格标签</x:v>
       </x:c>
       <x:c r="C59" s="16" t="str">
         <x:v>shop-card</x:v>
@@ -6092,16 +6999,16 @@
         <x:v>SVG/PNG，透明</x:v>
       </x:c>
       <x:c r="F59" s="16" t="str">
-        <x:v>可购买/金币不足/容量受限</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G59" s="16" t="str">
-        <x:v>关间整备</x:v>
+        <x:v>主营地招募</x:v>
       </x:c>
       <x:c r="H59" s="16" t="str">
-        <x:v>兵/车/马/炮4类</x:v>
+        <x:v>普通队友及仕商品</x:v>
       </x:c>
       <x:c r="I59" s="16" t="str">
-        <x:v>棋子像复用，价格由程序写入</x:v>
+        <x:v>不足仅禁用且保留价格，不显示差额；部署满员仍可招募至后备，仕最多两座。 来源：US020 R03/R04</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="76" customHeight="1">
@@ -6133,7 +7040,7 @@
         <x:v>统计数字和操作按钮独立</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="76" customHeight="1">
+    <x:row r="61" ht="98" customHeight="1">
       <x:c r="A61" s="16" t="str">
         <x:v>A-128</x:v>
       </x:c>
@@ -6150,7 +7057,7 @@
         <x:v>SVG/PNG，透明</x:v>
       </x:c>
       <x:c r="F61" s="16" t="str">
-        <x:v>默认/选中/提示</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G61" s="16" t="str">
         <x:v>队伍/技能/敌情/更多</x:v>
@@ -6159,10 +7066,10 @@
         <x:v>4款</x:v>
       </x:c>
       <x:c r="I61" s="16" t="str">
-        <x:v>448×924逻辑视口，3倍参考导出；保持一屏</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="76" customHeight="1">
+        <x:v>448×924逻辑视口，3倍参考导出；保持一屏；手机横版844×390存在棋盘不可辨问题，最终布局/切图规格TBD，不标全端通过。 来源：US015；US020；US021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="98" customHeight="1">
       <x:c r="A62" s="19" t="str">
         <x:v>A-129</x:v>
       </x:c>
@@ -6179,7 +7086,7 @@
         <x:v>PNG九宫格或CSS</x:v>
       </x:c>
       <x:c r="F62" s="19" t="str">
-        <x:v>展开/收起</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G62" s="19" t="str">
         <x:v>完整详情、敌情、战况记录</x:v>
@@ -6188,10 +7095,10 @@
         <x:v>1套</x:v>
       </x:c>
       <x:c r="I62" s="19" t="str">
-        <x:v>内容可内部滚动，主战斗页不滚动</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="76" customHeight="1">
+        <x:v>内容可内部滚动，主战斗页不滚动；手机横版844×390存在棋盘不可辨问题，最终布局/切图规格TBD，不标全端通过。 来源：US015；US020；US021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="98" customHeight="1">
       <x:c r="A63" s="16" t="str">
         <x:v>A-130</x:v>
       </x:c>
@@ -6208,7 +7115,7 @@
         <x:v>PNG九宫格或CSS</x:v>
       </x:c>
       <x:c r="F63" s="16" t="str">
-        <x:v>常态/警告/无选择</x:v>
+        <x:v>预留／待制作</x:v>
       </x:c>
       <x:c r="G63" s="16" t="str">
         <x:v>棋盘下方摘要</x:v>
@@ -6217,7 +7124,7 @@
         <x:v>2套</x:v>
       </x:c>
       <x:c r="I63" s="16" t="str">
-        <x:v>与桌面信息同源，文本不烘焙</x:v>
+        <x:v>与桌面信息同源，文本不烘焙；手机横版844×390存在棋盘不可辨问题，最终布局/切图规格TBD，不标全端通过。 来源：US015；US020；US021</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="76" customHeight="1">
@@ -6247,6 +7154,905 @@
       </x:c>
       <x:c r="I64" s="19" t="str">
         <x:v>字体授权 TBD；资源尺寸为制作建议，最终风格待确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="98" customHeight="1">
+      <x:c r="A65" s="16" t="str">
+        <x:v>A-132</x:v>
+      </x:c>
+      <x:c r="B65" s="16" t="str">
+        <x:v>主营地背景</x:v>
+      </x:c>
+      <x:c r="C65" s="16" t="str">
+        <x:v>主营地全屏</x:v>
+      </x:c>
+      <x:c r="D65" s="16" t="str">
+        <x:v>桌面1920×1080；手机构图TBD</x:v>
+      </x:c>
+      <x:c r="E65" s="16" t="str">
+        <x:v>背景PNG/WebP</x:v>
+      </x:c>
+      <x:c r="F65" s="16" t="str">
+        <x:v>桌面/手机构图</x:v>
+      </x:c>
+      <x:c r="G65" s="16" t="str">
+        <x:v>主营地全屏</x:v>
+      </x:c>
+      <x:c r="H65" s="16" t="str">
+        <x:v>桌面/手机构图</x:v>
+      </x:c>
+      <x:c r="I65" s="16" t="str">
+        <x:v>待制作。营地氛围插画可复用菜单元素；视觉风格TBD。 来源：US020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="98" customHeight="1">
+      <x:c r="A66" s="19" t="str">
+        <x:v>A-133</x:v>
+      </x:c>
+      <x:c r="B66" s="19" t="str">
+        <x:v>营地功能分区底板</x:v>
+      </x:c>
+      <x:c r="C66" s="19" t="str">
+        <x:v>主营地布局</x:v>
+      </x:c>
+      <x:c r="D66" s="19" t="str">
+        <x:v>自适应；九宫格基准TBD</x:v>
+      </x:c>
+      <x:c r="E66" s="19" t="str">
+        <x:v>面板九宫格PNG/SVG</x:v>
+      </x:c>
+      <x:c r="F66" s="19" t="str">
+        <x:v>资源/名单/招募/成长/技能5区</x:v>
+      </x:c>
+      <x:c r="G66" s="19" t="str">
+        <x:v>主营地布局</x:v>
+      </x:c>
+      <x:c r="H66" s="19" t="str">
+        <x:v>资源/名单/招募/成长/技能5区</x:v>
+      </x:c>
+      <x:c r="I66" s="19" t="str">
+        <x:v>复用／待制作。复用A-109/110；分区标题为动态文字，不制作五套重复底板。 来源：US020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="98" customHeight="1">
+      <x:c r="A67" s="16" t="str">
+        <x:v>A-134</x:v>
+      </x:c>
+      <x:c r="B67" s="16" t="str">
+        <x:v>队友总数与部署上限组件</x:v>
+      </x:c>
+      <x:c r="C67" s="16" t="str">
+        <x:v>营地和布阵</x:v>
+      </x:c>
+      <x:c r="D67" s="16" t="str">
+        <x:v>图标96×96建议；组件自适应</x:v>
+      </x:c>
+      <x:c r="E67" s="16" t="str">
+        <x:v>SVG图标＋实时文字</x:v>
+      </x:c>
+      <x:c r="F67" s="16" t="str">
+        <x:v>总数/后备数/部署数/扩编状态</x:v>
+      </x:c>
+      <x:c r="G67" s="16" t="str">
+        <x:v>营地和布阵</x:v>
+      </x:c>
+      <x:c r="H67" s="16" t="str">
+        <x:v>总数/后备数/部署数/扩编状态</x:v>
+      </x:c>
+      <x:c r="I67" s="16" t="str">
+        <x:v>待制作。库存不限、部署4→8；主帅与仕单列；价格和人数不烘焙。 来源：US020 R04（2026-10-21）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="98" customHeight="1">
+      <x:c r="A68" s="19" t="str">
+        <x:v>A-135</x:v>
+      </x:c>
+      <x:c r="B68" s="19" t="str">
+        <x:v>旅程增益解锁顺序与状态连接</x:v>
+      </x:c>
+      <x:c r="C68" s="19" t="str">
+        <x:v>主营地增益区</x:v>
+      </x:c>
+      <x:c r="D68" s="19" t="str">
+        <x:v>图标96×96建议；连接线自适应</x:v>
+      </x:c>
+      <x:c r="E68" s="19" t="str">
+        <x:v>SVG/CSS</x:v>
+      </x:c>
+      <x:c r="F68" s="19" t="str">
+        <x:v>锁定/可购买/已解锁</x:v>
+      </x:c>
+      <x:c r="G68" s="19" t="str">
+        <x:v>主营地增益区</x:v>
+      </x:c>
+      <x:c r="H68" s="19" t="str">
+        <x:v>锁定/可购买/已解锁</x:v>
+      </x:c>
+      <x:c r="I68" s="19" t="str">
+        <x:v>待制作。坚守→疾行→救援；复用A-120三图标，增加前置关系及同时生效状态。 来源：US020 R05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="98" customHeight="1">
+      <x:c r="A69" s="16" t="str">
+        <x:v>A-136</x:v>
+      </x:c>
+      <x:c r="B69" s="16" t="str">
+        <x:v>主营地首次指引与帮助卡</x:v>
+      </x:c>
+      <x:c r="C69" s="16" t="str">
+        <x:v>首次入营与帮助</x:v>
+      </x:c>
+      <x:c r="D69" s="16" t="str">
+        <x:v>双端自适应；内部可滚动</x:v>
+      </x:c>
+      <x:c r="E69" s="16" t="str">
+        <x:v>通用面板＋代码文字</x:v>
+      </x:c>
+      <x:c r="F69" s="16" t="str">
+        <x:v>首次/跳过/帮助重看</x:v>
+      </x:c>
+      <x:c r="G69" s="16" t="str">
+        <x:v>首次入营与帮助</x:v>
+      </x:c>
+      <x:c r="H69" s="16" t="str">
+        <x:v>首次/跳过/帮助重看</x:v>
+      </x:c>
+      <x:c r="I69" s="16" t="str">
+        <x:v>待制作。解释猫粮、库存/部署、招募、公共SP及增益顺序；复用通用弹窗，无新引导角色。 来源：US020 R10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="98" customHeight="1">
+      <x:c r="A70" s="19" t="str">
+        <x:v>A-137</x:v>
+      </x:c>
+      <x:c r="B70" s="19" t="str">
+        <x:v>回营恢复反馈</x:v>
+      </x:c>
+      <x:c r="C70" s="19" t="str">
+        <x:v>非最终关胜利回营</x:v>
+      </x:c>
+      <x:c r="D70" s="19" t="str">
+        <x:v>特效原点/时长TBD</x:v>
+      </x:c>
+      <x:c r="E70" s="19" t="str">
+        <x:v>透明序列或代码动画</x:v>
+      </x:c>
+      <x:c r="F70" s="19" t="str">
+        <x:v>伤员恢复/普通队友与仕恢复</x:v>
+      </x:c>
+      <x:c r="G70" s="19" t="str">
+        <x:v>非最终关胜利回营</x:v>
+      </x:c>
+      <x:c r="H70" s="19" t="str">
+        <x:v>伤员恢复/普通队友与仕恢复</x:v>
+      </x:c>
+      <x:c r="I70" s="19" t="str">
+        <x:v>待制作。复用治疗/复活主体，回营恢复不误表现为关内治疗仕。 来源：US020 R07</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="98" customHeight="1">
+      <x:c r="A71" s="16" t="str">
+        <x:v>A-138</x:v>
+      </x:c>
+      <x:c r="B71" s="16" t="str">
+        <x:v>本地保存与保存失败反馈</x:v>
+      </x:c>
+      <x:c r="C71" s="16" t="str">
+        <x:v>营地消费、继续旅程和存储异常</x:v>
+      </x:c>
+      <x:c r="D71" s="16" t="str">
+        <x:v>图标96×96建议</x:v>
+      </x:c>
+      <x:c r="E71" s="16" t="str">
+        <x:v>SVG图标＋实时文字</x:v>
+      </x:c>
+      <x:c r="F71" s="16" t="str">
+        <x:v>已保存/失败/本次会话</x:v>
+      </x:c>
+      <x:c r="G71" s="16" t="str">
+        <x:v>营地消费、继续旅程和存储异常</x:v>
+      </x:c>
+      <x:c r="H71" s="16" t="str">
+        <x:v>已保存/失败/本次会话</x:v>
+      </x:c>
+      <x:c r="I71" s="16" t="str">
+        <x:v>待制作。复用A-085/111，保存失败不能显示成功；不承诺云同步。 来源：US020 R09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="98" customHeight="1">
+      <x:c r="A72" s="19" t="str">
+        <x:v>A-139</x:v>
+      </x:c>
+      <x:c r="B72" s="19" t="str">
+        <x:v>关卡战术缩略图及棋种图例</x:v>
+      </x:c>
+      <x:c r="C72" s="19" t="str">
+        <x:v>三关选关详情</x:v>
+      </x:c>
+      <x:c r="D72" s="19" t="str">
+        <x:v>自适应；图例96×96建议</x:v>
+      </x:c>
+      <x:c r="E72" s="19" t="str">
+        <x:v>代码绘制＋复用棋子地形</x:v>
+      </x:c>
+      <x:c r="F72" s="19" t="str">
+        <x:v>地形/首波敌方站位</x:v>
+      </x:c>
+      <x:c r="G72" s="19" t="str">
+        <x:v>三关选关详情</x:v>
+      </x:c>
+      <x:c r="H72" s="19" t="str">
+        <x:v>地形/首波敌方站位</x:v>
+      </x:c>
+      <x:c r="I72" s="19" t="str">
+        <x:v>复用／待制作。复用地形与敌方棋子缩略像；程序生成，不手绘三张易失真的战局图；不泄露第二波。 来源：US020 R08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="98" customHeight="1">
+      <x:c r="A73" s="16" t="str">
+        <x:v>A-140</x:v>
+      </x:c>
+      <x:c r="B73" s="16" t="str">
+        <x:v>第0关演武场入口卡</x:v>
+      </x:c>
+      <x:c r="C73" s="16" t="str">
+        <x:v>新旅程教学入口</x:v>
+      </x:c>
+      <x:c r="D73" s="16" t="str">
+        <x:v>双端自适应</x:v>
+      </x:c>
+      <x:c r="E73" s="16" t="str">
+        <x:v>复用通用面板/按钮</x:v>
+      </x:c>
+      <x:c r="F73" s="16" t="str">
+        <x:v>首次必修/曾完成可跳过</x:v>
+      </x:c>
+      <x:c r="G73" s="16" t="str">
+        <x:v>新旅程教学入口</x:v>
+      </x:c>
+      <x:c r="H73" s="16" t="str">
+        <x:v>首次必修/曾完成可跳过</x:v>
+      </x:c>
+      <x:c r="I73" s="16" t="str">
+        <x:v>待制作。首次必须完成；曾完成才可跳过；完成/合法跳过先入营地，覆盖US016旧首次可跳过方案。 来源：US020 R01；US016内容</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="98" customHeight="1">
+      <x:c r="A74" s="19" t="str">
+        <x:v>A-141</x:v>
+      </x:c>
+      <x:c r="B74" s="19" t="str">
+        <x:v>教学步骤卡与进度</x:v>
+      </x:c>
+      <x:c r="C74" s="19" t="str">
+        <x:v>教学战斗提示区</x:v>
+      </x:c>
+      <x:c r="D74" s="19" t="str">
+        <x:v>双端自适应；手机留棋盘空间</x:v>
+      </x:c>
+      <x:c r="E74" s="19" t="str">
+        <x:v>面板＋实时文字</x:v>
+      </x:c>
+      <x:c r="F74" s="19" t="str">
+        <x:v>7步/当前/完成</x:v>
+      </x:c>
+      <x:c r="G74" s="19" t="str">
+        <x:v>教学战斗提示区</x:v>
+      </x:c>
+      <x:c r="H74" s="19" t="str">
+        <x:v>7步/当前/完成</x:v>
+      </x:c>
+      <x:c r="I74" s="19" t="str">
+        <x:v>待制作。进度由操作事件驱动；不把步骤文字烘焙到图内。 来源：US020；US016教学内容</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="98" customHeight="1">
+      <x:c r="A75" s="16" t="str">
+        <x:v>A-142</x:v>
+      </x:c>
+      <x:c r="B75" s="16" t="str">
+        <x:v>教学聚焦框与指向箭头</x:v>
+      </x:c>
+      <x:c r="C75" s="16" t="str">
+        <x:v>教学指定操作目标</x:v>
+      </x:c>
+      <x:c r="D75" s="16" t="str">
+        <x:v>矢量自适应</x:v>
+      </x:c>
+      <x:c r="E75" s="16" t="str">
+        <x:v>SVG/CSS</x:v>
+      </x:c>
+      <x:c r="F75" s="16" t="str">
+        <x:v>棋子/格子/按钮高亮</x:v>
+      </x:c>
+      <x:c r="G75" s="16" t="str">
+        <x:v>教学指定操作目标</x:v>
+      </x:c>
+      <x:c r="H75" s="16" t="str">
+        <x:v>棋子/格子/按钮高亮</x:v>
+      </x:c>
+      <x:c r="I75" s="16" t="str">
+        <x:v>待制作。复用A-066～071/118；描边和文字共同提示，避免只靠颜色。 来源：US016；US020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="98" customHeight="1">
+      <x:c r="A76" s="19" t="str">
+        <x:v>A-143</x:v>
+      </x:c>
+      <x:c r="B76" s="19" t="str">
+        <x:v>教学完成与失败反馈</x:v>
+      </x:c>
+      <x:c r="C76" s="19" t="str">
+        <x:v>教学结果层</x:v>
+      </x:c>
+      <x:c r="D76" s="19" t="str">
+        <x:v>自适应；装饰尺寸TBD</x:v>
+      </x:c>
+      <x:c r="E76" s="19" t="str">
+        <x:v>通用弹窗＋标题装饰</x:v>
+      </x:c>
+      <x:c r="F76" s="19" t="str">
+        <x:v>完成/重试/入营</x:v>
+      </x:c>
+      <x:c r="G76" s="19" t="str">
+        <x:v>教学结果层</x:v>
+      </x:c>
+      <x:c r="H76" s="19" t="str">
+        <x:v>完成/重试/入营</x:v>
+      </x:c>
+      <x:c r="I76" s="19" t="str">
+        <x:v>待制作。完成所得猫粮保留，教学技能/伤亡清空；失败只重试；复用A-127标题装饰。 来源：US020 R01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="98" customHeight="1">
+      <x:c r="A77" s="16" t="str">
+        <x:v>A-144</x:v>
+      </x:c>
+      <x:c r="B77" s="16" t="str">
+        <x:v>合法跳过教学确认弹窗</x:v>
+      </x:c>
+      <x:c r="C77" s="16" t="str">
+        <x:v>曾完成教学的新旅程</x:v>
+      </x:c>
+      <x:c r="D77" s="16" t="str">
+        <x:v>双端自适应</x:v>
+      </x:c>
+      <x:c r="E77" s="16" t="str">
+        <x:v>通用弹窗＋实时文字</x:v>
+      </x:c>
+      <x:c r="F77" s="16" t="str">
+        <x:v>返回学习/确认跳过</x:v>
+      </x:c>
+      <x:c r="G77" s="16" t="str">
+        <x:v>曾完成教学的新旅程</x:v>
+      </x:c>
+      <x:c r="H77" s="16" t="str">
+        <x:v>返回学习/确认跳过</x:v>
+      </x:c>
+      <x:c r="I77" s="16" t="str">
+        <x:v>复用／待制作。二次确认，仅曾完成者可用；跳过不给教学收益；复用A-109/110/114。 来源：US020 R01；US016</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="98" customHeight="1">
+      <x:c r="A78" s="19" t="str">
+        <x:v>A-145</x:v>
+      </x:c>
+      <x:c r="B78" s="19" t="str">
+        <x:v>演武场独立地图地区</x:v>
+      </x:c>
+      <x:c r="C78" s="19" t="str">
+        <x:v>初始地图独立教学地区</x:v>
+      </x:c>
+      <x:c r="D78" s="19" t="str">
+        <x:v>地图矢量区域；旗帜尺寸TBD</x:v>
+      </x:c>
+      <x:c r="E78" s="19" t="str">
+        <x:v>SVG区域/透明旗帜</x:v>
+      </x:c>
+      <x:c r="F78" s="19" t="str">
+        <x:v>区域/旗帜/选中描边</x:v>
+      </x:c>
+      <x:c r="G78" s="19" t="str">
+        <x:v>初始地图独立教学地区</x:v>
+      </x:c>
+      <x:c r="H78" s="19" t="str">
+        <x:v>区域/旗帜/选中描边</x:v>
+      </x:c>
+      <x:c r="I78" s="19" t="str">
+        <x:v>WIP／仅预留。第0关教学已接入不代表独立地图地区已实现；位置、入口关系和最终布局TBD。 来源：US016（US020未覆盖的草案）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="98" customHeight="1">
+      <x:c r="A79" s="16" t="str">
+        <x:v>A-146</x:v>
+      </x:c>
+      <x:c r="B79" s="16" t="str">
+        <x:v>演武场地图状态徽记</x:v>
+      </x:c>
+      <x:c r="C79" s="16" t="str">
+        <x:v>教学地图地区</x:v>
+      </x:c>
+      <x:c r="D79" s="16" t="str">
+        <x:v>96×96建议</x:v>
+      </x:c>
+      <x:c r="E79" s="16" t="str">
+        <x:v>SVG＋文字</x:v>
+      </x:c>
+      <x:c r="F79" s="16" t="str">
+        <x:v>待学习/已完成/已跳过</x:v>
+      </x:c>
+      <x:c r="G79" s="16" t="str">
+        <x:v>教学地图地区</x:v>
+      </x:c>
+      <x:c r="H79" s="16" t="str">
+        <x:v>待学习/已完成/已跳过</x:v>
+      </x:c>
+      <x:c r="I79" s="16" t="str">
+        <x:v>WIP／仅预留。必须遵循首次必修的新规则；是否展示已跳过及重学去向TBD。 来源：US016</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="98" customHeight="1">
+      <x:c r="A80" s="19" t="str">
+        <x:v>A-147</x:v>
+      </x:c>
+      <x:c r="B80" s="19" t="str">
+        <x:v>正式流程首次规则提示</x:v>
+      </x:c>
+      <x:c r="C80" s="19" t="str">
+        <x:v>首次遇到相关玩法</x:v>
+      </x:c>
+      <x:c r="D80" s="19" t="str">
+        <x:v>自适应</x:v>
+      </x:c>
+      <x:c r="E80" s="19" t="str">
+        <x:v>通用提示卡/图标复用</x:v>
+      </x:c>
+      <x:c r="F80" s="19" t="str">
+        <x:v>部署/地形/弓炮/SP/友伤等</x:v>
+      </x:c>
+      <x:c r="G80" s="19" t="str">
+        <x:v>首次遇到相关玩法</x:v>
+      </x:c>
+      <x:c r="H80" s="19" t="str">
+        <x:v>部署/地形/弓炮/SP/友伤等</x:v>
+      </x:c>
+      <x:c r="I80" s="19" t="str">
+        <x:v>WIP／仅预留。仅预留通用提示皮肤与小图；精确触发、频率、帮助入口TBD，复用现有图标。 来源：US016 §4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="98" customHeight="1">
+      <x:c r="A81" s="16" t="str">
+        <x:v>A-148</x:v>
+      </x:c>
+      <x:c r="B81" s="16" t="str">
+        <x:v>仕｜被毁残骸</x:v>
+      </x:c>
+      <x:c r="C81" s="16" t="str">
+        <x:v>仕阵亡占格</x:v>
+      </x:c>
+      <x:c r="D81" s="16" t="str">
+        <x:v>随棋子比例；具体像素TBD</x:v>
+      </x:c>
+      <x:c r="E81" s="16" t="str">
+        <x:v>透明PNG/WebP</x:v>
+      </x:c>
+      <x:c r="F81" s="16" t="str">
+        <x:v>1套，双侧共用</x:v>
+      </x:c>
+      <x:c r="G81" s="16" t="str">
+        <x:v>仕阵亡占格</x:v>
+      </x:c>
+      <x:c r="H81" s="16" t="str">
+        <x:v>1套，双侧共用</x:v>
+      </x:c>
+      <x:c r="I81" s="16" t="str">
+        <x:v>待制作。活塔不能移动，残骸可推动、作炮架、入水销毁；不能被关内救援。 来源：US018 §6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="98" customHeight="1">
+      <x:c r="A82" s="19" t="str">
+        <x:v>A-149</x:v>
+      </x:c>
+      <x:c r="B82" s="19" t="str">
+        <x:v>仕｜自动射击弹道与命中</x:v>
+      </x:c>
+      <x:c r="C82" s="19" t="str">
+        <x:v>结束回合后敌攻前</x:v>
+      </x:c>
+      <x:c r="D82" s="19" t="str">
+        <x:v>随棋盘缩放；时长TBD</x:v>
+      </x:c>
+      <x:c r="E82" s="19" t="str">
+        <x:v>透明序列/代码弹道</x:v>
+      </x:c>
+      <x:c r="F82" s="19" t="str">
+        <x:v>发射/命中/闪避</x:v>
+      </x:c>
+      <x:c r="G82" s="19" t="str">
+        <x:v>结束回合后敌攻前</x:v>
+      </x:c>
+      <x:c r="H82" s="19" t="str">
+        <x:v>发射/命中/闪避</x:v>
+      </x:c>
+      <x:c r="I82" s="19" t="str">
+        <x:v>待制作。八邻格选1敌人，双塔可同目标；动画顺序不改变同时锁定规则；复用A-117/024。 来源：US018 §3～4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="98" customHeight="1">
+      <x:c r="A83" s="16" t="str">
+        <x:v>A-150</x:v>
+      </x:c>
+      <x:c r="B83" s="16" t="str">
+        <x:v>仕｜就绪与冷却标识</x:v>
+      </x:c>
+      <x:c r="C83" s="16" t="str">
+        <x:v>仕详情、棋盘、名单</x:v>
+      </x:c>
+      <x:c r="D83" s="16" t="str">
+        <x:v>状态图标96×96建议</x:v>
+      </x:c>
+      <x:c r="E83" s="16" t="str">
+        <x:v>SVG＋实时数字</x:v>
+      </x:c>
+      <x:c r="F83" s="16" t="str">
+        <x:v>就绪有目标/就绪无目标/冷却</x:v>
+      </x:c>
+      <x:c r="G83" s="16" t="str">
+        <x:v>仕详情、棋盘、名单</x:v>
+      </x:c>
+      <x:c r="H83" s="16" t="str">
+        <x:v>就绪有目标/就绪无目标/冷却</x:v>
+      </x:c>
+      <x:c r="I83" s="16" t="str">
+        <x:v>待制作。间隔3→2→1；剩余回合实时文字；0不表示点击即开火。 来源：US018 §5/7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="98" customHeight="1">
+      <x:c r="A84" s="19" t="str">
+        <x:v>A-151</x:v>
+      </x:c>
+      <x:c r="B84" s="19" t="str">
+        <x:v>仕｜自动目标预览连线</x:v>
+      </x:c>
+      <x:c r="C84" s="19" t="str">
+        <x:v>当前局面的回合末预测</x:v>
+      </x:c>
+      <x:c r="D84" s="19" t="str">
+        <x:v>矢量随棋盘缩放</x:v>
+      </x:c>
+      <x:c r="E84" s="19" t="str">
+        <x:v>SVG/CSS连线</x:v>
+      </x:c>
+      <x:c r="F84" s="19" t="str">
+        <x:v>候选目标/条件命中</x:v>
+      </x:c>
+      <x:c r="G84" s="19" t="str">
+        <x:v>当前局面的回合末预测</x:v>
+      </x:c>
+      <x:c r="H84" s="19" t="str">
+        <x:v>候选目标/条件命中</x:v>
+      </x:c>
+      <x:c r="I84" s="19" t="str">
+        <x:v>待制作。与敌方锁定意图区分；玩家行动后可更新，树林结果为条件预览。 来源：US018 §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="98" customHeight="1">
+      <x:c r="A85" s="16" t="str">
+        <x:v>A-152</x:v>
+      </x:c>
+      <x:c r="B85" s="16" t="str">
+        <x:v>仕｜左右固定侧位与占用标记</x:v>
+      </x:c>
+      <x:c r="C85" s="16" t="str">
+        <x:v>仕布阵</x:v>
+      </x:c>
+      <x:c r="D85" s="16" t="str">
+        <x:v>随棋位缩放</x:v>
+      </x:c>
+      <x:c r="E85" s="16" t="str">
+        <x:v>SVG/棋位标记</x:v>
+      </x:c>
+      <x:c r="F85" s="16" t="str">
+        <x:v>左/右/空置/占用/冲突</x:v>
+      </x:c>
+      <x:c r="G85" s="16" t="str">
+        <x:v>仕布阵</x:v>
+      </x:c>
+      <x:c r="H85" s="16" t="str">
+        <x:v>左/右/空置/占用/冲突</x:v>
+      </x:c>
+      <x:c r="I85" s="16" t="str">
+        <x:v>待制作。(4,2)/(6,2)；最多2座，不占部署人口且无装置后备；复用A-124。 来源：US018；US020 R04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="98" customHeight="1">
+      <x:c r="A86" s="19" t="str">
+        <x:v>A-153</x:v>
+      </x:c>
+      <x:c r="B86" s="19" t="str">
+        <x:v>仕｜间隔升级图标与档位</x:v>
+      </x:c>
+      <x:c r="C86" s="19" t="str">
+        <x:v>营地/布阵/战斗技能栏</x:v>
+      </x:c>
+      <x:c r="D86" s="19" t="str">
+        <x:v>96×96建议</x:v>
+      </x:c>
+      <x:c r="E86" s="19" t="str">
+        <x:v>SVG＋动态档位</x:v>
+      </x:c>
+      <x:c r="F86" s="19" t="str">
+        <x:v>3回合/2回合/1回合</x:v>
+      </x:c>
+      <x:c r="G86" s="19" t="str">
+        <x:v>营地/布阵/战斗技能栏</x:v>
+      </x:c>
+      <x:c r="H86" s="19" t="str">
+        <x:v>3回合/2回合/1回合</x:v>
+      </x:c>
+      <x:c r="I86" s="19" t="str">
+        <x:v>待制作。两座独立升级、共享SP，3/5SP；只升间隔，不暗示伤害或射程升级。 来源：US018 §5；US020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="98" customHeight="1">
+      <x:c r="A87" s="16" t="str">
+        <x:v>A-154</x:v>
+      </x:c>
+      <x:c r="B87" s="16" t="str">
+        <x:v>马｜起跳、越障与落地</x:v>
+      </x:c>
+      <x:c r="C87" s="16" t="str">
+        <x:v>主动跳跃攻击</x:v>
+      </x:c>
+      <x:c r="D87" s="16" t="str">
+        <x:v>随棋子比例；时长TBD</x:v>
+      </x:c>
+      <x:c r="E87" s="16" t="str">
+        <x:v>代码位移＋透明特效</x:v>
+      </x:c>
+      <x:c r="F87" s="16" t="str">
+        <x:v>起跳/空中/落地</x:v>
+      </x:c>
+      <x:c r="G87" s="16" t="str">
+        <x:v>主动跳跃攻击</x:v>
+      </x:c>
+      <x:c r="H87" s="16" t="str">
+        <x:v>起跳/空中/落地</x:v>
+      </x:c>
+      <x:c r="I87" s="16" t="str">
+        <x:v>待制作。上下左右空格落点，基础2格、最高4格；不能把普通日字移动做成落地攻击。 来源：US021 §3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="98" customHeight="1">
+      <x:c r="A88" s="19" t="str">
+        <x:v>A-155</x:v>
+      </x:c>
+      <x:c r="B88" s="19" t="str">
+        <x:v>马｜落点四邻冲击与友伤</x:v>
+      </x:c>
+      <x:c r="C88" s="19" t="str">
+        <x:v>跳跃落地结算</x:v>
+      </x:c>
+      <x:c r="D88" s="19" t="str">
+        <x:v>随棋盘缩放</x:v>
+      </x:c>
+      <x:c r="E88" s="19" t="str">
+        <x:v>透明冲击效果＋代码裁切</x:v>
+      </x:c>
+      <x:c r="F88" s="19" t="str">
+        <x:v>1～3伤害档/边缘裁切</x:v>
+      </x:c>
+      <x:c r="G88" s="19" t="str">
+        <x:v>跳跃落地结算</x:v>
+      </x:c>
+      <x:c r="H88" s="19" t="str">
+        <x:v>1～3伤害档/边缘裁切</x:v>
+      </x:c>
+      <x:c r="I88" s="19" t="str">
+        <x:v>待制作。只作用上下左右四邻；包含友军和山，非斜邻群伤；复用伤害数字、山体受击和树林闪避。 来源：US021 §3/5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="98" customHeight="1">
+      <x:c r="A89" s="16" t="str">
+        <x:v>A-156</x:v>
+      </x:c>
+      <x:c r="B89" s="16" t="str">
+        <x:v>马｜推动与碰撞反馈</x:v>
+      </x:c>
+      <x:c r="C89" s="16" t="str">
+        <x:v>解锁推动后的跳跃落地</x:v>
+      </x:c>
+      <x:c r="D89" s="16" t="str">
+        <x:v>矢量/方向由代码旋转</x:v>
+      </x:c>
+      <x:c r="E89" s="16" t="str">
+        <x:v>复用箭头＋位移动画</x:v>
+      </x:c>
+      <x:c r="F89" s="16" t="str">
+        <x:v>向外推/受阻/入水/尸体推动</x:v>
+      </x:c>
+      <x:c r="G89" s="16" t="str">
+        <x:v>解锁推动后的跳跃落地</x:v>
+      </x:c>
+      <x:c r="H89" s="16" t="str">
+        <x:v>向外推/受阻/入水/尸体推动</x:v>
+      </x:c>
+      <x:c r="I89" s="16" t="str">
+        <x:v>待制作。先四邻伤害再推动存活者与尸体；复用A-018/118及碰撞反馈，不另画四方向套图。 来源：US021 §5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="98" customHeight="1">
+      <x:c r="A90" s="19" t="str">
+        <x:v>A-157</x:v>
+      </x:c>
+      <x:c r="B90" s="19" t="str">
+        <x:v>马｜跳跃落点与四邻预览</x:v>
+      </x:c>
+      <x:c r="C90" s="19" t="str">
+        <x:v>马技能预览</x:v>
+      </x:c>
+      <x:c r="D90" s="19" t="str">
+        <x:v>随棋盘缩放</x:v>
+      </x:c>
+      <x:c r="E90" s="19" t="str">
+        <x:v>SVG/CSS格标</x:v>
+      </x:c>
+      <x:c r="F90" s="19" t="str">
+        <x:v>合法落点/选中落点/伤害/推动/友伤</x:v>
+      </x:c>
+      <x:c r="G90" s="19" t="str">
+        <x:v>马技能预览</x:v>
+      </x:c>
+      <x:c r="H90" s="19" t="str">
+        <x:v>合法落点/选中落点/伤害/推动/友伤</x:v>
+      </x:c>
+      <x:c r="I90" s="19" t="str">
+        <x:v>待制作。落点必须为空，落点不受伤；中心与四邻不同标记，明确友伤，边缘裁切。 来源：US021 H20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="98" customHeight="1">
+      <x:c r="A91" s="16" t="str">
+        <x:v>A-158</x:v>
+      </x:c>
+      <x:c r="B91" s="16" t="str">
+        <x:v>马｜三项独立升级图标</x:v>
+      </x:c>
+      <x:c r="C91" s="16" t="str">
+        <x:v>营地、布阵和战斗技能区</x:v>
+      </x:c>
+      <x:c r="D91" s="16" t="str">
+        <x:v>96×96建议</x:v>
+      </x:c>
+      <x:c r="E91" s="16" t="str">
+        <x:v>SVG图标</x:v>
+      </x:c>
+      <x:c r="F91" s="16" t="str">
+        <x:v>推动解除马腿/距离/伤害3款</x:v>
+      </x:c>
+      <x:c r="G91" s="16" t="str">
+        <x:v>营地、布阵和战斗技能区</x:v>
+      </x:c>
+      <x:c r="H91" s="16" t="str">
+        <x:v>推动解除马腿/距离/伤害3款</x:v>
+      </x:c>
+      <x:c r="I91" s="16" t="str">
+        <x:v>待制作。推动2SP一次；距离1SP/级至4格；伤害2SP/级至3；三项无相互前置，价格实时文字。 来源：US021 §4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="98" customHeight="1">
+      <x:c r="A92" s="19" t="str">
+        <x:v>A-159</x:v>
+      </x:c>
+      <x:c r="B92" s="19" t="str">
+        <x:v>马｜双模式与独立行动额度</x:v>
+      </x:c>
+      <x:c r="C92" s="19" t="str">
+        <x:v>马操作区、详情与名单</x:v>
+      </x:c>
+      <x:c r="D92" s="19" t="str">
+        <x:v>双端自适应；热区44逻辑像素建议</x:v>
+      </x:c>
+      <x:c r="E92" s="19" t="str">
+        <x:v>通用按钮＋SVG状态</x:v>
+      </x:c>
+      <x:c r="F92" s="19" t="str">
+        <x:v>普通移动/跳跃攻击；可用/耗尽</x:v>
+      </x:c>
+      <x:c r="G92" s="19" t="str">
+        <x:v>马操作区、详情与名单</x:v>
+      </x:c>
+      <x:c r="H92" s="19" t="str">
+        <x:v>普通移动/跳跃攻击；可用/耗尽</x:v>
+      </x:c>
+      <x:c r="I92" s="19" t="str">
+        <x:v>待制作。可移动后跳跃；跳跃后不能再移动。无旧普通攻击入口，升级不恢复行动；复用A-077。 来源：US021 §2/6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="98" customHeight="1">
+      <x:c r="A93" s="16" t="str">
+        <x:v>A-160</x:v>
+      </x:c>
+      <x:c r="B93" s="16" t="str">
+        <x:v>猫粮货币图标</x:v>
+      </x:c>
+      <x:c r="C93" s="16" t="str">
+        <x:v>营地、战斗、结算、教学</x:v>
+      </x:c>
+      <x:c r="D93" s="16" t="str">
+        <x:v>96×96建议</x:v>
+      </x:c>
+      <x:c r="E93" s="16" t="str">
+        <x:v>SVG/透明PNG</x:v>
+      </x:c>
+      <x:c r="F93" s="16" t="str">
+        <x:v>普通/收入/支出/不足</x:v>
+      </x:c>
+      <x:c r="G93" s="16" t="str">
+        <x:v>营地、战斗、结算、教学</x:v>
+      </x:c>
+      <x:c r="H93" s="16" t="str">
+        <x:v>普通/收入/支出/不足</x:v>
+      </x:c>
+      <x:c r="I93" s="16" t="str">
+        <x:v>待制作。替换金币图标，仍单钱包；数值与价格代码生成，不新增第二货币。 来源：US020 R03</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="98" customHeight="1">
+      <x:c r="A94" s="19" t="str">
+        <x:v>A-161</x:v>
+      </x:c>
+      <x:c r="B94" s="19" t="str">
+        <x:v>公共SP获得与消费反馈</x:v>
+      </x:c>
+      <x:c r="C94" s="19" t="str">
+        <x:v>击杀、营地及战斗升级</x:v>
+      </x:c>
+      <x:c r="D94" s="19" t="str">
+        <x:v>图标96×96建议；动效TBD</x:v>
+      </x:c>
+      <x:c r="E94" s="19" t="str">
+        <x:v>SVG＋代码动画</x:v>
+      </x:c>
+      <x:c r="F94" s="19" t="str">
+        <x:v>获得/消费/不足/满级</x:v>
+      </x:c>
+      <x:c r="G94" s="19" t="str">
+        <x:v>击杀、营地及战斗升级</x:v>
+      </x:c>
+      <x:c r="H94" s="19" t="str">
+        <x:v>获得/消费/不足/满级</x:v>
+      </x:c>
+      <x:c r="I94" s="19" t="str">
+        <x:v>待制作。指向唯一公共SP栏；个人等级/击杀仍独立，复用A-112和A-042。 来源：US017；US020；US021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="98" customHeight="1">
+      <x:c r="A95" s="16" t="str">
+        <x:v>A-162</x:v>
+      </x:c>
+      <x:c r="B95" s="16" t="str">
+        <x:v>救援｜治疗与原位复活</x:v>
+      </x:c>
+      <x:c r="C95" s="16" t="str">
+        <x:v>第二波开始前救援</x:v>
+      </x:c>
+      <x:c r="D95" s="16" t="str">
+        <x:v>随棋子比例；时长TBD</x:v>
+      </x:c>
+      <x:c r="E95" s="16" t="str">
+        <x:v>透明特效/代码动画</x:v>
+      </x:c>
+      <x:c r="F95" s="16" t="str">
+        <x:v>伤员回满/尸体1HP复活</x:v>
+      </x:c>
+      <x:c r="G95" s="16" t="str">
+        <x:v>第二波开始前救援</x:v>
+      </x:c>
+      <x:c r="H95" s="16" t="str">
+        <x:v>伤员回满/尸体1HP复活</x:v>
+      </x:c>
+      <x:c r="I95" s="16" t="str">
+        <x:v>待制作。区别治疗和复活；复用A-125卡片，主帅/仕不适用，不表现异地传送。 来源：US020 R06</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6255,7 +8061,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5846739d9be04a9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R901c00f123764e7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6280,9 +8086,9 @@
         <x:v>三关地图美术分区</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="25" customHeight="1">
+    <x:row r="2" ht="35" customHeight="1">
       <x:c r="A2" s="13" t="str">
-        <x:v>三关是新的美术预留，不等同于战斗内的两波敌军。示意图只表达西→中→东南的关卡构图，不是战国七国疆界复原。三关敌阵、解锁方式、具体疆界与年代均 TBD。</x:v>
+        <x:v>正式三关已按1→2→3顺序接入；全部可预览地形/首波，只有下一关可挑战。演武场独立地图地区仍为US016 WIP，不算第4个正式关卡。历史疆界和最终构图TBD。</x:v>
       </x:c>
       <x:c r="B2" s="13"/>
       <x:c r="C2" s="13"/>
@@ -6293,7 +8099,7 @@
       <x:c r="H2" s="13"/>
       <x:c r="I2" s="13"/>
     </x:row>
-    <x:row r="3" ht="25" customHeight="1">
+    <x:row r="3" ht="35" customHeight="1">
       <x:c r="A3" s="13"/>
       <x:c r="B3" s="13"/>
       <x:c r="C3" s="13"/>
@@ -6353,10 +8159,10 @@
         <x:v>区域高亮、节点、山隘插画</x:v>
       </x:c>
       <x:c r="G6" s="19" t="str">
-        <x:v>未解锁/可挑战/选中/通关</x:v>
+        <x:v>未解锁/可挑战/选中/通关；均可查看</x:v>
       </x:c>
       <x:c r="H6" s="19" t="str">
-        <x:v>TBD，美术样稿未接入战斗</x:v>
+        <x:v>US020 R08：预览读有效地图与首波站位；未解锁及通关关卡不可进入</x:v>
       </x:c>
       <x:c r="I6" s="19" t="str">
         <x:v>地理题材参考；关卡边界为设计草案。https://commons.wikimedia.org/wiki/File:ZH-战国七雄地图.jpg</x:v>
@@ -6382,10 +8188,10 @@
         <x:v>区域高亮、节点、城邑插画</x:v>
       </x:c>
       <x:c r="G7" s="16" t="str">
-        <x:v>未解锁/可挑战/选中/通关</x:v>
+        <x:v>未解锁/可挑战/选中/通关；均可查看</x:v>
       </x:c>
       <x:c r="H7" s="16" t="str">
-        <x:v>TBD，美术样稿未接入战斗</x:v>
+        <x:v>US020 R08：预览读有效地图与首波站位；未解锁及通关关卡不可进入</x:v>
       </x:c>
       <x:c r="I7" s="16" t="str">
         <x:v>国别归属、地图年代不作精确标注。https://commons.wikimedia.org/wiki/File:ZH-战国七雄地图.jpg</x:v>
@@ -6411,10 +8217,10 @@
         <x:v>区域高亮、节点、水泽插画</x:v>
       </x:c>
       <x:c r="G8" s="19" t="str">
-        <x:v>未解锁/可挑战/选中/通关</x:v>
+        <x:v>未解锁/可挑战/选中/通关；均可查看</x:v>
       </x:c>
       <x:c r="H8" s="19" t="str">
-        <x:v>TBD，美术样稿未接入战斗</x:v>
+        <x:v>US020 R08：预览读有效地图与首波站位；未解锁及通关关卡不可进入</x:v>
       </x:c>
       <x:c r="I8" s="19" t="str">
         <x:v>战国题材局部地图，非现代全国行政图。https://commons.wikimedia.org/wiki/File:ZH-战国七雄地图.jpg</x:v>
@@ -6426,7 +8232,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a7e71c6ab774eb1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52a2eb3fa5bb478a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>